<commit_message>
Informe de Lululemon (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$17</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -313,20 +313,20 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Lululemon</t>
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C2" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
@@ -341,41 +341,41 @@
       </c>
       <c r="G2" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I2" s="2">
-        <v>26.48</v>
+        <v>93.61</v>
       </c>
       <c r="J2" s="2">
-        <v>27.68</v>
+        <v>132.71</v>
       </c>
       <c r="K2" s="2">
-        <v>36.62</v>
+        <v>146.21</v>
       </c>
       <c r="L2" s="3">
-        <v>0.045</v>
+        <v>0.418</v>
       </c>
       <c r="M2" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.562</v>
       </c>
       <c r="N2" s="2">
-        <v>36.11</v>
+        <v>104.91</v>
       </c>
       <c r="O2" s="2">
-        <v>30.75</v>
+        <v>127.14</v>
       </c>
       <c r="P2" s="2">
-        <v>40.69</v>
+        <v>162.3</v>
       </c>
       <c r="Q2" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R2" s="13" t="inlineStr">
@@ -398,9 +398,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V2" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V2" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W2" s="4" t="inlineStr">
@@ -423,26 +423,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA2" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB2" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="C3" s="10">
@@ -450,12 +450,12 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -470,32 +470,32 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="I3" s="2">
-        <v>78.3</v>
+        <v>26.48</v>
       </c>
       <c r="J3" s="2">
-        <v>84.06</v>
+        <v>27.68</v>
       </c>
       <c r="K3" s="2">
-        <v>97.98</v>
+        <v>36.62</v>
       </c>
       <c r="L3" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="M3" s="3">
-        <v>0.271</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="N3" s="2">
-        <v>69.22</v>
+        <v>36.11</v>
       </c>
       <c r="O3" s="2">
-        <v>86.5</v>
+        <v>30.75</v>
       </c>
       <c r="P3" s="2">
-        <v>110.62</v>
+        <v>40.69</v>
       </c>
       <c r="Q3" s="13" t="inlineStr">
         <is>
@@ -522,19 +522,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X3" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W3" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y3" s="4" t="inlineStr">
@@ -547,26 +547,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA3" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB3" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C4" s="10">
@@ -579,7 +579,7 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -598,28 +598,28 @@
         </is>
       </c>
       <c r="I4" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J4" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K4" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L4" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M4" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N4" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O4" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P4" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
@@ -631,9 +631,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T4" s="4" t="inlineStr">
@@ -646,19 +646,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -671,30 +671,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C5" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
@@ -703,56 +703,56 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+          <t>Consumo básico</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I5" s="2">
+        <v>52.9</v>
+      </c>
+      <c r="J5" s="2">
+        <v>55.98</v>
+      </c>
+      <c r="K5" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0.244</v>
+      </c>
+      <c r="N5" s="2">
+        <v>69.29</v>
+      </c>
+      <c r="O5" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="P5" s="2">
+        <v>65.83</v>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I5" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J5" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K5" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L5" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M5" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N5" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O5" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P5" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R5" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
@@ -760,9 +760,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
@@ -770,9 +770,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W5" s="6" t="inlineStr">
@@ -780,14 +780,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
@@ -802,23 +802,23 @@
       </c>
       <c r="AB5" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C6" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="I6" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="J6" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="K6" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="L6" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M6" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="N6" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="O6" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="P6" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
@@ -879,14 +879,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -919,34 +919,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB6" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C7" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -966,32 +966,32 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I7" s="2">
-        <v>26.82</v>
+        <v>59.72</v>
       </c>
       <c r="J7" s="2">
-        <v>25.71</v>
+        <v>58.59</v>
       </c>
       <c r="K7" s="2">
-        <v>27.88</v>
+        <v>66.22</v>
       </c>
       <c r="L7" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M7" s="3">
-        <v>0.04</v>
+        <v>0.114</v>
       </c>
       <c r="N7" s="2">
-        <v>39</v>
+        <v>67.12</v>
       </c>
       <c r="O7" s="2">
-        <v>24.22</v>
+        <v>57.83</v>
       </c>
       <c r="P7" s="2">
-        <v>30.98</v>
+        <v>73.94</v>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
@@ -1018,24 +1018,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1043,26 +1043,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB7" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C8" s="10">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -1090,36 +1090,36 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I8" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="J8" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="K8" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="L8" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M8" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="N8" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="O8" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="P8" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R8" s="13" t="inlineStr">
@@ -1127,9 +1127,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T8" s="4" t="inlineStr">
@@ -1142,29 +1142,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA8" s="4" t="inlineStr">
@@ -1174,19 +1174,19 @@
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C9" s="10">
@@ -1194,12 +1194,12 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1218,28 +1218,28 @@
         </is>
       </c>
       <c r="I9" s="2">
-        <v>16.22</v>
+        <v>577.5</v>
       </c>
       <c r="J9" s="2">
-        <v>13.97</v>
+        <v>466.62</v>
       </c>
       <c r="K9" s="2">
-        <v>14.66</v>
+        <v>564.55</v>
       </c>
       <c r="L9" s="3">
-        <v>-0.077</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M9" s="3">
-        <v>-0.035</v>
+        <v>0.005</v>
       </c>
       <c r="N9" s="2">
-        <v>17.05</v>
+        <v>795.86</v>
       </c>
       <c r="O9" s="2">
-        <v>13.61</v>
+        <v>504.42</v>
       </c>
       <c r="P9" s="2">
-        <v>16.41</v>
+        <v>645.34</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
@@ -1251,34 +1251,34 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y9" s="5" t="inlineStr">
@@ -1286,31 +1286,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C10" s="10">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1338,32 +1338,32 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I10" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="J10" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="K10" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="L10" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="M10" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="N10" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="O10" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="P10" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
@@ -1375,19 +1375,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
@@ -1395,14 +1395,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y10" s="5" t="inlineStr">
@@ -1410,98 +1410,98 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C11" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I11" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J11" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K11" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L11" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M11" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N11" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O11" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P11" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I11" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J11" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K11" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L11" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M11" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N11" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O11" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P11" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T11" s="4" t="inlineStr">
@@ -1514,9 +1514,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W11" s="4" t="inlineStr">
@@ -1524,9 +1524,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y11" s="5" t="inlineStr">
@@ -1534,44 +1534,44 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -1586,32 +1586,32 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I12" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="J12" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="K12" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="L12" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="M12" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N12" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="O12" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="P12" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
@@ -1623,9 +1623,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S12" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="S12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr">
@@ -1638,9 +1638,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W12" s="4" t="inlineStr">
@@ -1648,9 +1648,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y12" s="5" t="inlineStr">
@@ -1663,26 +1663,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C13" s="10">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -1710,32 +1710,32 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I13" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="J13" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="K13" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="L13" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="M13" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="N13" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="O13" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="P13" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
@@ -1747,14 +1747,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S13" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
@@ -1762,9 +1762,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -1794,19 +1794,19 @@
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C14" s="10">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -1834,32 +1834,32 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I14" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="J14" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="K14" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="M14" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="N14" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="O14" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="P14" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -1871,14 +1871,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -1891,9 +1891,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X14" s="6" t="inlineStr">
@@ -1918,23 +1918,23 @@
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C15" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -1962,28 +1962,28 @@
         </is>
       </c>
       <c r="I15" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="J15" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="K15" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="M15" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N15" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="O15" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="P15" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -2010,14 +2010,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X15" s="6" t="inlineStr">
@@ -2042,19 +2042,19 @@
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,116 +2062,240 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I16" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J16" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K16" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L16" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M16" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N16" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O16" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P16" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R16" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB16" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="C17" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E16" s="0" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I16" s="2">
+      <c r="I17" s="2">
         <v>698.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J17" s="2">
         <v>272.01</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K17" s="2">
         <v>348.9</v>
       </c>
-      <c r="L16" s="3">
+      <c r="L17" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M16" s="3">
+      <c r="M17" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N17" s="2">
         <v>713.11</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O17" s="2">
         <v>282.35</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P17" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R16" s="13" t="inlineStr">
+      <c r="R17" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB16" s="11" t="inlineStr">
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB17" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB16"/>
+  <autoFilter ref="A1:AB17"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2188,6 +2312,7 @@
     <hyperlink ref="AB14" r:id="rId13"/>
     <hyperlink ref="AB15" r:id="rId14"/>
     <hyperlink ref="AB16" r:id="rId15"/>
+    <hyperlink ref="AB17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Edenred (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$18</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -313,12 +313,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>Lululemon</t>
+          <t>Edenred</t>
         </is>
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>EDEN</t>
         </is>
       </c>
       <c r="C2" s="10">
@@ -326,12 +326,12 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -346,32 +346,32 @@
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I2" s="2">
-        <v>93.61</v>
+        <v>27.61</v>
       </c>
       <c r="J2" s="2">
-        <v>132.71</v>
+        <v>42.22</v>
       </c>
       <c r="K2" s="2">
-        <v>146.21</v>
+        <v>54.1</v>
       </c>
       <c r="L2" s="3">
-        <v>0.418</v>
+        <v>0.5770000000000001</v>
       </c>
       <c r="M2" s="3">
-        <v>0.562</v>
+        <v>1.008</v>
       </c>
       <c r="N2" s="2">
-        <v>104.91</v>
+        <v>30.57</v>
       </c>
       <c r="O2" s="2">
-        <v>127.14</v>
+        <v>48.17</v>
       </c>
       <c r="P2" s="2">
-        <v>162.3</v>
+        <v>61.6</v>
       </c>
       <c r="Q2" s="13" t="inlineStr">
         <is>
@@ -393,9 +393,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V2" s="4" t="inlineStr">
@@ -403,14 +403,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y2" s="4" t="inlineStr">
@@ -430,27 +430,27 @@
       </c>
       <c r="AB2" s="11" t="inlineStr">
         <is>
-          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
+          <t>informes/edenred-2026-10-07/Edenred - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Lululemon</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C3" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
@@ -465,41 +465,41 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I3" s="2">
-        <v>26.48</v>
+        <v>93.61</v>
       </c>
       <c r="J3" s="2">
-        <v>27.68</v>
+        <v>132.71</v>
       </c>
       <c r="K3" s="2">
-        <v>36.62</v>
+        <v>146.21</v>
       </c>
       <c r="L3" s="3">
-        <v>0.045</v>
+        <v>0.418</v>
       </c>
       <c r="M3" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.562</v>
       </c>
       <c r="N3" s="2">
-        <v>36.11</v>
+        <v>104.91</v>
       </c>
       <c r="O3" s="2">
-        <v>30.75</v>
+        <v>127.14</v>
       </c>
       <c r="P3" s="2">
-        <v>40.69</v>
+        <v>162.3</v>
       </c>
       <c r="Q3" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R3" s="13" t="inlineStr">
@@ -522,9 +522,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V3" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W3" s="4" t="inlineStr">
@@ -547,26 +547,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA3" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB3" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="C4" s="10">
@@ -574,12 +574,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -594,32 +594,32 @@
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="I4" s="2">
-        <v>78.3</v>
+        <v>26.48</v>
       </c>
       <c r="J4" s="2">
-        <v>84.06</v>
+        <v>27.68</v>
       </c>
       <c r="K4" s="2">
-        <v>97.98</v>
+        <v>36.62</v>
       </c>
       <c r="L4" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="M4" s="3">
-        <v>0.271</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="N4" s="2">
-        <v>69.22</v>
+        <v>36.11</v>
       </c>
       <c r="O4" s="2">
-        <v>86.5</v>
+        <v>30.75</v>
       </c>
       <c r="P4" s="2">
-        <v>110.62</v>
+        <v>40.69</v>
       </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
@@ -646,19 +646,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -671,26 +671,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C5" s="10">
@@ -703,7 +703,7 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -722,28 +722,28 @@
         </is>
       </c>
       <c r="I5" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J5" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K5" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L5" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M5" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N5" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O5" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P5" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
@@ -755,9 +755,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
@@ -770,19 +770,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -795,30 +795,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB5" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C6" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
@@ -827,56 +827,56 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
+          <t>Consumo básico</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I6" s="2">
+        <v>52.9</v>
+      </c>
+      <c r="J6" s="2">
+        <v>55.98</v>
+      </c>
+      <c r="K6" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="M6" s="3">
+        <v>0.244</v>
+      </c>
+      <c r="N6" s="2">
+        <v>69.29</v>
+      </c>
+      <c r="O6" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="P6" s="2">
+        <v>65.83</v>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I6" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J6" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K6" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L6" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M6" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N6" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O6" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P6" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q6" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R6" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -884,9 +884,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -894,9 +894,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W6" s="6" t="inlineStr">
@@ -904,14 +904,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -926,23 +926,23 @@
       </c>
       <c r="AB6" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C7" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -970,28 +970,28 @@
         </is>
       </c>
       <c r="I7" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="J7" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="K7" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="L7" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M7" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="N7" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="O7" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="P7" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
@@ -1003,14 +1003,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
@@ -1043,34 +1043,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB7" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C8" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -1090,32 +1090,32 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I8" s="2">
-        <v>26.82</v>
+        <v>59.72</v>
       </c>
       <c r="J8" s="2">
-        <v>25.71</v>
+        <v>58.59</v>
       </c>
       <c r="K8" s="2">
-        <v>27.88</v>
+        <v>66.22</v>
       </c>
       <c r="L8" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M8" s="3">
-        <v>0.04</v>
+        <v>0.114</v>
       </c>
       <c r="N8" s="2">
-        <v>39</v>
+        <v>67.12</v>
       </c>
       <c r="O8" s="2">
-        <v>24.22</v>
+        <v>57.83</v>
       </c>
       <c r="P8" s="2">
-        <v>30.98</v>
+        <v>73.94</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
@@ -1142,24 +1142,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1167,26 +1167,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C9" s="10">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1214,36 +1214,36 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I9" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="J9" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="K9" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="L9" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M9" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="N9" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="O9" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="P9" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R9" s="13" t="inlineStr">
@@ -1251,9 +1251,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T9" s="4" t="inlineStr">
@@ -1266,29 +1266,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA9" s="4" t="inlineStr">
@@ -1298,19 +1298,19 @@
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C10" s="10">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -1342,28 +1342,28 @@
         </is>
       </c>
       <c r="I10" s="2">
-        <v>16.22</v>
+        <v>577.5</v>
       </c>
       <c r="J10" s="2">
-        <v>13.97</v>
+        <v>466.62</v>
       </c>
       <c r="K10" s="2">
-        <v>14.66</v>
+        <v>564.55</v>
       </c>
       <c r="L10" s="3">
-        <v>-0.077</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M10" s="3">
-        <v>-0.035</v>
+        <v>0.005</v>
       </c>
       <c r="N10" s="2">
-        <v>17.05</v>
+        <v>795.86</v>
       </c>
       <c r="O10" s="2">
-        <v>13.61</v>
+        <v>504.42</v>
       </c>
       <c r="P10" s="2">
-        <v>16.41</v>
+        <v>645.34</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
@@ -1375,34 +1375,34 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y10" s="5" t="inlineStr">
@@ -1410,31 +1410,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1462,32 +1462,32 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I11" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="J11" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="K11" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="L11" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="M11" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="N11" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="O11" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="P11" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
@@ -1499,19 +1499,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
@@ -1519,14 +1519,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y11" s="5" t="inlineStr">
@@ -1534,98 +1534,98 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I12" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J12" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K12" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L12" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M12" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N12" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O12" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P12" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I12" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J12" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K12" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L12" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M12" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N12" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O12" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P12" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr">
@@ -1638,9 +1638,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W12" s="4" t="inlineStr">
@@ -1648,9 +1648,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y12" s="5" t="inlineStr">
@@ -1658,44 +1658,44 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C13" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -1710,32 +1710,32 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I13" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="J13" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="K13" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="L13" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="M13" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N13" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="O13" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="P13" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
@@ -1747,9 +1747,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S13" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -1762,9 +1762,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -1772,9 +1772,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y13" s="5" t="inlineStr">
@@ -1787,26 +1787,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C14" s="10">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -1834,32 +1834,32 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I14" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="J14" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="K14" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="M14" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="N14" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="O14" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="P14" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -1871,14 +1871,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S14" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -1886,9 +1886,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W14" s="4" t="inlineStr">
@@ -1918,19 +1918,19 @@
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C15" s="10">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -1958,32 +1958,32 @@
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I15" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="J15" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="K15" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="M15" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="N15" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="O15" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="P15" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -1995,14 +1995,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
@@ -2015,9 +2015,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X15" s="6" t="inlineStr">
@@ -2042,23 +2042,23 @@
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C16" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -2086,28 +2086,28 @@
         </is>
       </c>
       <c r="I16" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="J16" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="K16" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L16" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N16" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="O16" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="P16" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
@@ -2134,14 +2134,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X16" s="6" t="inlineStr">
@@ -2166,19 +2166,19 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C17" s="10">
@@ -2186,116 +2186,240 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I17" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J17" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K17" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L17" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M17" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N17" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O17" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P17" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB17" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E17" s="0" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
+      <c r="H18" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I17" s="2">
+      <c r="I18" s="2">
         <v>698.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J18" s="2">
         <v>272.01</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K18" s="2">
         <v>348.9</v>
       </c>
-      <c r="L17" s="3">
+      <c r="L18" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M17" s="3">
+      <c r="M18" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N18" s="2">
         <v>713.11</v>
       </c>
-      <c r="O17" s="2">
+      <c r="O18" s="2">
         <v>282.35</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P18" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R17" s="13" t="inlineStr">
+      <c r="R18" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB17" s="11" t="inlineStr">
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB18" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB17"/>
+  <autoFilter ref="A1:AB18"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2313,6 +2437,7 @@
     <hyperlink ref="AB15" r:id="rId14"/>
     <hyperlink ref="AB16" r:id="rId15"/>
     <hyperlink ref="AB17" r:id="rId16"/>
+    <hyperlink ref="AB18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Dassault Systèmes (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$19</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -561,25 +561,25 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="C4" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -589,41 +589,41 @@
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I4" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="J4" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="K4" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="L4" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="M4" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="N4" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="O4" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="P4" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R4" s="13" t="inlineStr">
@@ -631,9 +631,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T4" s="4" t="inlineStr">
@@ -646,9 +646,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W4" s="4" t="inlineStr">
@@ -656,9 +656,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -671,26 +671,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="C5" s="10">
@@ -698,12 +698,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -718,32 +718,32 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="I5" s="2">
-        <v>78.3</v>
+        <v>26.48</v>
       </c>
       <c r="J5" s="2">
-        <v>84.06</v>
+        <v>27.68</v>
       </c>
       <c r="K5" s="2">
-        <v>97.98</v>
+        <v>36.62</v>
       </c>
       <c r="L5" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="M5" s="3">
-        <v>0.271</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="N5" s="2">
-        <v>69.22</v>
+        <v>36.11</v>
       </c>
       <c r="O5" s="2">
-        <v>86.5</v>
+        <v>30.75</v>
       </c>
       <c r="P5" s="2">
-        <v>110.62</v>
+        <v>40.69</v>
       </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
@@ -770,19 +770,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -795,26 +795,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB5" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C6" s="10">
@@ -827,7 +827,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="I6" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J6" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K6" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L6" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M6" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N6" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O6" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P6" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
@@ -879,9 +879,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
@@ -894,19 +894,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
@@ -919,30 +919,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB6" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C7" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
@@ -951,56 +951,56 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
+          <t>Consumo básico</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I7" s="2">
+        <v>52.9</v>
+      </c>
+      <c r="J7" s="2">
+        <v>55.98</v>
+      </c>
+      <c r="K7" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="L7" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="M7" s="3">
+        <v>0.244</v>
+      </c>
+      <c r="N7" s="2">
+        <v>69.29</v>
+      </c>
+      <c r="O7" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="P7" s="2">
+        <v>65.83</v>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I7" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J7" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K7" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L7" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M7" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N7" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O7" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P7" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
@@ -1008,9 +1008,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
@@ -1018,9 +1018,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W7" s="6" t="inlineStr">
@@ -1028,14 +1028,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1050,23 +1050,23 @@
       </c>
       <c r="AB7" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C8" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -1094,28 +1094,28 @@
         </is>
       </c>
       <c r="I8" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="J8" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="K8" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="L8" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M8" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="N8" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="O8" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="P8" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
@@ -1127,14 +1127,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1167,34 +1167,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C9" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1214,32 +1214,32 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I9" s="2">
-        <v>26.82</v>
+        <v>59.72</v>
       </c>
       <c r="J9" s="2">
-        <v>25.71</v>
+        <v>58.59</v>
       </c>
       <c r="K9" s="2">
-        <v>27.88</v>
+        <v>66.22</v>
       </c>
       <c r="L9" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M9" s="3">
-        <v>0.04</v>
+        <v>0.114</v>
       </c>
       <c r="N9" s="2">
-        <v>39</v>
+        <v>67.12</v>
       </c>
       <c r="O9" s="2">
-        <v>24.22</v>
+        <v>57.83</v>
       </c>
       <c r="P9" s="2">
-        <v>30.98</v>
+        <v>73.94</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
@@ -1266,24 +1266,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1291,26 +1291,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C10" s="10">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1338,36 +1338,36 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I10" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="J10" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="K10" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="L10" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M10" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="N10" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="O10" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="P10" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R10" s="13" t="inlineStr">
@@ -1375,9 +1375,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T10" s="4" t="inlineStr">
@@ -1390,29 +1390,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA10" s="4" t="inlineStr">
@@ -1422,19 +1422,19 @@
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
@@ -1466,28 +1466,28 @@
         </is>
       </c>
       <c r="I11" s="2">
-        <v>16.22</v>
+        <v>577.5</v>
       </c>
       <c r="J11" s="2">
-        <v>13.97</v>
+        <v>466.62</v>
       </c>
       <c r="K11" s="2">
-        <v>14.66</v>
+        <v>564.55</v>
       </c>
       <c r="L11" s="3">
-        <v>-0.077</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M11" s="3">
-        <v>-0.035</v>
+        <v>0.005</v>
       </c>
       <c r="N11" s="2">
-        <v>17.05</v>
+        <v>795.86</v>
       </c>
       <c r="O11" s="2">
-        <v>13.61</v>
+        <v>504.42</v>
       </c>
       <c r="P11" s="2">
-        <v>16.41</v>
+        <v>645.34</v>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
@@ -1499,34 +1499,34 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y11" s="5" t="inlineStr">
@@ -1534,31 +1534,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C12" s="10">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -1586,32 +1586,32 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I12" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="J12" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="K12" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="L12" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="M12" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="N12" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="O12" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="P12" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
@@ -1623,19 +1623,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
@@ -1643,14 +1643,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y12" s="5" t="inlineStr">
@@ -1658,98 +1658,98 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C13" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I13" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J13" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K13" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L13" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M13" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N13" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O13" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P13" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I13" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J13" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K13" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L13" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M13" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N13" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O13" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P13" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -1762,9 +1762,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -1772,9 +1772,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y13" s="5" t="inlineStr">
@@ -1782,44 +1782,44 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C14" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1834,32 +1834,32 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I14" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="J14" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="K14" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="M14" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N14" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="O14" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="P14" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -1871,9 +1871,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S14" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -1886,9 +1886,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W14" s="4" t="inlineStr">
@@ -1896,9 +1896,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y14" s="5" t="inlineStr">
@@ -1911,26 +1911,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C15" s="10">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -1958,32 +1958,32 @@
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I15" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="J15" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="K15" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="M15" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="N15" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="O15" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="P15" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -1995,14 +1995,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S15" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
@@ -2010,9 +2010,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W15" s="4" t="inlineStr">
@@ -2042,19 +2042,19 @@
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2082,32 +2082,32 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I16" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="J16" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="K16" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="L16" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="N16" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="O16" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="P16" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
@@ -2119,14 +2119,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2139,9 +2139,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X16" s="6" t="inlineStr">
@@ -2166,23 +2166,23 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2210,28 +2210,28 @@
         </is>
       </c>
       <c r="I17" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="J17" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="K17" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L17" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N17" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="O17" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="P17" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
@@ -2258,14 +2258,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X17" s="6" t="inlineStr">
@@ -2290,19 +2290,19 @@
       </c>
       <c r="AB17" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C18" s="10">
@@ -2310,116 +2310,240 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I18" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J18" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K18" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L18" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M18" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N18" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O18" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P18" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R18" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB18" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E18" s="0" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="G19" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I18" s="2">
+      <c r="I19" s="2">
         <v>698.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J19" s="2">
         <v>272.01</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K19" s="2">
         <v>348.9</v>
       </c>
-      <c r="L18" s="3">
+      <c r="L19" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M18" s="3">
+      <c r="M19" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N19" s="2">
         <v>713.11</v>
       </c>
-      <c r="O18" s="2">
+      <c r="O19" s="2">
         <v>282.35</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P19" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R18" s="13" t="inlineStr">
+      <c r="R19" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB18" s="11" t="inlineStr">
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB19" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB18"/>
+  <autoFilter ref="A1:AB19"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2438,6 +2562,7 @@
     <hyperlink ref="AB16" r:id="rId15"/>
     <hyperlink ref="AB17" r:id="rId16"/>
     <hyperlink ref="AB18" r:id="rId17"/>
+    <hyperlink ref="AB19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Zoetis (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$20</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -561,12 +561,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C4" s="10">
@@ -574,12 +574,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -594,32 +594,32 @@
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I4" s="2">
-        <v>21.51</v>
+        <v>71.33</v>
       </c>
       <c r="J4" s="2">
-        <v>25.08</v>
+        <v>91.77</v>
       </c>
       <c r="K4" s="2">
-        <v>30.22</v>
+        <v>101.61</v>
       </c>
       <c r="L4" s="3">
-        <v>0.179</v>
+        <v>0.316</v>
       </c>
       <c r="M4" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="N4" s="2">
-        <v>23.32</v>
+        <v>96</v>
       </c>
       <c r="O4" s="2">
-        <v>25.73</v>
+        <v>90.12</v>
       </c>
       <c r="P4" s="2">
-        <v>31.95</v>
+        <v>108.2</v>
       </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
@@ -641,9 +641,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V4" s="4" t="inlineStr">
@@ -656,9 +656,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -671,39 +671,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="C5" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -713,41 +713,41 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I5" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="J5" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="K5" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="L5" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="M5" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="N5" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="O5" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="P5" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R5" s="13" t="inlineStr">
@@ -755,9 +755,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
@@ -770,9 +770,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W5" s="4" t="inlineStr">
@@ -780,9 +780,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -795,26 +795,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB5" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="C6" s="10">
@@ -822,12 +822,12 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -842,32 +842,32 @@
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="I6" s="2">
-        <v>78.3</v>
+        <v>26.48</v>
       </c>
       <c r="J6" s="2">
-        <v>84.06</v>
+        <v>27.68</v>
       </c>
       <c r="K6" s="2">
-        <v>97.98</v>
+        <v>36.62</v>
       </c>
       <c r="L6" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="M6" s="3">
-        <v>0.271</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="N6" s="2">
-        <v>69.22</v>
+        <v>36.11</v>
       </c>
       <c r="O6" s="2">
-        <v>86.5</v>
+        <v>30.75</v>
       </c>
       <c r="P6" s="2">
-        <v>110.62</v>
+        <v>40.69</v>
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
@@ -894,19 +894,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
@@ -919,26 +919,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB6" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C7" s="10">
@@ -951,7 +951,7 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -970,28 +970,28 @@
         </is>
       </c>
       <c r="I7" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J7" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K7" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L7" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M7" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N7" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O7" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P7" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
@@ -1003,9 +1003,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr">
@@ -1018,19 +1018,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y7" s="4" t="inlineStr">
@@ -1043,30 +1043,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB7" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C8" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
@@ -1075,56 +1075,56 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
+          <t>Consumo básico</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I8" s="2">
+        <v>52.9</v>
+      </c>
+      <c r="J8" s="2">
+        <v>55.98</v>
+      </c>
+      <c r="K8" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="L8" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="M8" s="3">
+        <v>0.244</v>
+      </c>
+      <c r="N8" s="2">
+        <v>69.29</v>
+      </c>
+      <c r="O8" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="P8" s="2">
+        <v>65.83</v>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I8" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J8" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K8" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L8" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M8" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N8" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O8" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P8" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S8" s="6" t="inlineStr">
@@ -1132,9 +1132,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1142,9 +1142,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W8" s="6" t="inlineStr">
@@ -1152,14 +1152,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1174,23 +1174,23 @@
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C9" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1218,28 +1218,28 @@
         </is>
       </c>
       <c r="I9" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="J9" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="K9" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="L9" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M9" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="N9" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="O9" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="P9" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
@@ -1251,14 +1251,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1291,34 +1291,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C10" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1338,32 +1338,32 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I10" s="2">
-        <v>26.82</v>
+        <v>59.72</v>
       </c>
       <c r="J10" s="2">
-        <v>25.71</v>
+        <v>58.59</v>
       </c>
       <c r="K10" s="2">
-        <v>27.88</v>
+        <v>66.22</v>
       </c>
       <c r="L10" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M10" s="3">
-        <v>0.04</v>
+        <v>0.114</v>
       </c>
       <c r="N10" s="2">
-        <v>39</v>
+        <v>67.12</v>
       </c>
       <c r="O10" s="2">
-        <v>24.22</v>
+        <v>57.83</v>
       </c>
       <c r="P10" s="2">
-        <v>30.98</v>
+        <v>73.94</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
@@ -1390,24 +1390,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1415,26 +1415,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -1462,36 +1462,36 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I11" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="J11" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="K11" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="L11" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M11" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="N11" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="O11" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="P11" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R11" s="13" t="inlineStr">
@@ -1499,9 +1499,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T11" s="4" t="inlineStr">
@@ -1514,29 +1514,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA11" s="4" t="inlineStr">
@@ -1546,19 +1546,19 @@
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C12" s="10">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
@@ -1590,28 +1590,28 @@
         </is>
       </c>
       <c r="I12" s="2">
-        <v>16.22</v>
+        <v>577.5</v>
       </c>
       <c r="J12" s="2">
-        <v>13.97</v>
+        <v>466.62</v>
       </c>
       <c r="K12" s="2">
-        <v>14.66</v>
+        <v>564.55</v>
       </c>
       <c r="L12" s="3">
-        <v>-0.077</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M12" s="3">
-        <v>-0.035</v>
+        <v>0.005</v>
       </c>
       <c r="N12" s="2">
-        <v>17.05</v>
+        <v>795.86</v>
       </c>
       <c r="O12" s="2">
-        <v>13.61</v>
+        <v>504.42</v>
       </c>
       <c r="P12" s="2">
-        <v>16.41</v>
+        <v>645.34</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
@@ -1623,34 +1623,34 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y12" s="5" t="inlineStr">
@@ -1658,31 +1658,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C13" s="10">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1710,32 +1710,32 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I13" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="J13" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="K13" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="L13" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="M13" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="N13" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="O13" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="P13" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
@@ -1747,19 +1747,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
@@ -1767,14 +1767,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y13" s="5" t="inlineStr">
@@ -1782,98 +1782,98 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C14" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I14" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J14" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K14" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L14" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M14" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N14" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O14" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P14" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H14" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I14" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J14" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K14" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L14" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M14" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N14" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O14" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P14" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -1886,9 +1886,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W14" s="4" t="inlineStr">
@@ -1896,9 +1896,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y14" s="5" t="inlineStr">
@@ -1906,44 +1906,44 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C15" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -1958,32 +1958,32 @@
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I15" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="J15" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="K15" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="M15" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N15" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="O15" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="P15" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -1995,9 +1995,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S15" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr">
@@ -2010,9 +2010,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W15" s="4" t="inlineStr">
@@ -2020,9 +2020,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y15" s="5" t="inlineStr">
@@ -2035,26 +2035,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2082,32 +2082,32 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I16" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="J16" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="K16" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="L16" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="N16" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="O16" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="P16" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
@@ -2119,14 +2119,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S16" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2134,9 +2134,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W16" s="4" t="inlineStr">
@@ -2166,19 +2166,19 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C17" s="10">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -2206,32 +2206,32 @@
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I17" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="J17" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="K17" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="L17" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="N17" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="O17" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="P17" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
@@ -2243,14 +2243,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
@@ -2263,9 +2263,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X17" s="6" t="inlineStr">
@@ -2290,23 +2290,23 @@
       </c>
       <c r="AB17" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C18" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -2334,28 +2334,28 @@
         </is>
       </c>
       <c r="I18" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="J18" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="K18" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L18" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="M18" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N18" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="O18" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="P18" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
@@ -2382,14 +2382,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X18" s="6" t="inlineStr">
@@ -2414,19 +2414,19 @@
       </c>
       <c r="AB18" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C19" s="10">
@@ -2434,116 +2434,240 @@
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I19" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J19" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K19" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L19" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M19" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N19" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O19" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P19" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB19" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="C20" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E19" s="0" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
+      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
+      <c r="H20" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I19" s="2">
+      <c r="I20" s="2">
         <v>698.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J20" s="2">
         <v>272.01</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K20" s="2">
         <v>348.9</v>
       </c>
-      <c r="L19" s="3">
+      <c r="L20" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M19" s="3">
+      <c r="M20" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N20" s="2">
         <v>713.11</v>
       </c>
-      <c r="O19" s="2">
+      <c r="O20" s="2">
         <v>282.35</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P20" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R19" s="13" t="inlineStr">
+      <c r="R20" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB19" s="11" t="inlineStr">
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB20" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB19"/>
+  <autoFilter ref="A1:AB20"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2563,6 +2687,7 @@
     <hyperlink ref="AB17" r:id="rId16"/>
     <hyperlink ref="AB18" r:id="rId17"/>
     <hyperlink ref="AB19" r:id="rId18"/>
+    <hyperlink ref="AB20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
seguimiento.xlsx con Zoetis, DSV y Rentokil
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$22</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -561,12 +561,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="C4" s="10">
@@ -574,12 +574,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -594,32 +594,32 @@
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="I4" s="2">
-        <v>71.33</v>
+        <v>1137.5</v>
       </c>
       <c r="J4" s="2">
-        <v>91.77</v>
+        <v>1357.81</v>
       </c>
       <c r="K4" s="2">
-        <v>101.61</v>
+        <v>1747.71</v>
       </c>
       <c r="L4" s="3">
-        <v>0.316</v>
+        <v>0.2</v>
       </c>
       <c r="M4" s="3">
-        <v>0.45399999999999996</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="N4" s="2">
-        <v>96</v>
+        <v>1939</v>
       </c>
       <c r="O4" s="2">
-        <v>90.12</v>
+        <v>1481.37</v>
       </c>
       <c r="P4" s="2">
-        <v>108.2</v>
+        <v>1949.82</v>
       </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
@@ -631,14 +631,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U4" s="6" t="inlineStr">
@@ -646,19 +646,19 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -678,19 +678,19 @@
       </c>
       <c r="AB4" s="11" t="inlineStr">
         <is>
-          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
+          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C5" s="10">
@@ -698,12 +698,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -718,32 +718,32 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I5" s="2">
-        <v>21.51</v>
+        <v>71.33</v>
       </c>
       <c r="J5" s="2">
-        <v>25.08</v>
+        <v>91.77</v>
       </c>
       <c r="K5" s="2">
-        <v>30.22</v>
+        <v>101.61</v>
       </c>
       <c r="L5" s="3">
-        <v>0.179</v>
+        <v>0.316</v>
       </c>
       <c r="M5" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="N5" s="2">
-        <v>23.32</v>
+        <v>96</v>
       </c>
       <c r="O5" s="2">
-        <v>25.73</v>
+        <v>90.12</v>
       </c>
       <c r="P5" s="2">
-        <v>31.95</v>
+        <v>108.2</v>
       </c>
       <c r="Q5" s="13" t="inlineStr">
         <is>
@@ -765,9 +765,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
@@ -780,9 +780,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -795,39 +795,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB5" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="C6" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -837,41 +837,41 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I6" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="J6" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="K6" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="L6" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="M6" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="N6" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="O6" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="P6" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R6" s="13" t="inlineStr">
@@ -879,9 +879,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
@@ -894,9 +894,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W6" s="4" t="inlineStr">
@@ -904,9 +904,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
@@ -919,26 +919,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB6" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="C7" s="10">
@@ -946,12 +946,12 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -966,32 +966,32 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="I7" s="2">
-        <v>78.3</v>
+        <v>26.48</v>
       </c>
       <c r="J7" s="2">
-        <v>84.06</v>
+        <v>27.68</v>
       </c>
       <c r="K7" s="2">
-        <v>97.98</v>
+        <v>36.62</v>
       </c>
       <c r="L7" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="M7" s="3">
-        <v>0.271</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="N7" s="2">
-        <v>69.22</v>
+        <v>36.11</v>
       </c>
       <c r="O7" s="2">
-        <v>86.5</v>
+        <v>30.75</v>
       </c>
       <c r="P7" s="2">
-        <v>110.62</v>
+        <v>40.69</v>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
@@ -1018,19 +1018,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y7" s="4" t="inlineStr">
@@ -1043,26 +1043,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB7" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C8" s="10">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1094,28 +1094,28 @@
         </is>
       </c>
       <c r="I8" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J8" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K8" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L8" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M8" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N8" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O8" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P8" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
@@ -1127,9 +1127,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T8" s="4" t="inlineStr">
@@ -1142,19 +1142,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y8" s="4" t="inlineStr">
@@ -1167,30 +1167,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C9" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
@@ -1199,56 +1199,56 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
+          <t>Consumo básico</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I9" s="2">
+        <v>52.9</v>
+      </c>
+      <c r="J9" s="2">
+        <v>55.98</v>
+      </c>
+      <c r="K9" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="L9" s="3">
+        <v>0.12</v>
+      </c>
+      <c r="M9" s="3">
+        <v>0.244</v>
+      </c>
+      <c r="N9" s="2">
+        <v>69.29</v>
+      </c>
+      <c r="O9" s="2">
+        <v>57.16</v>
+      </c>
+      <c r="P9" s="2">
+        <v>65.83</v>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I9" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J9" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K9" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L9" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M9" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N9" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O9" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P9" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S9" s="6" t="inlineStr">
@@ -1256,9 +1256,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1266,9 +1266,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W9" s="6" t="inlineStr">
@@ -1276,14 +1276,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1298,27 +1298,27 @@
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="C10" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1326,53 +1326,53 @@
           <t>Industria</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I10" s="2">
+        <v>3.97</v>
+      </c>
+      <c r="J10" s="2">
+        <v>3.76</v>
+      </c>
+      <c r="K10" s="2">
+        <v>4.53</v>
+      </c>
+      <c r="L10" s="3">
+        <v>-0.021</v>
+      </c>
+      <c r="M10" s="3">
+        <v>0.17300000000000001</v>
+      </c>
+      <c r="N10" s="2">
+        <v>6.15</v>
+      </c>
+      <c r="O10" s="2">
+        <v>4.05</v>
+      </c>
+      <c r="P10" s="2">
+        <v>5.05</v>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I10" s="2">
-        <v>59.72</v>
-      </c>
-      <c r="J10" s="2">
-        <v>58.59</v>
-      </c>
-      <c r="K10" s="2">
-        <v>66.22</v>
-      </c>
-      <c r="L10" s="3">
-        <v>-0.013999999999999999</v>
-      </c>
-      <c r="M10" s="3">
-        <v>0.114</v>
-      </c>
-      <c r="N10" s="2">
-        <v>67.12</v>
-      </c>
-      <c r="O10" s="2">
-        <v>57.83</v>
-      </c>
-      <c r="P10" s="2">
-        <v>73.94</v>
-      </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S10" s="4" t="inlineStr">
@@ -1380,19 +1380,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W10" s="6" t="inlineStr">
@@ -1400,14 +1400,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1415,26 +1415,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1457,37 +1457,37 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I11" s="2">
-        <v>26.82</v>
+        <v>10.18</v>
       </c>
       <c r="J11" s="2">
-        <v>25.71</v>
+        <v>10.41</v>
       </c>
       <c r="K11" s="2">
-        <v>27.88</v>
+        <v>11.23</v>
       </c>
       <c r="L11" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M11" s="3">
-        <v>0.04</v>
+        <v>0.122</v>
       </c>
       <c r="N11" s="2">
-        <v>39</v>
+        <v>14.33</v>
       </c>
       <c r="O11" s="2">
-        <v>24.22</v>
+        <v>9.92</v>
       </c>
       <c r="P11" s="2">
-        <v>30.98</v>
+        <v>12.34</v>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
@@ -1499,14 +1499,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U11" s="4" t="inlineStr">
@@ -1514,24 +1514,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z11" s="4" t="inlineStr">
@@ -1546,27 +1546,27 @@
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -1590,32 +1590,32 @@
         </is>
       </c>
       <c r="I12" s="2">
-        <v>577.5</v>
+        <v>59.72</v>
       </c>
       <c r="J12" s="2">
-        <v>466.62</v>
+        <v>58.59</v>
       </c>
       <c r="K12" s="2">
-        <v>564.55</v>
+        <v>66.22</v>
       </c>
       <c r="L12" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M12" s="3">
-        <v>0.005</v>
+        <v>0.114</v>
       </c>
       <c r="N12" s="2">
-        <v>795.86</v>
+        <v>67.12</v>
       </c>
       <c r="O12" s="2">
-        <v>504.42</v>
+        <v>57.83</v>
       </c>
       <c r="P12" s="2">
-        <v>645.34</v>
+        <v>73.94</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R12" s="13" t="inlineStr">
@@ -1623,9 +1623,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr">
@@ -1658,31 +1658,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C13" s="10">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1705,41 +1705,41 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I13" s="2">
-        <v>16.22</v>
+        <v>26.82</v>
       </c>
       <c r="J13" s="2">
-        <v>13.97</v>
+        <v>25.71</v>
       </c>
       <c r="K13" s="2">
-        <v>14.66</v>
+        <v>27.88</v>
       </c>
       <c r="L13" s="3">
-        <v>-0.077</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M13" s="3">
-        <v>-0.035</v>
+        <v>0.04</v>
       </c>
       <c r="N13" s="2">
-        <v>17.05</v>
+        <v>39</v>
       </c>
       <c r="O13" s="2">
-        <v>13.61</v>
+        <v>24.22</v>
       </c>
       <c r="P13" s="2">
-        <v>16.41</v>
+        <v>30.98</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R13" s="13" t="inlineStr">
@@ -1747,66 +1747,66 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C14" s="10">
@@ -1814,12 +1814,12 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1829,37 +1829,37 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I14" s="2">
-        <v>81490</v>
+        <v>577.5</v>
       </c>
       <c r="J14" s="2">
-        <v>66566.47</v>
+        <v>466.62</v>
       </c>
       <c r="K14" s="2">
-        <v>75201.52</v>
+        <v>564.55</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M14" s="3">
-        <v>-0.07</v>
+        <v>0.005</v>
       </c>
       <c r="N14" s="2">
-        <v>97866.67</v>
+        <v>795.86</v>
       </c>
       <c r="O14" s="2">
-        <v>65834.24</v>
+        <v>504.42</v>
       </c>
       <c r="P14" s="2">
-        <v>84206.58</v>
+        <v>645.34</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -1871,9 +1871,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -1886,14 +1886,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X14" s="6" t="inlineStr">
@@ -1918,23 +1918,23 @@
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C15" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
@@ -1943,81 +1943,81 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I15" s="2">
+        <v>16.22</v>
+      </c>
+      <c r="J15" s="2">
+        <v>13.97</v>
+      </c>
+      <c r="K15" s="2">
+        <v>14.66</v>
+      </c>
+      <c r="L15" s="3">
+        <v>-0.077</v>
+      </c>
+      <c r="M15" s="3">
+        <v>-0.035</v>
+      </c>
+      <c r="N15" s="2">
+        <v>17.05</v>
+      </c>
+      <c r="O15" s="2">
+        <v>13.61</v>
+      </c>
+      <c r="P15" s="2">
+        <v>16.41</v>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I15" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J15" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K15" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L15" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M15" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N15" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O15" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P15" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X15" s="4" t="inlineStr">
@@ -2042,19 +2042,19 @@
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,66 +2062,66 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I16" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J16" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K16" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L16" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M16" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N16" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O16" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P16" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>NOK</t>
-        </is>
-      </c>
-      <c r="I16" s="2">
-        <v>299</v>
-      </c>
-      <c r="J16" s="2">
-        <v>204.75</v>
-      </c>
-      <c r="K16" s="2">
-        <v>239.87</v>
-      </c>
-      <c r="L16" s="3">
-        <v>-0.308</v>
-      </c>
-      <c r="M16" s="3">
-        <v>-0.19</v>
-      </c>
-      <c r="N16" s="2">
-        <v>397.27</v>
-      </c>
-      <c r="O16" s="2">
-        <v>210.48</v>
-      </c>
-      <c r="P16" s="2">
-        <v>269.04</v>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S16" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -2154,9 +2154,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2166,32 +2166,32 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -2206,32 +2206,32 @@
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I17" s="2">
-        <v>6220</v>
+        <v>53.82</v>
       </c>
       <c r="J17" s="2">
-        <v>4460.49</v>
+        <v>44.48</v>
       </c>
       <c r="K17" s="2">
-        <v>4713.09</v>
+        <v>44.65</v>
       </c>
       <c r="L17" s="3">
-        <v>-0.266</v>
+        <v>-0.151</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.225</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N17" s="2">
-        <v>7278.89</v>
+        <v>60.39</v>
       </c>
       <c r="O17" s="2">
-        <v>4188.4</v>
+        <v>39.85</v>
       </c>
       <c r="P17" s="2">
-        <v>4821.79</v>
+        <v>48.84</v>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
@@ -2248,9 +2248,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
@@ -2268,9 +2268,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y17" s="5" t="inlineStr">
@@ -2283,26 +2283,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB17" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C18" s="10">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -2330,32 +2330,32 @@
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I18" s="2">
-        <v>253.14</v>
+        <v>299</v>
       </c>
       <c r="J18" s="2">
-        <v>168.18</v>
+        <v>204.75</v>
       </c>
       <c r="K18" s="2">
-        <v>168.18</v>
+        <v>239.87</v>
       </c>
       <c r="L18" s="3">
-        <v>-0.335</v>
+        <v>-0.308</v>
       </c>
       <c r="M18" s="3">
-        <v>-0.335</v>
+        <v>-0.19</v>
       </c>
       <c r="N18" s="2">
-        <v>337.43</v>
+        <v>397.27</v>
       </c>
       <c r="O18" s="2">
-        <v>146.32</v>
+        <v>210.48</v>
       </c>
       <c r="P18" s="2">
-        <v>187.18</v>
+        <v>269.04</v>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
@@ -2367,9 +2367,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S18" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -2382,14 +2382,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X18" s="6" t="inlineStr">
@@ -2414,32 +2414,32 @@
       </c>
       <c r="AB18" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C19" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -2454,32 +2454,32 @@
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I19" s="2">
-        <v>404.76</v>
+        <v>6220</v>
       </c>
       <c r="J19" s="2">
-        <v>222.49</v>
+        <v>4460.49</v>
       </c>
       <c r="K19" s="2">
-        <v>222.49</v>
+        <v>4713.09</v>
       </c>
       <c r="L19" s="3">
-        <v>-0.45</v>
+        <v>-0.266</v>
       </c>
       <c r="M19" s="3">
-        <v>-0.45</v>
+        <v>-0.225</v>
       </c>
       <c r="N19" s="2">
-        <v>477.21</v>
+        <v>7278.89</v>
       </c>
       <c r="O19" s="2">
-        <v>193.34</v>
+        <v>4188.4</v>
       </c>
       <c r="P19" s="2">
-        <v>247.41</v>
+        <v>4821.79</v>
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
@@ -2491,14 +2491,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr">
@@ -2506,9 +2506,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2538,136 +2538,384 @@
       </c>
       <c r="AB19" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
+          <t>Vertiv</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="C20" s="10">
+        <v>46302</v>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>Industria</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I20" s="2">
+        <v>253.14</v>
+      </c>
+      <c r="J20" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="K20" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="L20" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="M20" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="N20" s="2">
+        <v>337.43</v>
+      </c>
+      <c r="O20" s="2">
+        <v>146.32</v>
+      </c>
+      <c r="P20" s="2">
+        <v>187.18</v>
+      </c>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB20" s="11" t="inlineStr">
+        <is>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Intuitive</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="C21" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I21" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J21" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K21" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L21" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M21" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N21" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O21" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P21" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R21" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB21" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>VACN</t>
         </is>
       </c>
-      <c r="C20" s="10">
+      <c r="C22" s="10">
         <v>46301</v>
       </c>
-      <c r="D20" s="0" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E20" s="0" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G20" s="13" t="inlineStr">
+      <c r="G22" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
+      <c r="H22" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I20" s="2">
+      <c r="I22" s="2">
         <v>698.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J22" s="2">
         <v>272.01</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K22" s="2">
         <v>348.9</v>
       </c>
-      <c r="L20" s="3">
+      <c r="L22" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M20" s="3">
+      <c r="M22" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N22" s="2">
         <v>713.11</v>
       </c>
-      <c r="O20" s="2">
+      <c r="O22" s="2">
         <v>282.35</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P22" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R20" s="13" t="inlineStr">
+      <c r="R22" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB20" s="11" t="inlineStr">
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB22" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB20"/>
+  <autoFilter ref="A1:AB22"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2688,6 +2936,8 @@
     <hyperlink ref="AB18" r:id="rId17"/>
     <hyperlink ref="AB19" r:id="rId18"/>
     <hyperlink ref="AB20" r:id="rId19"/>
+    <hyperlink ref="AB21" r:id="rId20"/>
+    <hyperlink ref="AB22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Tomra (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$24</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1057,20 +1057,20 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="C8" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -1094,28 +1094,28 @@
         </is>
       </c>
       <c r="I8" s="2">
-        <v>78.3</v>
+        <v>8.677</v>
       </c>
       <c r="J8" s="2">
-        <v>84.06</v>
+        <v>9.45</v>
       </c>
       <c r="K8" s="2">
-        <v>97.98</v>
+        <v>11.42</v>
       </c>
       <c r="L8" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="M8" s="3">
-        <v>0.271</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="N8" s="2">
-        <v>69.22</v>
+        <v>11.81</v>
       </c>
       <c r="O8" s="2">
-        <v>86.5</v>
+        <v>9.65</v>
       </c>
       <c r="P8" s="2">
-        <v>110.62</v>
+        <v>12.54</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
@@ -1127,19 +1127,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
@@ -1147,9 +1147,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X8" s="6" t="inlineStr">
@@ -1157,9 +1157,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1167,26 +1167,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C9" s="10">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1218,28 +1218,28 @@
         </is>
       </c>
       <c r="I9" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J9" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K9" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L9" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M9" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N9" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O9" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P9" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
@@ -1251,9 +1251,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T9" s="4" t="inlineStr">
@@ -1266,19 +1266,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y9" s="4" t="inlineStr">
@@ -1291,39 +1291,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C10" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1338,32 +1338,32 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I10" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="J10" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="K10" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="L10" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="M10" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="N10" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="O10" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="P10" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
@@ -1375,19 +1375,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr">
@@ -1405,9 +1405,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1422,19 +1422,19 @@
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="C11" s="10">
@@ -1442,66 +1442,66 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+          <t>Industria</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I11" s="2">
+        <v>3.97</v>
+      </c>
+      <c r="J11" s="2">
+        <v>3.76</v>
+      </c>
+      <c r="K11" s="2">
+        <v>4.53</v>
+      </c>
+      <c r="L11" s="3">
+        <v>-0.021</v>
+      </c>
+      <c r="M11" s="3">
+        <v>0.17300000000000001</v>
+      </c>
+      <c r="N11" s="2">
+        <v>6.15</v>
+      </c>
+      <c r="O11" s="2">
+        <v>4.05</v>
+      </c>
+      <c r="P11" s="2">
+        <v>5.05</v>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I11" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J11" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K11" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L11" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M11" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N11" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O11" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P11" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="S11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T11" s="5" t="inlineStr">
@@ -1509,14 +1509,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W11" s="6" t="inlineStr">
@@ -1524,14 +1524,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z11" s="4" t="inlineStr">
@@ -1546,91 +1546,91 @@
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I12" s="2">
+        <v>80.75</v>
+      </c>
+      <c r="J12" s="2">
+        <v>80.93</v>
+      </c>
+      <c r="K12" s="2">
+        <v>93.63</v>
+      </c>
+      <c r="L12" s="3">
+        <v>0.013999999999999999</v>
+      </c>
+      <c r="M12" s="3">
+        <v>0.172</v>
+      </c>
+      <c r="N12" s="2">
+        <v>79.54</v>
+      </c>
+      <c r="O12" s="2">
+        <v>81.9</v>
+      </c>
+      <c r="P12" s="2">
+        <v>98.17</v>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I12" s="2">
-        <v>59.72</v>
-      </c>
-      <c r="J12" s="2">
-        <v>58.59</v>
-      </c>
-      <c r="K12" s="2">
-        <v>66.22</v>
-      </c>
-      <c r="L12" s="3">
-        <v>-0.013999999999999999</v>
-      </c>
-      <c r="M12" s="3">
-        <v>0.114</v>
-      </c>
-      <c r="N12" s="2">
-        <v>67.12</v>
-      </c>
-      <c r="O12" s="2">
-        <v>57.83</v>
-      </c>
-      <c r="P12" s="2">
-        <v>73.94</v>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="S12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="S12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -1638,19 +1638,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y12" s="5" t="inlineStr">
@@ -1663,26 +1663,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.docx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C13" s="10">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1705,37 +1705,37 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I13" s="2">
-        <v>26.82</v>
+        <v>10.18</v>
       </c>
       <c r="J13" s="2">
-        <v>25.71</v>
+        <v>10.41</v>
       </c>
       <c r="K13" s="2">
-        <v>27.88</v>
+        <v>11.23</v>
       </c>
       <c r="L13" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M13" s="3">
-        <v>0.04</v>
+        <v>0.122</v>
       </c>
       <c r="N13" s="2">
-        <v>39</v>
+        <v>14.33</v>
       </c>
       <c r="O13" s="2">
-        <v>24.22</v>
+        <v>9.92</v>
       </c>
       <c r="P13" s="2">
-        <v>30.98</v>
+        <v>12.34</v>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
@@ -1747,14 +1747,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
@@ -1762,24 +1762,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z13" s="4" t="inlineStr">
@@ -1794,27 +1794,27 @@
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C14" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -1838,32 +1838,32 @@
         </is>
       </c>
       <c r="I14" s="2">
-        <v>577.5</v>
+        <v>59.72</v>
       </c>
       <c r="J14" s="2">
-        <v>466.62</v>
+        <v>58.59</v>
       </c>
       <c r="K14" s="2">
-        <v>564.55</v>
+        <v>66.22</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M14" s="3">
-        <v>0.005</v>
+        <v>0.114</v>
       </c>
       <c r="N14" s="2">
-        <v>795.86</v>
+        <v>67.12</v>
       </c>
       <c r="O14" s="2">
-        <v>504.42</v>
+        <v>57.83</v>
       </c>
       <c r="P14" s="2">
-        <v>645.34</v>
+        <v>73.94</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R14" s="13" t="inlineStr">
@@ -1871,9 +1871,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -1906,31 +1906,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C15" s="10">
@@ -1938,12 +1938,12 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1953,41 +1953,41 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I15" s="2">
-        <v>16.22</v>
+        <v>26.82</v>
       </c>
       <c r="J15" s="2">
-        <v>13.97</v>
+        <v>25.71</v>
       </c>
       <c r="K15" s="2">
-        <v>14.66</v>
+        <v>27.88</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.077</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M15" s="3">
-        <v>-0.035</v>
+        <v>0.04</v>
       </c>
       <c r="N15" s="2">
-        <v>17.05</v>
+        <v>39</v>
       </c>
       <c r="O15" s="2">
-        <v>13.61</v>
+        <v>24.22</v>
       </c>
       <c r="P15" s="2">
-        <v>16.41</v>
+        <v>30.98</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R15" s="13" t="inlineStr">
@@ -1995,66 +1995,66 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,12 +2062,12 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -2077,37 +2077,37 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I16" s="2">
-        <v>81490</v>
+        <v>577.5</v>
       </c>
       <c r="J16" s="2">
-        <v>66566.47</v>
+        <v>466.62</v>
       </c>
       <c r="K16" s="2">
-        <v>75201.52</v>
+        <v>564.55</v>
       </c>
       <c r="L16" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.07</v>
+        <v>0.005</v>
       </c>
       <c r="N16" s="2">
-        <v>97866.67</v>
+        <v>795.86</v>
       </c>
       <c r="O16" s="2">
-        <v>65834.24</v>
+        <v>504.42</v>
       </c>
       <c r="P16" s="2">
-        <v>84206.58</v>
+        <v>645.34</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
@@ -2119,9 +2119,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -2134,14 +2134,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X16" s="6" t="inlineStr">
@@ -2166,23 +2166,23 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
@@ -2191,81 +2191,81 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I17" s="2">
+        <v>16.22</v>
+      </c>
+      <c r="J17" s="2">
+        <v>13.97</v>
+      </c>
+      <c r="K17" s="2">
+        <v>14.66</v>
+      </c>
+      <c r="L17" s="3">
+        <v>-0.077</v>
+      </c>
+      <c r="M17" s="3">
+        <v>-0.035</v>
+      </c>
+      <c r="N17" s="2">
+        <v>17.05</v>
+      </c>
+      <c r="O17" s="2">
+        <v>13.61</v>
+      </c>
+      <c r="P17" s="2">
+        <v>16.41</v>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I17" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J17" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K17" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L17" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M17" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N17" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O17" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P17" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X17" s="4" t="inlineStr">
@@ -2290,19 +2290,19 @@
       </c>
       <c r="AB17" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C18" s="10">
@@ -2310,66 +2310,66 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I18" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J18" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K18" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L18" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M18" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N18" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O18" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P18" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>NOK</t>
-        </is>
-      </c>
-      <c r="I18" s="2">
-        <v>299</v>
-      </c>
-      <c r="J18" s="2">
-        <v>204.75</v>
-      </c>
-      <c r="K18" s="2">
-        <v>239.87</v>
-      </c>
-      <c r="L18" s="3">
-        <v>-0.308</v>
-      </c>
-      <c r="M18" s="3">
-        <v>-0.19</v>
-      </c>
-      <c r="N18" s="2">
-        <v>397.27</v>
-      </c>
-      <c r="O18" s="2">
-        <v>210.48</v>
-      </c>
-      <c r="P18" s="2">
-        <v>269.04</v>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S18" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -2402,9 +2402,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2414,32 +2414,32 @@
       </c>
       <c r="AB18" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C19" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -2454,32 +2454,32 @@
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I19" s="2">
-        <v>6220</v>
+        <v>53.82</v>
       </c>
       <c r="J19" s="2">
-        <v>4460.49</v>
+        <v>44.48</v>
       </c>
       <c r="K19" s="2">
-        <v>4713.09</v>
+        <v>44.65</v>
       </c>
       <c r="L19" s="3">
-        <v>-0.266</v>
+        <v>-0.151</v>
       </c>
       <c r="M19" s="3">
-        <v>-0.225</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N19" s="2">
-        <v>7278.89</v>
+        <v>60.39</v>
       </c>
       <c r="O19" s="2">
-        <v>4188.4</v>
+        <v>39.85</v>
       </c>
       <c r="P19" s="2">
-        <v>4821.79</v>
+        <v>48.84</v>
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
@@ -2496,9 +2496,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr">
@@ -2516,9 +2516,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y19" s="5" t="inlineStr">
@@ -2531,26 +2531,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB19" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C20" s="10">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -2578,32 +2578,32 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I20" s="2">
-        <v>253.14</v>
+        <v>299</v>
       </c>
       <c r="J20" s="2">
-        <v>168.18</v>
+        <v>204.75</v>
       </c>
       <c r="K20" s="2">
-        <v>168.18</v>
+        <v>239.87</v>
       </c>
       <c r="L20" s="3">
-        <v>-0.335</v>
+        <v>-0.308</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.335</v>
+        <v>-0.19</v>
       </c>
       <c r="N20" s="2">
-        <v>337.43</v>
+        <v>397.27</v>
       </c>
       <c r="O20" s="2">
-        <v>146.32</v>
+        <v>210.48</v>
       </c>
       <c r="P20" s="2">
-        <v>187.18</v>
+        <v>269.04</v>
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
@@ -2615,9 +2615,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S20" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="T20" s="4" t="inlineStr">
@@ -2630,14 +2630,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X20" s="6" t="inlineStr">
@@ -2662,32 +2662,32 @@
       </c>
       <c r="AB20" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C21" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -2702,32 +2702,32 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I21" s="2">
-        <v>404.76</v>
+        <v>6220</v>
       </c>
       <c r="J21" s="2">
-        <v>222.49</v>
+        <v>4460.49</v>
       </c>
       <c r="K21" s="2">
-        <v>222.49</v>
+        <v>4713.09</v>
       </c>
       <c r="L21" s="3">
-        <v>-0.45</v>
+        <v>-0.266</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.45</v>
+        <v>-0.225</v>
       </c>
       <c r="N21" s="2">
-        <v>477.21</v>
+        <v>7278.89</v>
       </c>
       <c r="O21" s="2">
-        <v>193.34</v>
+        <v>4188.4</v>
       </c>
       <c r="P21" s="2">
-        <v>247.41</v>
+        <v>4821.79</v>
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
@@ -2739,14 +2739,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
@@ -2754,9 +2754,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2786,136 +2786,384 @@
       </c>
       <c r="AB21" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
+          <t>Vertiv</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="C22" s="10">
+        <v>46302</v>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>Industria</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I22" s="2">
+        <v>253.14</v>
+      </c>
+      <c r="J22" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="K22" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="L22" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="M22" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="N22" s="2">
+        <v>337.43</v>
+      </c>
+      <c r="O22" s="2">
+        <v>146.32</v>
+      </c>
+      <c r="P22" s="2">
+        <v>187.18</v>
+      </c>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R22" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB22" s="11" t="inlineStr">
+        <is>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Intuitive</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="C23" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I23" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J23" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K23" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L23" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M23" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N23" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O23" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P23" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R23" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB23" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>VACN</t>
         </is>
       </c>
-      <c r="C22" s="10">
+      <c r="C24" s="10">
         <v>46301</v>
       </c>
-      <c r="D22" s="0" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E22" s="0" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H24" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I22" s="2">
+      <c r="I24" s="2">
         <v>698.2</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J24" s="2">
         <v>272.01</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K24" s="2">
         <v>348.9</v>
       </c>
-      <c r="L22" s="3">
+      <c r="L24" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M22" s="3">
+      <c r="M24" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N24" s="2">
         <v>713.11</v>
       </c>
-      <c r="O22" s="2">
+      <c r="O24" s="2">
         <v>282.35</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P24" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R22" s="13" t="inlineStr">
+      <c r="R24" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB22" s="11" t="inlineStr">
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB24" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB22"/>
+  <autoFilter ref="A1:AB24"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -2938,6 +3186,8 @@
     <hyperlink ref="AB20" r:id="rId19"/>
     <hyperlink ref="AB21" r:id="rId20"/>
     <hyperlink ref="AB22" r:id="rId21"/>
+    <hyperlink ref="AB23" r:id="rId22"/>
+    <hyperlink ref="AB24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de PepsiCo (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AB$25</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1057,12 +1057,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="C8" s="10">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1090,36 +1090,36 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I8" s="2">
-        <v>8.677</v>
+        <v>123.73</v>
       </c>
       <c r="J8" s="2">
-        <v>9.45</v>
+        <v>151.16</v>
       </c>
       <c r="K8" s="2">
-        <v>11.42</v>
+        <v>164.85</v>
       </c>
       <c r="L8" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.268</v>
       </c>
       <c r="M8" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.379</v>
       </c>
       <c r="N8" s="2">
-        <v>11.81</v>
+        <v>148.64</v>
       </c>
       <c r="O8" s="2">
-        <v>9.65</v>
+        <v>148.29</v>
       </c>
       <c r="P8" s="2">
-        <v>12.54</v>
+        <v>181.24</v>
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="R8" s="13" t="inlineStr">
@@ -1132,9 +1132,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -1142,9 +1142,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W8" s="6" t="inlineStr">
@@ -1152,14 +1152,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1174,27 +1174,27 @@
       </c>
       <c r="AB8" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="C9" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1218,28 +1218,28 @@
         </is>
       </c>
       <c r="I9" s="2">
-        <v>78.3</v>
+        <v>8.677</v>
       </c>
       <c r="J9" s="2">
-        <v>84.06</v>
+        <v>9.45</v>
       </c>
       <c r="K9" s="2">
-        <v>97.98</v>
+        <v>11.42</v>
       </c>
       <c r="L9" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="M9" s="3">
-        <v>0.271</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="N9" s="2">
-        <v>69.22</v>
+        <v>11.81</v>
       </c>
       <c r="O9" s="2">
-        <v>86.5</v>
+        <v>9.65</v>
       </c>
       <c r="P9" s="2">
-        <v>110.62</v>
+        <v>12.54</v>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
@@ -1251,19 +1251,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V9" s="5" t="inlineStr">
@@ -1271,9 +1271,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X9" s="6" t="inlineStr">
@@ -1281,9 +1281,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1291,26 +1291,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB9" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C10" s="10">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1342,28 +1342,28 @@
         </is>
       </c>
       <c r="I10" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="J10" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="K10" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="L10" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="M10" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="N10" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="O10" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="P10" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
@@ -1375,9 +1375,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T10" s="4" t="inlineStr">
@@ -1390,19 +1390,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y10" s="4" t="inlineStr">
@@ -1415,39 +1415,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB10" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="C11" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1462,32 +1462,32 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I11" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="J11" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="K11" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="L11" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="M11" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="N11" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="O11" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="P11" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
@@ -1499,19 +1499,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V11" s="4" t="inlineStr">
@@ -1529,9 +1529,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z11" s="4" t="inlineStr">
@@ -1546,32 +1546,32 @@
       </c>
       <c r="AB11" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1586,32 +1586,32 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I12" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="J12" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="K12" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="L12" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="M12" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="N12" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="O12" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="P12" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
@@ -1623,19 +1623,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V12" s="4" t="inlineStr">
@@ -1643,19 +1643,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z12" s="4" t="inlineStr">
@@ -1663,34 +1663,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="C13" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -1698,53 +1698,53 @@
           <t>Salud</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I13" s="2">
+        <v>80.75</v>
+      </c>
+      <c r="J13" s="2">
+        <v>80.93</v>
+      </c>
+      <c r="K13" s="2">
+        <v>93.63</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0.013999999999999999</v>
+      </c>
+      <c r="M13" s="3">
+        <v>0.172</v>
+      </c>
+      <c r="N13" s="2">
+        <v>79.54</v>
+      </c>
+      <c r="O13" s="2">
+        <v>81.9</v>
+      </c>
+      <c r="P13" s="2">
+        <v>98.17</v>
+      </c>
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I13" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="J13" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="K13" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="L13" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="M13" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="N13" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="O13" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="P13" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S13" s="6" t="inlineStr">
@@ -1752,9 +1752,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
@@ -1762,19 +1762,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y13" s="5" t="inlineStr">
@@ -1787,30 +1787,30 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB13" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C14" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1838,28 +1838,28 @@
         </is>
       </c>
       <c r="I14" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="J14" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="K14" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="L14" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="M14" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="N14" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="O14" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="P14" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
@@ -1871,14 +1871,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -1911,34 +1911,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB14" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="C15" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -1958,32 +1958,32 @@
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I15" s="2">
-        <v>26.82</v>
+        <v>59.72</v>
       </c>
       <c r="J15" s="2">
-        <v>25.71</v>
+        <v>58.59</v>
       </c>
       <c r="K15" s="2">
-        <v>27.88</v>
+        <v>66.22</v>
       </c>
       <c r="L15" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="M15" s="3">
-        <v>0.04</v>
+        <v>0.114</v>
       </c>
       <c r="N15" s="2">
-        <v>39</v>
+        <v>67.12</v>
       </c>
       <c r="O15" s="2">
-        <v>24.22</v>
+        <v>57.83</v>
       </c>
       <c r="P15" s="2">
-        <v>30.98</v>
+        <v>73.94</v>
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
@@ -2010,24 +2010,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z15" s="4" t="inlineStr">
@@ -2035,26 +2035,26 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB15" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="C16" s="10">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2082,36 +2082,36 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I16" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="J16" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="K16" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="L16" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="M16" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="N16" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="O16" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="P16" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="R16" s="13" t="inlineStr">
@@ -2119,9 +2119,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -2134,29 +2134,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2166,19 +2166,19 @@
       </c>
       <c r="AB16" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="C17" s="10">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -2210,28 +2210,28 @@
         </is>
       </c>
       <c r="I17" s="2">
-        <v>16.22</v>
+        <v>577.5</v>
       </c>
       <c r="J17" s="2">
-        <v>13.97</v>
+        <v>466.62</v>
       </c>
       <c r="K17" s="2">
-        <v>14.66</v>
+        <v>564.55</v>
       </c>
       <c r="L17" s="3">
-        <v>-0.077</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.035</v>
+        <v>0.005</v>
       </c>
       <c r="N17" s="2">
-        <v>17.05</v>
+        <v>795.86</v>
       </c>
       <c r="O17" s="2">
-        <v>13.61</v>
+        <v>504.42</v>
       </c>
       <c r="P17" s="2">
-        <v>16.41</v>
+        <v>645.34</v>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
@@ -2243,34 +2243,34 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="T17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y17" s="5" t="inlineStr">
@@ -2278,31 +2278,31 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB17" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="C18" s="10">
@@ -2310,12 +2310,12 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -2330,32 +2330,32 @@
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I18" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="J18" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="K18" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="L18" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="M18" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="N18" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="O18" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="P18" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
@@ -2367,19 +2367,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2387,14 +2387,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y18" s="5" t="inlineStr">
@@ -2402,98 +2402,98 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB18" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="C19" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="I19" s="2">
+        <v>81490</v>
+      </c>
+      <c r="J19" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="K19" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="L19" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="M19" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="N19" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="O19" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="P19" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="I19" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="J19" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="K19" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="L19" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="M19" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="N19" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="O19" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="P19" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="Q19" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="S19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="T19" s="4" t="inlineStr">
@@ -2506,9 +2506,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2516,9 +2516,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y19" s="5" t="inlineStr">
@@ -2526,44 +2526,44 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Z19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB19" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="C20" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -2578,32 +2578,32 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="I20" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="J20" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="K20" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="L20" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="N20" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="O20" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="P20" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
@@ -2615,9 +2615,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S20" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="S20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="T20" s="4" t="inlineStr">
@@ -2630,9 +2630,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -2640,9 +2640,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y20" s="5" t="inlineStr">
@@ -2655,26 +2655,26 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB20" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="C21" s="10">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -2702,32 +2702,32 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="I21" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="J21" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="K21" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="L21" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="N21" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="O21" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="P21" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
@@ -2739,14 +2739,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="S21" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
@@ -2754,9 +2754,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2786,19 +2786,19 @@
       </c>
       <c r="AB21" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="C22" s="10">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -2826,32 +2826,32 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="I22" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="J22" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="K22" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="L22" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="M22" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="N22" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="O22" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="P22" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
@@ -2863,14 +2863,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="S22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2883,9 +2883,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X22" s="6" t="inlineStr">
@@ -2910,23 +2910,23 @@
       </c>
       <c r="AB22" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C23" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -2954,28 +2954,28 @@
         </is>
       </c>
       <c r="I23" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="J23" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="K23" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L23" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N23" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="O23" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="P23" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="Q23" s="13" t="inlineStr">
         <is>
@@ -3002,14 +3002,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X23" s="6" t="inlineStr">
@@ -3034,19 +3034,19 @@
       </c>
       <c r="AB23" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="C24" s="10">
@@ -3054,116 +3054,240 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I24" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="J24" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="K24" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L24" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N24" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="O24" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="P24" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="R24" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB24" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="C25" s="10">
+        <v>46301</v>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="E24" s="0" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="G24" s="13" t="inlineStr">
+      <c r="G25" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="I24" s="2">
+      <c r="I25" s="2">
         <v>698.2</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J25" s="2">
         <v>272.01</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K25" s="2">
         <v>348.9</v>
       </c>
-      <c r="L24" s="3">
+      <c r="L25" s="3">
         <v>-0.6</v>
       </c>
-      <c r="M24" s="3">
+      <c r="M25" s="3">
         <v>-0.49</v>
       </c>
-      <c r="N24" s="2">
+      <c r="N25" s="2">
         <v>713.11</v>
       </c>
-      <c r="O24" s="2">
+      <c r="O25" s="2">
         <v>282.35</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P25" s="2">
         <v>395.5</v>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="R24" s="13" t="inlineStr">
+      <c r="R25" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="T24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB24" s="11" t="inlineStr">
+      <c r="S25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB25" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB24"/>
+  <autoFilter ref="A1:AB25"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1"/>
     <hyperlink ref="AB3" r:id="rId2"/>
@@ -3188,6 +3312,7 @@
     <hyperlink ref="AB22" r:id="rId21"/>
     <hyperlink ref="AB23" r:id="rId22"/>
     <hyperlink ref="AB24" r:id="rId23"/>
+    <hyperlink ref="AB25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Microsoft (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$28</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -2641,32 +2641,32 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K20" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L20" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N20" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O20" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P20" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q20" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,19 +2678,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -2698,9 +2698,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D21" s="10">
@@ -2748,12 +2748,12 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -2768,32 +2768,32 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K21" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L21" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N21" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O21" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P21" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q21" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,19 +2805,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W21" s="5" t="inlineStr">
@@ -2825,14 +2825,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z21" s="5" t="inlineStr">
@@ -2840,19 +2840,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,79 +2862,79 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J22" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K22" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L22" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M22" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N22" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O22" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P22" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R22" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J22" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="K22" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="L22" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="M22" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="N22" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="O22" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="P22" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="Q22" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="R22" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S22" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="T22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2947,9 +2947,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X22" s="4" t="inlineStr">
@@ -2957,9 +2957,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z22" s="5" t="inlineStr">
@@ -2967,19 +2967,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,25 +2989,25 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -3022,32 +3022,32 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K23" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L23" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N23" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O23" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P23" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q23" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3059,9 +3059,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T23" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U23" s="4" t="inlineStr">
@@ -3074,9 +3074,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X23" s="4" t="inlineStr">
@@ -3084,9 +3084,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z23" s="5" t="inlineStr">
@@ -3099,14 +3099,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D24" s="10">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
@@ -3149,32 +3149,32 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="K24" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="L24" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="N24" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="O24" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="P24" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="Q24" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3186,14 +3186,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T24" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V24" s="4" t="inlineStr">
@@ -3201,9 +3201,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,12 +3243,12 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D25" s="10">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
@@ -3276,32 +3276,32 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K25" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L25" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N25" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O25" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P25" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q25" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3313,14 +3313,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr">
@@ -3333,9 +3333,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y25" s="6" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,16 +3370,16 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -3407,28 +3407,28 @@
         </is>
       </c>
       <c r="J26" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K26" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L26" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N26" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O26" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P26" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q26" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3455,14 +3455,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y26" s="6" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D27" s="10">
@@ -3510,116 +3510,243 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J27" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K27" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L27" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M27" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N27" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O27" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P27" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R27" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S27" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC27" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13">
+        <v>1</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D28" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F27" s="0" t="inlineStr">
+      <c r="F28" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="H28" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I27" s="13" t="inlineStr">
+      <c r="I28" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J27" s="2">
+      <c r="J28" s="2">
         <v>698.2</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K28" s="2">
         <v>272.01</v>
       </c>
-      <c r="L27" s="2">
+      <c r="L28" s="2">
         <v>348.9</v>
       </c>
-      <c r="M27" s="3">
+      <c r="M28" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N27" s="3">
+      <c r="N28" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O27" s="2">
+      <c r="O28" s="2">
         <v>713.11</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P28" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q28" s="2">
         <v>395.5</v>
       </c>
-      <c r="R27" s="13" t="inlineStr">
+      <c r="R28" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S27" s="13" t="inlineStr">
+      <c r="S28" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC27" s="11" t="inlineStr">
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC28" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC27"/>
+  <autoFilter ref="A1:AC28"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -3647,6 +3774,7 @@
     <hyperlink ref="AC25" r:id="rId24"/>
     <hyperlink ref="AC26" r:id="rId25"/>
     <hyperlink ref="AC27" r:id="rId26"/>
+    <hyperlink ref="AC28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de ICE (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$29</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1973,79 +1973,79 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D15" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J15" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K15" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L15" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M15" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N15" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O15" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P15" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R15" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J15" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="K15" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="L15" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="M15" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="N15" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="O15" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="P15" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="Q15" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="R15" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S15" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
@@ -2053,14 +2053,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="V15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X15" s="6" t="inlineStr">
@@ -2073,9 +2073,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,16 +2100,16 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D16" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I16" s="13" t="inlineStr">
@@ -2137,28 +2137,28 @@
         </is>
       </c>
       <c r="J16" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K16" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L16" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N16" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O16" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P16" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q16" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2170,14 +2170,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr">
@@ -2210,14 +2210,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,25 +2227,25 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -2260,32 +2260,32 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J17" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K17" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L17" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M17" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N17" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O17" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P17" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q17" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2312,14 +2312,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y17" s="6" t="inlineStr">
@@ -2327,9 +2327,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA17" s="4" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,25 +2354,25 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J18" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K18" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L18" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M18" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N18" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O18" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P18" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q18" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2439,24 +2439,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D19" s="10">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
@@ -2514,36 +2514,36 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K19" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L19" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M19" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N19" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O19" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P19" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q19" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S19" s="13" t="inlineStr">
@@ -2551,9 +2551,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr">
@@ -2566,29 +2566,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB19" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -2636,37 +2636,37 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K20" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L20" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N20" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O20" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P20" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q20" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,9 +2678,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2693,19 +2693,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z20" s="5" t="inlineStr">
@@ -2713,19 +2713,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,25 +2735,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -2768,32 +2768,32 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K21" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L21" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N21" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O21" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P21" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q21" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,19 +2805,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W21" s="5" t="inlineStr">
@@ -2825,9 +2825,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y21" s="4" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D22" s="10">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2895,32 +2895,32 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K22" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L22" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M22" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N22" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O22" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P22" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q22" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2932,19 +2932,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -2952,14 +2952,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z22" s="5" t="inlineStr">
@@ -2967,19 +2967,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,79 +2989,79 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J23" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K23" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L23" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M23" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N23" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O23" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P23" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R23" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J23" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="K23" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="L23" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="M23" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="N23" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="O23" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="P23" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="Q23" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="R23" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S23" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U23" s="4" t="inlineStr">
@@ -3074,9 +3074,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X23" s="4" t="inlineStr">
@@ -3084,9 +3084,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z23" s="5" t="inlineStr">
@@ -3094,19 +3094,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,25 +3116,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -3149,32 +3149,32 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K24" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L24" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N24" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O24" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P24" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q24" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3186,9 +3186,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T24" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3201,9 +3201,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
@@ -3211,9 +3211,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z24" s="5" t="inlineStr">
@@ -3226,14 +3226,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,12 +3243,12 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D25" s="10">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
@@ -3276,32 +3276,32 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="K25" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="L25" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="N25" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="O25" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="P25" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="Q25" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3313,14 +3313,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T25" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr">
@@ -3328,9 +3328,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X25" s="4" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D26" s="10">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
@@ -3403,32 +3403,32 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K26" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L26" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N26" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O26" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P26" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q26" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3440,14 +3440,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr">
@@ -3460,9 +3460,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y26" s="6" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,16 +3497,16 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
@@ -3534,28 +3534,28 @@
         </is>
       </c>
       <c r="J27" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K27" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L27" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O27" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P27" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q27" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3582,14 +3582,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y27" s="6" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D28" s="10">
@@ -3637,116 +3637,243 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J28" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K28" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L28" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M28" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N28" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O28" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P28" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R28" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S28" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC28" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13">
+        <v>1</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D29" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F28" s="0" t="inlineStr">
+      <c r="F29" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="H29" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="I29" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J28" s="2">
+      <c r="J29" s="2">
         <v>698.2</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K29" s="2">
         <v>272.01</v>
       </c>
-      <c r="L28" s="2">
+      <c r="L29" s="2">
         <v>348.9</v>
       </c>
-      <c r="M28" s="3">
+      <c r="M29" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N28" s="3">
+      <c r="N29" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O28" s="2">
+      <c r="O29" s="2">
         <v>713.11</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P29" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q29" s="2">
         <v>395.5</v>
       </c>
-      <c r="R28" s="13" t="inlineStr">
+      <c r="R29" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S28" s="13" t="inlineStr">
+      <c r="S29" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC28" s="11" t="inlineStr">
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC29" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC28"/>
+  <autoFilter ref="A1:AC29"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -3775,6 +3902,7 @@
     <hyperlink ref="AC26" r:id="rId25"/>
     <hyperlink ref="AC27" r:id="rId26"/>
     <hyperlink ref="AC28" r:id="rId27"/>
+    <hyperlink ref="AC29" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Novo Nordisk (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$30</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -830,25 +830,25 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>NOVO B</t>
         </is>
       </c>
       <c r="D6" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -863,32 +863,32 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J6" s="2">
-        <v>21.51</v>
+        <v>249.9</v>
       </c>
       <c r="K6" s="2">
-        <v>25.08</v>
+        <v>315.19</v>
       </c>
       <c r="L6" s="2">
-        <v>30.22</v>
+        <v>350.05</v>
       </c>
       <c r="M6" s="3">
-        <v>0.179</v>
+        <v>0.308</v>
       </c>
       <c r="N6" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.44799999999999995</v>
       </c>
       <c r="O6" s="2">
-        <v>23.32</v>
+        <v>305.82</v>
       </c>
       <c r="P6" s="2">
-        <v>25.73</v>
+        <v>314.56</v>
       </c>
       <c r="Q6" s="2">
-        <v>31.95</v>
+        <v>377.91</v>
       </c>
       <c r="R6" s="13" t="inlineStr">
         <is>
@@ -900,9 +900,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -920,14 +920,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -940,14 +940,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC6" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -957,25 +957,25 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -985,41 +985,41 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J7" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="K7" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="L7" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="M7" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="N7" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="O7" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="P7" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="Q7" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S7" s="13" t="inlineStr">
@@ -1027,9 +1027,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
@@ -1042,9 +1042,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X7" s="4" t="inlineStr">
@@ -1052,9 +1052,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1067,14 +1067,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1084,25 +1084,25 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>On</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="D8" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1117,46 +1117,46 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="J8" s="2">
-        <v>123.73</v>
+        <v>26.48</v>
       </c>
       <c r="K8" s="2">
-        <v>151.16</v>
+        <v>27.68</v>
       </c>
       <c r="L8" s="2">
-        <v>164.85</v>
+        <v>36.62</v>
       </c>
       <c r="M8" s="3">
-        <v>0.268</v>
+        <v>0.045</v>
       </c>
       <c r="N8" s="3">
-        <v>0.379</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="O8" s="2">
-        <v>148.64</v>
+        <v>36.11</v>
       </c>
       <c r="P8" s="2">
-        <v>148.29</v>
+        <v>30.75</v>
       </c>
       <c r="Q8" s="2">
-        <v>181.24</v>
+        <v>40.69</v>
       </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S8" s="13" t="inlineStr">
+        <is>
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S8" s="13" t="inlineStr">
-        <is>
-          <t>Comprar</t>
-        </is>
-      </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1164,24 +1164,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D9" s="10">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1248,28 +1248,28 @@
         </is>
       </c>
       <c r="J9" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="K9" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="L9" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="M9" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="N9" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="O9" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="P9" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="Q9" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
@@ -1286,9 +1286,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V9" s="6" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,12 +1338,12 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D10" s="10">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1371,36 +1371,36 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J10" s="2">
-        <v>8.677</v>
+        <v>142.43</v>
       </c>
       <c r="K10" s="2">
-        <v>9.45</v>
+        <v>162.26</v>
       </c>
       <c r="L10" s="2">
-        <v>11.42</v>
+        <v>191.49</v>
       </c>
       <c r="M10" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.154</v>
       </c>
       <c r="N10" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.359</v>
       </c>
       <c r="O10" s="2">
-        <v>11.81</v>
+        <v>203.9</v>
       </c>
       <c r="P10" s="2">
-        <v>9.65</v>
+        <v>164.86</v>
       </c>
       <c r="Q10" s="2">
-        <v>12.54</v>
+        <v>208.83</v>
       </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S10" s="13" t="inlineStr">
@@ -1413,9 +1413,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V10" s="6" t="inlineStr">
@@ -1423,9 +1423,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X10" s="6" t="inlineStr">
@@ -1433,14 +1433,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA10" s="4" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,20 +1465,20 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D11" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
@@ -1502,28 +1502,28 @@
         </is>
       </c>
       <c r="J11" s="2">
-        <v>78.3</v>
+        <v>8.677</v>
       </c>
       <c r="K11" s="2">
-        <v>84.06</v>
+        <v>9.45</v>
       </c>
       <c r="L11" s="2">
-        <v>97.98</v>
+        <v>11.42</v>
       </c>
       <c r="M11" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="N11" s="3">
-        <v>0.271</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="O11" s="2">
-        <v>69.22</v>
+        <v>11.81</v>
       </c>
       <c r="P11" s="2">
-        <v>86.5</v>
+        <v>9.65</v>
       </c>
       <c r="Q11" s="2">
-        <v>110.62</v>
+        <v>12.54</v>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
@@ -1535,19 +1535,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -1555,9 +1555,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y11" s="6" t="inlineStr">
@@ -1565,9 +1565,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA11" s="4" t="inlineStr">
@@ -1575,14 +1575,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D12" s="10">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1629,28 +1629,28 @@
         </is>
       </c>
       <c r="J12" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="K12" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="L12" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="M12" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N12" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="O12" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="P12" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="Q12" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
@@ -1662,9 +1662,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -1677,19 +1677,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z12" s="4" t="inlineStr">
@@ -1702,14 +1702,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -1719,25 +1719,25 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D13" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1752,32 +1752,32 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J13" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="K13" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="L13" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="M13" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="N13" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="O13" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="P13" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="Q13" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
@@ -1789,19 +1789,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -1819,9 +1819,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA13" s="4" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,25 +1846,25 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D14" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1879,32 +1879,32 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J14" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K14" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L14" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M14" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N14" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O14" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P14" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q14" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1916,19 +1916,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W14" s="4" t="inlineStr">
@@ -1936,19 +1936,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1956,14 +1956,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D15" s="10">
@@ -1986,12 +1986,12 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2006,32 +2006,32 @@
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J15" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K15" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L15" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M15" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N15" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O15" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P15" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q15" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2043,19 +2043,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W15" s="4" t="inlineStr">
@@ -2063,19 +2063,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,79 +2100,79 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D16" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J16" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K16" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L16" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M16" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N16" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O16" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P16" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R16" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J16" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="K16" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="L16" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="M16" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="N16" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="O16" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="P16" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="Q16" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="R16" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S16" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
@@ -2180,14 +2180,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="V16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X16" s="6" t="inlineStr">
@@ -2200,9 +2200,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,16 +2227,16 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I17" s="13" t="inlineStr">
@@ -2264,28 +2264,28 @@
         </is>
       </c>
       <c r="J17" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K17" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L17" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N17" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O17" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P17" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q17" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2297,14 +2297,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,25 +2354,25 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J18" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K18" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L18" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M18" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N18" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O18" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P18" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q18" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2439,14 +2439,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y18" s="6" t="inlineStr">
@@ -2454,9 +2454,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2464,14 +2464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,25 +2481,25 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D19" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -2514,32 +2514,32 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K19" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L19" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M19" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N19" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O19" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P19" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q19" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2566,24 +2566,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,12 +2608,12 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D20" s="10">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
@@ -2641,36 +2641,36 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K20" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L20" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N20" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O20" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P20" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q20" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S20" s="13" t="inlineStr">
@@ -2678,9 +2678,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2693,29 +2693,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,25 +2735,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -2763,37 +2763,37 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K21" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L21" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N21" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O21" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P21" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q21" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,9 +2805,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
@@ -2820,19 +2820,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z21" s="5" t="inlineStr">
@@ -2840,19 +2840,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,25 +2862,25 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2895,32 +2895,32 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K22" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L22" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M22" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N22" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O22" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P22" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q22" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2932,19 +2932,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -2952,9 +2952,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y22" s="4" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D23" s="10">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3022,32 +3022,32 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K23" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L23" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N23" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O23" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P23" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q23" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3059,19 +3059,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W23" s="5" t="inlineStr">
@@ -3079,14 +3079,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z23" s="5" t="inlineStr">
@@ -3094,19 +3094,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,79 +3116,79 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J24" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K24" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L24" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N24" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O24" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P24" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R24" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J24" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="K24" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="L24" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="M24" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="N24" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="O24" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="P24" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="Q24" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="R24" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S24" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3201,9 +3201,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
@@ -3211,9 +3211,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z24" s="5" t="inlineStr">
@@ -3221,19 +3221,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,25 +3243,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -3276,32 +3276,32 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K25" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L25" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N25" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O25" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P25" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q25" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3313,9 +3313,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T25" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3328,9 +3328,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X25" s="4" t="inlineStr">
@@ -3338,9 +3338,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z25" s="5" t="inlineStr">
@@ -3353,14 +3353,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D26" s="10">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
@@ -3403,32 +3403,32 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>6220</v>
+        <v>299</v>
       </c>
       <c r="K26" s="2">
-        <v>4460.49</v>
+        <v>204.75</v>
       </c>
       <c r="L26" s="2">
-        <v>4713.09</v>
+        <v>239.87</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.266</v>
+        <v>-0.308</v>
       </c>
       <c r="N26" s="3">
-        <v>-0.225</v>
+        <v>-0.19</v>
       </c>
       <c r="O26" s="2">
-        <v>7278.89</v>
+        <v>397.27</v>
       </c>
       <c r="P26" s="2">
-        <v>4188.4</v>
+        <v>210.48</v>
       </c>
       <c r="Q26" s="2">
-        <v>4821.79</v>
+        <v>269.04</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3440,14 +3440,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T26" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr">
@@ -3455,9 +3455,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X26" s="4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D27" s="10">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K27" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L27" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O27" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P27" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q27" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3567,14 +3567,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V27" s="4" t="inlineStr">
@@ -3587,9 +3587,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y27" s="6" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,16 +3624,16 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -3661,28 +3661,28 @@
         </is>
       </c>
       <c r="J28" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K28" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L28" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O28" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P28" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q28" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3709,14 +3709,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y28" s="6" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D29" s="10">
@@ -3764,116 +3764,243 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J29" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K29" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L29" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M29" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N29" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O29" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P29" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R29" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S29" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC29" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13">
+        <v>1</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D30" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F29" s="0" t="inlineStr">
+      <c r="F30" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H29" s="13" t="inlineStr">
+      <c r="H30" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I29" s="13" t="inlineStr">
+      <c r="I30" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J29" s="2">
+      <c r="J30" s="2">
         <v>698.2</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K30" s="2">
         <v>272.01</v>
       </c>
-      <c r="L29" s="2">
+      <c r="L30" s="2">
         <v>348.9</v>
       </c>
-      <c r="M29" s="3">
+      <c r="M30" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N29" s="3">
+      <c r="N30" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O29" s="2">
+      <c r="O30" s="2">
         <v>713.11</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P30" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q30" s="2">
         <v>395.5</v>
       </c>
-      <c r="R29" s="13" t="inlineStr">
+      <c r="R30" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S29" s="13" t="inlineStr">
+      <c r="S30" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC29" s="11" t="inlineStr">
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC30" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC29"/>
+  <autoFilter ref="A1:AC30"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -3903,6 +4030,7 @@
     <hyperlink ref="AC27" r:id="rId26"/>
     <hyperlink ref="AC28" r:id="rId27"/>
     <hyperlink ref="AC29" r:id="rId28"/>
+    <hyperlink ref="AC30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Alphabet (Vender, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$31</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3497,25 +3497,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K27" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L27" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O27" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P27" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q27" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3567,14 +3567,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V27" s="4" t="inlineStr">
@@ -3582,9 +3582,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X27" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D28" s="10">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -3657,32 +3657,32 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K28" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L28" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O28" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P28" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q28" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3694,14 +3694,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V28" s="4" t="inlineStr">
@@ -3714,9 +3714,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y28" s="6" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,16 +3751,16 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
@@ -3788,28 +3788,28 @@
         </is>
       </c>
       <c r="J29" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K29" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L29" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O29" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P29" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q29" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3836,14 +3836,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y29" s="6" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,12 +3878,12 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D30" s="10">
@@ -3891,116 +3891,243 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J30" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K30" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L30" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M30" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N30" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O30" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P30" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R30" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S30" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC30" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13">
+        <v>1</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D31" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F30" s="0" t="inlineStr">
+      <c r="F31" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H30" s="13" t="inlineStr">
+      <c r="H31" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I30" s="13" t="inlineStr">
+      <c r="I31" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J30" s="2">
+      <c r="J31" s="2">
         <v>698.2</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K31" s="2">
         <v>272.01</v>
       </c>
-      <c r="L30" s="2">
+      <c r="L31" s="2">
         <v>348.9</v>
       </c>
-      <c r="M30" s="3">
+      <c r="M31" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N30" s="3">
+      <c r="N31" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O30" s="2">
+      <c r="O31" s="2">
         <v>713.11</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P31" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q31" s="2">
         <v>395.5</v>
       </c>
-      <c r="R30" s="13" t="inlineStr">
+      <c r="R31" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S30" s="13" t="inlineStr">
+      <c r="S31" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC30" s="11" t="inlineStr">
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC31" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC30"/>
+  <autoFilter ref="A1:AC31"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -4031,6 +4158,7 @@
     <hyperlink ref="AC28" r:id="rId27"/>
     <hyperlink ref="AC29" r:id="rId28"/>
     <hyperlink ref="AC30" r:id="rId29"/>
+    <hyperlink ref="AC31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Seguimiento con LVMH, Uber, Cochlear y Wolters Kluwer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$35</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -449,25 +449,25 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Lululemon</t>
+          <t>Wolters Kluwer</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>WKL</t>
         </is>
       </c>
       <c r="D3" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
+          <t>Países Bajos</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -482,32 +482,32 @@
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J3" s="2">
-        <v>93.61</v>
+        <v>71.78</v>
       </c>
       <c r="K3" s="2">
-        <v>132.71</v>
+        <v>113.57</v>
       </c>
       <c r="L3" s="2">
-        <v>146.21</v>
+        <v>135.3</v>
       </c>
       <c r="M3" s="3">
-        <v>0.418</v>
+        <v>0.618</v>
       </c>
       <c r="N3" s="3">
-        <v>0.562</v>
+        <v>0.9209999999999999</v>
       </c>
       <c r="O3" s="2">
-        <v>104.91</v>
+        <v>89.78</v>
       </c>
       <c r="P3" s="2">
-        <v>127.14</v>
+        <v>119.82</v>
       </c>
       <c r="Q3" s="2">
-        <v>162.3</v>
+        <v>153.32</v>
       </c>
       <c r="R3" s="13" t="inlineStr">
         <is>
@@ -519,9 +519,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T3" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr">
@@ -529,9 +529,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W3" s="4" t="inlineStr">
@@ -539,14 +539,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y3" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X3" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y3" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z3" s="4" t="inlineStr">
@@ -559,14 +559,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB3" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC3" s="11" t="inlineStr">
         <is>
-          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
+          <t>informes/wolters-kluwer-2026-10-08/Wolters Kluwer - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -576,12 +576,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>Lululemon</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="D4" s="10">
@@ -589,12 +589,12 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -609,32 +609,32 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J4" s="2">
-        <v>1137.5</v>
+        <v>93.61</v>
       </c>
       <c r="K4" s="2">
-        <v>1357.81</v>
+        <v>132.71</v>
       </c>
       <c r="L4" s="2">
-        <v>1747.71</v>
+        <v>146.21</v>
       </c>
       <c r="M4" s="3">
-        <v>0.2</v>
+        <v>0.418</v>
       </c>
       <c r="N4" s="3">
-        <v>0.5429999999999999</v>
+        <v>0.562</v>
       </c>
       <c r="O4" s="2">
-        <v>1939</v>
+        <v>104.91</v>
       </c>
       <c r="P4" s="2">
-        <v>1481.37</v>
+        <v>127.14</v>
       </c>
       <c r="Q4" s="2">
-        <v>1949.82</v>
+        <v>162.3</v>
       </c>
       <c r="R4" s="13" t="inlineStr">
         <is>
@@ -651,29 +651,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z4" s="4" t="inlineStr">
@@ -686,14 +686,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC4" s="11" t="inlineStr">
         <is>
-          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
+          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -703,12 +703,12 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="D5" s="10">
@@ -716,12 +716,12 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -736,32 +736,32 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J5" s="2">
-        <v>71.33</v>
+        <v>1137.5</v>
       </c>
       <c r="K5" s="2">
-        <v>91.77</v>
+        <v>1357.81</v>
       </c>
       <c r="L5" s="2">
-        <v>101.61</v>
+        <v>1747.71</v>
       </c>
       <c r="M5" s="3">
-        <v>0.316</v>
+        <v>0.2</v>
       </c>
       <c r="N5" s="3">
-        <v>0.45399999999999996</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="O5" s="2">
-        <v>96</v>
+        <v>1939</v>
       </c>
       <c r="P5" s="2">
-        <v>90.12</v>
+        <v>1481.37</v>
       </c>
       <c r="Q5" s="2">
-        <v>108.2</v>
+        <v>1949.82</v>
       </c>
       <c r="R5" s="13" t="inlineStr">
         <is>
@@ -773,14 +773,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V5" s="6" t="inlineStr">
@@ -788,19 +788,19 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="AC5" s="11" t="inlineStr">
         <is>
-          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
+          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -830,20 +830,20 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>NOVO B</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="D6" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
@@ -863,32 +863,32 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J6" s="2">
-        <v>249.9</v>
+        <v>71.33</v>
       </c>
       <c r="K6" s="2">
-        <v>315.19</v>
+        <v>91.77</v>
       </c>
       <c r="L6" s="2">
-        <v>350.05</v>
+        <v>101.61</v>
       </c>
       <c r="M6" s="3">
-        <v>0.308</v>
+        <v>0.316</v>
       </c>
       <c r="N6" s="3">
-        <v>0.44799999999999995</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="O6" s="2">
-        <v>305.82</v>
+        <v>96</v>
       </c>
       <c r="P6" s="2">
-        <v>314.56</v>
+        <v>90.12</v>
       </c>
       <c r="Q6" s="2">
-        <v>377.91</v>
+        <v>108.2</v>
       </c>
       <c r="R6" s="13" t="inlineStr">
         <is>
@@ -900,9 +900,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -910,9 +910,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W6" s="4" t="inlineStr">
@@ -920,14 +920,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="AC6" s="11" t="inlineStr">
         <is>
-          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -957,25 +957,25 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>NOVO B</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -990,32 +990,32 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J7" s="2">
-        <v>21.51</v>
+        <v>249.9</v>
       </c>
       <c r="K7" s="2">
-        <v>25.08</v>
+        <v>315.19</v>
       </c>
       <c r="L7" s="2">
-        <v>30.22</v>
+        <v>350.05</v>
       </c>
       <c r="M7" s="3">
-        <v>0.179</v>
+        <v>0.308</v>
       </c>
       <c r="N7" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.44799999999999995</v>
       </c>
       <c r="O7" s="2">
-        <v>23.32</v>
+        <v>305.82</v>
       </c>
       <c r="P7" s="2">
-        <v>25.73</v>
+        <v>314.56</v>
       </c>
       <c r="Q7" s="2">
-        <v>31.95</v>
+        <v>377.91</v>
       </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
@@ -1027,9 +1027,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
@@ -1047,14 +1047,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1067,14 +1067,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1084,25 +1084,25 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="D8" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1112,41 +1112,41 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J8" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="K8" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="L8" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="M8" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="N8" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="O8" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="P8" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="Q8" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S8" s="13" t="inlineStr">
@@ -1154,9 +1154,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1169,9 +1169,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X8" s="4" t="inlineStr">
@@ -1179,9 +1179,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1194,14 +1194,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1211,25 +1211,25 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>On</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="D9" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1244,46 +1244,46 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="J9" s="2">
-        <v>123.73</v>
+        <v>26.48</v>
       </c>
       <c r="K9" s="2">
-        <v>151.16</v>
+        <v>27.68</v>
       </c>
       <c r="L9" s="2">
-        <v>164.85</v>
+        <v>36.62</v>
       </c>
       <c r="M9" s="3">
-        <v>0.268</v>
+        <v>0.045</v>
       </c>
       <c r="N9" s="3">
-        <v>0.379</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="O9" s="2">
-        <v>148.64</v>
+        <v>36.11</v>
       </c>
       <c r="P9" s="2">
-        <v>148.29</v>
+        <v>30.75</v>
       </c>
       <c r="Q9" s="2">
-        <v>181.24</v>
+        <v>40.69</v>
       </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S9" s="13" t="inlineStr">
+        <is>
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S9" s="13" t="inlineStr">
-        <is>
-          <t>Comprar</t>
-        </is>
-      </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1291,24 +1291,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,12 +1338,12 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D10" s="10">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1375,28 +1375,28 @@
         </is>
       </c>
       <c r="J10" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="K10" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="L10" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="M10" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="N10" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="O10" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="P10" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="Q10" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
@@ -1413,9 +1413,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V10" s="6" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D11" s="10">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1498,36 +1498,36 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J11" s="2">
-        <v>8.677</v>
+        <v>142.43</v>
       </c>
       <c r="K11" s="2">
-        <v>9.45</v>
+        <v>162.26</v>
       </c>
       <c r="L11" s="2">
-        <v>11.42</v>
+        <v>191.49</v>
       </c>
       <c r="M11" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.154</v>
       </c>
       <c r="N11" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.359</v>
       </c>
       <c r="O11" s="2">
-        <v>11.81</v>
+        <v>203.9</v>
       </c>
       <c r="P11" s="2">
-        <v>9.65</v>
+        <v>164.86</v>
       </c>
       <c r="Q11" s="2">
-        <v>12.54</v>
+        <v>208.83</v>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S11" s="13" t="inlineStr">
@@ -1540,9 +1540,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V11" s="6" t="inlineStr">
@@ -1550,9 +1550,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X11" s="6" t="inlineStr">
@@ -1560,14 +1560,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA11" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1592,20 +1592,20 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D12" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
@@ -1629,28 +1629,28 @@
         </is>
       </c>
       <c r="J12" s="2">
-        <v>78.3</v>
+        <v>8.677</v>
       </c>
       <c r="K12" s="2">
-        <v>84.06</v>
+        <v>9.45</v>
       </c>
       <c r="L12" s="2">
-        <v>97.98</v>
+        <v>11.42</v>
       </c>
       <c r="M12" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="N12" s="3">
-        <v>0.271</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="O12" s="2">
-        <v>69.22</v>
+        <v>11.81</v>
       </c>
       <c r="P12" s="2">
-        <v>86.5</v>
+        <v>9.65</v>
       </c>
       <c r="Q12" s="2">
-        <v>110.62</v>
+        <v>12.54</v>
       </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
@@ -1662,19 +1662,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1682,9 +1682,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y12" s="6" t="inlineStr">
@@ -1692,9 +1692,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA12" s="4" t="inlineStr">
@@ -1702,14 +1702,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1719,25 +1719,25 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D13" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1756,28 +1756,28 @@
         </is>
       </c>
       <c r="J13" s="2">
-        <v>52.9</v>
+        <v>380.9</v>
       </c>
       <c r="K13" s="2">
-        <v>55.98</v>
+        <v>410</v>
       </c>
       <c r="L13" s="2">
-        <v>62.5</v>
+        <v>478.01</v>
       </c>
       <c r="M13" s="3">
-        <v>0.12</v>
+        <v>0.111</v>
       </c>
       <c r="N13" s="3">
-        <v>0.244</v>
+        <v>0.289</v>
       </c>
       <c r="O13" s="2">
-        <v>69.29</v>
+        <v>526.49</v>
       </c>
       <c r="P13" s="2">
-        <v>57.16</v>
+        <v>422.71</v>
       </c>
       <c r="Q13" s="2">
-        <v>65.83</v>
+        <v>530.95</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
@@ -1794,9 +1794,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V13" s="4" t="inlineStr">
@@ -1809,19 +1809,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA13" s="4" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,20 +1846,20 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D14" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -1879,32 +1879,32 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J14" s="2">
-        <v>3.97</v>
+        <v>78.3</v>
       </c>
       <c r="K14" s="2">
-        <v>3.76</v>
+        <v>84.06</v>
       </c>
       <c r="L14" s="2">
-        <v>4.53</v>
+        <v>97.98</v>
       </c>
       <c r="M14" s="3">
-        <v>-0.021</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N14" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.271</v>
       </c>
       <c r="O14" s="2">
-        <v>6.15</v>
+        <v>69.22</v>
       </c>
       <c r="P14" s="2">
-        <v>4.05</v>
+        <v>86.5</v>
       </c>
       <c r="Q14" s="2">
-        <v>5.05</v>
+        <v>110.62</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1921,34 +1921,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1956,14 +1956,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,25 +1973,25 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D15" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2010,28 +2010,28 @@
         </is>
       </c>
       <c r="J15" s="2">
-        <v>80.75</v>
+        <v>52.9</v>
       </c>
       <c r="K15" s="2">
-        <v>80.93</v>
+        <v>55.98</v>
       </c>
       <c r="L15" s="2">
-        <v>93.63</v>
+        <v>62.5</v>
       </c>
       <c r="M15" s="3">
-        <v>0.013999999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="N15" s="3">
-        <v>0.172</v>
+        <v>0.244</v>
       </c>
       <c r="O15" s="2">
-        <v>79.54</v>
+        <v>69.29</v>
       </c>
       <c r="P15" s="2">
-        <v>81.9</v>
+        <v>57.16</v>
       </c>
       <c r="Q15" s="2">
-        <v>98.17</v>
+        <v>65.83</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2048,9 +2048,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr">
@@ -2063,19 +2063,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,25 +2100,25 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D16" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2137,28 +2137,28 @@
         </is>
       </c>
       <c r="J16" s="2">
-        <v>152.59</v>
+        <v>3.97</v>
       </c>
       <c r="K16" s="2">
-        <v>160.42</v>
+        <v>3.76</v>
       </c>
       <c r="L16" s="2">
-        <v>173.73</v>
+        <v>4.53</v>
       </c>
       <c r="M16" s="3">
-        <v>0.064</v>
+        <v>-0.021</v>
       </c>
       <c r="N16" s="3">
-        <v>0.152</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O16" s="2">
-        <v>185.33</v>
+        <v>6.15</v>
       </c>
       <c r="P16" s="2">
-        <v>152.72</v>
+        <v>4.05</v>
       </c>
       <c r="Q16" s="2">
-        <v>186.57</v>
+        <v>5.05</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2195,9 +2195,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z16" s="6" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,20 +2227,20 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
@@ -2248,53 +2248,53 @@
           <t>Salud</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J17" s="2">
+        <v>80.75</v>
+      </c>
+      <c r="K17" s="2">
+        <v>80.93</v>
+      </c>
+      <c r="L17" s="2">
+        <v>93.63</v>
+      </c>
+      <c r="M17" s="3">
+        <v>0.013999999999999999</v>
+      </c>
+      <c r="N17" s="3">
+        <v>0.172</v>
+      </c>
+      <c r="O17" s="2">
+        <v>79.54</v>
+      </c>
+      <c r="P17" s="2">
+        <v>81.9</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>98.17</v>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J17" s="2">
-        <v>10.18</v>
-      </c>
-      <c r="K17" s="2">
-        <v>10.41</v>
-      </c>
-      <c r="L17" s="2">
-        <v>11.23</v>
-      </c>
-      <c r="M17" s="3">
-        <v>0.040999999999999995</v>
-      </c>
-      <c r="N17" s="3">
-        <v>0.122</v>
-      </c>
-      <c r="O17" s="2">
-        <v>14.33</v>
-      </c>
-      <c r="P17" s="2">
-        <v>9.92</v>
-      </c>
-      <c r="Q17" s="2">
-        <v>12.34</v>
-      </c>
-      <c r="R17" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S17" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T17" s="6" t="inlineStr">
@@ -2302,9 +2302,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr">
@@ -2312,19 +2312,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z17" s="5" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,74 +2354,74 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J18" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K18" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L18" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M18" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N18" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O18" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P18" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R18" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J18" s="2">
-        <v>59.72</v>
-      </c>
-      <c r="K18" s="2">
-        <v>58.59</v>
-      </c>
-      <c r="L18" s="2">
-        <v>66.22</v>
-      </c>
-      <c r="M18" s="3">
-        <v>-0.013999999999999999</v>
-      </c>
-      <c r="N18" s="3">
-        <v>0.114</v>
-      </c>
-      <c r="O18" s="2">
-        <v>67.12</v>
-      </c>
-      <c r="P18" s="2">
-        <v>57.83</v>
-      </c>
-      <c r="Q18" s="2">
-        <v>73.94</v>
-      </c>
-      <c r="R18" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S18" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -2429,19 +2429,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X18" s="6" t="inlineStr">
@@ -2454,9 +2454,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2464,14 +2464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D19" s="10">
@@ -2494,12 +2494,12 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -2514,32 +2514,32 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>2702.5</v>
+        <v>70.24</v>
       </c>
       <c r="K19" s="2">
-        <v>2888.64</v>
+        <v>73.56</v>
       </c>
       <c r="L19" s="2">
-        <v>2897.35</v>
+        <v>80.39</v>
       </c>
       <c r="M19" s="3">
-        <v>0.098</v>
+        <v>0.047</v>
       </c>
       <c r="N19" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.145</v>
       </c>
       <c r="O19" s="2">
-        <v>4077.5</v>
+        <v>100.86</v>
       </c>
       <c r="P19" s="2">
-        <v>2585.33</v>
+        <v>69.88</v>
       </c>
       <c r="Q19" s="2">
-        <v>3307.49</v>
+        <v>89.38</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2566,19 +2566,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z19" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,12 +2608,12 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D20" s="10">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -2636,37 +2636,37 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>26.82</v>
+        <v>10.18</v>
       </c>
       <c r="K20" s="2">
-        <v>25.71</v>
+        <v>10.41</v>
       </c>
       <c r="L20" s="2">
-        <v>27.88</v>
+        <v>11.23</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N20" s="3">
-        <v>0.04</v>
+        <v>0.122</v>
       </c>
       <c r="O20" s="2">
-        <v>39</v>
+        <v>14.33</v>
       </c>
       <c r="P20" s="2">
-        <v>24.22</v>
+        <v>9.92</v>
       </c>
       <c r="Q20" s="2">
-        <v>30.98</v>
+        <v>12.34</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,14 +2678,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr">
@@ -2693,24 +2693,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,20 +2735,20 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
@@ -2772,32 +2772,32 @@
         </is>
       </c>
       <c r="J21" s="2">
-        <v>577.5</v>
+        <v>59.72</v>
       </c>
       <c r="K21" s="2">
-        <v>466.62</v>
+        <v>58.59</v>
       </c>
       <c r="L21" s="2">
-        <v>564.55</v>
+        <v>66.22</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N21" s="3">
-        <v>0.005</v>
+        <v>0.114</v>
       </c>
       <c r="O21" s="2">
-        <v>795.86</v>
+        <v>67.12</v>
       </c>
       <c r="P21" s="2">
-        <v>504.42</v>
+        <v>57.83</v>
       </c>
       <c r="Q21" s="2">
-        <v>645.34</v>
+        <v>73.94</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S21" s="13" t="inlineStr">
@@ -2805,9 +2805,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
@@ -2840,19 +2840,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D22" s="10">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2890,41 +2890,41 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>529.76</v>
+        <v>2702.5</v>
       </c>
       <c r="K22" s="2">
-        <v>450.46</v>
+        <v>2888.64</v>
       </c>
       <c r="L22" s="2">
-        <v>511.38</v>
+        <v>2897.35</v>
       </c>
       <c r="M22" s="3">
-        <v>-0.14300000000000002</v>
+        <v>0.098</v>
       </c>
       <c r="N22" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O22" s="2">
-        <v>587.63</v>
+        <v>4077.5</v>
       </c>
       <c r="P22" s="2">
-        <v>447.76</v>
+        <v>2585.33</v>
       </c>
       <c r="Q22" s="2">
-        <v>568.48</v>
+        <v>3307.49</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S22" s="13" t="inlineStr">
@@ -2952,34 +2952,34 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D23" s="10">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3017,41 +3017,41 @@
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>16.22</v>
+        <v>26.82</v>
       </c>
       <c r="K23" s="2">
-        <v>13.97</v>
+        <v>25.71</v>
       </c>
       <c r="L23" s="2">
-        <v>14.66</v>
+        <v>27.88</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.077</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N23" s="3">
-        <v>-0.035</v>
+        <v>0.04</v>
       </c>
       <c r="O23" s="2">
-        <v>17.05</v>
+        <v>39</v>
       </c>
       <c r="P23" s="2">
-        <v>13.61</v>
+        <v>24.22</v>
       </c>
       <c r="Q23" s="2">
-        <v>16.41</v>
+        <v>30.98</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S23" s="13" t="inlineStr">
@@ -3059,54 +3059,54 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D24" s="10">
@@ -3129,12 +3129,12 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3144,37 +3144,37 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>81490</v>
+        <v>577.5</v>
       </c>
       <c r="K24" s="2">
-        <v>66566.47</v>
+        <v>466.62</v>
       </c>
       <c r="L24" s="2">
-        <v>75201.52</v>
+        <v>564.55</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N24" s="3">
-        <v>-0.07</v>
+        <v>0.005</v>
       </c>
       <c r="O24" s="2">
-        <v>97866.67</v>
+        <v>795.86</v>
       </c>
       <c r="P24" s="2">
-        <v>65834.24</v>
+        <v>504.42</v>
       </c>
       <c r="Q24" s="2">
-        <v>84206.58</v>
+        <v>645.34</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3186,9 +3186,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3201,14 +3201,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y24" s="6" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,79 +3243,79 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J25" s="2">
+        <v>529.76</v>
+      </c>
+      <c r="K25" s="2">
+        <v>450.46</v>
+      </c>
+      <c r="L25" s="2">
+        <v>511.38</v>
+      </c>
+      <c r="M25" s="3">
+        <v>-0.14300000000000002</v>
+      </c>
+      <c r="N25" s="3">
+        <v>-0.027999999999999997</v>
+      </c>
+      <c r="O25" s="2">
+        <v>587.63</v>
+      </c>
+      <c r="P25" s="2">
+        <v>447.76</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>568.48</v>
+      </c>
+      <c r="R25" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="J25" s="2">
-        <v>53.82</v>
-      </c>
-      <c r="K25" s="2">
-        <v>44.48</v>
-      </c>
-      <c r="L25" s="2">
-        <v>44.65</v>
-      </c>
-      <c r="M25" s="3">
-        <v>-0.151</v>
-      </c>
-      <c r="N25" s="3">
-        <v>-0.14800000000000002</v>
-      </c>
-      <c r="O25" s="2">
-        <v>60.39</v>
-      </c>
-      <c r="P25" s="2">
-        <v>39.85</v>
-      </c>
-      <c r="Q25" s="2">
-        <v>48.84</v>
-      </c>
-      <c r="R25" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S25" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3328,9 +3328,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X25" s="4" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D26" s="10">
@@ -3383,76 +3383,76 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J26" s="2">
+        <v>16.22</v>
+      </c>
+      <c r="K26" s="2">
+        <v>13.97</v>
+      </c>
+      <c r="L26" s="2">
+        <v>14.66</v>
+      </c>
+      <c r="M26" s="3">
+        <v>-0.077</v>
+      </c>
+      <c r="N26" s="3">
+        <v>-0.035</v>
+      </c>
+      <c r="O26" s="2">
+        <v>17.05</v>
+      </c>
+      <c r="P26" s="2">
+        <v>13.61</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>16.41</v>
+      </c>
+      <c r="R26" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I26" s="13" t="inlineStr">
-        <is>
-          <t>NOK</t>
-        </is>
-      </c>
-      <c r="J26" s="2">
-        <v>299</v>
-      </c>
-      <c r="K26" s="2">
-        <v>204.75</v>
-      </c>
-      <c r="L26" s="2">
-        <v>239.87</v>
-      </c>
-      <c r="M26" s="3">
-        <v>-0.308</v>
-      </c>
-      <c r="N26" s="3">
-        <v>-0.19</v>
-      </c>
-      <c r="O26" s="2">
-        <v>397.27</v>
-      </c>
-      <c r="P26" s="2">
-        <v>210.48</v>
-      </c>
-      <c r="Q26" s="2">
-        <v>269.04</v>
-      </c>
-      <c r="R26" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S26" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
-        </is>
-      </c>
-      <c r="T26" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3460,14 +3460,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z26" s="5" t="inlineStr">
@@ -3480,14 +3480,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,74 +3497,74 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J27" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K27" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L27" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M27" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N27" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O27" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P27" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R27" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J27" s="2">
-        <v>350.5</v>
-      </c>
-      <c r="K27" s="2">
-        <v>252.74</v>
-      </c>
-      <c r="L27" s="2">
-        <v>281.33</v>
-      </c>
-      <c r="M27" s="3">
-        <v>-0.276</v>
-      </c>
-      <c r="N27" s="3">
-        <v>-0.195</v>
-      </c>
-      <c r="O27" s="2">
-        <v>429.47</v>
-      </c>
-      <c r="P27" s="2">
-        <v>245.16</v>
-      </c>
-      <c r="Q27" s="2">
-        <v>313.65</v>
-      </c>
-      <c r="R27" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S27" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T27" s="4" t="inlineStr">
@@ -3602,9 +3602,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB27" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,25 +3624,25 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -3657,32 +3657,32 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>6220</v>
+        <v>129</v>
       </c>
       <c r="K28" s="2">
-        <v>4460.49</v>
+        <v>100.16</v>
       </c>
       <c r="L28" s="2">
-        <v>4713.09</v>
+        <v>115.11</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.266</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.225</v>
+        <v>-0.081</v>
       </c>
       <c r="O28" s="2">
-        <v>7278.89</v>
+        <v>137.09</v>
       </c>
       <c r="P28" s="2">
-        <v>4188.4</v>
+        <v>103.06</v>
       </c>
       <c r="Q28" s="2">
-        <v>4821.79</v>
+        <v>128.2</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3694,14 +3694,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V28" s="4" t="inlineStr">
@@ -3719,9 +3719,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z28" s="5" t="inlineStr">
@@ -3734,14 +3734,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,25 +3751,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
@@ -3784,32 +3784,32 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>253.14</v>
+        <v>53.82</v>
       </c>
       <c r="K29" s="2">
-        <v>168.18</v>
+        <v>44.48</v>
       </c>
       <c r="L29" s="2">
-        <v>168.18</v>
+        <v>44.65</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.335</v>
+        <v>-0.151</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.335</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O29" s="2">
-        <v>337.43</v>
+        <v>60.39</v>
       </c>
       <c r="P29" s="2">
-        <v>146.32</v>
+        <v>39.85</v>
       </c>
       <c r="Q29" s="2">
-        <v>187.18</v>
+        <v>48.84</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3821,9 +3821,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr">
@@ -3841,14 +3841,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z29" s="5" t="inlineStr">
@@ -3861,14 +3861,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,25 +3878,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
@@ -3911,32 +3911,32 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>404.76</v>
+        <v>299</v>
       </c>
       <c r="K30" s="2">
-        <v>222.49</v>
+        <v>204.75</v>
       </c>
       <c r="L30" s="2">
-        <v>222.49</v>
+        <v>239.87</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.45</v>
+        <v>-0.308</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.45</v>
+        <v>-0.19</v>
       </c>
       <c r="O30" s="2">
-        <v>477.21</v>
+        <v>397.27</v>
       </c>
       <c r="P30" s="2">
-        <v>193.34</v>
+        <v>210.48</v>
       </c>
       <c r="Q30" s="2">
-        <v>247.41</v>
+        <v>269.04</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,9 +3948,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T30" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,129 +4005,637 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
+          <t>Alphabet</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D31" s="10">
+        <v>46303</v>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>Servicios de comunicación</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J31" s="2">
+        <v>350.5</v>
+      </c>
+      <c r="K31" s="2">
+        <v>252.74</v>
+      </c>
+      <c r="L31" s="2">
+        <v>281.33</v>
+      </c>
+      <c r="M31" s="3">
+        <v>-0.276</v>
+      </c>
+      <c r="N31" s="3">
+        <v>-0.195</v>
+      </c>
+      <c r="O31" s="2">
+        <v>429.47</v>
+      </c>
+      <c r="P31" s="2">
+        <v>245.16</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>313.65</v>
+      </c>
+      <c r="R31" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S31" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC31" s="11" t="inlineStr">
+        <is>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13">
+        <v>1</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>Fanuc</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>6954</t>
+        </is>
+      </c>
+      <c r="D32" s="10">
+        <v>46302</v>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>Japón</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>Industria</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J32" s="2">
+        <v>6220</v>
+      </c>
+      <c r="K32" s="2">
+        <v>4460.49</v>
+      </c>
+      <c r="L32" s="2">
+        <v>4713.09</v>
+      </c>
+      <c r="M32" s="3">
+        <v>-0.266</v>
+      </c>
+      <c r="N32" s="3">
+        <v>-0.225</v>
+      </c>
+      <c r="O32" s="2">
+        <v>7278.89</v>
+      </c>
+      <c r="P32" s="2">
+        <v>4188.4</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>4821.79</v>
+      </c>
+      <c r="R32" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S32" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC32" s="11" t="inlineStr">
+        <is>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13">
+        <v>1</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>Vertiv</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="D33" s="10">
+        <v>46302</v>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>Industria</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J33" s="2">
+        <v>253.14</v>
+      </c>
+      <c r="K33" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="L33" s="2">
+        <v>168.18</v>
+      </c>
+      <c r="M33" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="N33" s="3">
+        <v>-0.335</v>
+      </c>
+      <c r="O33" s="2">
+        <v>337.43</v>
+      </c>
+      <c r="P33" s="2">
+        <v>146.32</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>187.18</v>
+      </c>
+      <c r="R33" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S33" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC33" s="11" t="inlineStr">
+        <is>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13">
+        <v>1</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>Intuitive</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="D34" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J34" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K34" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L34" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M34" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N34" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O34" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P34" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R34" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S34" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC34" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13">
+        <v>1</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>VACN</t>
         </is>
       </c>
-      <c r="D31" s="10">
+      <c r="D35" s="10">
         <v>46301</v>
       </c>
-      <c r="E31" s="0" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F31" s="0" t="inlineStr">
+      <c r="F35" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H31" s="13" t="inlineStr">
+      <c r="H35" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I31" s="13" t="inlineStr">
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J31" s="2">
+      <c r="J35" s="2">
         <v>698.2</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K35" s="2">
         <v>272.01</v>
       </c>
-      <c r="L31" s="2">
+      <c r="L35" s="2">
         <v>348.9</v>
       </c>
-      <c r="M31" s="3">
+      <c r="M35" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N31" s="3">
+      <c r="N35" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O31" s="2">
+      <c r="O35" s="2">
         <v>713.11</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P35" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q35" s="2">
         <v>395.5</v>
       </c>
-      <c r="R31" s="13" t="inlineStr">
+      <c r="R35" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S31" s="13" t="inlineStr">
+      <c r="S35" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC31" s="11" t="inlineStr">
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC35" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC31"/>
+  <autoFilter ref="A1:AC35"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -4159,6 +4667,10 @@
     <hyperlink ref="AC29" r:id="rId28"/>
     <hyperlink ref="AC30" r:id="rId29"/>
     <hyperlink ref="AC31" r:id="rId30"/>
+    <hyperlink ref="AC32" r:id="rId31"/>
+    <hyperlink ref="AC33" r:id="rId32"/>
+    <hyperlink ref="AC34" r:id="rId33"/>
+    <hyperlink ref="AC35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Evolution (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$36</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D13" s="10">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -1756,28 +1756,28 @@
         </is>
       </c>
       <c r="J13" s="2">
-        <v>380.9</v>
+        <v>72.2709</v>
       </c>
       <c r="K13" s="2">
-        <v>410</v>
+        <v>81.5</v>
       </c>
       <c r="L13" s="2">
-        <v>478.01</v>
+        <v>95.8</v>
       </c>
       <c r="M13" s="3">
-        <v>0.111</v>
+        <v>0.128</v>
       </c>
       <c r="N13" s="3">
-        <v>0.289</v>
+        <v>0.326</v>
       </c>
       <c r="O13" s="2">
-        <v>526.49</v>
+        <v>67.88</v>
       </c>
       <c r="P13" s="2">
-        <v>422.71</v>
+        <v>83.29</v>
       </c>
       <c r="Q13" s="2">
-        <v>530.95</v>
+        <v>103.75</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
@@ -1789,14 +1789,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V13" s="4" t="inlineStr">
@@ -1809,9 +1809,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y13" s="6" t="inlineStr">
@@ -1819,9 +1819,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA13" s="4" t="inlineStr">
@@ -1829,14 +1829,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,25 +1846,25 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D14" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1883,28 +1883,28 @@
         </is>
       </c>
       <c r="J14" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="K14" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="L14" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="M14" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="N14" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="O14" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="P14" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="Q14" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1916,14 +1916,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V14" s="4" t="inlineStr">
@@ -1931,14 +1931,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y14" s="6" t="inlineStr">
@@ -1946,9 +1946,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1956,14 +1956,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D15" s="10">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2010,28 +2010,28 @@
         </is>
       </c>
       <c r="J15" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="K15" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="L15" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="M15" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N15" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="O15" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="P15" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="Q15" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2043,9 +2043,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
@@ -2058,19 +2058,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,25 +2100,25 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D16" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2133,32 +2133,32 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J16" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="K16" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="L16" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="M16" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="N16" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="O16" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="P16" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="Q16" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2170,19 +2170,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W16" s="4" t="inlineStr">
@@ -2200,9 +2200,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,25 +2227,25 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2260,32 +2260,32 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J17" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K17" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L17" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M17" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N17" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O17" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P17" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q17" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2297,19 +2297,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W17" s="4" t="inlineStr">
@@ -2317,19 +2317,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA17" s="4" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D18" s="10">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J18" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K18" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L18" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M18" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N18" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O18" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P18" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q18" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2424,19 +2424,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2444,19 +2444,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2464,14 +2464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D19" s="10">
@@ -2499,56 +2499,56 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J19" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K19" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L19" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M19" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N19" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O19" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P19" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I19" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J19" s="2">
-        <v>70.24</v>
-      </c>
-      <c r="K19" s="2">
-        <v>73.56</v>
-      </c>
-      <c r="L19" s="2">
-        <v>80.39</v>
-      </c>
-      <c r="M19" s="3">
-        <v>0.047</v>
-      </c>
-      <c r="N19" s="3">
-        <v>0.145</v>
-      </c>
-      <c r="O19" s="2">
-        <v>100.86</v>
-      </c>
-      <c r="P19" s="2">
-        <v>69.88</v>
-      </c>
-      <c r="Q19" s="2">
-        <v>89.38</v>
-      </c>
-      <c r="R19" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S19" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T19" s="4" t="inlineStr">
@@ -2556,14 +2556,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2571,19 +2571,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -2636,37 +2636,37 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>10.18</v>
+        <v>70.24</v>
       </c>
       <c r="K20" s="2">
-        <v>10.41</v>
+        <v>73.56</v>
       </c>
       <c r="L20" s="2">
-        <v>11.23</v>
+        <v>80.39</v>
       </c>
       <c r="M20" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.047</v>
       </c>
       <c r="N20" s="3">
-        <v>0.122</v>
+        <v>0.145</v>
       </c>
       <c r="O20" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="P20" s="2">
-        <v>9.92</v>
+        <v>69.88</v>
       </c>
       <c r="Q20" s="2">
-        <v>12.34</v>
+        <v>89.38</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,14 +2678,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr">
@@ -2693,24 +2693,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,16 +2735,16 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
@@ -2772,28 +2772,28 @@
         </is>
       </c>
       <c r="J21" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K21" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L21" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N21" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O21" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P21" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q21" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,14 +2805,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V21" s="4" t="inlineStr">
@@ -2845,14 +2845,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,25 +2862,25 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2895,32 +2895,32 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K22" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L22" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M22" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N22" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O22" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P22" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q22" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2947,14 +2947,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y22" s="6" t="inlineStr">
@@ -2962,9 +2962,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA22" s="4" t="inlineStr">
@@ -2972,14 +2972,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,25 +2989,25 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3022,32 +3022,32 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K23" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L23" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N23" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O23" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P23" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q23" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3074,24 +3074,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA23" s="4" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D24" s="10">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
@@ -3149,36 +3149,36 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K24" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L24" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N24" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O24" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P24" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q24" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S24" s="13" t="inlineStr">
@@ -3186,9 +3186,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3201,29 +3201,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB24" s="4" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,25 +3243,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3271,37 +3271,37 @@
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K25" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L25" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N25" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O25" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P25" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q25" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3313,9 +3313,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3328,19 +3328,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z25" s="5" t="inlineStr">
@@ -3348,19 +3348,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,25 +3370,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3403,32 +3403,32 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K26" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L26" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N26" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O26" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P26" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q26" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3440,19 +3440,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3460,9 +3460,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y26" s="4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D27" s="10">
@@ -3510,12 +3510,12 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K27" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L27" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O27" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P27" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q27" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3567,19 +3567,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W27" s="5" t="inlineStr">
@@ -3587,14 +3587,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z27" s="5" t="inlineStr">
@@ -3602,19 +3602,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,74 +3624,74 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J28" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K28" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L28" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M28" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N28" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O28" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P28" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R28" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J28" s="2">
-        <v>129</v>
-      </c>
-      <c r="K28" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L28" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M28" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N28" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O28" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P28" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q28" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R28" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S28" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T28" s="4" t="inlineStr">
@@ -3709,9 +3709,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X28" s="4" t="inlineStr">
@@ -3719,9 +3719,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z28" s="5" t="inlineStr">
@@ -3729,19 +3729,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,25 +3751,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
@@ -3784,32 +3784,32 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K29" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L29" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O29" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P29" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q29" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3821,9 +3821,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,25 +3878,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
@@ -3911,32 +3911,32 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K30" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L30" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O30" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P30" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q30" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,9 +3948,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T30" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3963,9 +3963,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X30" s="4" t="inlineStr">
@@ -3973,9 +3973,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z30" s="5" t="inlineStr">
@@ -3988,14 +3988,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,25 +4005,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -4038,32 +4038,32 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K31" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L31" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O31" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P31" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q31" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -4075,9 +4075,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T31" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,25 +4132,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K32" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L32" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O32" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P32" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q32" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,14 +4202,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V32" s="4" t="inlineStr">
@@ -4217,9 +4217,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X32" s="4" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D33" s="10">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K33" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L33" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O33" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P33" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q33" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,14 +4329,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V33" s="4" t="inlineStr">
@@ -4349,9 +4349,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y33" s="6" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,16 +4386,16 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -4404,7 +4404,7 @@
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -4423,28 +4423,28 @@
         </is>
       </c>
       <c r="J34" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K34" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L34" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O34" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P34" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q34" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4471,14 +4471,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y34" s="6" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,12 +4513,12 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D35" s="10">
@@ -4526,116 +4526,243 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J35" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K35" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L35" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M35" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N35" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O35" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P35" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R35" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S35" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC35" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13">
+        <v>1</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D36" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F35" s="0" t="inlineStr">
+      <c r="F36" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H35" s="13" t="inlineStr">
+      <c r="H36" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr">
+      <c r="I36" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J35" s="2">
+      <c r="J36" s="2">
         <v>698.2</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K36" s="2">
         <v>272.01</v>
       </c>
-      <c r="L35" s="2">
+      <c r="L36" s="2">
         <v>348.9</v>
       </c>
-      <c r="M35" s="3">
+      <c r="M36" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N35" s="3">
+      <c r="N36" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O35" s="2">
+      <c r="O36" s="2">
         <v>713.11</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P36" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q36" s="2">
         <v>395.5</v>
       </c>
-      <c r="R35" s="13" t="inlineStr">
+      <c r="R36" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S35" s="13" t="inlineStr">
+      <c r="S36" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC35" s="11" t="inlineStr">
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC36" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC35"/>
+  <autoFilter ref="A1:AC36"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -4671,6 +4798,7 @@
     <hyperlink ref="AC33" r:id="rId32"/>
     <hyperlink ref="AC34" r:id="rId33"/>
     <hyperlink ref="AC35" r:id="rId34"/>
+    <hyperlink ref="AC36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Fluidra (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$37</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -576,25 +576,25 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Lululemon</t>
+          <t>Fluidra</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>FDR</t>
         </is>
       </c>
       <c r="D4" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -609,32 +609,32 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J4" s="2">
-        <v>93.61</v>
+        <v>17</v>
       </c>
       <c r="K4" s="2">
-        <v>132.71</v>
+        <v>22.22</v>
       </c>
       <c r="L4" s="2">
-        <v>146.21</v>
+        <v>26.89</v>
       </c>
       <c r="M4" s="3">
-        <v>0.418</v>
+        <v>0.345</v>
       </c>
       <c r="N4" s="3">
-        <v>0.562</v>
+        <v>0.62</v>
       </c>
       <c r="O4" s="2">
-        <v>104.91</v>
+        <v>26.03</v>
       </c>
       <c r="P4" s="2">
-        <v>127.14</v>
+        <v>23.89</v>
       </c>
       <c r="Q4" s="2">
-        <v>162.3</v>
+        <v>30.42</v>
       </c>
       <c r="R4" s="13" t="inlineStr">
         <is>
@@ -646,19 +646,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W4" s="4" t="inlineStr">
@@ -666,14 +666,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z4" s="4" t="inlineStr">
@@ -686,14 +686,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC4" s="11" t="inlineStr">
         <is>
-          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
+          <t>informes/fluidra-2026-10-08/Fluidra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -703,12 +703,12 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>Lululemon</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="D5" s="10">
@@ -716,12 +716,12 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -736,32 +736,32 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J5" s="2">
-        <v>1137.5</v>
+        <v>93.61</v>
       </c>
       <c r="K5" s="2">
-        <v>1357.81</v>
+        <v>132.71</v>
       </c>
       <c r="L5" s="2">
-        <v>1747.71</v>
+        <v>146.21</v>
       </c>
       <c r="M5" s="3">
-        <v>0.2</v>
+        <v>0.418</v>
       </c>
       <c r="N5" s="3">
-        <v>0.5429999999999999</v>
+        <v>0.562</v>
       </c>
       <c r="O5" s="2">
-        <v>1939</v>
+        <v>104.91</v>
       </c>
       <c r="P5" s="2">
-        <v>1481.37</v>
+        <v>127.14</v>
       </c>
       <c r="Q5" s="2">
-        <v>1949.82</v>
+        <v>162.3</v>
       </c>
       <c r="R5" s="13" t="inlineStr">
         <is>
@@ -778,29 +778,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
@@ -813,14 +813,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC5" s="11" t="inlineStr">
         <is>
-          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
+          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="D6" s="10">
@@ -843,12 +843,12 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -863,32 +863,32 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J6" s="2">
-        <v>71.33</v>
+        <v>1137.5</v>
       </c>
       <c r="K6" s="2">
-        <v>91.77</v>
+        <v>1357.81</v>
       </c>
       <c r="L6" s="2">
-        <v>101.61</v>
+        <v>1747.71</v>
       </c>
       <c r="M6" s="3">
-        <v>0.316</v>
+        <v>0.2</v>
       </c>
       <c r="N6" s="3">
-        <v>0.45399999999999996</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="O6" s="2">
-        <v>96</v>
+        <v>1939</v>
       </c>
       <c r="P6" s="2">
-        <v>90.12</v>
+        <v>1481.37</v>
       </c>
       <c r="Q6" s="2">
-        <v>108.2</v>
+        <v>1949.82</v>
       </c>
       <c r="R6" s="13" t="inlineStr">
         <is>
@@ -900,14 +900,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V6" s="6" t="inlineStr">
@@ -915,19 +915,19 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="AC6" s="11" t="inlineStr">
         <is>
-          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
+          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -957,20 +957,20 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>NOVO B</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
@@ -990,32 +990,32 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J7" s="2">
-        <v>249.9</v>
+        <v>71.33</v>
       </c>
       <c r="K7" s="2">
-        <v>315.19</v>
+        <v>91.77</v>
       </c>
       <c r="L7" s="2">
-        <v>350.05</v>
+        <v>101.61</v>
       </c>
       <c r="M7" s="3">
-        <v>0.308</v>
+        <v>0.316</v>
       </c>
       <c r="N7" s="3">
-        <v>0.44799999999999995</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="O7" s="2">
-        <v>305.82</v>
+        <v>96</v>
       </c>
       <c r="P7" s="2">
-        <v>314.56</v>
+        <v>90.12</v>
       </c>
       <c r="Q7" s="2">
-        <v>377.91</v>
+        <v>108.2</v>
       </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
@@ -1027,9 +1027,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
@@ -1037,9 +1037,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W7" s="4" t="inlineStr">
@@ -1047,14 +1047,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1084,25 +1084,25 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>NOVO B</t>
         </is>
       </c>
       <c r="D8" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1117,32 +1117,32 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J8" s="2">
-        <v>21.51</v>
+        <v>249.9</v>
       </c>
       <c r="K8" s="2">
-        <v>25.08</v>
+        <v>315.19</v>
       </c>
       <c r="L8" s="2">
-        <v>30.22</v>
+        <v>350.05</v>
       </c>
       <c r="M8" s="3">
-        <v>0.179</v>
+        <v>0.308</v>
       </c>
       <c r="N8" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.44799999999999995</v>
       </c>
       <c r="O8" s="2">
-        <v>23.32</v>
+        <v>305.82</v>
       </c>
       <c r="P8" s="2">
-        <v>25.73</v>
+        <v>314.56</v>
       </c>
       <c r="Q8" s="2">
-        <v>31.95</v>
+        <v>377.91</v>
       </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
@@ -1154,9 +1154,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1174,14 +1174,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1194,14 +1194,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1211,25 +1211,25 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="D9" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1239,41 +1239,41 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J9" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="K9" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="L9" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="M9" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="N9" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="O9" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="P9" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="Q9" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S9" s="13" t="inlineStr">
@@ -1281,9 +1281,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1296,9 +1296,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X9" s="4" t="inlineStr">
@@ -1306,9 +1306,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1321,14 +1321,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,25 +1338,25 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>On</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="D10" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1371,46 +1371,46 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="J10" s="2">
-        <v>123.73</v>
+        <v>26.48</v>
       </c>
       <c r="K10" s="2">
-        <v>151.16</v>
+        <v>27.68</v>
       </c>
       <c r="L10" s="2">
-        <v>164.85</v>
+        <v>36.62</v>
       </c>
       <c r="M10" s="3">
-        <v>0.268</v>
+        <v>0.045</v>
       </c>
       <c r="N10" s="3">
-        <v>0.379</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="O10" s="2">
-        <v>148.64</v>
+        <v>36.11</v>
       </c>
       <c r="P10" s="2">
-        <v>148.29</v>
+        <v>30.75</v>
       </c>
       <c r="Q10" s="2">
-        <v>181.24</v>
+        <v>40.69</v>
       </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S10" s="13" t="inlineStr">
+        <is>
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S10" s="13" t="inlineStr">
-        <is>
-          <t>Comprar</t>
-        </is>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1418,24 +1418,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D11" s="10">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1502,28 +1502,28 @@
         </is>
       </c>
       <c r="J11" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="K11" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="L11" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="M11" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="N11" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="O11" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="P11" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="Q11" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
@@ -1540,9 +1540,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V11" s="6" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D12" s="10">
@@ -1605,12 +1605,12 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1625,36 +1625,36 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J12" s="2">
-        <v>8.677</v>
+        <v>142.43</v>
       </c>
       <c r="K12" s="2">
-        <v>9.45</v>
+        <v>162.26</v>
       </c>
       <c r="L12" s="2">
-        <v>11.42</v>
+        <v>191.49</v>
       </c>
       <c r="M12" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.154</v>
       </c>
       <c r="N12" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.359</v>
       </c>
       <c r="O12" s="2">
-        <v>11.81</v>
+        <v>203.9</v>
       </c>
       <c r="P12" s="2">
-        <v>9.65</v>
+        <v>164.86</v>
       </c>
       <c r="Q12" s="2">
-        <v>12.54</v>
+        <v>208.83</v>
       </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S12" s="13" t="inlineStr">
@@ -1667,9 +1667,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V12" s="6" t="inlineStr">
@@ -1677,9 +1677,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X12" s="6" t="inlineStr">
@@ -1687,14 +1687,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA12" s="4" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Evolution</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>EVO</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D13" s="10">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1756,28 +1756,28 @@
         </is>
       </c>
       <c r="J13" s="2">
-        <v>72.2709</v>
+        <v>8.677</v>
       </c>
       <c r="K13" s="2">
-        <v>81.5</v>
+        <v>9.45</v>
       </c>
       <c r="L13" s="2">
-        <v>95.8</v>
+        <v>11.42</v>
       </c>
       <c r="M13" s="3">
-        <v>0.128</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="N13" s="3">
-        <v>0.326</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="O13" s="2">
-        <v>67.88</v>
+        <v>11.81</v>
       </c>
       <c r="P13" s="2">
-        <v>83.29</v>
+        <v>9.65</v>
       </c>
       <c r="Q13" s="2">
-        <v>103.75</v>
+        <v>12.54</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
@@ -1789,24 +1789,24 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X13" s="6" t="inlineStr">
@@ -1819,9 +1819,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z13" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA13" s="4" t="inlineStr">
@@ -1829,14 +1829,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D14" s="10">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -1883,28 +1883,28 @@
         </is>
       </c>
       <c r="J14" s="2">
-        <v>380.9</v>
+        <v>72.2709</v>
       </c>
       <c r="K14" s="2">
-        <v>410</v>
+        <v>81.5</v>
       </c>
       <c r="L14" s="2">
-        <v>478.01</v>
+        <v>95.8</v>
       </c>
       <c r="M14" s="3">
-        <v>0.111</v>
+        <v>0.128</v>
       </c>
       <c r="N14" s="3">
-        <v>0.289</v>
+        <v>0.326</v>
       </c>
       <c r="O14" s="2">
-        <v>526.49</v>
+        <v>67.88</v>
       </c>
       <c r="P14" s="2">
-        <v>422.71</v>
+        <v>83.29</v>
       </c>
       <c r="Q14" s="2">
-        <v>530.95</v>
+        <v>103.75</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1916,14 +1916,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V14" s="4" t="inlineStr">
@@ -1936,9 +1936,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y14" s="6" t="inlineStr">
@@ -1946,9 +1946,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1956,14 +1956,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,25 +1973,25 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D15" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2010,28 +2010,28 @@
         </is>
       </c>
       <c r="J15" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="K15" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="L15" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="M15" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="N15" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="O15" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="P15" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="Q15" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2043,14 +2043,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr">
@@ -2058,14 +2058,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y15" s="6" t="inlineStr">
@@ -2073,9 +2073,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D16" s="10">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2137,28 +2137,28 @@
         </is>
       </c>
       <c r="J16" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="K16" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="L16" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="M16" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N16" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="O16" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="P16" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="Q16" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2170,9 +2170,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2185,19 +2185,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z16" s="4" t="inlineStr">
@@ -2210,14 +2210,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,25 +2227,25 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2260,32 +2260,32 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J17" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="K17" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="L17" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="M17" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="N17" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="O17" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="P17" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="Q17" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2297,19 +2297,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W17" s="4" t="inlineStr">
@@ -2327,9 +2327,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA17" s="4" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,25 +2354,25 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J18" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K18" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L18" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M18" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N18" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O18" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P18" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q18" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2424,19 +2424,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2444,19 +2444,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2464,14 +2464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D19" s="10">
@@ -2494,12 +2494,12 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2514,32 +2514,32 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K19" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L19" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M19" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N19" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O19" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P19" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q19" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2551,19 +2551,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2571,19 +2571,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2591,14 +2591,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,12 +2608,12 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D20" s="10">
@@ -2626,56 +2626,56 @@
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J20" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K20" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L20" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M20" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N20" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O20" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P20" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J20" s="2">
-        <v>70.24</v>
-      </c>
-      <c r="K20" s="2">
-        <v>73.56</v>
-      </c>
-      <c r="L20" s="2">
-        <v>80.39</v>
-      </c>
-      <c r="M20" s="3">
-        <v>0.047</v>
-      </c>
-      <c r="N20" s="3">
-        <v>0.145</v>
-      </c>
-      <c r="O20" s="2">
-        <v>100.86</v>
-      </c>
-      <c r="P20" s="2">
-        <v>69.88</v>
-      </c>
-      <c r="Q20" s="2">
-        <v>89.38</v>
-      </c>
-      <c r="R20" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S20" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T20" s="4" t="inlineStr">
@@ -2683,14 +2683,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -2698,19 +2698,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,25 +2735,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -2763,37 +2763,37 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>10.18</v>
+        <v>70.24</v>
       </c>
       <c r="K21" s="2">
-        <v>10.41</v>
+        <v>73.56</v>
       </c>
       <c r="L21" s="2">
-        <v>11.23</v>
+        <v>80.39</v>
       </c>
       <c r="M21" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.047</v>
       </c>
       <c r="N21" s="3">
-        <v>0.122</v>
+        <v>0.145</v>
       </c>
       <c r="O21" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="P21" s="2">
-        <v>9.92</v>
+        <v>69.88</v>
       </c>
       <c r="Q21" s="2">
-        <v>12.34</v>
+        <v>89.38</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,14 +2805,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V21" s="4" t="inlineStr">
@@ -2820,24 +2820,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA21" s="4" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,16 +2862,16 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
@@ -2899,28 +2899,28 @@
         </is>
       </c>
       <c r="J22" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K22" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L22" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M22" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N22" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O22" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P22" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q22" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2932,14 +2932,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V22" s="4" t="inlineStr">
@@ -2972,14 +2972,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,25 +2989,25 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3022,32 +3022,32 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K23" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L23" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M23" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N23" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O23" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P23" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q23" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3074,14 +3074,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y23" s="6" t="inlineStr">
@@ -3089,9 +3089,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA23" s="4" t="inlineStr">
@@ -3099,14 +3099,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,25 +3116,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3149,32 +3149,32 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K24" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L24" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N24" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O24" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P24" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q24" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3201,24 +3201,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA24" s="4" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,12 +3243,12 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D25" s="10">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
@@ -3276,36 +3276,36 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K25" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L25" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N25" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O25" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P25" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q25" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S25" s="13" t="inlineStr">
@@ -3313,9 +3313,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3328,29 +3328,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB25" s="4" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,25 +3370,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3398,37 +3398,37 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K26" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L26" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N26" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O26" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P26" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q26" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3440,9 +3440,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
@@ -3455,19 +3455,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z26" s="5" t="inlineStr">
@@ -3475,19 +3475,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,25 +3497,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K27" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L27" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O27" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P27" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q27" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3567,19 +3567,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W27" s="5" t="inlineStr">
@@ -3587,9 +3587,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y27" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D28" s="10">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3657,32 +3657,32 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K28" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L28" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O28" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P28" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q28" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3694,19 +3694,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W28" s="5" t="inlineStr">
@@ -3714,14 +3714,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z28" s="5" t="inlineStr">
@@ -3729,19 +3729,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,74 +3751,74 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J29" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K29" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L29" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M29" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N29" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O29" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P29" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R29" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J29" s="2">
-        <v>129</v>
-      </c>
-      <c r="K29" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L29" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M29" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N29" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O29" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P29" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q29" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R29" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S29" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T29" s="4" t="inlineStr">
@@ -3836,9 +3836,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X29" s="4" t="inlineStr">
@@ -3846,9 +3846,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z29" s="5" t="inlineStr">
@@ -3856,19 +3856,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,25 +3878,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
@@ -3911,32 +3911,32 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K30" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L30" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O30" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P30" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q30" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,9 +3948,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,25 +4005,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -4038,32 +4038,32 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K31" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L31" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O31" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P31" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q31" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -4075,9 +4075,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T31" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr">
@@ -4090,9 +4090,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X31" s="4" t="inlineStr">
@@ -4100,9 +4100,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z31" s="5" t="inlineStr">
@@ -4115,14 +4115,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,25 +4132,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K32" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L32" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O32" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P32" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q32" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,9 +4202,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T32" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,25 +4259,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K33" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L33" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O33" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P33" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q33" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,14 +4329,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V33" s="4" t="inlineStr">
@@ -4344,9 +4344,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X33" s="4" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,12 +4386,12 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D34" s="10">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J34" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K34" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L34" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O34" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P34" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q34" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4456,14 +4456,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V34" s="4" t="inlineStr">
@@ -4476,9 +4476,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y34" s="6" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,16 +4513,16 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -4550,28 +4550,28 @@
         </is>
       </c>
       <c r="J35" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K35" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L35" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O35" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P35" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q35" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4598,14 +4598,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y35" s="6" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,12 +4640,12 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D36" s="10">
@@ -4653,116 +4653,243 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J36" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K36" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L36" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M36" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N36" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O36" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P36" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R36" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S36" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC36" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13">
+        <v>1</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D37" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F36" s="0" t="inlineStr">
+      <c r="F37" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H36" s="13" t="inlineStr">
+      <c r="H37" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I36" s="13" t="inlineStr">
+      <c r="I37" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J36" s="2">
+      <c r="J37" s="2">
         <v>698.2</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K37" s="2">
         <v>272.01</v>
       </c>
-      <c r="L36" s="2">
+      <c r="L37" s="2">
         <v>348.9</v>
       </c>
-      <c r="M36" s="3">
+      <c r="M37" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N36" s="3">
+      <c r="N37" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O36" s="2">
+      <c r="O37" s="2">
         <v>713.11</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P37" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q37" s="2">
         <v>395.5</v>
       </c>
-      <c r="R36" s="13" t="inlineStr">
+      <c r="R37" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S36" s="13" t="inlineStr">
+      <c r="S37" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC36" s="11" t="inlineStr">
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC37" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC36"/>
+  <autoFilter ref="A1:AC37"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -4799,6 +4926,7 @@
     <hyperlink ref="AC34" r:id="rId33"/>
     <hyperlink ref="AC35" r:id="rId34"/>
     <hyperlink ref="AC36" r:id="rId35"/>
+    <hyperlink ref="AC37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Krones (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$38</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -957,25 +957,25 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>Krones</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -990,32 +990,32 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J7" s="2">
-        <v>71.33</v>
+        <v>104</v>
       </c>
       <c r="K7" s="2">
-        <v>91.77</v>
+        <v>131.42</v>
       </c>
       <c r="L7" s="2">
-        <v>101.61</v>
+        <v>157.08</v>
       </c>
       <c r="M7" s="3">
-        <v>0.316</v>
+        <v>0.29100000000000004</v>
       </c>
       <c r="N7" s="3">
-        <v>0.45399999999999996</v>
+        <v>0.537</v>
       </c>
       <c r="O7" s="2">
-        <v>96</v>
+        <v>147.9</v>
       </c>
       <c r="P7" s="2">
-        <v>90.12</v>
+        <v>138.91</v>
       </c>
       <c r="Q7" s="2">
-        <v>108.2</v>
+        <v>173.47</v>
       </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
@@ -1037,24 +1037,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
+          <t>informes/krones-2026-10-09/Krones - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -1084,20 +1084,20 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>NOVO B</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="D8" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
@@ -1117,32 +1117,32 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J8" s="2">
-        <v>249.9</v>
+        <v>71.33</v>
       </c>
       <c r="K8" s="2">
-        <v>315.19</v>
+        <v>91.77</v>
       </c>
       <c r="L8" s="2">
-        <v>350.05</v>
+        <v>101.61</v>
       </c>
       <c r="M8" s="3">
-        <v>0.308</v>
+        <v>0.316</v>
       </c>
       <c r="N8" s="3">
-        <v>0.44799999999999995</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="O8" s="2">
-        <v>305.82</v>
+        <v>96</v>
       </c>
       <c r="P8" s="2">
-        <v>314.56</v>
+        <v>90.12</v>
       </c>
       <c r="Q8" s="2">
-        <v>377.91</v>
+        <v>108.2</v>
       </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
@@ -1154,9 +1154,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1164,9 +1164,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W8" s="4" t="inlineStr">
@@ -1174,14 +1174,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y8" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1211,25 +1211,25 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>NOVO B</t>
         </is>
       </c>
       <c r="D9" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1244,32 +1244,32 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J9" s="2">
-        <v>21.51</v>
+        <v>249.9</v>
       </c>
       <c r="K9" s="2">
-        <v>25.08</v>
+        <v>315.19</v>
       </c>
       <c r="L9" s="2">
-        <v>30.22</v>
+        <v>350.05</v>
       </c>
       <c r="M9" s="3">
-        <v>0.179</v>
+        <v>0.308</v>
       </c>
       <c r="N9" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.44799999999999995</v>
       </c>
       <c r="O9" s="2">
-        <v>23.32</v>
+        <v>305.82</v>
       </c>
       <c r="P9" s="2">
-        <v>25.73</v>
+        <v>314.56</v>
       </c>
       <c r="Q9" s="2">
-        <v>31.95</v>
+        <v>377.91</v>
       </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
@@ -1281,9 +1281,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1301,14 +1301,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1321,14 +1321,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,25 +1338,25 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="D10" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1366,41 +1366,41 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J10" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="K10" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="L10" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="M10" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="N10" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="O10" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="P10" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="Q10" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S10" s="13" t="inlineStr">
@@ -1408,9 +1408,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1423,9 +1423,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X10" s="4" t="inlineStr">
@@ -1433,9 +1433,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y10" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1448,14 +1448,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,25 +1465,25 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>On</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="D11" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1498,46 +1498,46 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="J11" s="2">
-        <v>123.73</v>
+        <v>26.48</v>
       </c>
       <c r="K11" s="2">
-        <v>151.16</v>
+        <v>27.68</v>
       </c>
       <c r="L11" s="2">
-        <v>164.85</v>
+        <v>36.62</v>
       </c>
       <c r="M11" s="3">
-        <v>0.268</v>
+        <v>0.045</v>
       </c>
       <c r="N11" s="3">
-        <v>0.379</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="O11" s="2">
-        <v>148.64</v>
+        <v>36.11</v>
       </c>
       <c r="P11" s="2">
-        <v>148.29</v>
+        <v>30.75</v>
       </c>
       <c r="Q11" s="2">
-        <v>181.24</v>
+        <v>40.69</v>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S11" s="13" t="inlineStr">
+        <is>
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S11" s="13" t="inlineStr">
-        <is>
-          <t>Comprar</t>
-        </is>
-      </c>
-      <c r="T11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U11" s="4" t="inlineStr">
@@ -1545,24 +1545,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z11" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D12" s="10">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1629,28 +1629,28 @@
         </is>
       </c>
       <c r="J12" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="K12" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="L12" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="M12" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="N12" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="O12" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="P12" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="Q12" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
@@ -1667,9 +1667,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U12" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V12" s="6" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D13" s="10">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1752,36 +1752,36 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J13" s="2">
-        <v>8.677</v>
+        <v>142.43</v>
       </c>
       <c r="K13" s="2">
-        <v>9.45</v>
+        <v>162.26</v>
       </c>
       <c r="L13" s="2">
-        <v>11.42</v>
+        <v>191.49</v>
       </c>
       <c r="M13" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.154</v>
       </c>
       <c r="N13" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.359</v>
       </c>
       <c r="O13" s="2">
-        <v>11.81</v>
+        <v>203.9</v>
       </c>
       <c r="P13" s="2">
-        <v>9.65</v>
+        <v>164.86</v>
       </c>
       <c r="Q13" s="2">
-        <v>12.54</v>
+        <v>208.83</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S13" s="13" t="inlineStr">
@@ -1794,9 +1794,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V13" s="6" t="inlineStr">
@@ -1804,9 +1804,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X13" s="6" t="inlineStr">
@@ -1814,14 +1814,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA13" s="4" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>Evolution</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>EVO</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D14" s="10">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1883,28 +1883,28 @@
         </is>
       </c>
       <c r="J14" s="2">
-        <v>72.2709</v>
+        <v>8.677</v>
       </c>
       <c r="K14" s="2">
-        <v>81.5</v>
+        <v>9.45</v>
       </c>
       <c r="L14" s="2">
-        <v>95.8</v>
+        <v>11.42</v>
       </c>
       <c r="M14" s="3">
-        <v>0.128</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="N14" s="3">
-        <v>0.326</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="O14" s="2">
-        <v>67.88</v>
+        <v>11.81</v>
       </c>
       <c r="P14" s="2">
-        <v>83.29</v>
+        <v>9.65</v>
       </c>
       <c r="Q14" s="2">
-        <v>103.75</v>
+        <v>12.54</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
@@ -1916,24 +1916,24 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X14" s="6" t="inlineStr">
@@ -1946,9 +1946,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z14" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z14" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1956,14 +1956,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D15" s="10">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -2010,28 +2010,28 @@
         </is>
       </c>
       <c r="J15" s="2">
-        <v>380.9</v>
+        <v>72.2709</v>
       </c>
       <c r="K15" s="2">
-        <v>410</v>
+        <v>81.5</v>
       </c>
       <c r="L15" s="2">
-        <v>478.01</v>
+        <v>95.8</v>
       </c>
       <c r="M15" s="3">
-        <v>0.111</v>
+        <v>0.128</v>
       </c>
       <c r="N15" s="3">
-        <v>0.289</v>
+        <v>0.326</v>
       </c>
       <c r="O15" s="2">
-        <v>526.49</v>
+        <v>67.88</v>
       </c>
       <c r="P15" s="2">
-        <v>422.71</v>
+        <v>83.29</v>
       </c>
       <c r="Q15" s="2">
-        <v>530.95</v>
+        <v>103.75</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2043,14 +2043,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr">
@@ -2063,9 +2063,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y15" s="6" t="inlineStr">
@@ -2073,9 +2073,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,25 +2100,25 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D16" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2137,28 +2137,28 @@
         </is>
       </c>
       <c r="J16" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="K16" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="L16" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="M16" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="N16" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="O16" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="P16" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="Q16" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2170,14 +2170,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr">
@@ -2185,14 +2185,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y16" s="6" t="inlineStr">
@@ -2200,9 +2200,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2210,14 +2210,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,12 +2227,12 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D17" s="10">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2264,28 +2264,28 @@
         </is>
       </c>
       <c r="J17" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="K17" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="L17" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="M17" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N17" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="O17" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="P17" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="Q17" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2297,9 +2297,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
@@ -2312,19 +2312,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z17" s="4" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,25 +2354,25 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J18" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="K18" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="L18" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="M18" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="N18" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="O18" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="P18" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="Q18" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2424,19 +2424,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2454,9 +2454,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA18" s="4" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,25 +2481,25 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D19" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2514,32 +2514,32 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K19" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L19" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M19" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N19" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O19" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P19" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q19" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2551,19 +2551,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2571,19 +2571,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2591,14 +2591,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,12 +2608,12 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D20" s="10">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2641,32 +2641,32 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K20" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L20" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M20" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N20" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O20" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P20" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q20" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,19 +2678,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -2698,19 +2698,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2718,14 +2718,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D21" s="10">
@@ -2753,56 +2753,56 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J21" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K21" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L21" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M21" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N21" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O21" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P21" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R21" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J21" s="2">
-        <v>70.24</v>
-      </c>
-      <c r="K21" s="2">
-        <v>73.56</v>
-      </c>
-      <c r="L21" s="2">
-        <v>80.39</v>
-      </c>
-      <c r="M21" s="3">
-        <v>0.047</v>
-      </c>
-      <c r="N21" s="3">
-        <v>0.145</v>
-      </c>
-      <c r="O21" s="2">
-        <v>100.86</v>
-      </c>
-      <c r="P21" s="2">
-        <v>69.88</v>
-      </c>
-      <c r="Q21" s="2">
-        <v>89.38</v>
-      </c>
-      <c r="R21" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S21" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T21" s="4" t="inlineStr">
@@ -2810,14 +2810,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2825,19 +2825,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA21" s="4" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,25 +2862,25 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -2890,37 +2890,37 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>10.18</v>
+        <v>70.24</v>
       </c>
       <c r="K22" s="2">
-        <v>10.41</v>
+        <v>73.56</v>
       </c>
       <c r="L22" s="2">
-        <v>11.23</v>
+        <v>80.39</v>
       </c>
       <c r="M22" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.047</v>
       </c>
       <c r="N22" s="3">
-        <v>0.122</v>
+        <v>0.145</v>
       </c>
       <c r="O22" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="P22" s="2">
-        <v>9.92</v>
+        <v>69.88</v>
       </c>
       <c r="Q22" s="2">
-        <v>12.34</v>
+        <v>89.38</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2932,14 +2932,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V22" s="4" t="inlineStr">
@@ -2947,24 +2947,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA22" s="4" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,16 +2989,16 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
@@ -3026,28 +3026,28 @@
         </is>
       </c>
       <c r="J23" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K23" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L23" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N23" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O23" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P23" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q23" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3059,14 +3059,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V23" s="4" t="inlineStr">
@@ -3099,14 +3099,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,25 +3116,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3149,32 +3149,32 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K24" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L24" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M24" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N24" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O24" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P24" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q24" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3201,14 +3201,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y24" s="6" t="inlineStr">
@@ -3216,9 +3216,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA24" s="4" t="inlineStr">
@@ -3226,14 +3226,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,25 +3243,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3276,32 +3276,32 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K25" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L25" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N25" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O25" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P25" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q25" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3328,24 +3328,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA25" s="4" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,12 +3370,12 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D26" s="10">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
@@ -3403,36 +3403,36 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K26" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L26" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N26" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O26" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P26" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q26" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S26" s="13" t="inlineStr">
@@ -3440,9 +3440,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
@@ -3455,29 +3455,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB26" s="4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,25 +3497,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3525,37 +3525,37 @@
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K27" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L27" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O27" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P27" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q27" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3567,9 +3567,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U27" s="4" t="inlineStr">
@@ -3582,19 +3582,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z27" s="5" t="inlineStr">
@@ -3602,19 +3602,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,25 +3624,25 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3657,32 +3657,32 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K28" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L28" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O28" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P28" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q28" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3694,19 +3694,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W28" s="5" t="inlineStr">
@@ -3714,9 +3714,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y28" s="4" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D29" s="10">
@@ -3764,12 +3764,12 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3784,32 +3784,32 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K29" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L29" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O29" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P29" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q29" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3821,19 +3821,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W29" s="5" t="inlineStr">
@@ -3841,14 +3841,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z29" s="5" t="inlineStr">
@@ -3856,19 +3856,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,74 +3878,74 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J30" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K30" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L30" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M30" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N30" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O30" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P30" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R30" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J30" s="2">
-        <v>129</v>
-      </c>
-      <c r="K30" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L30" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M30" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N30" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O30" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P30" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q30" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R30" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T30" s="4" t="inlineStr">
@@ -3963,9 +3963,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X30" s="4" t="inlineStr">
@@ -3973,9 +3973,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z30" s="5" t="inlineStr">
@@ -3983,19 +3983,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,25 +4005,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -4038,32 +4038,32 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K31" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L31" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O31" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P31" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q31" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -4075,9 +4075,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,25 +4132,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K32" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L32" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O32" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P32" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q32" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,9 +4202,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T32" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -4217,9 +4217,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X32" s="4" t="inlineStr">
@@ -4227,9 +4227,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z32" s="5" t="inlineStr">
@@ -4242,14 +4242,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,25 +4259,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K33" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L33" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O33" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P33" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q33" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,9 +4329,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T33" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,25 +4386,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J34" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K34" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L34" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O34" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P34" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q34" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4456,14 +4456,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V34" s="4" t="inlineStr">
@@ -4471,9 +4471,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X34" s="4" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,12 +4513,12 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D35" s="10">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -4546,32 +4546,32 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J35" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K35" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L35" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O35" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P35" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q35" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4583,14 +4583,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V35" s="4" t="inlineStr">
@@ -4603,9 +4603,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y35" s="6" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,16 +4640,16 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -4677,28 +4677,28 @@
         </is>
       </c>
       <c r="J36" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K36" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L36" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M36" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O36" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P36" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q36" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R36" s="13" t="inlineStr">
         <is>
@@ -4725,14 +4725,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y36" s="6" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4767,12 +4767,12 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D37" s="10">
@@ -4780,116 +4780,243 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J37" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K37" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L37" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M37" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N37" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O37" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P37" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R37" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S37" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC37" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13">
+        <v>1</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D38" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F37" s="0" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H37" s="13" t="inlineStr">
+      <c r="H38" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I37" s="13" t="inlineStr">
+      <c r="I38" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J37" s="2">
+      <c r="J38" s="2">
         <v>698.2</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K38" s="2">
         <v>272.01</v>
       </c>
-      <c r="L37" s="2">
+      <c r="L38" s="2">
         <v>348.9</v>
       </c>
-      <c r="M37" s="3">
+      <c r="M38" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N37" s="3">
+      <c r="N38" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O37" s="2">
+      <c r="O38" s="2">
         <v>713.11</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P38" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q38" s="2">
         <v>395.5</v>
       </c>
-      <c r="R37" s="13" t="inlineStr">
+      <c r="R38" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S37" s="13" t="inlineStr">
+      <c r="S38" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC37" s="11" t="inlineStr">
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC38" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC37"/>
+  <autoFilter ref="A1:AC38"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -4927,6 +5054,7 @@
     <hyperlink ref="AC35" r:id="rId34"/>
     <hyperlink ref="AC36" r:id="rId35"/>
     <hyperlink ref="AC37" r:id="rId36"/>
+    <hyperlink ref="AC38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Fielmann (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$39</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -576,25 +576,25 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Fluidra</t>
+          <t>Fielmann</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>FDR</t>
+          <t>FIE</t>
         </is>
       </c>
       <c r="D4" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -613,28 +613,28 @@
         </is>
       </c>
       <c r="J4" s="2">
-        <v>17</v>
+        <v>37.15</v>
       </c>
       <c r="K4" s="2">
-        <v>22.22</v>
+        <v>49.13</v>
       </c>
       <c r="L4" s="2">
-        <v>26.89</v>
+        <v>59.79</v>
       </c>
       <c r="M4" s="3">
-        <v>0.345</v>
+        <v>0.36</v>
       </c>
       <c r="N4" s="3">
-        <v>0.62</v>
+        <v>0.647</v>
       </c>
       <c r="O4" s="2">
-        <v>26.03</v>
+        <v>55.25</v>
       </c>
       <c r="P4" s="2">
-        <v>23.89</v>
+        <v>51.14</v>
       </c>
       <c r="Q4" s="2">
-        <v>30.42</v>
+        <v>64.46</v>
       </c>
       <c r="R4" s="13" t="inlineStr">
         <is>
@@ -646,19 +646,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W4" s="4" t="inlineStr">
@@ -666,14 +666,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y4" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z4" s="4" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="AC4" s="11" t="inlineStr">
         <is>
-          <t>informes/fluidra-2026-10-08/Fluidra - 2026-10-08.pdf</t>
+          <t>informes/fielmann-2026-10-09/Fielmann Group - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -703,25 +703,25 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Lululemon</t>
+          <t>Fluidra</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>FDR</t>
         </is>
       </c>
       <c r="D5" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -736,32 +736,32 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J5" s="2">
-        <v>93.61</v>
+        <v>17</v>
       </c>
       <c r="K5" s="2">
-        <v>132.71</v>
+        <v>22.22</v>
       </c>
       <c r="L5" s="2">
-        <v>146.21</v>
+        <v>26.89</v>
       </c>
       <c r="M5" s="3">
-        <v>0.418</v>
+        <v>0.345</v>
       </c>
       <c r="N5" s="3">
-        <v>0.562</v>
+        <v>0.62</v>
       </c>
       <c r="O5" s="2">
-        <v>104.91</v>
+        <v>26.03</v>
       </c>
       <c r="P5" s="2">
-        <v>127.14</v>
+        <v>23.89</v>
       </c>
       <c r="Q5" s="2">
-        <v>162.3</v>
+        <v>30.42</v>
       </c>
       <c r="R5" s="13" t="inlineStr">
         <is>
@@ -773,19 +773,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W5" s="4" t="inlineStr">
@@ -793,14 +793,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X5" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X5" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
@@ -813,14 +813,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB5" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB5" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC5" s="11" t="inlineStr">
         <is>
-          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
+          <t>informes/fluidra-2026-10-08/Fluidra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>Lululemon</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>DSV</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="D6" s="10">
@@ -843,12 +843,12 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos (sede operativa en Vancouver, Canadá)</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -863,32 +863,32 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J6" s="2">
-        <v>1137.5</v>
+        <v>93.61</v>
       </c>
       <c r="K6" s="2">
-        <v>1357.81</v>
+        <v>132.71</v>
       </c>
       <c r="L6" s="2">
-        <v>1747.71</v>
+        <v>146.21</v>
       </c>
       <c r="M6" s="3">
-        <v>0.2</v>
+        <v>0.418</v>
       </c>
       <c r="N6" s="3">
-        <v>0.5429999999999999</v>
+        <v>0.562</v>
       </c>
       <c r="O6" s="2">
-        <v>1939</v>
+        <v>104.91</v>
       </c>
       <c r="P6" s="2">
-        <v>1481.37</v>
+        <v>127.14</v>
       </c>
       <c r="Q6" s="2">
-        <v>1949.82</v>
+        <v>162.3</v>
       </c>
       <c r="R6" s="13" t="inlineStr">
         <is>
@@ -905,29 +905,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y6" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X6" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -940,14 +940,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB6" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB6" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC6" s="11" t="inlineStr">
         <is>
-          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
+          <t>informes/lululemon-2026-10-07/Lululemon - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -957,20 +957,20 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Krones</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>DSV</t>
         </is>
       </c>
       <c r="D7" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
@@ -990,32 +990,32 @@
       </c>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J7" s="2">
-        <v>104</v>
+        <v>1137.5</v>
       </c>
       <c r="K7" s="2">
-        <v>131.42</v>
+        <v>1357.81</v>
       </c>
       <c r="L7" s="2">
-        <v>157.08</v>
+        <v>1747.71</v>
       </c>
       <c r="M7" s="3">
-        <v>0.29100000000000004</v>
+        <v>0.2</v>
       </c>
       <c r="N7" s="3">
-        <v>0.537</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="O7" s="2">
-        <v>147.9</v>
+        <v>1939</v>
       </c>
       <c r="P7" s="2">
-        <v>138.91</v>
+        <v>1481.37</v>
       </c>
       <c r="Q7" s="2">
-        <v>173.47</v>
+        <v>1949.82</v>
       </c>
       <c r="R7" s="13" t="inlineStr">
         <is>
@@ -1027,19 +1027,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T7" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W7" s="6" t="inlineStr">
@@ -1052,9 +1052,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y7" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="AC7" s="11" t="inlineStr">
         <is>
-          <t>informes/krones-2026-10-09/Krones - 2026-10-09.pdf</t>
+          <t>informes/dsv-2026-10-07/DSV - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1084,25 +1084,25 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>Krones</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="D8" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1117,32 +1117,32 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J8" s="2">
-        <v>71.33</v>
+        <v>104</v>
       </c>
       <c r="K8" s="2">
-        <v>91.77</v>
+        <v>131.42</v>
       </c>
       <c r="L8" s="2">
-        <v>101.61</v>
+        <v>157.08</v>
       </c>
       <c r="M8" s="3">
-        <v>0.316</v>
+        <v>0.29100000000000004</v>
       </c>
       <c r="N8" s="3">
-        <v>0.45399999999999996</v>
+        <v>0.537</v>
       </c>
       <c r="O8" s="2">
-        <v>96</v>
+        <v>147.9</v>
       </c>
       <c r="P8" s="2">
-        <v>90.12</v>
+        <v>138.91</v>
       </c>
       <c r="Q8" s="2">
-        <v>108.2</v>
+        <v>173.47</v>
       </c>
       <c r="R8" s="13" t="inlineStr">
         <is>
@@ -1164,24 +1164,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X8" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="AC8" s="11" t="inlineStr">
         <is>
-          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
+          <t>informes/krones-2026-10-09/Krones - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -1211,20 +1211,20 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>NOVO B</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="D9" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>Dinamarca</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
@@ -1244,32 +1244,32 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>DKK</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J9" s="2">
-        <v>249.9</v>
+        <v>71.33</v>
       </c>
       <c r="K9" s="2">
-        <v>315.19</v>
+        <v>91.77</v>
       </c>
       <c r="L9" s="2">
-        <v>350.05</v>
+        <v>101.61</v>
       </c>
       <c r="M9" s="3">
-        <v>0.308</v>
+        <v>0.316</v>
       </c>
       <c r="N9" s="3">
-        <v>0.44799999999999995</v>
+        <v>0.45399999999999996</v>
       </c>
       <c r="O9" s="2">
-        <v>305.82</v>
+        <v>96</v>
       </c>
       <c r="P9" s="2">
-        <v>314.56</v>
+        <v>90.12</v>
       </c>
       <c r="Q9" s="2">
-        <v>377.91</v>
+        <v>108.2</v>
       </c>
       <c r="R9" s="13" t="inlineStr">
         <is>
@@ -1281,9 +1281,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
@@ -1291,9 +1291,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W9" s="4" t="inlineStr">
@@ -1301,14 +1301,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X9" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z9" s="4" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="AC9" s="11" t="inlineStr">
         <is>
-          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
+          <t>informes/zoetis-2026-10-07/Zoetis - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,25 +1338,25 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Dassault Systèmes</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>DSY</t>
+          <t>NOVO B</t>
         </is>
       </c>
       <c r="D10" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Dinamarca</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1371,32 +1371,32 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>DKK</t>
         </is>
       </c>
       <c r="J10" s="2">
-        <v>21.51</v>
+        <v>249.9</v>
       </c>
       <c r="K10" s="2">
-        <v>25.08</v>
+        <v>315.19</v>
       </c>
       <c r="L10" s="2">
-        <v>30.22</v>
+        <v>350.05</v>
       </c>
       <c r="M10" s="3">
-        <v>0.179</v>
+        <v>0.308</v>
       </c>
       <c r="N10" s="3">
-        <v>0.41700000000000004</v>
+        <v>0.44799999999999995</v>
       </c>
       <c r="O10" s="2">
-        <v>23.32</v>
+        <v>305.82</v>
       </c>
       <c r="P10" s="2">
-        <v>25.73</v>
+        <v>314.56</v>
       </c>
       <c r="Q10" s="2">
-        <v>31.95</v>
+        <v>377.91</v>
       </c>
       <c r="R10" s="13" t="inlineStr">
         <is>
@@ -1408,9 +1408,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1428,14 +1428,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X10" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z10" s="4" t="inlineStr">
@@ -1448,14 +1448,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB10" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB10" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC10" s="11" t="inlineStr">
         <is>
-          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
+          <t>informes/novo-nordisk-2026-10-08/Novo Nordisk - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1465,25 +1465,25 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>On</t>
+          <t>Dassault Systèmes</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="D11" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1493,41 +1493,41 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J11" s="2">
-        <v>26.48</v>
+        <v>21.51</v>
       </c>
       <c r="K11" s="2">
-        <v>27.68</v>
+        <v>25.08</v>
       </c>
       <c r="L11" s="2">
-        <v>36.62</v>
+        <v>30.22</v>
       </c>
       <c r="M11" s="3">
-        <v>0.045</v>
+        <v>0.179</v>
       </c>
       <c r="N11" s="3">
-        <v>0.38299999999999995</v>
+        <v>0.41700000000000004</v>
       </c>
       <c r="O11" s="2">
-        <v>36.11</v>
+        <v>23.32</v>
       </c>
       <c r="P11" s="2">
-        <v>30.75</v>
+        <v>25.73</v>
       </c>
       <c r="Q11" s="2">
-        <v>40.69</v>
+        <v>31.95</v>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S11" s="13" t="inlineStr">
@@ -1535,9 +1535,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U11" s="4" t="inlineStr">
@@ -1550,9 +1550,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W11" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X11" s="4" t="inlineStr">
@@ -1560,9 +1560,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y11" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z11" s="4" t="inlineStr">
@@ -1575,14 +1575,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB11" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB11" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC11" s="11" t="inlineStr">
         <is>
-          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
+          <t>informes/dassault-2026-10-07/Dassault Systèmes - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -1592,25 +1592,25 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>On</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="D12" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1625,46 +1625,46 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="J12" s="2">
-        <v>123.73</v>
+        <v>26.48</v>
       </c>
       <c r="K12" s="2">
-        <v>151.16</v>
+        <v>27.68</v>
       </c>
       <c r="L12" s="2">
-        <v>164.85</v>
+        <v>36.62</v>
       </c>
       <c r="M12" s="3">
-        <v>0.268</v>
+        <v>0.045</v>
       </c>
       <c r="N12" s="3">
-        <v>0.379</v>
+        <v>0.38299999999999995</v>
       </c>
       <c r="O12" s="2">
-        <v>148.64</v>
+        <v>36.11</v>
       </c>
       <c r="P12" s="2">
-        <v>148.29</v>
+        <v>30.75</v>
       </c>
       <c r="Q12" s="2">
-        <v>181.24</v>
+        <v>40.69</v>
       </c>
       <c r="R12" s="13" t="inlineStr">
         <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="S12" s="13" t="inlineStr">
+        <is>
           <t>Comprar</t>
         </is>
       </c>
-      <c r="S12" s="13" t="inlineStr">
-        <is>
-          <t>Comprar</t>
-        </is>
-      </c>
-      <c r="T12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -1672,24 +1672,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X12" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y12" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W12" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y12" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z12" s="4" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="AC12" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/on-2026-10-06/On Holding - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D13" s="10">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1756,28 +1756,28 @@
         </is>
       </c>
       <c r="J13" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="K13" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="L13" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="M13" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="N13" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="O13" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="P13" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="Q13" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="R13" s="13" t="inlineStr">
         <is>
@@ -1794,9 +1794,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V13" s="6" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="AC13" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D14" s="10">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1879,36 +1879,36 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J14" s="2">
-        <v>8.677</v>
+        <v>142.43</v>
       </c>
       <c r="K14" s="2">
-        <v>9.45</v>
+        <v>162.26</v>
       </c>
       <c r="L14" s="2">
-        <v>11.42</v>
+        <v>191.49</v>
       </c>
       <c r="M14" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.154</v>
       </c>
       <c r="N14" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.359</v>
       </c>
       <c r="O14" s="2">
-        <v>11.81</v>
+        <v>203.9</v>
       </c>
       <c r="P14" s="2">
-        <v>9.65</v>
+        <v>164.86</v>
       </c>
       <c r="Q14" s="2">
-        <v>12.54</v>
+        <v>208.83</v>
       </c>
       <c r="R14" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="S14" s="13" t="inlineStr">
@@ -1921,9 +1921,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V14" s="6" t="inlineStr">
@@ -1931,9 +1931,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="W14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X14" s="6" t="inlineStr">
@@ -1941,14 +1941,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z14" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA14" s="4" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="AC14" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>Evolution</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>EVO</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D15" s="10">
@@ -1986,12 +1986,12 @@
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2010,28 +2010,28 @@
         </is>
       </c>
       <c r="J15" s="2">
-        <v>72.2709</v>
+        <v>8.677</v>
       </c>
       <c r="K15" s="2">
-        <v>81.5</v>
+        <v>9.45</v>
       </c>
       <c r="L15" s="2">
-        <v>95.8</v>
+        <v>11.42</v>
       </c>
       <c r="M15" s="3">
-        <v>0.128</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="N15" s="3">
-        <v>0.326</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="O15" s="2">
-        <v>67.88</v>
+        <v>11.81</v>
       </c>
       <c r="P15" s="2">
-        <v>83.29</v>
+        <v>9.65</v>
       </c>
       <c r="Q15" s="2">
-        <v>103.75</v>
+        <v>12.54</v>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
@@ -2043,24 +2043,24 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X15" s="6" t="inlineStr">
@@ -2073,9 +2073,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA15" s="4" t="inlineStr">
@@ -2083,14 +2083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC15" s="11" t="inlineStr">
         <is>
-          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D16" s="10">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
@@ -2137,28 +2137,28 @@
         </is>
       </c>
       <c r="J16" s="2">
-        <v>380.9</v>
+        <v>72.2709</v>
       </c>
       <c r="K16" s="2">
-        <v>410</v>
+        <v>81.5</v>
       </c>
       <c r="L16" s="2">
-        <v>478.01</v>
+        <v>95.8</v>
       </c>
       <c r="M16" s="3">
-        <v>0.111</v>
+        <v>0.128</v>
       </c>
       <c r="N16" s="3">
-        <v>0.289</v>
+        <v>0.326</v>
       </c>
       <c r="O16" s="2">
-        <v>526.49</v>
+        <v>67.88</v>
       </c>
       <c r="P16" s="2">
-        <v>422.71</v>
+        <v>83.29</v>
       </c>
       <c r="Q16" s="2">
-        <v>530.95</v>
+        <v>103.75</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2170,14 +2170,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr">
@@ -2190,9 +2190,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y16" s="6" t="inlineStr">
@@ -2200,9 +2200,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z16" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA16" s="4" t="inlineStr">
@@ -2210,14 +2210,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC16" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2227,25 +2227,25 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D17" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2264,28 +2264,28 @@
         </is>
       </c>
       <c r="J17" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="K17" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="L17" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="M17" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="N17" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="O17" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="P17" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="Q17" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
@@ -2297,14 +2297,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr">
@@ -2312,14 +2312,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y17" s="6" t="inlineStr">
@@ -2327,9 +2327,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA17" s="4" t="inlineStr">
@@ -2337,14 +2337,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB17" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC17" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2354,12 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D18" s="10">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2391,28 +2391,28 @@
         </is>
       </c>
       <c r="J18" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="K18" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="L18" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="M18" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="N18" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="O18" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="P18" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="Q18" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
@@ -2424,9 +2424,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
@@ -2439,19 +2439,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X18" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z18" s="4" t="inlineStr">
@@ -2464,14 +2464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB18" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2481,25 +2481,25 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D19" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2514,32 +2514,32 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J19" s="2">
-        <v>3.97</v>
+        <v>52.9</v>
       </c>
       <c r="K19" s="2">
-        <v>3.76</v>
+        <v>55.98</v>
       </c>
       <c r="L19" s="2">
-        <v>4.53</v>
+        <v>62.5</v>
       </c>
       <c r="M19" s="3">
-        <v>-0.021</v>
+        <v>0.12</v>
       </c>
       <c r="N19" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.244</v>
       </c>
       <c r="O19" s="2">
-        <v>6.15</v>
+        <v>69.29</v>
       </c>
       <c r="P19" s="2">
-        <v>4.05</v>
+        <v>57.16</v>
       </c>
       <c r="Q19" s="2">
-        <v>5.05</v>
+        <v>65.83</v>
       </c>
       <c r="R19" s="13" t="inlineStr">
         <is>
@@ -2551,19 +2551,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2581,9 +2581,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2641,32 +2641,32 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J20" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K20" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L20" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M20" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N20" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O20" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P20" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q20" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2678,19 +2678,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -2698,19 +2698,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2718,14 +2718,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D21" s="10">
@@ -2748,12 +2748,12 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2768,32 +2768,32 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K21" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L21" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M21" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N21" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O21" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P21" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q21" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,19 +2805,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2825,19 +2825,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA21" s="4" t="inlineStr">
@@ -2845,14 +2845,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D22" s="10">
@@ -2880,56 +2880,56 @@
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J22" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K22" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L22" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M22" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N22" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O22" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P22" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R22" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J22" s="2">
-        <v>70.24</v>
-      </c>
-      <c r="K22" s="2">
-        <v>73.56</v>
-      </c>
-      <c r="L22" s="2">
-        <v>80.39</v>
-      </c>
-      <c r="M22" s="3">
-        <v>0.047</v>
-      </c>
-      <c r="N22" s="3">
-        <v>0.145</v>
-      </c>
-      <c r="O22" s="2">
-        <v>100.86</v>
-      </c>
-      <c r="P22" s="2">
-        <v>69.88</v>
-      </c>
-      <c r="Q22" s="2">
-        <v>89.38</v>
-      </c>
-      <c r="R22" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S22" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T22" s="4" t="inlineStr">
@@ -2937,14 +2937,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W22" s="4" t="inlineStr">
@@ -2952,19 +2952,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA22" s="4" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,25 +2989,25 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D23" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3017,37 +3017,37 @@
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J23" s="2">
-        <v>10.18</v>
+        <v>70.24</v>
       </c>
       <c r="K23" s="2">
-        <v>10.41</v>
+        <v>73.56</v>
       </c>
       <c r="L23" s="2">
-        <v>11.23</v>
+        <v>80.39</v>
       </c>
       <c r="M23" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.047</v>
       </c>
       <c r="N23" s="3">
-        <v>0.122</v>
+        <v>0.145</v>
       </c>
       <c r="O23" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="P23" s="2">
-        <v>9.92</v>
+        <v>69.88</v>
       </c>
       <c r="Q23" s="2">
-        <v>12.34</v>
+        <v>89.38</v>
       </c>
       <c r="R23" s="13" t="inlineStr">
         <is>
@@ -3059,14 +3059,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V23" s="4" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z23" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA23" s="4" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,16 +3116,16 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
@@ -3153,28 +3153,28 @@
         </is>
       </c>
       <c r="J24" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K24" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L24" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N24" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O24" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P24" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q24" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3186,14 +3186,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V24" s="4" t="inlineStr">
@@ -3226,14 +3226,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,25 +3243,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3276,32 +3276,32 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K25" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L25" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M25" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N25" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O25" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P25" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q25" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3328,14 +3328,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y25" s="6" t="inlineStr">
@@ -3343,9 +3343,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA25" s="4" t="inlineStr">
@@ -3353,14 +3353,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,25 +3370,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3403,32 +3403,32 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K26" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L26" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N26" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O26" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P26" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q26" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3455,24 +3455,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA26" s="4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D27" s="10">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
@@ -3530,36 +3530,36 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K27" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L27" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N27" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O27" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P27" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q27" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S27" s="13" t="inlineStr">
@@ -3567,9 +3567,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U27" s="4" t="inlineStr">
@@ -3582,29 +3582,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB27" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,25 +3624,25 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3652,37 +3652,37 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K28" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L28" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O28" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P28" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q28" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3694,9 +3694,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
@@ -3709,19 +3709,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z28" s="5" t="inlineStr">
@@ -3729,19 +3729,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,25 +3751,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3784,32 +3784,32 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K29" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L29" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O29" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P29" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q29" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3821,19 +3821,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W29" s="5" t="inlineStr">
@@ -3841,9 +3841,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y29" s="4" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,12 +3878,12 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D30" s="10">
@@ -3891,12 +3891,12 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -3911,32 +3911,32 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K30" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L30" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O30" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P30" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q30" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,19 +3948,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W30" s="5" t="inlineStr">
@@ -3968,14 +3968,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z30" s="5" t="inlineStr">
@@ -3983,19 +3983,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,74 +4005,74 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J31" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K31" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L31" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M31" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N31" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O31" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P31" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q31" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R31" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I31" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J31" s="2">
-        <v>129</v>
-      </c>
-      <c r="K31" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L31" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M31" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N31" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O31" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P31" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q31" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R31" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S31" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T31" s="4" t="inlineStr">
@@ -4090,9 +4090,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X31" s="4" t="inlineStr">
@@ -4100,9 +4100,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z31" s="5" t="inlineStr">
@@ -4110,19 +4110,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,25 +4132,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K32" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L32" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O32" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P32" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q32" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,9 +4202,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,25 +4259,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K33" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L33" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O33" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P33" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q33" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,9 +4329,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T33" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
@@ -4344,9 +4344,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X33" s="4" t="inlineStr">
@@ -4354,9 +4354,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z33" s="5" t="inlineStr">
@@ -4369,14 +4369,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,25 +4386,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J34" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K34" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L34" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O34" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P34" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q34" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4456,9 +4456,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T34" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,25 +4513,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -4546,32 +4546,32 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J35" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K35" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L35" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O35" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P35" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q35" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4583,14 +4583,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V35" s="4" t="inlineStr">
@@ -4598,9 +4598,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X35" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,12 +4640,12 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D36" s="10">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
@@ -4673,32 +4673,32 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J36" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K36" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L36" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M36" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O36" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P36" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q36" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R36" s="13" t="inlineStr">
         <is>
@@ -4710,14 +4710,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V36" s="4" t="inlineStr">
@@ -4730,9 +4730,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y36" s="6" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4767,16 +4767,16 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -4804,28 +4804,28 @@
         </is>
       </c>
       <c r="J37" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K37" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L37" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M37" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O37" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P37" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q37" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R37" s="13" t="inlineStr">
         <is>
@@ -4852,14 +4852,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y37" s="6" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AC37" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4894,12 +4894,12 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D38" s="10">
@@ -4907,116 +4907,243 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J38" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K38" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L38" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M38" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N38" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O38" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P38" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R38" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S38" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC38" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13">
+        <v>1</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D39" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F38" s="0" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H38" s="13" t="inlineStr">
+      <c r="H39" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I38" s="13" t="inlineStr">
+      <c r="I39" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J38" s="2">
+      <c r="J39" s="2">
         <v>698.2</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K39" s="2">
         <v>272.01</v>
       </c>
-      <c r="L38" s="2">
+      <c r="L39" s="2">
         <v>348.9</v>
       </c>
-      <c r="M38" s="3">
+      <c r="M39" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N38" s="3">
+      <c r="N39" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O38" s="2">
+      <c r="O39" s="2">
         <v>713.11</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P39" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q39" s="2">
         <v>395.5</v>
       </c>
-      <c r="R38" s="13" t="inlineStr">
+      <c r="R39" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S38" s="13" t="inlineStr">
+      <c r="S39" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC38" s="11" t="inlineStr">
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC39" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC38"/>
+  <autoFilter ref="A1:AC39"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -5055,6 +5182,7 @@
     <hyperlink ref="AC36" r:id="rId35"/>
     <hyperlink ref="AC37" r:id="rId36"/>
     <hyperlink ref="AC38" r:id="rId37"/>
+    <hyperlink ref="AC39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de A. O. Smith (Mantener, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$40</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3116,25 +3116,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3144,37 +3144,37 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J24" s="2">
-        <v>10.18</v>
+        <v>56.56</v>
       </c>
       <c r="K24" s="2">
-        <v>10.41</v>
+        <v>55.24</v>
       </c>
       <c r="L24" s="2">
-        <v>11.23</v>
+        <v>62.35</v>
       </c>
       <c r="M24" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.002</v>
       </c>
       <c r="N24" s="3">
-        <v>0.122</v>
+        <v>0.127</v>
       </c>
       <c r="O24" s="2">
-        <v>14.33</v>
+        <v>69.91</v>
       </c>
       <c r="P24" s="2">
-        <v>9.92</v>
+        <v>55.41</v>
       </c>
       <c r="Q24" s="2">
-        <v>12.34</v>
+        <v>65.9</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3191,9 +3191,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V24" s="4" t="inlineStr">
@@ -3201,14 +3201,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y24" s="6" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,16 +3243,16 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
@@ -3280,28 +3280,28 @@
         </is>
       </c>
       <c r="J25" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K25" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L25" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M25" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N25" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O25" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P25" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q25" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3313,14 +3313,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr">
@@ -3353,14 +3353,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,25 +3370,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3403,32 +3403,32 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J26" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K26" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L26" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M26" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N26" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O26" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P26" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q26" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3455,14 +3455,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y26" s="6" t="inlineStr">
@@ -3470,9 +3470,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA26" s="4" t="inlineStr">
@@ -3480,14 +3480,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,25 +3497,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K27" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L27" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M27" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N27" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O27" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P27" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q27" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3582,24 +3582,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA27" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D28" s="10">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -3657,36 +3657,36 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K28" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L28" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N28" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O28" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P28" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q28" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S28" s="13" t="inlineStr">
@@ -3694,9 +3694,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
@@ -3709,29 +3709,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB28" s="4" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,25 +3751,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3779,37 +3779,37 @@
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K29" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L29" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O29" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P29" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q29" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
@@ -3821,9 +3821,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr">
@@ -3836,19 +3836,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z29" s="5" t="inlineStr">
@@ -3856,19 +3856,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,25 +3878,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -3911,32 +3911,32 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K30" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L30" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O30" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P30" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q30" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,19 +3948,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W30" s="5" t="inlineStr">
@@ -3968,9 +3968,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y30" s="4" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,12 +4005,12 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D31" s="10">
@@ -4018,12 +4018,12 @@
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -4038,32 +4038,32 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K31" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L31" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O31" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P31" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q31" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -4075,19 +4075,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W31" s="5" t="inlineStr">
@@ -4095,14 +4095,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z31" s="5" t="inlineStr">
@@ -4110,19 +4110,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,74 +4132,74 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J32" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K32" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L32" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M32" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N32" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O32" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P32" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q32" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R32" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H32" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I32" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J32" s="2">
-        <v>129</v>
-      </c>
-      <c r="K32" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L32" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M32" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N32" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O32" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P32" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q32" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R32" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S32" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T32" s="4" t="inlineStr">
@@ -4217,9 +4217,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X32" s="4" t="inlineStr">
@@ -4227,9 +4227,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z32" s="5" t="inlineStr">
@@ -4237,19 +4237,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,25 +4259,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K33" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L33" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O33" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P33" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q33" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,9 +4329,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,25 +4386,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J34" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K34" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L34" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O34" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P34" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q34" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4456,9 +4456,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T34" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -4471,9 +4471,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X34" s="4" t="inlineStr">
@@ -4481,9 +4481,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z34" s="5" t="inlineStr">
@@ -4496,14 +4496,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,25 +4513,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -4546,32 +4546,32 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J35" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K35" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L35" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O35" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P35" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q35" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4583,9 +4583,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T35" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,25 +4640,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -4673,32 +4673,32 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J36" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K36" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L36" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M36" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O36" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P36" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q36" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R36" s="13" t="inlineStr">
         <is>
@@ -4710,14 +4710,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V36" s="4" t="inlineStr">
@@ -4725,9 +4725,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X36" s="4" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4767,12 +4767,12 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D37" s="10">
@@ -4780,7 +4780,7 @@
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
@@ -4800,32 +4800,32 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J37" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K37" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L37" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M37" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O37" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P37" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q37" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R37" s="13" t="inlineStr">
         <is>
@@ -4837,14 +4837,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V37" s="4" t="inlineStr">
@@ -4857,9 +4857,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y37" s="6" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AC37" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4894,16 +4894,16 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -4931,28 +4931,28 @@
         </is>
       </c>
       <c r="J38" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K38" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L38" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M38" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O38" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P38" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q38" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R38" s="13" t="inlineStr">
         <is>
@@ -4979,14 +4979,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y38" s="6" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="AC38" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5021,12 +5021,12 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D39" s="10">
@@ -5034,116 +5034,243 @@
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J39" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K39" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L39" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M39" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N39" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O39" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P39" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R39" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S39" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC39" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13">
+        <v>1</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D40" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F39" s="0" t="inlineStr">
+      <c r="F40" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H39" s="13" t="inlineStr">
+      <c r="H40" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I39" s="13" t="inlineStr">
+      <c r="I40" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J39" s="2">
+      <c r="J40" s="2">
         <v>698.2</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K40" s="2">
         <v>272.01</v>
       </c>
-      <c r="L39" s="2">
+      <c r="L40" s="2">
         <v>348.9</v>
       </c>
-      <c r="M39" s="3">
+      <c r="M40" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N39" s="3">
+      <c r="N40" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O39" s="2">
+      <c r="O40" s="2">
         <v>713.11</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P40" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q40" s="2">
         <v>395.5</v>
       </c>
-      <c r="R39" s="13" t="inlineStr">
+      <c r="R40" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S39" s="13" t="inlineStr">
+      <c r="S40" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC39" s="11" t="inlineStr">
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC40" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC39"/>
+  <autoFilter ref="A1:AC40"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -5183,6 +5310,7 @@
     <hyperlink ref="AC37" r:id="rId36"/>
     <hyperlink ref="AC38" r:id="rId37"/>
     <hyperlink ref="AC39" r:id="rId38"/>
+    <hyperlink ref="AC40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Cooper Companies (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$41</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Cooper</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2645,28 +2645,28 @@
         </is>
       </c>
       <c r="J20" s="2">
-        <v>3.97</v>
+        <v>54.3</v>
       </c>
       <c r="K20" s="2">
-        <v>3.76</v>
+        <v>57.1</v>
       </c>
       <c r="L20" s="2">
-        <v>4.53</v>
+        <v>66.21</v>
       </c>
       <c r="M20" s="3">
-        <v>-0.021</v>
+        <v>0.052000000000000005</v>
       </c>
       <c r="N20" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.21899999999999997</v>
       </c>
       <c r="O20" s="2">
-        <v>6.15</v>
+        <v>65.8</v>
       </c>
       <c r="P20" s="2">
-        <v>4.05</v>
+        <v>57.56</v>
       </c>
       <c r="Q20" s="2">
-        <v>5.05</v>
+        <v>73.6</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -2708,9 +2708,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/cooper-companies-2026-10-09/Cooper Companies - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -2735,25 +2735,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2768,32 +2768,32 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J21" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="K21" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="L21" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="M21" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="N21" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="O21" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="P21" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="Q21" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
@@ -2805,19 +2805,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2825,19 +2825,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X21" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z21" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA21" s="4" t="inlineStr">
@@ -2845,14 +2845,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB21" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D22" s="10">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -2895,32 +2895,32 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J22" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="K22" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="L22" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="M22" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="N22" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="O22" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="P22" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="Q22" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="R22" s="13" t="inlineStr">
         <is>
@@ -2932,19 +2932,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W22" s="4" t="inlineStr">
@@ -2952,19 +2952,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA22" s="4" t="inlineStr">
@@ -2972,14 +2972,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D23" s="10">
@@ -3007,56 +3007,56 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J23" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="K23" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="L23" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="M23" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="N23" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="O23" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="P23" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="R23" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J23" s="2">
-        <v>70.24</v>
-      </c>
-      <c r="K23" s="2">
-        <v>73.56</v>
-      </c>
-      <c r="L23" s="2">
-        <v>80.39</v>
-      </c>
-      <c r="M23" s="3">
-        <v>0.047</v>
-      </c>
-      <c r="N23" s="3">
-        <v>0.145</v>
-      </c>
-      <c r="O23" s="2">
-        <v>100.86</v>
-      </c>
-      <c r="P23" s="2">
-        <v>69.88</v>
-      </c>
-      <c r="Q23" s="2">
-        <v>89.38</v>
-      </c>
-      <c r="R23" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="S23" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T23" s="4" t="inlineStr">
@@ -3064,14 +3064,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W23" s="4" t="inlineStr">
@@ -3079,19 +3079,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA23" s="4" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3116,16 +3116,16 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -3153,28 +3153,28 @@
         </is>
       </c>
       <c r="J24" s="2">
-        <v>56.56</v>
+        <v>70.24</v>
       </c>
       <c r="K24" s="2">
-        <v>55.24</v>
+        <v>73.56</v>
       </c>
       <c r="L24" s="2">
-        <v>62.35</v>
+        <v>80.39</v>
       </c>
       <c r="M24" s="3">
-        <v>0.002</v>
+        <v>0.047</v>
       </c>
       <c r="N24" s="3">
-        <v>0.127</v>
+        <v>0.145</v>
       </c>
       <c r="O24" s="2">
-        <v>69.91</v>
+        <v>100.86</v>
       </c>
       <c r="P24" s="2">
-        <v>55.41</v>
+        <v>69.88</v>
       </c>
       <c r="Q24" s="2">
-        <v>65.9</v>
+        <v>89.38</v>
       </c>
       <c r="R24" s="13" t="inlineStr">
         <is>
@@ -3186,9 +3186,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3211,14 +3211,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA24" s="4" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3243,25 +3243,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3271,37 +3271,37 @@
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J25" s="2">
-        <v>10.18</v>
+        <v>56.56</v>
       </c>
       <c r="K25" s="2">
-        <v>10.41</v>
+        <v>55.24</v>
       </c>
       <c r="L25" s="2">
-        <v>11.23</v>
+        <v>62.35</v>
       </c>
       <c r="M25" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.002</v>
       </c>
       <c r="N25" s="3">
-        <v>0.122</v>
+        <v>0.127</v>
       </c>
       <c r="O25" s="2">
-        <v>14.33</v>
+        <v>69.91</v>
       </c>
       <c r="P25" s="2">
-        <v>9.92</v>
+        <v>55.41</v>
       </c>
       <c r="Q25" s="2">
-        <v>12.34</v>
+        <v>65.9</v>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
@@ -3318,9 +3318,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="U25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr">
@@ -3328,14 +3328,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y25" s="6" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3370,16 +3370,16 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
@@ -3407,28 +3407,28 @@
         </is>
       </c>
       <c r="J26" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="K26" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="L26" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="M26" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="N26" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="O26" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="P26" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="Q26" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="R26" s="13" t="inlineStr">
         <is>
@@ -3440,14 +3440,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr">
@@ -3480,14 +3480,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3497,25 +3497,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3530,32 +3530,32 @@
       </c>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J27" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="K27" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="L27" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="M27" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="N27" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="O27" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="P27" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="Q27" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="R27" s="13" t="inlineStr">
         <is>
@@ -3582,14 +3582,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y27" s="6" t="inlineStr">
@@ -3597,9 +3597,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA27" s="4" t="inlineStr">
@@ -3607,14 +3607,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AB27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3624,25 +3624,25 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3657,32 +3657,32 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J28" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="K28" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="L28" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="M28" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="N28" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="O28" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="P28" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="Q28" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="R28" s="13" t="inlineStr">
         <is>
@@ -3709,24 +3709,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA28" s="4" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D29" s="10">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
@@ -3784,36 +3784,36 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J29" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="K29" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="L29" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="M29" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="N29" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="O29" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="P29" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="Q29" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="R29" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S29" s="13" t="inlineStr">
@@ -3821,9 +3821,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr">
@@ -3836,29 +3836,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB29" s="4" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3878,25 +3878,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -3906,37 +3906,37 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J30" s="2">
-        <v>529.76</v>
+        <v>577.5</v>
       </c>
       <c r="K30" s="2">
-        <v>450.46</v>
+        <v>466.62</v>
       </c>
       <c r="L30" s="2">
-        <v>511.38</v>
+        <v>564.55</v>
       </c>
       <c r="M30" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.027999999999999997</v>
+        <v>0.005</v>
       </c>
       <c r="O30" s="2">
-        <v>587.63</v>
+        <v>795.86</v>
       </c>
       <c r="P30" s="2">
-        <v>447.76</v>
+        <v>504.42</v>
       </c>
       <c r="Q30" s="2">
-        <v>568.48</v>
+        <v>645.34</v>
       </c>
       <c r="R30" s="13" t="inlineStr">
         <is>
@@ -3948,9 +3948,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3963,19 +3963,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z30" s="5" t="inlineStr">
@@ -3983,19 +3983,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4005,25 +4005,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -4038,32 +4038,32 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K31" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L31" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O31" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P31" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q31" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
@@ -4075,19 +4075,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W31" s="5" t="inlineStr">
@@ -4095,9 +4095,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y31" s="4" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,12 +4132,12 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D32" s="10">
@@ -4145,12 +4145,12 @@
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K32" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L32" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O32" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P32" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q32" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,19 +4202,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
@@ -4222,14 +4222,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z32" s="5" t="inlineStr">
@@ -4237,19 +4237,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,74 +4259,74 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J33" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K33" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L33" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M33" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N33" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O33" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P33" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q33" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R33" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H33" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J33" s="2">
-        <v>129</v>
-      </c>
-      <c r="K33" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L33" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M33" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N33" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O33" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P33" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q33" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R33" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S33" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T33" s="4" t="inlineStr">
@@ -4344,9 +4344,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X33" s="4" t="inlineStr">
@@ -4354,9 +4354,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z33" s="5" t="inlineStr">
@@ -4364,19 +4364,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,25 +4386,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J34" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K34" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L34" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M34" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O34" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P34" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q34" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R34" s="13" t="inlineStr">
         <is>
@@ -4456,9 +4456,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,25 +4513,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -4546,32 +4546,32 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J35" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K35" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L35" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O35" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P35" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q35" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4583,9 +4583,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr">
@@ -4598,9 +4598,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X35" s="4" t="inlineStr">
@@ -4608,9 +4608,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z35" s="5" t="inlineStr">
@@ -4623,14 +4623,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,25 +4640,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -4673,32 +4673,32 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J36" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K36" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L36" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M36" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O36" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P36" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q36" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R36" s="13" t="inlineStr">
         <is>
@@ -4710,9 +4710,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T36" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4767,25 +4767,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -4800,32 +4800,32 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J37" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K37" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L37" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M37" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O37" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P37" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q37" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R37" s="13" t="inlineStr">
         <is>
@@ -4837,14 +4837,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V37" s="4" t="inlineStr">
@@ -4852,9 +4852,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X37" s="4" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AC37" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4894,12 +4894,12 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D38" s="10">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
@@ -4927,32 +4927,32 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J38" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K38" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L38" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M38" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O38" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P38" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q38" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R38" s="13" t="inlineStr">
         <is>
@@ -4964,14 +4964,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -4984,9 +4984,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y38" s="6" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="AC38" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5021,16 +5021,16 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -5058,28 +5058,28 @@
         </is>
       </c>
       <c r="J39" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K39" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L39" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M39" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O39" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P39" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q39" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R39" s="13" t="inlineStr">
         <is>
@@ -5106,14 +5106,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y39" s="6" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="AC39" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5148,12 +5148,12 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D40" s="10">
@@ -5161,116 +5161,243 @@
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J40" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K40" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L40" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M40" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N40" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O40" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P40" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R40" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S40" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC40" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13">
+        <v>1</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D41" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F40" s="0" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H40" s="13" t="inlineStr">
+      <c r="H41" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I40" s="13" t="inlineStr">
+      <c r="I41" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J40" s="2">
+      <c r="J41" s="2">
         <v>698.2</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K41" s="2">
         <v>272.01</v>
       </c>
-      <c r="L40" s="2">
+      <c r="L41" s="2">
         <v>348.9</v>
       </c>
-      <c r="M40" s="3">
+      <c r="M41" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N40" s="3">
+      <c r="N41" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O40" s="2">
+      <c r="O41" s="2">
         <v>713.11</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P41" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q41" s="2">
         <v>395.5</v>
       </c>
-      <c r="R40" s="13" t="inlineStr">
+      <c r="R41" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S40" s="13" t="inlineStr">
+      <c r="S41" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W40" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z40" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA40" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC40" s="11" t="inlineStr">
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC41" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC40"/>
+  <autoFilter ref="A1:AC41"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -5311,6 +5438,7 @@
     <hyperlink ref="AC38" r:id="rId37"/>
     <hyperlink ref="AC39" r:id="rId38"/>
     <hyperlink ref="AC40" r:id="rId39"/>
+    <hyperlink ref="AC41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Olympus (Mantener, convicción media)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AC$42</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -4005,25 +4005,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -4033,41 +4033,41 @@
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J31" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="K31" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="L31" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="M31" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="O31" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="P31" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="Q31" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="R31" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="S31" s="13" t="inlineStr">
@@ -4075,14 +4075,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V31" s="4" t="inlineStr">
@@ -4100,14 +4100,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA31" s="5" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4132,25 +4132,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4165,32 +4165,32 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J32" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="K32" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="L32" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="M32" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="O32" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="P32" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="Q32" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="R32" s="13" t="inlineStr">
         <is>
@@ -4202,19 +4202,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="U32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
@@ -4222,9 +4222,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y32" s="4" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D33" s="10">
@@ -4272,12 +4272,12 @@
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -4292,32 +4292,32 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J33" s="2">
-        <v>81490</v>
+        <v>16.22</v>
       </c>
       <c r="K33" s="2">
-        <v>66566.47</v>
+        <v>13.97</v>
       </c>
       <c r="L33" s="2">
-        <v>75201.52</v>
+        <v>14.66</v>
       </c>
       <c r="M33" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.07</v>
+        <v>-0.035</v>
       </c>
       <c r="O33" s="2">
-        <v>97866.67</v>
+        <v>17.05</v>
       </c>
       <c r="P33" s="2">
-        <v>65834.24</v>
+        <v>13.61</v>
       </c>
       <c r="Q33" s="2">
-        <v>84206.58</v>
+        <v>16.41</v>
       </c>
       <c r="R33" s="13" t="inlineStr">
         <is>
@@ -4329,19 +4329,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="U33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W33" s="5" t="inlineStr">
@@ -4349,14 +4349,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="X33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z33" s="5" t="inlineStr">
@@ -4364,19 +4364,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,74 +4386,74 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="J34" s="2">
+        <v>81490</v>
+      </c>
+      <c r="K34" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="L34" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="M34" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="N34" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="O34" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="P34" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="R34" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H34" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="J34" s="2">
-        <v>129</v>
-      </c>
-      <c r="K34" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="L34" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="M34" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="N34" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="O34" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="P34" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="Q34" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="R34" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T34" s="4" t="inlineStr">
@@ -4471,9 +4471,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X34" s="4" t="inlineStr">
@@ -4481,9 +4481,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z34" s="5" t="inlineStr">
@@ -4491,19 +4491,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AA34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4513,25 +4513,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -4546,32 +4546,32 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="J35" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="K35" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="L35" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="M35" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="O35" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="P35" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="Q35" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="R35" s="13" t="inlineStr">
         <is>
@@ -4583,9 +4583,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4640,25 +4640,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -4673,32 +4673,32 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="J36" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="K36" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="L36" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="M36" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="O36" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="P36" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="Q36" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="R36" s="13" t="inlineStr">
         <is>
@@ -4710,9 +4710,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T36" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="T36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -4725,9 +4725,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="W36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X36" s="4" t="inlineStr">
@@ -4735,9 +4735,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z36" s="5" t="inlineStr">
@@ -4750,14 +4750,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC36" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4767,25 +4767,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -4800,32 +4800,32 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="J37" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="K37" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="L37" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="M37" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="O37" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="P37" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="Q37" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="R37" s="13" t="inlineStr">
         <is>
@@ -4837,9 +4837,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T37" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="U37" s="4" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="AC37" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4894,25 +4894,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -4927,32 +4927,32 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J38" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="K38" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="L38" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="M38" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="O38" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="P38" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="Q38" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="R38" s="13" t="inlineStr">
         <is>
@@ -4964,14 +4964,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="U38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -4979,9 +4979,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X38" s="4" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="AC38" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5021,12 +5021,12 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D39" s="10">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
@@ -5054,32 +5054,32 @@
       </c>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="J39" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="K39" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="L39" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="M39" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="O39" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="P39" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="Q39" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="R39" s="13" t="inlineStr">
         <is>
@@ -5091,14 +5091,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="T39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="T39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="U39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V39" s="4" t="inlineStr">
@@ -5111,9 +5111,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y39" s="6" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="AC39" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5148,16 +5148,16 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -5185,28 +5185,28 @@
         </is>
       </c>
       <c r="J40" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="K40" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="L40" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M40" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O40" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="P40" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="Q40" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="R40" s="13" t="inlineStr">
         <is>
@@ -5233,14 +5233,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W40" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y40" s="6" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="AC40" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5275,12 +5275,12 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D41" s="10">
@@ -5288,116 +5288,243 @@
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="J41" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="K41" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="L41" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M41" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="N41" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O41" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="P41" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="R41" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="S41" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AC41" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13">
+        <v>1</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D42" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F41" s="0" t="inlineStr">
+      <c r="F42" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G42" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H41" s="13" t="inlineStr">
+      <c r="H42" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I41" s="13" t="inlineStr">
+      <c r="I42" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="J41" s="2">
+      <c r="J42" s="2">
         <v>698.2</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K42" s="2">
         <v>272.01</v>
       </c>
-      <c r="L41" s="2">
+      <c r="L42" s="2">
         <v>348.9</v>
       </c>
-      <c r="M41" s="3">
+      <c r="M42" s="3">
         <v>-0.6</v>
       </c>
-      <c r="N41" s="3">
+      <c r="N42" s="3">
         <v>-0.49</v>
       </c>
-      <c r="O41" s="2">
+      <c r="O42" s="2">
         <v>713.11</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P42" s="2">
         <v>282.35</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q42" s="2">
         <v>395.5</v>
       </c>
-      <c r="R41" s="13" t="inlineStr">
+      <c r="R42" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="S41" s="13" t="inlineStr">
+      <c r="S42" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="U41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="X41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC41" s="11" t="inlineStr">
+      <c r="T42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC42" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC41"/>
+  <autoFilter ref="A1:AC42"/>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1"/>
     <hyperlink ref="AC3" r:id="rId2"/>
@@ -5439,6 +5566,7 @@
     <hyperlink ref="AC39" r:id="rId38"/>
     <hyperlink ref="AC40" r:id="rId39"/>
     <hyperlink ref="AC41" r:id="rId40"/>
+    <hyperlink ref="AC42" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de CSL (Mantener, convicción Baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$43</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -4552,25 +4552,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -4590,32 +4590,32 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K34" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L34" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M34" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O34" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P34" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q34" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R34" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
@@ -4632,29 +4632,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA34" s="5" t="inlineStr">
@@ -4662,19 +4662,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4684,79 +4684,79 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K35" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L35" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M35" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N35" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O35" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P35" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R35" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S35" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I35" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J35" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K35" s="2">
-        <v>129</v>
-      </c>
-      <c r="L35" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M35" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N35" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O35" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P35" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q35" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R35" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S35" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr">
@@ -4774,9 +4774,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y35" s="4" t="inlineStr">
@@ -4784,9 +4784,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA35" s="5" t="inlineStr">
@@ -4794,19 +4794,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4816,25 +4816,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -4849,37 +4849,37 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K36" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L36" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M36" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O36" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P36" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q36" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R36" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S36" s="13" t="inlineStr">
         <is>
@@ -4891,9 +4891,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V36" s="4" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="AD36" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4948,25 +4948,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -4981,37 +4981,37 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K37" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L37" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M37" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O37" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P37" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q37" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R37" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S37" s="13" t="inlineStr">
         <is>
@@ -5023,9 +5023,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U37" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V37" s="4" t="inlineStr">
@@ -5038,9 +5038,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y37" s="4" t="inlineStr">
@@ -5048,9 +5048,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA37" s="5" t="inlineStr">
@@ -5063,14 +5063,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD37" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5080,25 +5080,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -5113,37 +5113,37 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L38" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M38" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O38" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P38" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q38" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R38" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
@@ -5155,9 +5155,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U38" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5212,25 +5212,25 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -5245,37 +5245,37 @@
       </c>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K39" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L39" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M39" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O39" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P39" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q39" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R39" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5287,14 +5287,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W39" s="4" t="inlineStr">
@@ -5302,9 +5302,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y39" s="4" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5344,12 +5344,12 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D40" s="10">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
@@ -5382,32 +5382,32 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K40" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="L40" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="M40" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="O40" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="P40" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="Q40" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="R40" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5419,14 +5419,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W40" s="4" t="inlineStr">
@@ -5439,9 +5439,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z40" s="6" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5476,16 +5476,16 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D41" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
@@ -5518,28 +5518,28 @@
         </is>
       </c>
       <c r="K41" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L41" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M41" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N41" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O41" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P41" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q41" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R41" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5566,14 +5566,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z41" s="6" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5608,12 +5608,12 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D42" s="10">
@@ -5621,121 +5621,253 @@
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K42" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L42" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M42" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N42" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O42" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P42" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R42" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S42" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T42" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD42" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13">
+        <v>1</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D43" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F42" s="0" t="inlineStr">
+      <c r="F43" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G42" s="9" t="inlineStr">
+      <c r="G43" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H42" s="13" t="inlineStr">
+      <c r="H43" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr">
+      <c r="I43" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J42" s="13" t="inlineStr">
+      <c r="J43" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K42" s="2">
+      <c r="K43" s="2">
         <v>698.2</v>
       </c>
-      <c r="L42" s="2">
+      <c r="L43" s="2">
         <v>272.01</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M43" s="2">
         <v>348.9</v>
       </c>
-      <c r="N42" s="3">
+      <c r="N43" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O42" s="3">
+      <c r="O43" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P43" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q43" s="2">
         <v>282.35</v>
       </c>
-      <c r="R42" s="2">
+      <c r="R43" s="2">
         <v>395.5</v>
       </c>
-      <c r="S42" s="13" t="inlineStr">
+      <c r="S43" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T42" s="13" t="inlineStr">
+      <c r="T43" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD42" s="11" t="inlineStr">
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD43" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD42"/>
+  <autoFilter ref="A1:AD43"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -5778,6 +5910,7 @@
     <hyperlink ref="AD40" r:id="rId39"/>
     <hyperlink ref="AD41" r:id="rId40"/>
     <hyperlink ref="AD42" r:id="rId41"/>
+    <hyperlink ref="AD43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de ICON (Mantener, convicción Baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$44</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3232,25 +3232,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICON</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Irlanda</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -3260,12 +3260,12 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr">
@@ -3274,37 +3274,37 @@
         </is>
       </c>
       <c r="K24" s="2">
-        <v>70.24</v>
+        <v>164.5</v>
       </c>
       <c r="L24" s="2">
-        <v>73.56</v>
+        <v>163.26</v>
       </c>
       <c r="M24" s="2">
-        <v>80.39</v>
+        <v>194.24</v>
       </c>
       <c r="N24" s="3">
-        <v>0.047</v>
+        <v>-0.008</v>
       </c>
       <c r="O24" s="3">
-        <v>0.145</v>
+        <v>0.18100000000000002</v>
       </c>
       <c r="P24" s="2">
-        <v>100.86</v>
+        <v>184.41</v>
       </c>
       <c r="Q24" s="2">
-        <v>69.88</v>
+        <v>155.42</v>
       </c>
       <c r="R24" s="2">
-        <v>89.38</v>
+        <v>202.28</v>
       </c>
       <c r="S24" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Vender</t>
         </is>
       </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3312,14 +3312,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
@@ -3327,19 +3327,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB24" s="4" t="inlineStr">
@@ -3347,14 +3347,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD24" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3364,16 +3364,16 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -3406,28 +3406,28 @@
         </is>
       </c>
       <c r="K25" s="2">
-        <v>56.56</v>
+        <v>70.24</v>
       </c>
       <c r="L25" s="2">
-        <v>55.24</v>
+        <v>73.56</v>
       </c>
       <c r="M25" s="2">
-        <v>62.35</v>
+        <v>80.39</v>
       </c>
       <c r="N25" s="3">
-        <v>0.002</v>
+        <v>0.047</v>
       </c>
       <c r="O25" s="3">
-        <v>0.127</v>
+        <v>0.145</v>
       </c>
       <c r="P25" s="2">
-        <v>69.91</v>
+        <v>100.86</v>
       </c>
       <c r="Q25" s="2">
-        <v>55.41</v>
+        <v>69.88</v>
       </c>
       <c r="R25" s="2">
-        <v>65.9</v>
+        <v>89.38</v>
       </c>
       <c r="S25" s="13" t="inlineStr">
         <is>
@@ -3439,9 +3439,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr">
@@ -3464,14 +3464,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA25" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB25" s="4" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="AD25" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3496,25 +3496,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
@@ -3534,32 +3534,32 @@
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K26" s="2">
-        <v>10.18</v>
+        <v>56.56</v>
       </c>
       <c r="L26" s="2">
-        <v>10.41</v>
+        <v>55.24</v>
       </c>
       <c r="M26" s="2">
-        <v>11.23</v>
+        <v>62.35</v>
       </c>
       <c r="N26" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.002</v>
       </c>
       <c r="O26" s="3">
-        <v>0.122</v>
+        <v>0.127</v>
       </c>
       <c r="P26" s="2">
-        <v>14.33</v>
+        <v>69.91</v>
       </c>
       <c r="Q26" s="2">
-        <v>9.92</v>
+        <v>55.41</v>
       </c>
       <c r="R26" s="2">
-        <v>12.34</v>
+        <v>65.9</v>
       </c>
       <c r="S26" s="13" t="inlineStr">
         <is>
@@ -3576,9 +3576,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W26" s="4" t="inlineStr">
@@ -3586,14 +3586,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z26" s="6" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="AD26" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3656,42 +3656,42 @@
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="K27" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="L27" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="M27" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="N27" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O27" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P27" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="Q27" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="R27" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="S27" s="13" t="inlineStr">
         <is>
@@ -3703,14 +3703,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W27" s="4" t="inlineStr">
@@ -3743,14 +3743,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD27" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3760,25 +3760,25 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3798,32 +3798,32 @@
       </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K28" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L28" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M28" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N28" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O28" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P28" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q28" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R28" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S28" s="13" t="inlineStr">
         <is>
@@ -3850,14 +3850,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y28" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z28" s="6" t="inlineStr">
@@ -3865,9 +3865,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB28" s="4" t="inlineStr">
@@ -3875,14 +3875,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3892,25 +3892,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3930,32 +3930,32 @@
       </c>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K29" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="L29" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="M29" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="N29" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="O29" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P29" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="Q29" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="R29" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="S29" s="13" t="inlineStr">
         <is>
@@ -3982,24 +3982,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB29" s="4" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="AD29" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4024,12 +4024,12 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D30" s="10">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
@@ -4057,41 +4057,41 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K30" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L30" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M30" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O30" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P30" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q30" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R30" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T30" s="13" t="inlineStr">
@@ -4099,9 +4099,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V30" s="4" t="inlineStr">
@@ -4114,29 +4114,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AA30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC30" s="4" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="AD30" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4156,25 +4156,25 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -4189,56 +4189,56 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K31" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L31" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M31" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O31" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P31" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q31" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R31" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S31" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T31" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T31" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U31" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W31" s="4" t="inlineStr">
@@ -4246,14 +4246,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y31" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z31" s="6" t="inlineStr">
@@ -4261,24 +4261,24 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD31" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4288,25 +4288,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4316,46 +4316,46 @@
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K32" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L32" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M32" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O32" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P32" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q32" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R32" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S32" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T32" s="13" t="inlineStr">
@@ -4363,14 +4363,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -4388,14 +4388,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB32" s="5" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="AD32" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4420,25 +4420,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -4458,32 +4458,32 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K33" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L33" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M33" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O33" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P33" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q33" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R33" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S33" s="13" t="inlineStr">
         <is>
@@ -4495,19 +4495,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="V33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X33" s="5" t="inlineStr">
@@ -4515,9 +4515,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Y33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z33" s="4" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="AD33" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4552,25 +4552,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -4590,32 +4590,32 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K34" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L34" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M34" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O34" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P34" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q34" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R34" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
@@ -4627,9 +4627,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
@@ -4637,19 +4637,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z34" s="4" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="AD34" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4684,25 +4684,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -4722,32 +4722,32 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K35" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L35" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M35" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O35" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P35" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q35" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R35" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S35" s="13" t="inlineStr">
         <is>
@@ -4764,29 +4764,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X35" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA35" s="5" t="inlineStr">
@@ -4794,19 +4794,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4816,79 +4816,79 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K36" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L36" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M36" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N36" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O36" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P36" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q36" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R36" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S36" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I36" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J36" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K36" s="2">
-        <v>129</v>
-      </c>
-      <c r="L36" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M36" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N36" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O36" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P36" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q36" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R36" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S36" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T36" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -4906,9 +4906,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y36" s="4" t="inlineStr">
@@ -4916,9 +4916,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA36" s="5" t="inlineStr">
@@ -4926,19 +4926,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD36" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4948,25 +4948,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -4981,37 +4981,37 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K37" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L37" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M37" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O37" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P37" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q37" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R37" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S37" s="13" t="inlineStr">
         <is>
@@ -5023,9 +5023,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V37" s="4" t="inlineStr">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="AD37" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5080,25 +5080,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -5113,37 +5113,37 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L38" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M38" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O38" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P38" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q38" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R38" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
@@ -5155,9 +5155,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U38" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -5170,9 +5170,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y38" s="4" t="inlineStr">
@@ -5180,9 +5180,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA38" s="5" t="inlineStr">
@@ -5195,14 +5195,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5212,25 +5212,25 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -5245,37 +5245,37 @@
       </c>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K39" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L39" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M39" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O39" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P39" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q39" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R39" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5287,9 +5287,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U39" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V39" s="4" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5344,25 +5344,25 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -5377,37 +5377,37 @@
       </c>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K40" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L40" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M40" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O40" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P40" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q40" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R40" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5419,14 +5419,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W40" s="4" t="inlineStr">
@@ -5434,9 +5434,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y40" s="4" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5476,12 +5476,12 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D41" s="10">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
@@ -5514,32 +5514,32 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="L41" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="M41" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="N41" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="O41" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="P41" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="Q41" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="R41" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5551,14 +5551,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W41" s="4" t="inlineStr">
@@ -5571,9 +5571,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z41" s="6" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5608,16 +5608,16 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
@@ -5650,28 +5650,28 @@
         </is>
       </c>
       <c r="K42" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L42" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M42" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N42" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O42" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P42" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q42" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R42" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
@@ -5698,14 +5698,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z42" s="6" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5740,12 +5740,12 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D43" s="10">
@@ -5753,121 +5753,253 @@
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K43" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L43" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M43" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N43" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O43" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P43" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R43" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S43" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T43" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB43" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD43" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13">
+        <v>1</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D44" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F43" s="0" t="inlineStr">
+      <c r="F44" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G43" s="9" t="inlineStr">
+      <c r="G44" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H43" s="13" t="inlineStr">
+      <c r="H44" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I43" s="13" t="inlineStr">
+      <c r="I44" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J43" s="13" t="inlineStr">
+      <c r="J44" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K43" s="2">
+      <c r="K44" s="2">
         <v>698.2</v>
       </c>
-      <c r="L43" s="2">
+      <c r="L44" s="2">
         <v>272.01</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M44" s="2">
         <v>348.9</v>
       </c>
-      <c r="N43" s="3">
+      <c r="N44" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O43" s="3">
+      <c r="O44" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P44" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q44" s="2">
         <v>282.35</v>
       </c>
-      <c r="R43" s="2">
+      <c r="R44" s="2">
         <v>395.5</v>
       </c>
-      <c r="S43" s="13" t="inlineStr">
+      <c r="S44" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T43" s="13" t="inlineStr">
+      <c r="T44" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD43" s="11" t="inlineStr">
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD44" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD43"/>
+  <autoFilter ref="A1:AD44"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -5911,6 +6043,7 @@
     <hyperlink ref="AD41" r:id="rId40"/>
     <hyperlink ref="AD42" r:id="rId41"/>
     <hyperlink ref="AD43" r:id="rId42"/>
+    <hyperlink ref="AD44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de PepsiCo, iteración 2 (Comprar, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$45</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1780,12 +1780,12 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Equifax</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>EFX</t>
         </is>
       </c>
       <c r="D13" s="10">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr">
@@ -1822,28 +1822,28 @@
         </is>
       </c>
       <c r="K13" s="2">
-        <v>123.73</v>
+        <v>142.43</v>
       </c>
       <c r="L13" s="2">
-        <v>151.16</v>
+        <v>162.26</v>
       </c>
       <c r="M13" s="2">
-        <v>164.85</v>
+        <v>191.49</v>
       </c>
       <c r="N13" s="3">
-        <v>0.268</v>
+        <v>0.154</v>
       </c>
       <c r="O13" s="3">
-        <v>0.379</v>
+        <v>0.359</v>
       </c>
       <c r="P13" s="2">
-        <v>148.64</v>
+        <v>203.9</v>
       </c>
       <c r="Q13" s="2">
-        <v>148.29</v>
+        <v>164.86</v>
       </c>
       <c r="R13" s="2">
-        <v>181.24</v>
+        <v>208.83</v>
       </c>
       <c r="S13" s="13" t="inlineStr">
         <is>
@@ -1860,9 +1860,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V13" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W13" s="6" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="AD13" s="11" t="inlineStr">
         <is>
-          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
+          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -1912,12 +1912,12 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>Equifax</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D14" s="10">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J14" s="13" t="inlineStr">
@@ -1954,28 +1954,28 @@
         </is>
       </c>
       <c r="K14" s="2">
-        <v>142.43</v>
+        <v>123.73</v>
       </c>
       <c r="L14" s="2">
-        <v>162.26</v>
+        <v>151.16</v>
       </c>
       <c r="M14" s="2">
-        <v>191.49</v>
+        <v>164.85</v>
       </c>
       <c r="N14" s="3">
-        <v>0.154</v>
+        <v>0.268</v>
       </c>
       <c r="O14" s="3">
-        <v>0.359</v>
+        <v>0.379</v>
       </c>
       <c r="P14" s="2">
-        <v>203.9</v>
+        <v>148.64</v>
       </c>
       <c r="Q14" s="2">
-        <v>164.86</v>
+        <v>148.29</v>
       </c>
       <c r="R14" s="2">
-        <v>208.83</v>
+        <v>181.24</v>
       </c>
       <c r="S14" s="13" t="inlineStr">
         <is>
@@ -1992,9 +1992,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V14" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W14" s="6" t="inlineStr">
@@ -2034,35 +2034,35 @@
       </c>
       <c r="AD14" s="11" t="inlineStr">
         <is>
-          <t>informes/equifax-2026-10-08/Equifax - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-08/PepsiCo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>Tomra</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
         <is>
-          <t>TOM</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D15" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2077,41 +2077,41 @@
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K15" s="2">
-        <v>8.677</v>
+        <v>128.34</v>
       </c>
       <c r="L15" s="2">
-        <v>9.45</v>
+        <v>152.55</v>
       </c>
       <c r="M15" s="2">
-        <v>11.42</v>
+        <v>166.39</v>
       </c>
       <c r="N15" s="3">
-        <v>0.11199999999999999</v>
+        <v>0.23399999999999999</v>
       </c>
       <c r="O15" s="3">
-        <v>0.33899999999999997</v>
+        <v>0.342</v>
       </c>
       <c r="P15" s="2">
-        <v>11.81</v>
+        <v>144.82</v>
       </c>
       <c r="Q15" s="2">
-        <v>9.65</v>
+        <v>149.65</v>
       </c>
       <c r="R15" s="2">
-        <v>12.54</v>
+        <v>182.91</v>
       </c>
       <c r="S15" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T15" s="13" t="inlineStr">
@@ -2124,9 +2124,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W15" s="6" t="inlineStr">
@@ -2134,9 +2134,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="X15" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y15" s="6" t="inlineStr">
@@ -2144,14 +2144,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Z15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA15" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA15" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB15" s="4" t="inlineStr">
@@ -2159,14 +2159,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC15" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC15" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD15" s="11" t="inlineStr">
         <is>
-          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
+          <t>informes/pepsico-2026-10-09/PepsiCo - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -2176,12 +2176,12 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>Evolution</t>
+          <t>Tomra</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>EVO</t>
+          <t>TOM</t>
         </is>
       </c>
       <c r="D16" s="10">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2218,28 +2218,28 @@
         </is>
       </c>
       <c r="K16" s="2">
-        <v>72.2709</v>
+        <v>8.677</v>
       </c>
       <c r="L16" s="2">
-        <v>81.5</v>
+        <v>9.45</v>
       </c>
       <c r="M16" s="2">
-        <v>95.8</v>
+        <v>11.42</v>
       </c>
       <c r="N16" s="3">
-        <v>0.128</v>
+        <v>0.11199999999999999</v>
       </c>
       <c r="O16" s="3">
-        <v>0.326</v>
+        <v>0.33899999999999997</v>
       </c>
       <c r="P16" s="2">
-        <v>67.88</v>
+        <v>11.81</v>
       </c>
       <c r="Q16" s="2">
-        <v>83.29</v>
+        <v>9.65</v>
       </c>
       <c r="R16" s="2">
-        <v>103.75</v>
+        <v>12.54</v>
       </c>
       <c r="S16" s="13" t="inlineStr">
         <is>
@@ -2251,24 +2251,24 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y16" s="6" t="inlineStr">
@@ -2281,9 +2281,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA16" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA16" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB16" s="4" t="inlineStr">
@@ -2291,14 +2291,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC16" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC16" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD16" s="11" t="inlineStr">
         <is>
-          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
+          <t>informes/tomra-2026-10-08/Tomra - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2308,12 +2308,12 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D17" s="10">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
@@ -2350,28 +2350,28 @@
         </is>
       </c>
       <c r="K17" s="2">
-        <v>380.9</v>
+        <v>72.2709</v>
       </c>
       <c r="L17" s="2">
-        <v>410</v>
+        <v>81.5</v>
       </c>
       <c r="M17" s="2">
-        <v>478.01</v>
+        <v>95.8</v>
       </c>
       <c r="N17" s="3">
-        <v>0.111</v>
+        <v>0.128</v>
       </c>
       <c r="O17" s="3">
-        <v>0.289</v>
+        <v>0.326</v>
       </c>
       <c r="P17" s="2">
-        <v>526.49</v>
+        <v>67.88</v>
       </c>
       <c r="Q17" s="2">
-        <v>422.71</v>
+        <v>83.29</v>
       </c>
       <c r="R17" s="2">
-        <v>530.95</v>
+        <v>103.75</v>
       </c>
       <c r="S17" s="13" t="inlineStr">
         <is>
@@ -2383,14 +2383,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W17" s="4" t="inlineStr">
@@ -2403,9 +2403,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y17" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z17" s="6" t="inlineStr">
@@ -2413,9 +2413,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA17" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA17" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB17" s="4" t="inlineStr">
@@ -2423,14 +2423,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC17" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD17" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2440,25 +2440,25 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D18" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2482,28 +2482,28 @@
         </is>
       </c>
       <c r="K18" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="L18" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="M18" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="N18" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="O18" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="P18" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="Q18" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="R18" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="S18" s="13" t="inlineStr">
         <is>
@@ -2515,14 +2515,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2530,14 +2530,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z18" s="6" t="inlineStr">
@@ -2545,9 +2545,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA18" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA18" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB18" s="4" t="inlineStr">
@@ -2555,14 +2555,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC18" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC18" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD18" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2572,12 +2572,12 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D19" s="10">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2614,28 +2614,28 @@
         </is>
       </c>
       <c r="K19" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="L19" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="M19" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="N19" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="O19" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="P19" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="Q19" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="R19" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="S19" s="13" t="inlineStr">
         <is>
@@ -2647,9 +2647,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V19" s="4" t="inlineStr">
@@ -2662,19 +2662,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2687,14 +2687,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD19" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -2704,25 +2704,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Cooper</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2742,32 +2742,32 @@
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K20" s="2">
-        <v>54.3</v>
+        <v>52.9</v>
       </c>
       <c r="L20" s="2">
-        <v>57.1</v>
+        <v>55.98</v>
       </c>
       <c r="M20" s="2">
-        <v>66.21</v>
+        <v>62.5</v>
       </c>
       <c r="N20" s="3">
-        <v>0.052000000000000005</v>
+        <v>0.12</v>
       </c>
       <c r="O20" s="3">
-        <v>0.21899999999999997</v>
+        <v>0.244</v>
       </c>
       <c r="P20" s="2">
-        <v>65.8</v>
+        <v>69.29</v>
       </c>
       <c r="Q20" s="2">
-        <v>57.56</v>
+        <v>57.16</v>
       </c>
       <c r="R20" s="2">
-        <v>73.6</v>
+        <v>65.83</v>
       </c>
       <c r="S20" s="13" t="inlineStr">
         <is>
@@ -2779,19 +2779,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V20" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W20" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X20" s="4" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="AD20" s="11" t="inlineStr">
         <is>
-          <t>informes/cooper-companies-2026-10-09/Cooper Companies - 2026-10-09.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -2836,25 +2836,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Cooper</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2878,28 +2878,28 @@
         </is>
       </c>
       <c r="K21" s="2">
-        <v>3.97</v>
+        <v>54.3</v>
       </c>
       <c r="L21" s="2">
-        <v>3.76</v>
+        <v>57.1</v>
       </c>
       <c r="M21" s="2">
-        <v>4.53</v>
+        <v>66.21</v>
       </c>
       <c r="N21" s="3">
-        <v>-0.021</v>
+        <v>0.052000000000000005</v>
       </c>
       <c r="O21" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.21899999999999997</v>
       </c>
       <c r="P21" s="2">
-        <v>6.15</v>
+        <v>65.8</v>
       </c>
       <c r="Q21" s="2">
-        <v>4.05</v>
+        <v>57.56</v>
       </c>
       <c r="R21" s="2">
-        <v>5.05</v>
+        <v>73.6</v>
       </c>
       <c r="S21" s="13" t="inlineStr">
         <is>
@@ -2941,9 +2941,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB21" s="4" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="AD21" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/cooper-companies-2026-10-09/Cooper Companies - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -2968,25 +2968,25 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -3006,32 +3006,32 @@
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K22" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="L22" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="M22" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="N22" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="O22" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="P22" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="Q22" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="R22" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="S22" s="13" t="inlineStr">
         <is>
@@ -3043,19 +3043,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V22" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X22" s="4" t="inlineStr">
@@ -3063,19 +3063,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB22" s="4" t="inlineStr">
@@ -3083,14 +3083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD22" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3100,12 +3100,12 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D23" s="10">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3138,32 +3138,32 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K23" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="L23" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="M23" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="N23" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="O23" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="P23" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="Q23" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="R23" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="S23" s="13" t="inlineStr">
         <is>
@@ -3175,39 +3175,39 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V23" s="5" t="inlineStr">
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z23" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB23" s="4" t="inlineStr">
@@ -3215,14 +3215,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD23" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3232,76 +3232,76 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>ICON</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Irlanda</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K24" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="L24" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="M24" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="N24" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="O24" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="P24" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="R24" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="S24" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="K24" s="2">
-        <v>164.5</v>
-      </c>
-      <c r="L24" s="2">
-        <v>163.26</v>
-      </c>
-      <c r="M24" s="2">
-        <v>194.24</v>
-      </c>
-      <c r="N24" s="3">
-        <v>-0.008</v>
-      </c>
-      <c r="O24" s="3">
-        <v>0.18100000000000002</v>
-      </c>
-      <c r="P24" s="2">
-        <v>184.41</v>
-      </c>
-      <c r="Q24" s="2">
-        <v>155.42</v>
-      </c>
-      <c r="R24" s="2">
-        <v>202.28</v>
-      </c>
-      <c r="S24" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
           <t>Comprar</t>
@@ -3347,14 +3347,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD24" s="11" t="inlineStr">
         <is>
-          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3364,25 +3364,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>ICON</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Irlanda</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -3392,12 +3392,12 @@
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr">
@@ -3406,37 +3406,37 @@
         </is>
       </c>
       <c r="K25" s="2">
-        <v>70.24</v>
+        <v>164.5</v>
       </c>
       <c r="L25" s="2">
-        <v>73.56</v>
+        <v>163.26</v>
       </c>
       <c r="M25" s="2">
-        <v>80.39</v>
+        <v>194.24</v>
       </c>
       <c r="N25" s="3">
-        <v>0.047</v>
+        <v>-0.008</v>
       </c>
       <c r="O25" s="3">
-        <v>0.145</v>
+        <v>0.18100000000000002</v>
       </c>
       <c r="P25" s="2">
-        <v>100.86</v>
+        <v>184.41</v>
       </c>
       <c r="Q25" s="2">
-        <v>69.88</v>
+        <v>155.42</v>
       </c>
       <c r="R25" s="2">
-        <v>89.38</v>
+        <v>202.28</v>
       </c>
       <c r="S25" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Vender</t>
         </is>
       </c>
       <c r="T25" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3444,14 +3444,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X25" s="4" t="inlineStr">
@@ -3459,19 +3459,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB25" s="4" t="inlineStr">
@@ -3479,14 +3479,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC25" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC25" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD25" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3496,16 +3496,16 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -3538,28 +3538,28 @@
         </is>
       </c>
       <c r="K26" s="2">
-        <v>56.56</v>
+        <v>70.24</v>
       </c>
       <c r="L26" s="2">
-        <v>55.24</v>
+        <v>73.56</v>
       </c>
       <c r="M26" s="2">
-        <v>62.35</v>
+        <v>80.39</v>
       </c>
       <c r="N26" s="3">
-        <v>0.002</v>
+        <v>0.047</v>
       </c>
       <c r="O26" s="3">
-        <v>0.127</v>
+        <v>0.145</v>
       </c>
       <c r="P26" s="2">
-        <v>69.91</v>
+        <v>100.86</v>
       </c>
       <c r="Q26" s="2">
-        <v>55.41</v>
+        <v>69.88</v>
       </c>
       <c r="R26" s="2">
-        <v>65.9</v>
+        <v>89.38</v>
       </c>
       <c r="S26" s="13" t="inlineStr">
         <is>
@@ -3571,9 +3571,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr">
@@ -3596,14 +3596,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB26" s="4" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="AD26" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3628,25 +3628,25 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D27" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I27" s="13" t="inlineStr">
@@ -3666,32 +3666,32 @@
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K27" s="2">
-        <v>10.18</v>
+        <v>56.56</v>
       </c>
       <c r="L27" s="2">
-        <v>10.41</v>
+        <v>55.24</v>
       </c>
       <c r="M27" s="2">
-        <v>11.23</v>
+        <v>62.35</v>
       </c>
       <c r="N27" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.002</v>
       </c>
       <c r="O27" s="3">
-        <v>0.122</v>
+        <v>0.127</v>
       </c>
       <c r="P27" s="2">
-        <v>14.33</v>
+        <v>69.91</v>
       </c>
       <c r="Q27" s="2">
-        <v>9.92</v>
+        <v>55.41</v>
       </c>
       <c r="R27" s="2">
-        <v>12.34</v>
+        <v>65.9</v>
       </c>
       <c r="S27" s="13" t="inlineStr">
         <is>
@@ -3708,36 +3708,36 @@
           <t>=</t>
         </is>
       </c>
-      <c r="V27" s="5" t="inlineStr">
+      <c r="V27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA27" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA27" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AB27" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="AD27" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3760,16 +3760,16 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -3778,7 +3778,7 @@
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -3788,42 +3788,42 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="K28" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="L28" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="M28" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="N28" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O28" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P28" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="Q28" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="R28" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="S28" s="13" t="inlineStr">
         <is>
@@ -3835,14 +3835,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V28" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U28" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V28" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W28" s="4" t="inlineStr">
@@ -3875,14 +3875,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3892,25 +3892,25 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3930,32 +3930,32 @@
       </c>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K29" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L29" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M29" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N29" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O29" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P29" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q29" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R29" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S29" s="13" t="inlineStr">
         <is>
@@ -3982,39 +3982,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X29" s="5" t="inlineStr">
+      <c r="X29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -4024,25 +4024,25 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -4062,32 +4062,32 @@
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K30" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="L30" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="M30" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="N30" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="O30" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P30" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="Q30" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="R30" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
@@ -4114,24 +4114,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z30" s="5" t="inlineStr">
+      <c r="X30" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB30" s="4" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="AD30" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4156,12 +4156,12 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D31" s="10">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
@@ -4189,41 +4189,41 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K31" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L31" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M31" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N31" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O31" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P31" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q31" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R31" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S31" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T31" s="13" t="inlineStr">
@@ -4231,9 +4231,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V31" s="4" t="inlineStr">
@@ -4246,29 +4246,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA31" s="5" t="inlineStr">
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z31" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC31" s="4" t="inlineStr">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="AD31" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4288,25 +4288,25 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4321,56 +4321,56 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K32" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L32" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M32" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O32" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P32" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q32" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R32" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S32" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T32" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T32" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U32" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -4378,39 +4378,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X32" s="5" t="inlineStr">
+      <c r="X32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA32" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD32" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4420,25 +4420,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -4448,46 +4448,46 @@
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K33" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L33" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M33" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O33" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P33" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q33" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R33" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S33" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T33" s="13" t="inlineStr">
@@ -4495,14 +4495,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W33" s="4" t="inlineStr">
@@ -4520,21 +4520,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA33" s="5" t="inlineStr">
+      <c r="Z33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB33" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC33" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="AD33" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4552,25 +4552,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -4590,32 +4590,32 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K34" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L34" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M34" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O34" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P34" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q34" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R34" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
@@ -4627,46 +4627,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U34" s="5" t="inlineStr">
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X34" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V34" s="5" t="inlineStr">
+      <c r="Y34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA34" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W34" s="5" t="inlineStr">
+      <c r="AB34" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC34" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="AD34" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4684,25 +4684,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -4722,32 +4722,32 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K35" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L35" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M35" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O35" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P35" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q35" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R35" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S35" s="13" t="inlineStr">
         <is>
@@ -4759,9 +4759,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V35" s="5" t="inlineStr">
@@ -4769,19 +4769,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z35" s="4" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="AD35" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4816,25 +4816,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
@@ -4854,32 +4854,32 @@
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K36" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L36" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M36" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O36" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P36" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q36" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R36" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S36" s="13" t="inlineStr">
         <is>
@@ -4896,29 +4896,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X36" s="5" t="inlineStr">
+      <c r="V36" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA36" s="5" t="inlineStr">
@@ -4926,19 +4926,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB36" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD36" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4948,79 +4948,79 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K37" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L37" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M37" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N37" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O37" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P37" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R37" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S37" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I37" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J37" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K37" s="2">
-        <v>129</v>
-      </c>
-      <c r="L37" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M37" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N37" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O37" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P37" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q37" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R37" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S37" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T37" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U37" s="4" t="inlineStr">
@@ -5038,9 +5038,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X37" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y37" s="4" t="inlineStr">
@@ -5048,9 +5048,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA37" s="5" t="inlineStr">
@@ -5058,19 +5058,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD37" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5080,25 +5080,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -5113,37 +5113,37 @@
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L38" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M38" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O38" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P38" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q38" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R38" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
@@ -5155,9 +5155,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5212,25 +5212,25 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -5245,37 +5245,37 @@
       </c>
       <c r="I39" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K39" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L39" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M39" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O39" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P39" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q39" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R39" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5287,9 +5287,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U39" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V39" s="4" t="inlineStr">
@@ -5302,39 +5302,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X39" s="5" t="inlineStr">
+      <c r="X39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA39" s="5" t="inlineStr">
+      <c r="AB39" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5344,25 +5344,25 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -5377,37 +5377,37 @@
       </c>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K40" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L40" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M40" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O40" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P40" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q40" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R40" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5419,9 +5419,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U40" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V40" s="4" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5476,25 +5476,25 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D41" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
@@ -5509,37 +5509,37 @@
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L41" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M41" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N41" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O41" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P41" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q41" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R41" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5551,14 +5551,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W41" s="4" t="inlineStr">
@@ -5566,9 +5566,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y41" s="4" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5608,12 +5608,12 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D42" s="10">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
@@ -5646,32 +5646,32 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K42" s="2">
-        <v>253.14</v>
+        <v>6220</v>
       </c>
       <c r="L42" s="2">
-        <v>168.18</v>
+        <v>4460.49</v>
       </c>
       <c r="M42" s="2">
-        <v>168.18</v>
+        <v>4713.09</v>
       </c>
       <c r="N42" s="3">
-        <v>-0.335</v>
+        <v>-0.266</v>
       </c>
       <c r="O42" s="3">
-        <v>-0.335</v>
+        <v>-0.225</v>
       </c>
       <c r="P42" s="2">
-        <v>337.43</v>
+        <v>7278.89</v>
       </c>
       <c r="Q42" s="2">
-        <v>146.32</v>
+        <v>4188.4</v>
       </c>
       <c r="R42" s="2">
-        <v>187.18</v>
+        <v>4821.79</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
@@ -5683,14 +5683,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W42" s="4" t="inlineStr">
@@ -5703,9 +5703,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z42" s="6" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5740,16 +5740,16 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -5782,28 +5782,28 @@
         </is>
       </c>
       <c r="K43" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L43" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M43" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N43" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O43" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P43" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q43" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R43" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
@@ -5830,31 +5830,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X43" s="5" t="inlineStr">
+      <c r="X43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA43" s="5" t="inlineStr">
+      <c r="AB43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC43" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5872,12 +5872,12 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D44" s="10">
@@ -5885,121 +5885,253 @@
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K44" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L44" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M44" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N44" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O44" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P44" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R44" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S44" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T44" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD44" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13">
+        <v>1</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D45" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F44" s="0" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G44" s="9" t="inlineStr">
+      <c r="G45" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H44" s="13" t="inlineStr">
+      <c r="H45" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I44" s="13" t="inlineStr">
+      <c r="I45" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J44" s="13" t="inlineStr">
+      <c r="J45" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K44" s="2">
+      <c r="K45" s="2">
         <v>698.2</v>
       </c>
-      <c r="L44" s="2">
+      <c r="L45" s="2">
         <v>272.01</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M45" s="2">
         <v>348.9</v>
       </c>
-      <c r="N44" s="3">
+      <c r="N45" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O44" s="3">
+      <c r="O45" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P45" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q45" s="2">
         <v>282.35</v>
       </c>
-      <c r="R44" s="2">
+      <c r="R45" s="2">
         <v>395.5</v>
       </c>
-      <c r="S44" s="13" t="inlineStr">
+      <c r="S45" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T44" s="13" t="inlineStr">
+      <c r="T45" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X44" s="5" t="inlineStr">
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X45" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA44" s="5" t="inlineStr">
+      <c r="Y45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA45" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB44" s="5" t="inlineStr">
+      <c r="AB45" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD44" s="11" t="inlineStr">
+      <c r="AC45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD45" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD44"/>
+  <autoFilter ref="A1:AD45"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -6044,6 +6176,7 @@
     <hyperlink ref="AD42" r:id="rId41"/>
     <hyperlink ref="AD43" r:id="rId42"/>
     <hyperlink ref="AD44" r:id="rId43"/>
+    <hyperlink ref="AD45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Uber, iteración 2 (Mantener, convicción media); sostenibilidad: activos ligeros si se reinvierte menos del 15 % del NOPAT
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$50</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -3892,16 +3892,16 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D29" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -3934,28 +3934,28 @@
         </is>
       </c>
       <c r="K29" s="2">
-        <v>70.24</v>
+        <v>56.56</v>
       </c>
       <c r="L29" s="2">
-        <v>73.56</v>
+        <v>55.24</v>
       </c>
       <c r="M29" s="2">
-        <v>80.39</v>
+        <v>62.35</v>
       </c>
       <c r="N29" s="3">
-        <v>0.047</v>
+        <v>0.002</v>
       </c>
       <c r="O29" s="3">
-        <v>0.145</v>
+        <v>0.127</v>
       </c>
       <c r="P29" s="2">
-        <v>100.86</v>
+        <v>69.91</v>
       </c>
       <c r="Q29" s="2">
-        <v>69.88</v>
+        <v>55.41</v>
       </c>
       <c r="R29" s="2">
-        <v>89.38</v>
+        <v>65.9</v>
       </c>
       <c r="S29" s="13" t="inlineStr">
         <is>
@@ -3967,9 +3967,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V29" s="4" t="inlineStr">
@@ -3992,14 +3992,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB29" s="4" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="AD29" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4024,16 +4024,16 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -4066,28 +4066,28 @@
         </is>
       </c>
       <c r="K30" s="2">
-        <v>56.56</v>
+        <v>70.24</v>
       </c>
       <c r="L30" s="2">
-        <v>55.24</v>
+        <v>73.56</v>
       </c>
       <c r="M30" s="2">
-        <v>62.35</v>
+        <v>80.39</v>
       </c>
       <c r="N30" s="3">
-        <v>0.002</v>
+        <v>0.047</v>
       </c>
       <c r="O30" s="3">
-        <v>0.127</v>
+        <v>0.145</v>
       </c>
       <c r="P30" s="2">
-        <v>69.91</v>
+        <v>100.86</v>
       </c>
       <c r="Q30" s="2">
-        <v>55.41</v>
+        <v>69.88</v>
       </c>
       <c r="R30" s="2">
-        <v>65.9</v>
+        <v>89.38</v>
       </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
@@ -4099,9 +4099,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V30" s="4" t="inlineStr">
@@ -4124,14 +4124,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z30" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA30" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Z30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA30" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB30" s="4" t="inlineStr">
@@ -4146,35 +4146,35 @@
       </c>
       <c r="AD30" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I31" s="13" t="inlineStr">
@@ -4194,32 +4194,32 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K31" s="2">
-        <v>10.18</v>
+        <v>71.51</v>
       </c>
       <c r="L31" s="2">
-        <v>10.41</v>
+        <v>73.59</v>
       </c>
       <c r="M31" s="2">
-        <v>11.23</v>
+        <v>80.42</v>
       </c>
       <c r="N31" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.028999999999999998</v>
       </c>
       <c r="O31" s="3">
-        <v>0.122</v>
+        <v>0.125</v>
       </c>
       <c r="P31" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="Q31" s="2">
-        <v>9.92</v>
+        <v>69.91</v>
       </c>
       <c r="R31" s="2">
-        <v>12.34</v>
+        <v>89.41</v>
       </c>
       <c r="S31" s="13" t="inlineStr">
         <is>
@@ -4231,14 +4231,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W31" s="4" t="inlineStr">
@@ -4246,24 +4246,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA31" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA31" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB31" s="4" t="inlineStr">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="AD31" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -4288,16 +4288,16 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
@@ -4306,7 +4306,7 @@
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4316,42 +4316,42 @@
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="K32" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="L32" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="M32" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="N32" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O32" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P32" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="Q32" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="R32" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="S32" s="13" t="inlineStr">
         <is>
@@ -4363,14 +4363,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V32" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -4403,14 +4403,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD32" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4420,25 +4420,25 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -4458,32 +4458,32 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K33" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L33" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M33" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N33" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O33" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P33" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q33" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R33" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S33" s="13" t="inlineStr">
         <is>
@@ -4510,39 +4510,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X33" s="5" t="inlineStr">
+      <c r="X33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA33" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y33" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB33" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -4552,25 +4552,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -4590,32 +4590,32 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K34" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="L34" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="M34" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="N34" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="O34" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P34" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="Q34" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="R34" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
@@ -4642,24 +4642,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z34" s="5" t="inlineStr">
+      <c r="X34" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y34" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA34" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB34" s="4" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="AD34" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4684,12 +4684,12 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D35" s="10">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
@@ -4717,41 +4717,41 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K35" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L35" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M35" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O35" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P35" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q35" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R35" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S35" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T35" s="13" t="inlineStr">
@@ -4759,9 +4759,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V35" s="4" t="inlineStr">
@@ -4774,29 +4774,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA35" s="5" t="inlineStr">
+      <c r="X35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z35" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC35" s="4" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="AD35" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4816,25 +4816,25 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D36" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
@@ -4849,56 +4849,56 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K36" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L36" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M36" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O36" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P36" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q36" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R36" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S36" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T36" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T36" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U36" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W36" s="4" t="inlineStr">
@@ -4906,39 +4906,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X36" s="5" t="inlineStr">
+      <c r="X36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA36" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y36" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB36" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD36" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4948,25 +4948,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -4976,46 +4976,46 @@
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K37" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L37" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M37" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O37" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P37" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q37" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R37" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S37" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T37" s="13" t="inlineStr">
@@ -5023,14 +5023,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W37" s="4" t="inlineStr">
@@ -5048,21 +5048,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA37" s="5" t="inlineStr">
+      <c r="Z37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB37" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC37" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="AD37" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -5080,25 +5080,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -5118,32 +5118,32 @@
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L38" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M38" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O38" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P38" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q38" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R38" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
@@ -5155,46 +5155,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U38" s="5" t="inlineStr">
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X38" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V38" s="5" t="inlineStr">
+      <c r="Y38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA38" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr">
+      <c r="AB38" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC38" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5212,25 +5212,25 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -5250,32 +5250,32 @@
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K39" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L39" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M39" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O39" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P39" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q39" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R39" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5287,9 +5287,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V39" s="5" t="inlineStr">
@@ -5297,19 +5297,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y39" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z39" s="4" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5344,25 +5344,25 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -5382,32 +5382,32 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K40" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L40" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M40" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O40" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P40" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q40" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R40" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5424,29 +5424,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X40" s="5" t="inlineStr">
+      <c r="V40" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA40" s="5" t="inlineStr">
@@ -5454,19 +5454,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -5476,79 +5476,79 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D41" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K41" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L41" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M41" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N41" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O41" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P41" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R41" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S41" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I41" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J41" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K41" s="2">
-        <v>129</v>
-      </c>
-      <c r="L41" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M41" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N41" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O41" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P41" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q41" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R41" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S41" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T41" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U41" s="4" t="inlineStr">
@@ -5566,9 +5566,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y41" s="4" t="inlineStr">
@@ -5576,9 +5576,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA41" s="5" t="inlineStr">
@@ -5586,19 +5586,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5608,25 +5608,25 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
@@ -5641,37 +5641,37 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K42" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L42" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M42" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N42" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O42" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P42" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q42" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R42" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
@@ -5683,9 +5683,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V42" s="4" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5740,25 +5740,25 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -5773,37 +5773,37 @@
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K43" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L43" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M43" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N43" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O43" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P43" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q43" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R43" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
@@ -5815,9 +5815,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U43" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V43" s="4" t="inlineStr">
@@ -5830,39 +5830,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X43" s="5" t="inlineStr">
+      <c r="X43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA43" s="5" t="inlineStr">
+      <c r="AB43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5872,25 +5872,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
@@ -5905,37 +5905,37 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K44" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L44" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M44" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O44" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P44" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q44" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R44" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
@@ -5947,9 +5947,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U44" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V44" s="4" t="inlineStr">
@@ -5994,7 +5994,7 @@
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6004,25 +6004,25 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
@@ -6037,37 +6037,37 @@
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K45" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L45" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M45" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N45" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O45" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P45" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q45" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R45" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
@@ -6079,14 +6079,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W45" s="4" t="inlineStr">
@@ -6094,9 +6094,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y45" s="4" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6136,25 +6136,25 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D46" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I46" s="13" t="inlineStr">
@@ -6174,32 +6174,32 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K46" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L46" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M46" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N46" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O46" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P46" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q46" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R46" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
@@ -6211,14 +6211,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6236,9 +6236,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA46" s="5" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6268,25 +6268,25 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
@@ -6306,32 +6306,32 @@
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K47" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L47" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M47" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N47" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O47" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P47" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q47" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R47" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
@@ -6363,14 +6363,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA47" s="5" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -6400,16 +6400,16 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D48" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -6442,28 +6442,28 @@
         </is>
       </c>
       <c r="K48" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L48" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M48" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N48" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O48" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P48" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q48" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R48" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
@@ -6490,31 +6490,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X48" s="5" t="inlineStr">
+      <c r="X48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA48" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y48" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA48" s="5" t="inlineStr">
+      <c r="AB48" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB48" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC48" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6532,12 +6532,12 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D49" s="10">
@@ -6545,121 +6545,253 @@
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K49" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L49" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M49" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N49" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O49" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P49" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q49" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R49" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S49" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T49" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X49" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD49" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="13">
+        <v>1</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D50" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F49" s="0" t="inlineStr">
+      <c r="F50" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
+      <c r="G50" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H49" s="13" t="inlineStr">
+      <c r="H50" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I49" s="13" t="inlineStr">
+      <c r="I50" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J49" s="13" t="inlineStr">
+      <c r="J50" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K49" s="2">
+      <c r="K50" s="2">
         <v>698.2</v>
       </c>
-      <c r="L49" s="2">
+      <c r="L50" s="2">
         <v>272.01</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M50" s="2">
         <v>348.9</v>
       </c>
-      <c r="N49" s="3">
+      <c r="N50" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O49" s="3">
+      <c r="O50" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P50" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q49" s="2">
+      <c r="Q50" s="2">
         <v>282.35</v>
       </c>
-      <c r="R49" s="2">
+      <c r="R50" s="2">
         <v>395.5</v>
       </c>
-      <c r="S49" s="13" t="inlineStr">
+      <c r="S50" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T49" s="13" t="inlineStr">
+      <c r="T50" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X49" s="5" t="inlineStr">
+      <c r="U50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA49" s="5" t="inlineStr">
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB49" s="5" t="inlineStr">
+      <c r="AB50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD49" s="11" t="inlineStr">
+      <c r="AC50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD50" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD49"/>
+  <autoFilter ref="A1:AD50"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -6709,6 +6841,7 @@
     <hyperlink ref="AD47" r:id="rId46"/>
     <hyperlink ref="AD48" r:id="rId47"/>
     <hyperlink ref="AD49" r:id="rId48"/>
+    <hyperlink ref="AD50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Dunelm (Comprar, convicción media)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$51</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2572,20 +2572,20 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>Evolution</t>
+          <t>Dunelm</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>EVO</t>
+          <t>DNLM</t>
         </is>
       </c>
       <c r="D19" s="10">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Suecia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
@@ -2600,46 +2600,46 @@
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K19" s="2">
-        <v>72.2709</v>
+        <v>7.995</v>
       </c>
       <c r="L19" s="2">
-        <v>81.5</v>
+        <v>8.79</v>
       </c>
       <c r="M19" s="2">
-        <v>95.8</v>
+        <v>10.23</v>
       </c>
       <c r="N19" s="3">
-        <v>0.128</v>
+        <v>0.156</v>
       </c>
       <c r="O19" s="3">
-        <v>0.326</v>
+        <v>0.336</v>
       </c>
       <c r="P19" s="2">
-        <v>67.88</v>
+        <v>9.935</v>
       </c>
       <c r="Q19" s="2">
-        <v>83.29</v>
+        <v>8.8</v>
       </c>
       <c r="R19" s="2">
-        <v>103.75</v>
+        <v>11.87</v>
       </c>
       <c r="S19" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="T19" s="13" t="inlineStr">
@@ -2647,9 +2647,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U19" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V19" s="4" t="inlineStr">
@@ -2667,14 +2667,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z19" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA19" s="4" t="inlineStr">
@@ -2687,14 +2687,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC19" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC19" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD19" s="11" t="inlineStr">
         <is>
-          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
+          <t>informes/dunelm-2026-10-10/Dunelm - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -2704,25 +2704,25 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>Constellation</t>
+          <t>Evolution</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>CSU</t>
+          <t>EVO</t>
         </is>
       </c>
       <c r="D20" s="10">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Canadá</t>
+          <t>Suecia</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>Tecnología de la información</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2742,32 +2742,32 @@
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K20" s="2">
-        <v>2104.75</v>
+        <v>72.2709</v>
       </c>
       <c r="L20" s="2">
-        <v>2320.86</v>
+        <v>81.5</v>
       </c>
       <c r="M20" s="2">
-        <v>2710.71</v>
+        <v>95.8</v>
       </c>
       <c r="N20" s="3">
-        <v>0.105</v>
+        <v>0.128</v>
       </c>
       <c r="O20" s="3">
-        <v>0.29</v>
+        <v>0.326</v>
       </c>
       <c r="P20" s="2">
-        <v>2836.45</v>
+        <v>67.88</v>
       </c>
       <c r="Q20" s="2">
-        <v>2214.1</v>
+        <v>83.29</v>
       </c>
       <c r="R20" s="2">
-        <v>3017.12</v>
+        <v>103.75</v>
       </c>
       <c r="S20" s="13" t="inlineStr">
         <is>
@@ -2799,14 +2799,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z20" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA20" s="4" t="inlineStr">
@@ -2819,14 +2819,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC20" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC20" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD20" s="11" t="inlineStr">
         <is>
-          <t>informes/constellation-software-2026-10-10/Constellation Software - 2026-10-10.pdf</t>
+          <t>informes/evolution-2026-10-08/Evolution - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -2836,25 +2836,25 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Constellation</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>CSU</t>
         </is>
       </c>
       <c r="D21" s="10">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Canadá</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Tecnología de la información</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2874,32 +2874,32 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K21" s="2">
-        <v>380.9</v>
+        <v>2104.75</v>
       </c>
       <c r="L21" s="2">
-        <v>410</v>
+        <v>2320.86</v>
       </c>
       <c r="M21" s="2">
-        <v>478.01</v>
+        <v>2710.71</v>
       </c>
       <c r="N21" s="3">
-        <v>0.111</v>
+        <v>0.105</v>
       </c>
       <c r="O21" s="3">
-        <v>0.289</v>
+        <v>0.29</v>
       </c>
       <c r="P21" s="2">
-        <v>526.49</v>
+        <v>2836.45</v>
       </c>
       <c r="Q21" s="2">
-        <v>422.71</v>
+        <v>2214.1</v>
       </c>
       <c r="R21" s="2">
-        <v>530.95</v>
+        <v>3017.12</v>
       </c>
       <c r="S21" s="13" t="inlineStr">
         <is>
@@ -2911,14 +2911,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W21" s="4" t="inlineStr">
@@ -2936,14 +2936,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA21" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA21" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB21" s="4" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="AD21" s="11" t="inlineStr">
         <is>
-          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
+          <t>informes/constellation-software-2026-10-10/Constellation Software - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -2968,25 +2968,25 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D22" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -3010,28 +3010,28 @@
         </is>
       </c>
       <c r="K22" s="2">
-        <v>78.3</v>
+        <v>380.9</v>
       </c>
       <c r="L22" s="2">
-        <v>84.06</v>
+        <v>410</v>
       </c>
       <c r="M22" s="2">
-        <v>97.98</v>
+        <v>478.01</v>
       </c>
       <c r="N22" s="3">
-        <v>0.09300000000000001</v>
+        <v>0.111</v>
       </c>
       <c r="O22" s="3">
-        <v>0.271</v>
+        <v>0.289</v>
       </c>
       <c r="P22" s="2">
-        <v>69.22</v>
+        <v>526.49</v>
       </c>
       <c r="Q22" s="2">
-        <v>86.5</v>
+        <v>422.71</v>
       </c>
       <c r="R22" s="2">
-        <v>110.62</v>
+        <v>530.95</v>
       </c>
       <c r="S22" s="13" t="inlineStr">
         <is>
@@ -3043,14 +3043,14 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W22" s="4" t="inlineStr">
@@ -3058,14 +3058,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z22" s="6" t="inlineStr">
@@ -3073,9 +3073,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA22" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AA22" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB22" s="4" t="inlineStr">
@@ -3083,14 +3083,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC22" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC22" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD22" s="11" t="inlineStr">
         <is>
-          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
+          <t>informes/lvmh-2026-10-08/LVMH - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3100,12 +3100,12 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>Viscofan</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>VIS</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="D23" s="10">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>Consumo básico</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3142,28 +3142,28 @@
         </is>
       </c>
       <c r="K23" s="2">
-        <v>52.9</v>
+        <v>78.3</v>
       </c>
       <c r="L23" s="2">
-        <v>55.98</v>
+        <v>84.06</v>
       </c>
       <c r="M23" s="2">
-        <v>62.5</v>
+        <v>97.98</v>
       </c>
       <c r="N23" s="3">
-        <v>0.12</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="O23" s="3">
-        <v>0.244</v>
+        <v>0.271</v>
       </c>
       <c r="P23" s="2">
-        <v>69.29</v>
+        <v>69.22</v>
       </c>
       <c r="Q23" s="2">
-        <v>57.16</v>
+        <v>86.5</v>
       </c>
       <c r="R23" s="2">
-        <v>65.83</v>
+        <v>110.62</v>
       </c>
       <c r="S23" s="13" t="inlineStr">
         <is>
@@ -3175,9 +3175,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V23" s="4" t="inlineStr">
@@ -3190,19 +3190,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z23" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA23" s="4" t="inlineStr">
@@ -3215,14 +3215,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC23" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC23" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD23" s="11" t="inlineStr">
         <is>
-          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
+          <t>informes/caf-2026-10-06/CAF - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -3232,25 +3232,25 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Cooper</t>
+          <t>Viscofan</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>VIS</t>
         </is>
       </c>
       <c r="D24" s="10">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo básico</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -3270,32 +3270,32 @@
       </c>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K24" s="2">
-        <v>54.3</v>
+        <v>52.9</v>
       </c>
       <c r="L24" s="2">
-        <v>57.1</v>
+        <v>55.98</v>
       </c>
       <c r="M24" s="2">
-        <v>66.21</v>
+        <v>62.5</v>
       </c>
       <c r="N24" s="3">
-        <v>0.052000000000000005</v>
+        <v>0.12</v>
       </c>
       <c r="O24" s="3">
-        <v>0.21899999999999997</v>
+        <v>0.244</v>
       </c>
       <c r="P24" s="2">
-        <v>65.8</v>
+        <v>69.29</v>
       </c>
       <c r="Q24" s="2">
-        <v>57.56</v>
+        <v>57.16</v>
       </c>
       <c r="R24" s="2">
-        <v>73.6</v>
+        <v>65.83</v>
       </c>
       <c r="S24" s="13" t="inlineStr">
         <is>
@@ -3307,19 +3307,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V24" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W24" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U24" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="AD24" s="11" t="inlineStr">
         <is>
-          <t>informes/cooper-companies-2026-10-09/Cooper Companies - 2026-10-09.pdf</t>
+          <t>informes/viscofan-2026-10-06/Viscofan - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -3364,25 +3364,25 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Rentokil</t>
+          <t>Cooper</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="D25" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3406,28 +3406,28 @@
         </is>
       </c>
       <c r="K25" s="2">
-        <v>3.97</v>
+        <v>54.3</v>
       </c>
       <c r="L25" s="2">
-        <v>3.76</v>
+        <v>57.1</v>
       </c>
       <c r="M25" s="2">
-        <v>4.53</v>
+        <v>66.21</v>
       </c>
       <c r="N25" s="3">
-        <v>-0.021</v>
+        <v>0.052000000000000005</v>
       </c>
       <c r="O25" s="3">
-        <v>0.17300000000000001</v>
+        <v>0.21899999999999997</v>
       </c>
       <c r="P25" s="2">
-        <v>6.15</v>
+        <v>65.8</v>
       </c>
       <c r="Q25" s="2">
-        <v>4.05</v>
+        <v>57.56</v>
       </c>
       <c r="R25" s="2">
-        <v>5.05</v>
+        <v>73.6</v>
       </c>
       <c r="S25" s="13" t="inlineStr">
         <is>
@@ -3469,9 +3469,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA25" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA25" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB25" s="4" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="AD25" s="11" t="inlineStr">
         <is>
-          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
+          <t>informes/cooper-companies-2026-10-09/Cooper Companies - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -3496,25 +3496,25 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>bioMérieux</t>
+          <t>Rentokil</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>RTO (LSE); RTO (NYSE, 1 ADS = 5 acciones)</t>
         </is>
       </c>
       <c r="D26" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -3534,32 +3534,32 @@
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K26" s="2">
-        <v>80.75</v>
+        <v>3.97</v>
       </c>
       <c r="L26" s="2">
-        <v>80.93</v>
+        <v>3.76</v>
       </c>
       <c r="M26" s="2">
-        <v>93.63</v>
+        <v>4.53</v>
       </c>
       <c r="N26" s="3">
-        <v>0.013999999999999999</v>
+        <v>-0.021</v>
       </c>
       <c r="O26" s="3">
-        <v>0.172</v>
+        <v>0.17300000000000001</v>
       </c>
       <c r="P26" s="2">
-        <v>79.54</v>
+        <v>6.15</v>
       </c>
       <c r="Q26" s="2">
-        <v>81.9</v>
+        <v>4.05</v>
       </c>
       <c r="R26" s="2">
-        <v>98.17</v>
+        <v>5.05</v>
       </c>
       <c r="S26" s="13" t="inlineStr">
         <is>
@@ -3571,19 +3571,19 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V26" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="W26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X26" s="4" t="inlineStr">
@@ -3591,19 +3591,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y26" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA26" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB26" s="4" t="inlineStr">
@@ -3611,14 +3611,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC26" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC26" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD26" s="11" t="inlineStr">
         <is>
-          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
+          <t>informes/rentokil-2026-10-07/Rentokil Initial - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -3628,12 +3628,12 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>bioMérieux</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="D27" s="10">
@@ -3641,12 +3641,12 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>Financieras</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3666,32 +3666,32 @@
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K27" s="2">
-        <v>152.59</v>
+        <v>80.75</v>
       </c>
       <c r="L27" s="2">
-        <v>160.42</v>
+        <v>80.93</v>
       </c>
       <c r="M27" s="2">
-        <v>173.73</v>
+        <v>93.63</v>
       </c>
       <c r="N27" s="3">
-        <v>0.064</v>
+        <v>0.013999999999999999</v>
       </c>
       <c r="O27" s="3">
-        <v>0.152</v>
+        <v>0.172</v>
       </c>
       <c r="P27" s="2">
-        <v>185.33</v>
+        <v>79.54</v>
       </c>
       <c r="Q27" s="2">
-        <v>152.72</v>
+        <v>81.9</v>
       </c>
       <c r="R27" s="2">
-        <v>186.57</v>
+        <v>98.17</v>
       </c>
       <c r="S27" s="13" t="inlineStr">
         <is>
@@ -3703,39 +3703,39 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V27" s="5" t="inlineStr">
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V27" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="W27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y27" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z27" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA27" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB27" s="4" t="inlineStr">
@@ -3743,14 +3743,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC27" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC27" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AD27" s="11" t="inlineStr">
         <is>
-          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
+          <t>informes/biomerieux-2026-10-08/bioMérieux - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3760,76 +3760,76 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>ICON</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D28" s="10">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Irlanda</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
+          <t>Financieras</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K28" s="2">
+        <v>152.59</v>
+      </c>
+      <c r="L28" s="2">
+        <v>160.42</v>
+      </c>
+      <c r="M28" s="2">
+        <v>173.73</v>
+      </c>
+      <c r="N28" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="O28" s="3">
+        <v>0.152</v>
+      </c>
+      <c r="P28" s="2">
+        <v>185.33</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>152.72</v>
+      </c>
+      <c r="R28" s="2">
+        <v>186.57</v>
+      </c>
+      <c r="S28" s="13" t="inlineStr">
         <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="K28" s="2">
-        <v>164.5</v>
-      </c>
-      <c r="L28" s="2">
-        <v>163.26</v>
-      </c>
-      <c r="M28" s="2">
-        <v>194.24</v>
-      </c>
-      <c r="N28" s="3">
-        <v>-0.008</v>
-      </c>
-      <c r="O28" s="3">
-        <v>0.18100000000000002</v>
-      </c>
-      <c r="P28" s="2">
-        <v>184.41</v>
-      </c>
-      <c r="Q28" s="2">
-        <v>155.42</v>
-      </c>
-      <c r="R28" s="2">
-        <v>202.28</v>
-      </c>
-      <c r="S28" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T28" s="13" t="inlineStr">
         <is>
           <t>Comprar</t>
@@ -3875,14 +3875,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC28" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC28" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
         <is>
-          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
+          <t>informes/ice-2026-10-08/Intercontinental Exchange - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -3892,12 +3892,12 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>ICON</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="D29" s="10">
@@ -3905,12 +3905,12 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Irlanda</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -3920,12 +3920,12 @@
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J29" s="13" t="inlineStr">
@@ -3934,52 +3934,52 @@
         </is>
       </c>
       <c r="K29" s="2">
-        <v>56.56</v>
+        <v>164.5</v>
       </c>
       <c r="L29" s="2">
-        <v>55.24</v>
+        <v>163.26</v>
       </c>
       <c r="M29" s="2">
-        <v>62.35</v>
+        <v>194.24</v>
       </c>
       <c r="N29" s="3">
-        <v>0.002</v>
+        <v>-0.008</v>
       </c>
       <c r="O29" s="3">
-        <v>0.127</v>
+        <v>0.18100000000000002</v>
       </c>
       <c r="P29" s="2">
-        <v>69.91</v>
+        <v>184.41</v>
       </c>
       <c r="Q29" s="2">
-        <v>55.41</v>
+        <v>155.42</v>
       </c>
       <c r="R29" s="2">
-        <v>65.9</v>
+        <v>202.28</v>
       </c>
       <c r="S29" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Vender</t>
         </is>
       </c>
       <c r="T29" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U29" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>Comprar</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V29" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X29" s="4" t="inlineStr">
@@ -3987,9 +3987,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z29" s="6" t="inlineStr">
@@ -3997,9 +3997,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AA29" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AA29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB29" s="4" t="inlineStr">
@@ -4007,14 +4007,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC29" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -4024,16 +4024,16 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D30" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -4066,28 +4066,28 @@
         </is>
       </c>
       <c r="K30" s="2">
-        <v>70.24</v>
+        <v>56.56</v>
       </c>
       <c r="L30" s="2">
-        <v>73.56</v>
+        <v>55.24</v>
       </c>
       <c r="M30" s="2">
-        <v>80.39</v>
+        <v>62.35</v>
       </c>
       <c r="N30" s="3">
-        <v>0.047</v>
+        <v>0.002</v>
       </c>
       <c r="O30" s="3">
-        <v>0.145</v>
+        <v>0.127</v>
       </c>
       <c r="P30" s="2">
-        <v>100.86</v>
+        <v>69.91</v>
       </c>
       <c r="Q30" s="2">
-        <v>69.88</v>
+        <v>55.41</v>
       </c>
       <c r="R30" s="2">
-        <v>89.38</v>
+        <v>65.9</v>
       </c>
       <c r="S30" s="13" t="inlineStr">
         <is>
@@ -4099,9 +4099,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V30" s="4" t="inlineStr">
@@ -4124,14 +4124,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA30" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z30" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA30" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB30" s="4" t="inlineStr">
@@ -4146,13 +4146,13 @@
       </c>
       <c r="AD30" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="D31" s="10">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -4198,28 +4198,28 @@
         </is>
       </c>
       <c r="K31" s="2">
-        <v>71.51</v>
+        <v>70.24</v>
       </c>
       <c r="L31" s="2">
-        <v>73.59</v>
+        <v>73.56</v>
       </c>
       <c r="M31" s="2">
-        <v>80.42</v>
+        <v>80.39</v>
       </c>
       <c r="N31" s="3">
-        <v>0.028999999999999998</v>
+        <v>0.047</v>
       </c>
       <c r="O31" s="3">
-        <v>0.125</v>
+        <v>0.145</v>
       </c>
       <c r="P31" s="2">
         <v>100.86</v>
       </c>
       <c r="Q31" s="2">
-        <v>69.91</v>
+        <v>69.88</v>
       </c>
       <c r="R31" s="2">
-        <v>89.41</v>
+        <v>89.38</v>
       </c>
       <c r="S31" s="13" t="inlineStr">
         <is>
@@ -4261,9 +4261,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA31" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA31" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB31" s="4" t="inlineStr">
@@ -4278,35 +4278,35 @@
       </c>
       <c r="AD31" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D32" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I32" s="13" t="inlineStr">
@@ -4326,32 +4326,32 @@
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K32" s="2">
-        <v>10.18</v>
+        <v>71.51</v>
       </c>
       <c r="L32" s="2">
-        <v>10.41</v>
+        <v>73.59</v>
       </c>
       <c r="M32" s="2">
-        <v>11.23</v>
+        <v>80.42</v>
       </c>
       <c r="N32" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.028999999999999998</v>
       </c>
       <c r="O32" s="3">
-        <v>0.122</v>
+        <v>0.125</v>
       </c>
       <c r="P32" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="Q32" s="2">
-        <v>9.92</v>
+        <v>69.91</v>
       </c>
       <c r="R32" s="2">
-        <v>12.34</v>
+        <v>89.41</v>
       </c>
       <c r="S32" s="13" t="inlineStr">
         <is>
@@ -4363,14 +4363,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -4378,24 +4378,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z32" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA32" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA32" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB32" s="4" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="AD32" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -4420,16 +4420,16 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D33" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -4448,42 +4448,42 @@
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="K33" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="L33" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="M33" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="N33" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O33" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P33" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="Q33" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="R33" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="S33" s="13" t="inlineStr">
         <is>
@@ -4495,14 +4495,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V33" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U33" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V33" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W33" s="4" t="inlineStr">
@@ -4535,14 +4535,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC33" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC33" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -4552,25 +4552,25 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D34" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -4590,32 +4590,32 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K34" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L34" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M34" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N34" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O34" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P34" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q34" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R34" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S34" s="13" t="inlineStr">
         <is>
@@ -4642,39 +4642,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X34" s="5" t="inlineStr">
+      <c r="X34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA34" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y34" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z34" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB34" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC34" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC34" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -4684,25 +4684,25 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D35" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -4722,32 +4722,32 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K35" s="2">
-        <v>26.82</v>
+        <v>2702.5</v>
       </c>
       <c r="L35" s="2">
-        <v>25.71</v>
+        <v>2888.64</v>
       </c>
       <c r="M35" s="2">
-        <v>27.88</v>
+        <v>2897.35</v>
       </c>
       <c r="N35" s="3">
-        <v>-0.040999999999999995</v>
+        <v>0.098</v>
       </c>
       <c r="O35" s="3">
-        <v>0.04</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P35" s="2">
-        <v>39</v>
+        <v>4077.5</v>
       </c>
       <c r="Q35" s="2">
-        <v>24.22</v>
+        <v>2585.33</v>
       </c>
       <c r="R35" s="2">
-        <v>30.98</v>
+        <v>3307.49</v>
       </c>
       <c r="S35" s="13" t="inlineStr">
         <is>
@@ -4774,24 +4774,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y35" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z35" s="5" t="inlineStr">
+      <c r="X35" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA35" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y35" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z35" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA35" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB35" s="4" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="AD35" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -4816,12 +4816,12 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D36" s="10">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F36" s="0" t="inlineStr">
@@ -4849,41 +4849,41 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K36" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L36" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M36" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N36" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O36" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P36" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q36" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R36" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S36" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T36" s="13" t="inlineStr">
@@ -4891,9 +4891,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V36" s="4" t="inlineStr">
@@ -4906,29 +4906,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA36" s="5" t="inlineStr">
+      <c r="X36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z36" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB36" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA36" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB36" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC36" s="4" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="AD36" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -4948,25 +4948,25 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D37" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -4981,56 +4981,56 @@
       </c>
       <c r="I37" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K37" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L37" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M37" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N37" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O37" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P37" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q37" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R37" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S37" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T37" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T37" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U37" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W37" s="4" t="inlineStr">
@@ -5038,39 +5038,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X37" s="5" t="inlineStr">
+      <c r="X37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA37" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y37" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB37" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC37" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB37" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC37" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD37" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5080,25 +5080,25 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -5108,46 +5108,46 @@
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L38" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M38" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N38" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O38" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P38" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q38" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R38" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T38" s="13" t="inlineStr">
@@ -5155,14 +5155,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W38" s="4" t="inlineStr">
@@ -5180,21 +5180,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z38" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA38" s="5" t="inlineStr">
+      <c r="Z38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA38" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB38" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB38" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC38" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -5212,25 +5212,25 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -5250,32 +5250,32 @@
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K39" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L39" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M39" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N39" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O39" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P39" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q39" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R39" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5287,46 +5287,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U39" s="5" t="inlineStr">
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X39" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V39" s="5" t="inlineStr">
+      <c r="Y39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z39" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W39" s="5" t="inlineStr">
+      <c r="AB39" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB39" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC39" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5334,7 +5334,7 @@
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5344,25 +5344,25 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -5382,32 +5382,32 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K40" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L40" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M40" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O40" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P40" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q40" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R40" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5419,9 +5419,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V40" s="5" t="inlineStr">
@@ -5429,19 +5429,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y40" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z40" s="4" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5476,25 +5476,25 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D41" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -5514,32 +5514,32 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L41" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M41" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N41" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O41" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P41" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q41" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R41" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5556,29 +5556,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X41" s="5" t="inlineStr">
+      <c r="V41" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA41" s="5" t="inlineStr">
@@ -5586,19 +5586,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB41" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -5608,79 +5608,79 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G42" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K42" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L42" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M42" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N42" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O42" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P42" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R42" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S42" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H42" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J42" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K42" s="2">
-        <v>129</v>
-      </c>
-      <c r="L42" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M42" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N42" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O42" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P42" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q42" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R42" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S42" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T42" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
@@ -5698,9 +5698,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y42" s="4" t="inlineStr">
@@ -5708,9 +5708,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA42" s="5" t="inlineStr">
@@ -5718,19 +5718,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5740,25 +5740,25 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -5773,37 +5773,37 @@
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K43" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L43" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M43" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N43" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O43" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P43" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q43" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R43" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
@@ -5815,9 +5815,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V43" s="4" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -5872,25 +5872,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
@@ -5905,37 +5905,37 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K44" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L44" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M44" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O44" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P44" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q44" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R44" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
@@ -5947,9 +5947,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U44" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V44" s="4" t="inlineStr">
@@ -5962,39 +5962,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X44" s="5" t="inlineStr">
+      <c r="X44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA44" s="5" t="inlineStr">
+      <c r="AB44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6004,25 +6004,25 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
@@ -6037,37 +6037,37 @@
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K45" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L45" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M45" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N45" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O45" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P45" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q45" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R45" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
@@ -6079,9 +6079,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U45" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V45" s="4" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6136,25 +6136,25 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D46" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
@@ -6169,37 +6169,37 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K46" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L46" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M46" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N46" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O46" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P46" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q46" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R46" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
@@ -6211,14 +6211,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6226,9 +6226,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X46" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y46" s="4" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6268,25 +6268,25 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
@@ -6306,32 +6306,32 @@
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K47" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L47" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M47" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N47" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O47" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P47" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q47" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R47" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
@@ -6343,14 +6343,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">
@@ -6368,9 +6368,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA47" s="5" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6400,25 +6400,25 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D48" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -6428,7 +6428,7 @@
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
@@ -6438,32 +6438,32 @@
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K48" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L48" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M48" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N48" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O48" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P48" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q48" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R48" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
@@ -6495,14 +6495,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA48" s="5" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -6532,16 +6532,16 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -6574,28 +6574,28 @@
         </is>
       </c>
       <c r="K49" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L49" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M49" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O49" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P49" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q49" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R49" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
@@ -6622,31 +6622,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X49" s="5" t="inlineStr">
+      <c r="X49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA49" s="5" t="inlineStr">
+      <c r="AB49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC49" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6664,12 +6664,12 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D50" s="10">
@@ -6677,121 +6677,253 @@
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F50" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J50" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K50" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L50" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M50" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N50" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O50" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P50" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q50" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R50" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S50" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD50" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13">
+        <v>1</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D51" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F50" s="0" t="inlineStr">
+      <c r="F51" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G50" s="9" t="inlineStr">
+      <c r="G51" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H50" s="13" t="inlineStr">
+      <c r="H51" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I50" s="13" t="inlineStr">
+      <c r="I51" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J50" s="13" t="inlineStr">
+      <c r="J51" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K50" s="2">
+      <c r="K51" s="2">
         <v>698.2</v>
       </c>
-      <c r="L50" s="2">
+      <c r="L51" s="2">
         <v>272.01</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M51" s="2">
         <v>348.9</v>
       </c>
-      <c r="N50" s="3">
+      <c r="N51" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O50" s="3">
+      <c r="O51" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P51" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q50" s="2">
+      <c r="Q51" s="2">
         <v>282.35</v>
       </c>
-      <c r="R50" s="2">
+      <c r="R51" s="2">
         <v>395.5</v>
       </c>
-      <c r="S50" s="13" t="inlineStr">
+      <c r="S51" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T50" s="13" t="inlineStr">
+      <c r="T51" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X50" s="5" t="inlineStr">
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA50" s="5" t="inlineStr">
+      <c r="Y51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB50" s="5" t="inlineStr">
+      <c r="AB51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD50" s="11" t="inlineStr">
+      <c r="AC51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD51" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD50"/>
+  <autoFilter ref="A1:AD51"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -6842,6 +6974,7 @@
     <hyperlink ref="AD48" r:id="rId47"/>
     <hyperlink ref="AD49" r:id="rId48"/>
     <hyperlink ref="AD50" r:id="rId49"/>
+    <hyperlink ref="AD51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Netflix (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$56</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -5340,16 +5340,16 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -5368,12 +5368,12 @@
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J40" s="13" t="inlineStr">
@@ -5382,39 +5382,39 @@
         </is>
       </c>
       <c r="K40" s="2">
-        <v>26.82</v>
+        <v>70.3</v>
       </c>
       <c r="L40" s="2">
-        <v>25.71</v>
+        <v>61.1</v>
       </c>
       <c r="M40" s="2">
-        <v>27.88</v>
+        <v>73.49</v>
       </c>
       <c r="N40" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.131</v>
       </c>
       <c r="O40" s="3">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="P40" s="2">
-        <v>39</v>
+        <v>92.55</v>
       </c>
       <c r="Q40" s="2">
-        <v>24.22</v>
+        <v>58.17</v>
       </c>
       <c r="R40" s="2">
-        <v>30.98</v>
+        <v>81.69</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T40" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T40" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5430,9 +5430,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y40" s="4" t="inlineStr">
@@ -5440,19 +5440,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z40" s="5" t="inlineStr">
+      <c r="Z40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA40" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB40" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB40" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC40" s="4" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -5472,12 +5472,12 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D41" s="10">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
@@ -5505,41 +5505,41 @@
       </c>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L41" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M41" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N41" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O41" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P41" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q41" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R41" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T41" s="13" t="inlineStr">
@@ -5547,9 +5547,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V41" s="4" t="inlineStr">
@@ -5562,29 +5562,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA41" s="5" t="inlineStr">
+      <c r="X41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z41" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC41" s="4" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5604,25 +5604,25 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -5637,56 +5637,56 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K42" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L42" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M42" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N42" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O42" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P42" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q42" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R42" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T42" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T42" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U42" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W42" s="4" t="inlineStr">
@@ -5694,39 +5694,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X42" s="5" t="inlineStr">
+      <c r="X42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA42" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB42" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -5736,25 +5736,25 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -5764,46 +5764,46 @@
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K43" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L43" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M43" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N43" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O43" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P43" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q43" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R43" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T43" s="13" t="inlineStr">
@@ -5811,14 +5811,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W43" s="4" t="inlineStr">
@@ -5836,21 +5836,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA43" s="5" t="inlineStr">
+      <c r="Z43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC43" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -5868,25 +5868,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -5906,32 +5906,32 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K44" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L44" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M44" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O44" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P44" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q44" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R44" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
@@ -5943,46 +5943,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U44" s="5" t="inlineStr">
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V44" s="5" t="inlineStr">
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W44" s="5" t="inlineStr">
+      <c r="AB44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC44" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6000,25 +6000,25 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -6038,32 +6038,32 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K45" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L45" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M45" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N45" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O45" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P45" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q45" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R45" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
@@ -6075,9 +6075,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V45" s="5" t="inlineStr">
@@ -6085,19 +6085,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z45" s="4" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6132,25 +6132,25 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D46" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -6170,32 +6170,32 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K46" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L46" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M46" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N46" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O46" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P46" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q46" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R46" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
@@ -6212,29 +6212,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X46" s="5" t="inlineStr">
+      <c r="V46" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA46" s="5" t="inlineStr">
@@ -6242,19 +6242,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB46" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6264,79 +6264,79 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K47" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L47" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M47" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N47" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O47" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P47" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R47" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S47" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H47" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I47" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J47" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K47" s="2">
-        <v>129</v>
-      </c>
-      <c r="L47" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M47" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N47" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O47" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P47" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q47" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R47" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S47" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T47" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U47" s="4" t="inlineStr">
@@ -6354,9 +6354,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X47" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y47" s="4" t="inlineStr">
@@ -6364,9 +6364,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA47" s="5" t="inlineStr">
@@ -6374,19 +6374,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB47" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6396,25 +6396,25 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D48" s="10">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -6429,37 +6429,37 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K48" s="2">
-        <v>53.82</v>
+        <v>129</v>
       </c>
       <c r="L48" s="2">
-        <v>44.48</v>
+        <v>100.16</v>
       </c>
       <c r="M48" s="2">
-        <v>44.65</v>
+        <v>115.11</v>
       </c>
       <c r="N48" s="3">
-        <v>-0.151</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O48" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.081</v>
       </c>
       <c r="P48" s="2">
-        <v>60.39</v>
+        <v>137.09</v>
       </c>
       <c r="Q48" s="2">
-        <v>39.85</v>
+        <v>103.06</v>
       </c>
       <c r="R48" s="2">
-        <v>48.84</v>
+        <v>128.2</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
@@ -6471,9 +6471,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V48" s="4" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6528,25 +6528,25 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -6561,37 +6561,37 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K49" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L49" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M49" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O49" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P49" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q49" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R49" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
@@ -6603,9 +6603,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U49" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V49" s="4" t="inlineStr">
@@ -6618,39 +6618,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X49" s="5" t="inlineStr">
+      <c r="X49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA49" s="5" t="inlineStr">
+      <c r="AB49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
@@ -6693,37 +6693,37 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L50" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M50" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O50" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P50" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q50" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R50" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
@@ -6735,9 +6735,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U50" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V50" s="4" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
@@ -6825,37 +6825,37 @@
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L51" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M51" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O51" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P51" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q51" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R51" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
@@ -6867,14 +6867,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W51" s="4" t="inlineStr">
@@ -6882,9 +6882,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X51" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y51" s="4" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -6952,7 +6952,7 @@
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I52" s="13" t="inlineStr">
@@ -6962,32 +6962,32 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L52" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M52" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N52" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O52" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P52" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q52" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R52" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
@@ -6999,14 +6999,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W52" s="4" t="inlineStr">
@@ -7024,9 +7024,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA52" s="5" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L53" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M53" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O53" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P53" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q53" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R53" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
@@ -7151,14 +7151,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA53" s="5" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,16 +7188,16 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -7230,28 +7230,28 @@
         </is>
       </c>
       <c r="K54" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L54" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M54" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O54" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P54" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q54" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R54" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
@@ -7278,31 +7278,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X54" s="5" t="inlineStr">
+      <c r="X54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA54" s="5" t="inlineStr">
+      <c r="AB54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB54" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC54" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7310,7 +7310,7 @@
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,12 +7320,12 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D55" s="10">
@@ -7333,121 +7333,253 @@
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K55" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L55" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M55" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N55" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O55" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P55" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q55" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R55" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S55" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T55" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X55" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB55" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD55" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13">
+        <v>1</v>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D56" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F55" s="0" t="inlineStr">
+      <c r="F56" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G56" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H55" s="13" t="inlineStr">
+      <c r="H56" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I55" s="13" t="inlineStr">
+      <c r="I56" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J55" s="13" t="inlineStr">
+      <c r="J56" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K55" s="2">
+      <c r="K56" s="2">
         <v>698.2</v>
       </c>
-      <c r="L55" s="2">
+      <c r="L56" s="2">
         <v>272.01</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M56" s="2">
         <v>348.9</v>
       </c>
-      <c r="N55" s="3">
+      <c r="N56" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O55" s="3">
+      <c r="O56" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P56" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q55" s="2">
+      <c r="Q56" s="2">
         <v>282.35</v>
       </c>
-      <c r="R55" s="2">
+      <c r="R56" s="2">
         <v>395.5</v>
       </c>
-      <c r="S55" s="13" t="inlineStr">
+      <c r="S56" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T55" s="13" t="inlineStr">
+      <c r="T56" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X55" s="5" t="inlineStr">
+      <c r="U56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA55" s="5" t="inlineStr">
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="5" t="inlineStr">
+      <c r="AB56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD55" s="11" t="inlineStr">
+      <c r="AC56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD56" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD55"/>
+  <autoFilter ref="A1:AD56"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -7503,6 +7635,7 @@
     <hyperlink ref="AD53" r:id="rId52"/>
     <hyperlink ref="AD54" r:id="rId53"/>
     <hyperlink ref="AD55" r:id="rId54"/>
+    <hyperlink ref="AD56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Hermès (Vender, convicción baja); lecciones de los cinco análisis de la cartera
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$57</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -6528,20 +6528,20 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
@@ -6570,28 +6570,28 @@
         </is>
       </c>
       <c r="K49" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L49" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M49" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O49" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P49" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q49" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R49" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
@@ -6603,9 +6603,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V49" s="4" t="inlineStr">
@@ -6628,9 +6628,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z49" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA49" s="5" t="inlineStr">
@@ -6643,14 +6643,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
@@ -6693,37 +6693,37 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L50" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M50" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O50" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P50" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q50" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R50" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
@@ -6735,9 +6735,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U50" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V50" s="4" t="inlineStr">
@@ -6750,39 +6750,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X50" s="5" t="inlineStr">
+      <c r="X50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA50" s="5" t="inlineStr">
+      <c r="AB50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB50" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
@@ -6825,37 +6825,37 @@
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L51" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M51" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O51" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P51" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q51" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R51" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
@@ -6867,9 +6867,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U51" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V51" s="4" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -6957,37 +6957,37 @@
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L52" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M52" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N52" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O52" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P52" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q52" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R52" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
@@ -6999,14 +6999,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W52" s="4" t="inlineStr">
@@ -7014,9 +7014,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y52" s="4" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -7084,7 +7084,7 @@
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L53" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M53" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O53" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P53" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q53" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R53" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
@@ -7131,14 +7131,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W53" s="4" t="inlineStr">
@@ -7156,9 +7156,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA53" s="5" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,25 +7188,25 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I54" s="13" t="inlineStr">
@@ -7226,32 +7226,32 @@
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K54" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L54" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M54" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O54" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P54" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q54" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R54" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
@@ -7283,14 +7283,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA54" s="5" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,16 +7320,16 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -7362,28 +7362,28 @@
         </is>
       </c>
       <c r="K55" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L55" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M55" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O55" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P55" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q55" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R55" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
@@ -7410,31 +7410,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X55" s="5" t="inlineStr">
+      <c r="X55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA55" s="5" t="inlineStr">
+      <c r="AB55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC55" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,12 +7452,12 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D56" s="10">
@@ -7465,121 +7465,253 @@
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K56" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L56" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M56" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N56" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O56" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P56" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q56" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R56" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S56" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T56" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD56" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13">
+        <v>1</v>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D57" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F56" s="0" t="inlineStr">
+      <c r="F57" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G56" s="9" t="inlineStr">
+      <c r="G57" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H56" s="13" t="inlineStr">
+      <c r="H57" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr">
+      <c r="I57" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J56" s="13" t="inlineStr">
+      <c r="J57" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K56" s="2">
+      <c r="K57" s="2">
         <v>698.2</v>
       </c>
-      <c r="L56" s="2">
+      <c r="L57" s="2">
         <v>272.01</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M57" s="2">
         <v>348.9</v>
       </c>
-      <c r="N56" s="3">
+      <c r="N57" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O56" s="3">
+      <c r="O57" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P57" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q56" s="2">
+      <c r="Q57" s="2">
         <v>282.35</v>
       </c>
-      <c r="R56" s="2">
+      <c r="R57" s="2">
         <v>395.5</v>
       </c>
-      <c r="S56" s="13" t="inlineStr">
+      <c r="S57" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T56" s="13" t="inlineStr">
+      <c r="T57" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X56" s="5" t="inlineStr">
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA56" s="5" t="inlineStr">
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB56" s="5" t="inlineStr">
+      <c r="AB57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD56" s="11" t="inlineStr">
+      <c r="AC57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD57" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD56"/>
+  <autoFilter ref="A1:AD57"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -7636,6 +7768,7 @@
     <hyperlink ref="AD54" r:id="rId53"/>
     <hyperlink ref="AD55" r:id="rId54"/>
     <hyperlink ref="AD56" r:id="rId55"/>
+    <hyperlink ref="AD57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Burkhalter (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$62</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -5076,20 +5076,20 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Burkhalter</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>BRKN</t>
         </is>
       </c>
       <c r="D38" s="10">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F38" s="0" t="inlineStr">
@@ -5104,56 +5104,56 @@
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="K38" s="2">
-        <v>56.56</v>
+        <v>124.6</v>
       </c>
       <c r="L38" s="2">
-        <v>55.24</v>
+        <v>111.78</v>
       </c>
       <c r="M38" s="2">
-        <v>62.35</v>
+        <v>136.6</v>
       </c>
       <c r="N38" s="3">
-        <v>0.002</v>
+        <v>-0.061</v>
       </c>
       <c r="O38" s="3">
-        <v>0.127</v>
+        <v>0.138</v>
       </c>
       <c r="P38" s="2">
-        <v>69.91</v>
+        <v>148.18</v>
       </c>
       <c r="Q38" s="2">
-        <v>55.41</v>
+        <v>111.33</v>
       </c>
       <c r="R38" s="2">
-        <v>65.9</v>
+        <v>151.46</v>
       </c>
       <c r="S38" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T38" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T38" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V38" s="4" t="inlineStr">
@@ -5176,9 +5176,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z38" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z38" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA38" s="5" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="AD38" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/burkhalter-2026-10-11/Burkhalter - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -5208,16 +5208,16 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D39" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -5250,28 +5250,28 @@
         </is>
       </c>
       <c r="K39" s="2">
-        <v>70.24</v>
+        <v>56.56</v>
       </c>
       <c r="L39" s="2">
-        <v>73.56</v>
+        <v>55.24</v>
       </c>
       <c r="M39" s="2">
-        <v>80.39</v>
+        <v>62.35</v>
       </c>
       <c r="N39" s="3">
-        <v>0.047</v>
+        <v>0.002</v>
       </c>
       <c r="O39" s="3">
-        <v>0.145</v>
+        <v>0.127</v>
       </c>
       <c r="P39" s="2">
-        <v>100.86</v>
+        <v>69.91</v>
       </c>
       <c r="Q39" s="2">
-        <v>69.88</v>
+        <v>55.41</v>
       </c>
       <c r="R39" s="2">
-        <v>89.38</v>
+        <v>65.9</v>
       </c>
       <c r="S39" s="13" t="inlineStr">
         <is>
@@ -5283,9 +5283,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V39" s="4" t="inlineStr">
@@ -5308,14 +5308,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA39" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z39" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB39" s="4" t="inlineStr">
@@ -5330,13 +5330,13 @@
       </c>
       <c r="AD39" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
@@ -5349,7 +5349,7 @@
         </is>
       </c>
       <c r="D40" s="10">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -5382,28 +5382,28 @@
         </is>
       </c>
       <c r="K40" s="2">
-        <v>71.51</v>
+        <v>70.24</v>
       </c>
       <c r="L40" s="2">
-        <v>73.59</v>
+        <v>73.56</v>
       </c>
       <c r="M40" s="2">
-        <v>80.42</v>
+        <v>80.39</v>
       </c>
       <c r="N40" s="3">
-        <v>0.028999999999999998</v>
+        <v>0.047</v>
       </c>
       <c r="O40" s="3">
-        <v>0.125</v>
+        <v>0.145</v>
       </c>
       <c r="P40" s="2">
         <v>100.86</v>
       </c>
       <c r="Q40" s="2">
-        <v>69.91</v>
+        <v>69.88</v>
       </c>
       <c r="R40" s="2">
-        <v>89.41</v>
+        <v>89.38</v>
       </c>
       <c r="S40" s="13" t="inlineStr">
         <is>
@@ -5445,9 +5445,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA40" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA40" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB40" s="4" t="inlineStr">
@@ -5462,35 +5462,35 @@
       </c>
       <c r="AD40" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D41" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I41" s="13" t="inlineStr">
@@ -5510,32 +5510,32 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>10.18</v>
+        <v>71.51</v>
       </c>
       <c r="L41" s="2">
-        <v>10.41</v>
+        <v>73.59</v>
       </c>
       <c r="M41" s="2">
-        <v>11.23</v>
+        <v>80.42</v>
       </c>
       <c r="N41" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.028999999999999998</v>
       </c>
       <c r="O41" s="3">
-        <v>0.122</v>
+        <v>0.125</v>
       </c>
       <c r="P41" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="Q41" s="2">
-        <v>9.92</v>
+        <v>69.91</v>
       </c>
       <c r="R41" s="2">
-        <v>12.34</v>
+        <v>89.41</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5547,14 +5547,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W41" s="4" t="inlineStr">
@@ -5562,24 +5562,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA41" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB41" s="4" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -5604,16 +5604,16 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -5632,42 +5632,42 @@
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="K42" s="2">
-        <v>59.72</v>
+        <v>10.18</v>
       </c>
       <c r="L42" s="2">
-        <v>58.59</v>
+        <v>10.41</v>
       </c>
       <c r="M42" s="2">
-        <v>66.22</v>
+        <v>11.23</v>
       </c>
       <c r="N42" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O42" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P42" s="2">
-        <v>67.12</v>
+        <v>14.33</v>
       </c>
       <c r="Q42" s="2">
-        <v>57.83</v>
+        <v>9.92</v>
       </c>
       <c r="R42" s="2">
-        <v>73.94</v>
+        <v>12.34</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
@@ -5679,14 +5679,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V42" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W42" s="4" t="inlineStr">
@@ -5719,14 +5719,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -5736,25 +5736,25 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -5774,32 +5774,32 @@
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K43" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L43" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M43" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N43" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O43" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P43" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q43" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R43" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
@@ -5826,39 +5826,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X43" s="5" t="inlineStr">
+      <c r="X43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB43" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -5868,25 +5868,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -5896,46 +5896,46 @@
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K44" s="2">
-        <v>70.3</v>
+        <v>2702.5</v>
       </c>
       <c r="L44" s="2">
-        <v>61.1</v>
+        <v>2888.64</v>
       </c>
       <c r="M44" s="2">
-        <v>73.49</v>
+        <v>2897.35</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.131</v>
+        <v>0.098</v>
       </c>
       <c r="O44" s="3">
-        <v>0.045</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P44" s="2">
-        <v>92.55</v>
+        <v>4077.5</v>
       </c>
       <c r="Q44" s="2">
-        <v>58.17</v>
+        <v>2585.33</v>
       </c>
       <c r="R44" s="2">
-        <v>81.69</v>
+        <v>3307.49</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T44" s="13" t="inlineStr">
@@ -5958,29 +5958,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA44" s="5" t="inlineStr">
+      <c r="X44" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC44" s="4" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6000,16 +6000,16 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -6028,12 +6028,12 @@
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
@@ -6042,39 +6042,39 @@
         </is>
       </c>
       <c r="K45" s="2">
-        <v>26.82</v>
+        <v>70.3</v>
       </c>
       <c r="L45" s="2">
-        <v>25.71</v>
+        <v>61.1</v>
       </c>
       <c r="M45" s="2">
-        <v>27.88</v>
+        <v>73.49</v>
       </c>
       <c r="N45" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.131</v>
       </c>
       <c r="O45" s="3">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="P45" s="2">
-        <v>39</v>
+        <v>92.55</v>
       </c>
       <c r="Q45" s="2">
-        <v>24.22</v>
+        <v>58.17</v>
       </c>
       <c r="R45" s="2">
-        <v>30.98</v>
+        <v>81.69</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T45" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T45" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U45" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6090,9 +6090,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y45" s="4" t="inlineStr">
@@ -6100,19 +6100,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z45" s="5" t="inlineStr">
+      <c r="Z45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA45" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC45" s="4" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6132,12 +6132,12 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D46" s="10">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
@@ -6165,41 +6165,41 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K46" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L46" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M46" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N46" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O46" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P46" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q46" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R46" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T46" s="13" t="inlineStr">
@@ -6207,9 +6207,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V46" s="4" t="inlineStr">
@@ -6222,29 +6222,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA46" s="5" t="inlineStr">
+      <c r="X46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z46" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC46" s="4" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6264,25 +6264,25 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -6297,56 +6297,56 @@
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K47" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L47" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M47" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N47" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O47" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P47" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q47" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R47" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T47" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T47" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U47" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">
@@ -6354,39 +6354,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X47" s="5" t="inlineStr">
+      <c r="X47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB47" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6396,25 +6396,25 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D48" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -6424,46 +6424,46 @@
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K48" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L48" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M48" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N48" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O48" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P48" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q48" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R48" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T48" s="13" t="inlineStr">
@@ -6471,14 +6471,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U48" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V48" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W48" s="4" t="inlineStr">
@@ -6496,21 +6496,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z48" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA48" s="5" t="inlineStr">
+      <c r="Z48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB48" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC48" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6528,25 +6528,25 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -6566,32 +6566,32 @@
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K49" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L49" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M49" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O49" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P49" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q49" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R49" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
@@ -6603,46 +6603,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U49" s="5" t="inlineStr">
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V49" s="5" t="inlineStr">
+      <c r="Y49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W49" s="5" t="inlineStr">
+      <c r="AB49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC49" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -6698,32 +6698,32 @@
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L50" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M50" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O50" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P50" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q50" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R50" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
@@ -6735,9 +6735,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V50" s="5" t="inlineStr">
@@ -6745,19 +6745,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z50" s="4" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -6830,32 +6830,32 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L51" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M51" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O51" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P51" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q51" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R51" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
@@ -6872,29 +6872,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X51" s="5" t="inlineStr">
+      <c r="V51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA51" s="5" t="inlineStr">
@@ -6902,19 +6902,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB51" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,79 +6924,79 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K52" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L52" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M52" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N52" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O52" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P52" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q52" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R52" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S52" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H52" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I52" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J52" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K52" s="2">
-        <v>129</v>
-      </c>
-      <c r="L52" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M52" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N52" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O52" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P52" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q52" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R52" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S52" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T52" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
@@ -7014,9 +7014,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y52" s="4" t="inlineStr">
@@ -7024,9 +7024,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA52" s="5" t="inlineStr">
@@ -7034,19 +7034,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Hermès</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>1283</v>
+        <v>129</v>
       </c>
       <c r="L53" s="2">
-        <v>937.64</v>
+        <v>100.16</v>
       </c>
       <c r="M53" s="2">
-        <v>1158.7</v>
+        <v>115.11</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.255</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O53" s="3">
-        <v>-0.083</v>
+        <v>-0.081</v>
       </c>
       <c r="P53" s="2">
-        <v>1657.61</v>
+        <v>137.09</v>
       </c>
       <c r="Q53" s="2">
-        <v>909.51</v>
+        <v>103.06</v>
       </c>
       <c r="R53" s="2">
-        <v>1263.94</v>
+        <v>128.2</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
@@ -7156,29 +7156,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z53" s="5" t="inlineStr">
+      <c r="Z53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA53" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA53" s="5" t="inlineStr">
+      <c r="AB53" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB53" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,20 +7188,20 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
@@ -7221,7 +7221,7 @@
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
@@ -7230,28 +7230,28 @@
         </is>
       </c>
       <c r="K54" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L54" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M54" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O54" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P54" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q54" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R54" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
@@ -7263,9 +7263,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V54" s="4" t="inlineStr">
@@ -7288,9 +7288,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z54" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA54" s="5" t="inlineStr">
@@ -7303,14 +7303,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,25 +7320,25 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -7353,37 +7353,37 @@
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K55" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L55" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M55" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O55" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P55" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q55" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R55" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
@@ -7395,9 +7395,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U55" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V55" s="4" t="inlineStr">
@@ -7410,39 +7410,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X55" s="5" t="inlineStr">
+      <c r="X55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA55" s="5" t="inlineStr">
+      <c r="AB55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,25 +7452,25 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
@@ -7485,37 +7485,37 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K56" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L56" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M56" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N56" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O56" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P56" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q56" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R56" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
@@ -7527,9 +7527,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U56" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V56" s="4" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,25 +7584,25 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
@@ -7617,37 +7617,37 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K57" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L57" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M57" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P57" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q57" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R57" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
@@ -7659,14 +7659,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W57" s="4" t="inlineStr">
@@ -7674,9 +7674,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X57" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y57" s="4" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7716,25 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I58" s="13" t="inlineStr">
@@ -7754,32 +7754,32 @@
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K58" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L58" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M58" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P58" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q58" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R58" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
@@ -7791,14 +7791,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W58" s="4" t="inlineStr">
@@ -7816,9 +7816,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA58" s="5" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I59" s="13" t="inlineStr">
@@ -7886,32 +7886,32 @@
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L59" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M59" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P59" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q59" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R59" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7943,14 +7943,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA59" s="5" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,16 +7980,16 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -8022,28 +8022,28 @@
         </is>
       </c>
       <c r="K60" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L60" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M60" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P60" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q60" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R60" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8070,31 +8070,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X60" s="5" t="inlineStr">
+      <c r="X60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA60" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA60" s="5" t="inlineStr">
+      <c r="AB60" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB60" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC60" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,12 +8112,12 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D61" s="10">
@@ -8125,121 +8125,253 @@
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K61" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L61" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M61" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N61" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O61" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P61" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q61" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R61" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S61" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T61" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X61" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA61" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB61" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD61" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13">
+        <v>1</v>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D62" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F61" s="0" t="inlineStr">
+      <c r="F62" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G61" s="9" t="inlineStr">
+      <c r="G62" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H61" s="13" t="inlineStr">
+      <c r="H62" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I61" s="13" t="inlineStr">
+      <c r="I62" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J61" s="13" t="inlineStr">
+      <c r="J62" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K61" s="2">
+      <c r="K62" s="2">
         <v>698.2</v>
       </c>
-      <c r="L61" s="2">
+      <c r="L62" s="2">
         <v>272.01</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M62" s="2">
         <v>348.9</v>
       </c>
-      <c r="N61" s="3">
+      <c r="N62" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O61" s="3">
+      <c r="O62" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P62" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q61" s="2">
+      <c r="Q62" s="2">
         <v>282.35</v>
       </c>
-      <c r="R61" s="2">
+      <c r="R62" s="2">
         <v>395.5</v>
       </c>
-      <c r="S61" s="13" t="inlineStr">
+      <c r="S62" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T61" s="13" t="inlineStr">
+      <c r="T62" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X61" s="5" t="inlineStr">
+      <c r="U62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X62" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA61" s="5" t="inlineStr">
+      <c r="Y62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA62" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB61" s="5" t="inlineStr">
+      <c r="AB62" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD61" s="11" t="inlineStr">
+      <c r="AC62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD62" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD61"/>
+  <autoFilter ref="A1:AD62"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -8301,6 +8433,7 @@
     <hyperlink ref="AD59" r:id="rId58"/>
     <hyperlink ref="AD60" r:id="rId59"/>
     <hyperlink ref="AD61" r:id="rId60"/>
+    <hyperlink ref="AD62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de ATOSS Software (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$64</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -5868,25 +5868,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>ATOSS</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>AOF</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
@@ -5910,39 +5910,39 @@
         </is>
       </c>
       <c r="K44" s="2">
-        <v>59.72</v>
+        <v>87.3</v>
       </c>
       <c r="L44" s="2">
-        <v>58.59</v>
+        <v>80.89</v>
       </c>
       <c r="M44" s="2">
-        <v>66.22</v>
+        <v>94.95</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.013999999999999999</v>
+        <v>-0.047</v>
       </c>
       <c r="O44" s="3">
         <v>0.114</v>
       </c>
       <c r="P44" s="2">
-        <v>67.12</v>
+        <v>120.78</v>
       </c>
       <c r="Q44" s="2">
-        <v>57.83</v>
+        <v>79.19</v>
       </c>
       <c r="R44" s="2">
-        <v>73.94</v>
+        <v>101.11</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T44" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T44" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5963,9 +5963,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z44" s="6" t="inlineStr">
@@ -5978,19 +5978,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AC44" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC44" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/atoss-2026-10-11/ATOSS Software - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6000,25 +6000,25 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -6038,32 +6038,32 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K45" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L45" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M45" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N45" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O45" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P45" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q45" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R45" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
@@ -6090,39 +6090,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X45" s="5" t="inlineStr">
+      <c r="X45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA45" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y45" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB45" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC45" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC45" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -6132,25 +6132,25 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D46" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -6160,46 +6160,46 @@
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K46" s="2">
-        <v>70.3</v>
+        <v>2702.5</v>
       </c>
       <c r="L46" s="2">
-        <v>61.1</v>
+        <v>2888.64</v>
       </c>
       <c r="M46" s="2">
-        <v>73.49</v>
+        <v>2897.35</v>
       </c>
       <c r="N46" s="3">
-        <v>-0.131</v>
+        <v>0.098</v>
       </c>
       <c r="O46" s="3">
-        <v>0.045</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P46" s="2">
-        <v>92.55</v>
+        <v>4077.5</v>
       </c>
       <c r="Q46" s="2">
-        <v>58.17</v>
+        <v>2585.33</v>
       </c>
       <c r="R46" s="2">
-        <v>81.69</v>
+        <v>3307.49</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T46" s="13" t="inlineStr">
@@ -6222,29 +6222,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA46" s="5" t="inlineStr">
+      <c r="X46" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB46" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y46" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB46" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC46" s="4" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6264,16 +6264,16 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -6292,12 +6292,12 @@
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J47" s="13" t="inlineStr">
@@ -6306,39 +6306,39 @@
         </is>
       </c>
       <c r="K47" s="2">
-        <v>26.82</v>
+        <v>70.3</v>
       </c>
       <c r="L47" s="2">
-        <v>25.71</v>
+        <v>61.1</v>
       </c>
       <c r="M47" s="2">
-        <v>27.88</v>
+        <v>73.49</v>
       </c>
       <c r="N47" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.131</v>
       </c>
       <c r="O47" s="3">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="P47" s="2">
-        <v>39</v>
+        <v>92.55</v>
       </c>
       <c r="Q47" s="2">
-        <v>24.22</v>
+        <v>58.17</v>
       </c>
       <c r="R47" s="2">
-        <v>30.98</v>
+        <v>81.69</v>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T47" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T47" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U47" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6354,9 +6354,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y47" s="4" t="inlineStr">
@@ -6364,19 +6364,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z47" s="5" t="inlineStr">
+      <c r="Z47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB47" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB47" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC47" s="4" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6396,12 +6396,12 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D48" s="10">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
@@ -6429,41 +6429,41 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K48" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L48" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M48" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N48" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O48" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P48" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q48" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R48" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T48" s="13" t="inlineStr">
@@ -6471,9 +6471,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V48" s="4" t="inlineStr">
@@ -6486,29 +6486,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA48" s="5" t="inlineStr">
+      <c r="X48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z48" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC48" s="4" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6528,25 +6528,25 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -6561,56 +6561,56 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K49" s="2">
-        <v>2000</v>
+        <v>577.5</v>
       </c>
       <c r="L49" s="2">
-        <v>1932.11</v>
+        <v>466.62</v>
       </c>
       <c r="M49" s="2">
-        <v>1939.91</v>
+        <v>564.55</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.019</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O49" s="3">
-        <v>-0.015</v>
+        <v>0.005</v>
       </c>
       <c r="P49" s="2">
-        <v>2184.62</v>
+        <v>795.86</v>
       </c>
       <c r="Q49" s="2">
-        <v>1711.85</v>
+        <v>504.42</v>
       </c>
       <c r="R49" s="2">
-        <v>2020.99</v>
+        <v>645.34</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T49" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T49" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U49" s="6" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="V49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="V49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W49" s="4" t="inlineStr">
@@ -6618,39 +6618,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X49" s="5" t="inlineStr">
+      <c r="X49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB49" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -6688,46 +6688,46 @@
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L50" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M50" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O50" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P50" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q50" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R50" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T50" s="13" t="inlineStr">
@@ -6735,14 +6735,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W50" s="4" t="inlineStr">
@@ -6760,21 +6760,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA50" s="5" t="inlineStr">
+      <c r="Z50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB50" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC50" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -6830,32 +6830,32 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L51" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M51" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O51" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P51" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q51" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R51" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
@@ -6867,46 +6867,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U51" s="5" t="inlineStr">
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V51" s="5" t="inlineStr">
+      <c r="Y51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W51" s="5" t="inlineStr">
+      <c r="AB51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC51" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -6962,32 +6962,32 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L52" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M52" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N52" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O52" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P52" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q52" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R52" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
@@ -6999,9 +6999,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V52" s="5" t="inlineStr">
@@ -7009,19 +7009,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z52" s="4" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L53" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M53" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O53" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P53" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q53" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R53" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
@@ -7136,29 +7136,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X53" s="5" t="inlineStr">
+      <c r="V53" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA53" s="5" t="inlineStr">
@@ -7166,19 +7166,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,79 +7188,79 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K54" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L54" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M54" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N54" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O54" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P54" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q54" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R54" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S54" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H54" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I54" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J54" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K54" s="2">
-        <v>129</v>
-      </c>
-      <c r="L54" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M54" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N54" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O54" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P54" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q54" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R54" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S54" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T54" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
@@ -7278,9 +7278,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X54" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y54" s="4" t="inlineStr">
@@ -7288,9 +7288,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA54" s="5" t="inlineStr">
@@ -7298,19 +7298,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB54" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,25 +7320,25 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Hermès</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -7358,32 +7358,32 @@
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K55" s="2">
-        <v>1283</v>
+        <v>129</v>
       </c>
       <c r="L55" s="2">
-        <v>937.64</v>
+        <v>100.16</v>
       </c>
       <c r="M55" s="2">
-        <v>1158.7</v>
+        <v>115.11</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.255</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O55" s="3">
-        <v>-0.083</v>
+        <v>-0.081</v>
       </c>
       <c r="P55" s="2">
-        <v>1657.61</v>
+        <v>137.09</v>
       </c>
       <c r="Q55" s="2">
-        <v>909.51</v>
+        <v>103.06</v>
       </c>
       <c r="R55" s="2">
-        <v>1263.94</v>
+        <v>128.2</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
@@ -7420,29 +7420,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z55" s="5" t="inlineStr">
+      <c r="Z55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA55" s="5" t="inlineStr">
+      <c r="AB55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,20 +7452,20 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
@@ -7494,28 +7494,28 @@
         </is>
       </c>
       <c r="K56" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L56" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M56" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N56" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O56" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P56" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q56" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R56" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
@@ -7527,9 +7527,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V56" s="4" t="inlineStr">
@@ -7552,9 +7552,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA56" s="5" t="inlineStr">
@@ -7567,14 +7567,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,25 +7584,25 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
@@ -7617,37 +7617,37 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K57" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L57" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M57" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P57" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q57" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R57" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
@@ -7659,9 +7659,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U57" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V57" s="4" t="inlineStr">
@@ -7674,39 +7674,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X57" s="5" t="inlineStr">
+      <c r="X57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA57" s="5" t="inlineStr">
+      <c r="AB57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB57" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7716,25 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -7749,37 +7749,37 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K58" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L58" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M58" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P58" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q58" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R58" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
@@ -7791,9 +7791,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U58" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V58" s="4" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -7881,37 +7881,37 @@
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L59" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M59" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P59" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q59" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R59" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7923,14 +7923,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W59" s="4" t="inlineStr">
@@ -7938,9 +7938,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X59" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y59" s="4" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,25 +7980,25 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I60" s="13" t="inlineStr">
@@ -8018,32 +8018,32 @@
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K60" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L60" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M60" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P60" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q60" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R60" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8055,14 +8055,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W60" s="4" t="inlineStr">
@@ -8080,9 +8080,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA60" s="5" t="inlineStr">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,25 +8112,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D61" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="H61" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I61" s="13" t="inlineStr">
@@ -8150,32 +8150,32 @@
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K61" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L61" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M61" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N61" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O61" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P61" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q61" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R61" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S61" s="13" t="inlineStr">
         <is>
@@ -8207,14 +8207,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA61" s="5" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="AD61" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -8244,16 +8244,16 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D62" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
@@ -8262,7 +8262,7 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
@@ -8286,28 +8286,28 @@
         </is>
       </c>
       <c r="K62" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L62" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M62" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N62" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O62" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P62" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q62" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R62" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S62" s="13" t="inlineStr">
         <is>
@@ -8334,31 +8334,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X62" s="5" t="inlineStr">
+      <c r="X62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA62" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y62" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z62" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA62" s="5" t="inlineStr">
+      <c r="AB62" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB62" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC62" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8366,7 +8366,7 @@
       </c>
       <c r="AD62" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8376,12 +8376,12 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D63" s="10">
@@ -8389,121 +8389,253 @@
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J63" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K63" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L63" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M63" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N63" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O63" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P63" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q63" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R63" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S63" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T63" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X63" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z63" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA63" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB63" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD63" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13">
+        <v>1</v>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D64" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F63" s="0" t="inlineStr">
+      <c r="F64" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G63" s="9" t="inlineStr">
+      <c r="G64" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H63" s="13" t="inlineStr">
+      <c r="H64" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I63" s="13" t="inlineStr">
+      <c r="I64" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J63" s="13" t="inlineStr">
+      <c r="J64" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K63" s="2">
+      <c r="K64" s="2">
         <v>698.2</v>
       </c>
-      <c r="L63" s="2">
+      <c r="L64" s="2">
         <v>272.01</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M64" s="2">
         <v>348.9</v>
       </c>
-      <c r="N63" s="3">
+      <c r="N64" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O63" s="3">
+      <c r="O64" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P64" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q63" s="2">
+      <c r="Q64" s="2">
         <v>282.35</v>
       </c>
-      <c r="R63" s="2">
+      <c r="R64" s="2">
         <v>395.5</v>
       </c>
-      <c r="S63" s="13" t="inlineStr">
+      <c r="S64" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T63" s="13" t="inlineStr">
+      <c r="T64" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X63" s="5" t="inlineStr">
+      <c r="U64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X64" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA63" s="5" t="inlineStr">
+      <c r="Y64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA64" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB63" s="5" t="inlineStr">
+      <c r="AB64" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC63" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD63" s="11" t="inlineStr">
+      <c r="AC64" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD64" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD63"/>
+  <autoFilter ref="A1:AD64"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -8567,6 +8699,7 @@
     <hyperlink ref="AD61" r:id="rId60"/>
     <hyperlink ref="AD62" r:id="rId61"/>
     <hyperlink ref="AD63" r:id="rId62"/>
+    <hyperlink ref="AD64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de S&P Global (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$65</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>SPGI</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -6688,61 +6688,61 @@
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>2000</v>
+        <v>407.82</v>
       </c>
       <c r="L50" s="2">
-        <v>1932.11</v>
+        <v>351.69</v>
       </c>
       <c r="M50" s="2">
-        <v>1939.91</v>
+        <v>398.1</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.019</v>
+        <v>-0.128</v>
       </c>
       <c r="O50" s="3">
-        <v>-0.015</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="P50" s="2">
-        <v>2184.62</v>
+        <v>516.86</v>
       </c>
       <c r="Q50" s="2">
-        <v>1711.85</v>
+        <v>338.33</v>
       </c>
       <c r="R50" s="2">
-        <v>2020.99</v>
+        <v>446.65</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T50" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V50" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W50" s="4" t="inlineStr">
@@ -6750,39 +6750,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X50" s="5" t="inlineStr">
+      <c r="X50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
       <c r="AB50" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/sp-global-2026-10-12/S&amp;P Global - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -6820,46 +6820,46 @@
       </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L51" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M51" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O51" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P51" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q51" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R51" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T51" s="13" t="inlineStr">
@@ -6867,14 +6867,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W51" s="4" t="inlineStr">
@@ -6892,21 +6892,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA51" s="5" t="inlineStr">
+      <c r="Z51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC51" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -6962,32 +6962,32 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L52" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M52" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N52" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O52" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P52" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q52" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R52" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
@@ -6999,46 +6999,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U52" s="5" t="inlineStr">
+      <c r="U52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X52" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V52" s="5" t="inlineStr">
+      <c r="Y52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W52" s="5" t="inlineStr">
+      <c r="AB52" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC52" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -7046,7 +7046,7 @@
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -7094,32 +7094,32 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>128.3</v>
+        <v>16.22</v>
       </c>
       <c r="L53" s="2">
-        <v>99</v>
+        <v>13.97</v>
       </c>
       <c r="M53" s="2">
-        <v>117</v>
+        <v>14.66</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.077</v>
       </c>
       <c r="O53" s="3">
-        <v>-0.065</v>
+        <v>-0.035</v>
       </c>
       <c r="P53" s="2">
-        <v>128.84</v>
+        <v>17.05</v>
       </c>
       <c r="Q53" s="2">
-        <v>97.02</v>
+        <v>13.61</v>
       </c>
       <c r="R53" s="2">
-        <v>132.07</v>
+        <v>16.41</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
@@ -7131,9 +7131,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="V53" s="5" t="inlineStr">
@@ -7141,19 +7141,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="W53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="X53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Z53" s="4" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,25 +7188,25 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
@@ -7226,32 +7226,32 @@
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K54" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L54" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M54" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O54" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P54" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q54" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R54" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
@@ -7268,29 +7268,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X54" s="5" t="inlineStr">
+      <c r="V54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA54" s="5" t="inlineStr">
@@ -7298,19 +7298,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB54" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,79 +7320,79 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K55" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L55" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M55" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N55" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O55" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P55" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q55" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R55" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S55" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H55" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I55" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J55" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K55" s="2">
-        <v>129</v>
-      </c>
-      <c r="L55" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M55" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N55" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O55" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P55" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q55" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R55" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S55" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T55" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U55" s="4" t="inlineStr">
@@ -7410,9 +7410,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X55" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y55" s="4" t="inlineStr">
@@ -7420,9 +7420,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA55" s="5" t="inlineStr">
@@ -7430,19 +7430,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,25 +7452,25 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>Hermès</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
@@ -7490,32 +7490,32 @@
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K56" s="2">
-        <v>1283</v>
+        <v>129</v>
       </c>
       <c r="L56" s="2">
-        <v>937.64</v>
+        <v>100.16</v>
       </c>
       <c r="M56" s="2">
-        <v>1158.7</v>
+        <v>115.11</v>
       </c>
       <c r="N56" s="3">
-        <v>-0.255</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O56" s="3">
-        <v>-0.083</v>
+        <v>-0.081</v>
       </c>
       <c r="P56" s="2">
-        <v>1657.61</v>
+        <v>137.09</v>
       </c>
       <c r="Q56" s="2">
-        <v>909.51</v>
+        <v>103.06</v>
       </c>
       <c r="R56" s="2">
-        <v>1263.94</v>
+        <v>128.2</v>
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
@@ -7552,29 +7552,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z56" s="5" t="inlineStr">
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA56" s="5" t="inlineStr">
+      <c r="AB56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB56" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,20 +7584,20 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
@@ -7617,7 +7617,7 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
@@ -7626,28 +7626,28 @@
         </is>
       </c>
       <c r="K57" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L57" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M57" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P57" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q57" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R57" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
@@ -7659,9 +7659,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V57" s="4" t="inlineStr">
@@ -7684,9 +7684,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z57" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA57" s="5" t="inlineStr">
@@ -7699,14 +7699,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7716,25 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -7749,37 +7749,37 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K58" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L58" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M58" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P58" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q58" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R58" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
@@ -7791,9 +7791,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U58" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V58" s="4" t="inlineStr">
@@ -7806,39 +7806,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X58" s="5" t="inlineStr">
+      <c r="X58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z58" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA58" s="5" t="inlineStr">
+      <c r="AB58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -7881,37 +7881,37 @@
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L59" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M59" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P59" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q59" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R59" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7923,9 +7923,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U59" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V59" s="4" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,25 +7980,25 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -8013,37 +8013,37 @@
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K60" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L60" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M60" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P60" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q60" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R60" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8055,14 +8055,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W60" s="4" t="inlineStr">
@@ -8070,9 +8070,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X60" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y60" s="4" t="inlineStr">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,25 +8112,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D61" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="H61" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I61" s="13" t="inlineStr">
@@ -8150,32 +8150,32 @@
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K61" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L61" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M61" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N61" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O61" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P61" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q61" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R61" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S61" s="13" t="inlineStr">
         <is>
@@ -8187,14 +8187,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W61" s="4" t="inlineStr">
@@ -8212,9 +8212,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA61" s="5" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="AD61" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8244,25 +8244,25 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D62" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I62" s="13" t="inlineStr">
@@ -8282,32 +8282,32 @@
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K62" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L62" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M62" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N62" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O62" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P62" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q62" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R62" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S62" s="13" t="inlineStr">
         <is>
@@ -8339,14 +8339,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y62" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z62" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA62" s="5" t="inlineStr">
@@ -8366,7 +8366,7 @@
       </c>
       <c r="AD62" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -8376,16 +8376,16 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D63" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
@@ -8418,28 +8418,28 @@
         </is>
       </c>
       <c r="K63" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L63" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M63" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N63" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O63" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P63" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q63" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R63" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S63" s="13" t="inlineStr">
         <is>
@@ -8466,31 +8466,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X63" s="5" t="inlineStr">
+      <c r="X63" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y63" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z63" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA63" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z63" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA63" s="5" t="inlineStr">
+      <c r="AB63" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB63" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC63" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD63" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8508,12 +8508,12 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D64" s="10">
@@ -8521,121 +8521,253 @@
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J64" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K64" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L64" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M64" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N64" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O64" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P64" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q64" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R64" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S64" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T64" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X64" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z64" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA64" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB64" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD64" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="13">
+        <v>1</v>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D65" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F64" s="0" t="inlineStr">
+      <c r="F65" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G64" s="9" t="inlineStr">
+      <c r="G65" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H64" s="13" t="inlineStr">
+      <c r="H65" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I64" s="13" t="inlineStr">
+      <c r="I65" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J64" s="13" t="inlineStr">
+      <c r="J65" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K64" s="2">
+      <c r="K65" s="2">
         <v>698.2</v>
       </c>
-      <c r="L64" s="2">
+      <c r="L65" s="2">
         <v>272.01</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M65" s="2">
         <v>348.9</v>
       </c>
-      <c r="N64" s="3">
+      <c r="N65" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O64" s="3">
+      <c r="O65" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P65" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q64" s="2">
+      <c r="Q65" s="2">
         <v>282.35</v>
       </c>
-      <c r="R64" s="2">
+      <c r="R65" s="2">
         <v>395.5</v>
       </c>
-      <c r="S64" s="13" t="inlineStr">
+      <c r="S65" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T64" s="13" t="inlineStr">
+      <c r="T65" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X64" s="5" t="inlineStr">
+      <c r="U65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X65" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA64" s="5" t="inlineStr">
+      <c r="Y65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA65" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB64" s="5" t="inlineStr">
+      <c r="AB65" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC64" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD64" s="11" t="inlineStr">
+      <c r="AC65" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD65" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD64"/>
+  <autoFilter ref="A1:AD65"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -8700,6 +8832,7 @@
     <hyperlink ref="AD62" r:id="rId61"/>
     <hyperlink ref="AD63" r:id="rId62"/>
     <hyperlink ref="AD64" r:id="rId63"/>
+    <hyperlink ref="AD65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Amazon (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$66</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -7188,25 +7188,25 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
@@ -7230,28 +7230,28 @@
         </is>
       </c>
       <c r="K54" s="2">
-        <v>128.3</v>
+        <v>262.43</v>
       </c>
       <c r="L54" s="2">
-        <v>99</v>
+        <v>213.96</v>
       </c>
       <c r="M54" s="2">
-        <v>117</v>
+        <v>251.97</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.185</v>
       </c>
       <c r="O54" s="3">
-        <v>-0.065</v>
+        <v>-0.04</v>
       </c>
       <c r="P54" s="2">
-        <v>128.84</v>
+        <v>331.36</v>
       </c>
       <c r="Q54" s="2">
-        <v>97.02</v>
+        <v>203.69</v>
       </c>
       <c r="R54" s="2">
-        <v>132.07</v>
+        <v>271.09</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
@@ -7268,29 +7268,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V54" s="5" t="inlineStr">
+      <c r="V54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA54" s="5" t="inlineStr">
@@ -7303,14 +7303,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/amazon-2026-10-12/Amazon - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,25 +7320,25 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -7358,32 +7358,32 @@
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K55" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L55" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M55" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O55" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P55" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q55" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R55" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
@@ -7400,29 +7400,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X55" s="5" t="inlineStr">
+      <c r="V55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA55" s="5" t="inlineStr">
@@ -7430,19 +7430,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB55" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,79 +7452,79 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K56" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L56" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M56" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N56" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O56" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P56" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q56" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R56" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S56" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H56" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I56" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K56" s="2">
-        <v>129</v>
-      </c>
-      <c r="L56" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M56" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N56" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O56" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P56" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q56" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R56" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S56" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T56" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
@@ -7542,9 +7542,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y56" s="4" t="inlineStr">
@@ -7552,9 +7552,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA56" s="5" t="inlineStr">
@@ -7562,19 +7562,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB56" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,25 +7584,25 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Hermès</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
@@ -7622,32 +7622,32 @@
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K57" s="2">
-        <v>1283</v>
+        <v>129</v>
       </c>
       <c r="L57" s="2">
-        <v>937.64</v>
+        <v>100.16</v>
       </c>
       <c r="M57" s="2">
-        <v>1158.7</v>
+        <v>115.11</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.255</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.083</v>
+        <v>-0.081</v>
       </c>
       <c r="P57" s="2">
-        <v>1657.61</v>
+        <v>137.09</v>
       </c>
       <c r="Q57" s="2">
-        <v>909.51</v>
+        <v>103.06</v>
       </c>
       <c r="R57" s="2">
-        <v>1263.94</v>
+        <v>128.2</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
@@ -7684,29 +7684,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z57" s="5" t="inlineStr">
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA57" s="5" t="inlineStr">
+      <c r="AB57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB57" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,20 +7716,20 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
@@ -7758,28 +7758,28 @@
         </is>
       </c>
       <c r="K58" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L58" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M58" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P58" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q58" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R58" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
@@ -7791,9 +7791,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U58" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V58" s="4" t="inlineStr">
@@ -7816,9 +7816,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z58" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA58" s="5" t="inlineStr">
@@ -7831,14 +7831,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC58" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -7881,37 +7881,37 @@
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L59" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M59" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P59" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q59" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R59" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7923,9 +7923,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U59" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U59" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V59" s="4" t="inlineStr">
@@ -7938,39 +7938,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X59" s="5" t="inlineStr">
+      <c r="X59" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA59" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA59" s="5" t="inlineStr">
+      <c r="AB59" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB59" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC59" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,25 +7980,25 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -8013,37 +8013,37 @@
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K60" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L60" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M60" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P60" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q60" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R60" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8055,9 +8055,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U60" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V60" s="4" t="inlineStr">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,25 +8112,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D61" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
@@ -8145,37 +8145,37 @@
       </c>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K61" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L61" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M61" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N61" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O61" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P61" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q61" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R61" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S61" s="13" t="inlineStr">
         <is>
@@ -8187,14 +8187,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W61" s="4" t="inlineStr">
@@ -8202,9 +8202,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X61" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y61" s="4" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="AD61" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -8244,25 +8244,25 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D62" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I62" s="13" t="inlineStr">
@@ -8282,32 +8282,32 @@
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K62" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L62" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M62" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N62" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O62" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P62" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q62" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R62" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S62" s="13" t="inlineStr">
         <is>
@@ -8319,14 +8319,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U62" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V62" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W62" s="4" t="inlineStr">
@@ -8344,9 +8344,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z62" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA62" s="5" t="inlineStr">
@@ -8366,7 +8366,7 @@
       </c>
       <c r="AD62" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8376,25 +8376,25 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D63" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
@@ -8404,7 +8404,7 @@
       </c>
       <c r="H63" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I63" s="13" t="inlineStr">
@@ -8414,32 +8414,32 @@
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K63" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L63" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M63" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N63" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O63" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P63" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q63" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R63" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S63" s="13" t="inlineStr">
         <is>
@@ -8471,14 +8471,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y63" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z63" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA63" s="5" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD63" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -8508,16 +8508,16 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D64" s="10">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
@@ -8526,7 +8526,7 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
@@ -8550,28 +8550,28 @@
         </is>
       </c>
       <c r="K64" s="2">
-        <v>404.76</v>
+        <v>253.14</v>
       </c>
       <c r="L64" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="M64" s="2">
-        <v>222.49</v>
+        <v>168.18</v>
       </c>
       <c r="N64" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="O64" s="3">
-        <v>-0.45</v>
+        <v>-0.335</v>
       </c>
       <c r="P64" s="2">
-        <v>477.21</v>
+        <v>337.43</v>
       </c>
       <c r="Q64" s="2">
-        <v>193.34</v>
+        <v>146.32</v>
       </c>
       <c r="R64" s="2">
-        <v>247.41</v>
+        <v>187.18</v>
       </c>
       <c r="S64" s="13" t="inlineStr">
         <is>
@@ -8598,31 +8598,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X64" s="5" t="inlineStr">
+      <c r="X64" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y64" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z64" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA64" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z64" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA64" s="5" t="inlineStr">
+      <c r="AB64" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB64" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC64" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8630,7 +8630,7 @@
       </c>
       <c r="AD64" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8640,12 +8640,12 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D65" s="10">
@@ -8653,121 +8653,253 @@
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H65" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J65" s="13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K65" s="2">
+        <v>404.76</v>
+      </c>
+      <c r="L65" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="M65" s="2">
+        <v>222.49</v>
+      </c>
+      <c r="N65" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="O65" s="3">
+        <v>-0.45</v>
+      </c>
+      <c r="P65" s="2">
+        <v>477.21</v>
+      </c>
+      <c r="Q65" s="2">
+        <v>193.34</v>
+      </c>
+      <c r="R65" s="2">
+        <v>247.41</v>
+      </c>
+      <c r="S65" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T65" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X65" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z65" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA65" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB65" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD65" s="11" t="inlineStr">
+        <is>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13">
+        <v>1</v>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D66" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="F65" s="0" t="inlineStr">
+      <c r="F66" s="0" t="inlineStr">
         <is>
           <t>Tecnologías de la información</t>
         </is>
       </c>
-      <c r="G65" s="9" t="inlineStr">
+      <c r="G66" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H65" s="13" t="inlineStr">
+      <c r="H66" s="13" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I65" s="13" t="inlineStr">
+      <c r="I66" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J65" s="13" t="inlineStr">
+      <c r="J66" s="13" t="inlineStr">
         <is>
           <t>CHF</t>
         </is>
       </c>
-      <c r="K65" s="2">
+      <c r="K66" s="2">
         <v>698.2</v>
       </c>
-      <c r="L65" s="2">
+      <c r="L66" s="2">
         <v>272.01</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M66" s="2">
         <v>348.9</v>
       </c>
-      <c r="N65" s="3">
+      <c r="N66" s="3">
         <v>-0.6</v>
       </c>
-      <c r="O65" s="3">
+      <c r="O66" s="3">
         <v>-0.49</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P66" s="2">
         <v>713.11</v>
       </c>
-      <c r="Q65" s="2">
+      <c r="Q66" s="2">
         <v>282.35</v>
       </c>
-      <c r="R65" s="2">
+      <c r="R66" s="2">
         <v>395.5</v>
       </c>
-      <c r="S65" s="13" t="inlineStr">
+      <c r="S66" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T65" s="13" t="inlineStr">
+      <c r="T66" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X65" s="5" t="inlineStr">
+      <c r="U66" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V66" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W66" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X66" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA65" s="5" t="inlineStr">
+      <c r="Y66" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z66" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA66" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB65" s="5" t="inlineStr">
+      <c r="AB66" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC65" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AD65" s="11" t="inlineStr">
+      <c r="AC66" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD66" s="11" t="inlineStr">
         <is>
           <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD65"/>
+  <autoFilter ref="A1:AD66"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -8833,6 +8965,7 @@
     <hyperlink ref="AD63" r:id="rId62"/>
     <hyperlink ref="AD64" r:id="rId63"/>
     <hyperlink ref="AD65" r:id="rId64"/>
+    <hyperlink ref="AD66" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Pro Medicus (Vender, convicción alta) y rentabilidad a 6 meses de las dos carteras
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$70</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -9294,8 +9294,140 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="13">
+        <v>1</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>Pro Medicus</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>PME</t>
+        </is>
+      </c>
+      <c r="D70" s="10">
+        <v>46307</v>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="K70" s="2">
+        <v>168.37</v>
+      </c>
+      <c r="L70" s="2">
+        <v>50.61</v>
+      </c>
+      <c r="M70" s="2">
+        <v>58.79</v>
+      </c>
+      <c r="N70" s="3">
+        <v>-0.695</v>
+      </c>
+      <c r="O70" s="3">
+        <v>-0.647</v>
+      </c>
+      <c r="P70" s="2">
+        <v>202.47</v>
+      </c>
+      <c r="Q70" s="2">
+        <v>48.84</v>
+      </c>
+      <c r="R70" s="2">
+        <v>66.1</v>
+      </c>
+      <c r="S70" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T70" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD70" s="11" t="inlineStr">
+        <is>
+          <t>informes/pro-medicus-2026-10-12/Pro Medicus - 2026-10-12.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AD69"/>
+  <autoFilter ref="A1:AD70"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -9365,6 +9497,7 @@
     <hyperlink ref="AD67" r:id="rId66"/>
     <hyperlink ref="AD68" r:id="rId67"/>
     <hyperlink ref="AD69" r:id="rId68"/>
+    <hyperlink ref="AD70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Medpace (Vender, convicción media)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$71</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -9036,16 +9036,16 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Medpace</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D68" s="10">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I68" s="13" t="inlineStr">
@@ -9078,28 +9078,28 @@
         </is>
       </c>
       <c r="K68" s="2">
-        <v>404.76</v>
+        <v>612.05</v>
       </c>
       <c r="L68" s="2">
-        <v>222.49</v>
+        <v>326.15</v>
       </c>
       <c r="M68" s="2">
-        <v>222.49</v>
+        <v>382.27</v>
       </c>
       <c r="N68" s="3">
-        <v>-0.45</v>
+        <v>-0.467</v>
       </c>
       <c r="O68" s="3">
-        <v>-0.45</v>
+        <v>-0.375</v>
       </c>
       <c r="P68" s="2">
-        <v>477.21</v>
+        <v>595.92</v>
       </c>
       <c r="Q68" s="2">
-        <v>193.34</v>
+        <v>310.49</v>
       </c>
       <c r="R68" s="2">
-        <v>247.41</v>
+        <v>424.97</v>
       </c>
       <c r="S68" s="13" t="inlineStr">
         <is>
@@ -9126,39 +9126,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X68" s="5" t="inlineStr">
+      <c r="X68" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y68" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z68" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA68" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y68" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z68" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA68" s="5" t="inlineStr">
+      <c r="AB68" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB68" s="5" t="inlineStr">
+      <c r="AC68" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC68" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AD68" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/medpace-2026-10-12/Medpace - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -9168,12 +9168,12 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D69" s="10">
@@ -9181,12 +9181,12 @@
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
@@ -9206,32 +9206,32 @@
       </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K69" s="2">
-        <v>698.2</v>
+        <v>404.76</v>
       </c>
       <c r="L69" s="2">
-        <v>272.01</v>
+        <v>222.49</v>
       </c>
       <c r="M69" s="2">
-        <v>348.9</v>
+        <v>222.49</v>
       </c>
       <c r="N69" s="3">
-        <v>-0.6</v>
+        <v>-0.45</v>
       </c>
       <c r="O69" s="3">
-        <v>-0.49</v>
+        <v>-0.45</v>
       </c>
       <c r="P69" s="2">
-        <v>713.11</v>
+        <v>477.21</v>
       </c>
       <c r="Q69" s="2">
-        <v>282.35</v>
+        <v>193.34</v>
       </c>
       <c r="R69" s="2">
-        <v>395.5</v>
+        <v>247.41</v>
       </c>
       <c r="S69" s="13" t="inlineStr">
         <is>
@@ -9268,9 +9268,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z69" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z69" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA69" s="5" t="inlineStr">
@@ -9283,14 +9283,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC69" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC69" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD69" s="11" t="inlineStr">
         <is>
-          <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -9300,134 +9300,266 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D70" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>Suiza</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="K70" s="2">
+        <v>698.2</v>
+      </c>
+      <c r="L70" s="2">
+        <v>272.01</v>
+      </c>
+      <c r="M70" s="2">
+        <v>348.9</v>
+      </c>
+      <c r="N70" s="3">
+        <v>-0.6</v>
+      </c>
+      <c r="O70" s="3">
+        <v>-0.49</v>
+      </c>
+      <c r="P70" s="2">
+        <v>713.11</v>
+      </c>
+      <c r="Q70" s="2">
+        <v>282.35</v>
+      </c>
+      <c r="R70" s="2">
+        <v>395.5</v>
+      </c>
+      <c r="S70" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T70" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB70" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC70" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD70" s="11" t="inlineStr">
+        <is>
+          <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="13">
+        <v>1</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
           <t>Pro Medicus</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C71" s="13" t="inlineStr">
         <is>
           <t>PME</t>
         </is>
       </c>
-      <c r="D70" s="10">
+      <c r="D71" s="10">
         <v>46307</v>
       </c>
-      <c r="E70" s="0" t="inlineStr">
+      <c r="E71" s="0" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="F70" s="0" t="inlineStr">
+      <c r="F71" s="0" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="G70" s="9" t="inlineStr">
+      <c r="G71" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H70" s="13" t="inlineStr">
+      <c r="H71" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I70" s="13" t="inlineStr">
+      <c r="I71" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J70" s="13" t="inlineStr">
+      <c r="J71" s="13" t="inlineStr">
         <is>
           <t>AUD</t>
         </is>
       </c>
-      <c r="K70" s="2">
+      <c r="K71" s="2">
         <v>168.37</v>
       </c>
-      <c r="L70" s="2">
+      <c r="L71" s="2">
         <v>50.61</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M71" s="2">
         <v>58.79</v>
       </c>
-      <c r="N70" s="3">
+      <c r="N71" s="3">
         <v>-0.695</v>
       </c>
-      <c r="O70" s="3">
+      <c r="O71" s="3">
         <v>-0.647</v>
       </c>
-      <c r="P70" s="2">
+      <c r="P71" s="2">
         <v>202.47</v>
       </c>
-      <c r="Q70" s="2">
+      <c r="Q71" s="2">
         <v>48.84</v>
       </c>
-      <c r="R70" s="2">
+      <c r="R71" s="2">
         <v>66.1</v>
       </c>
-      <c r="S70" s="13" t="inlineStr">
+      <c r="S71" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T70" s="13" t="inlineStr">
+      <c r="T71" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X70" s="5" t="inlineStr">
+      <c r="U71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA70" s="5" t="inlineStr">
+      <c r="Y71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB70" s="5" t="inlineStr">
+      <c r="AB71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AD70" s="11" t="inlineStr">
+      <c r="AC71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD71" s="11" t="inlineStr">
         <is>
           <t>informes/pro-medicus-2026-10-12/Pro Medicus - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD70"/>
+  <autoFilter ref="A1:AD71"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -9498,6 +9630,7 @@
     <hyperlink ref="AD68" r:id="rId67"/>
     <hyperlink ref="AD69" r:id="rId68"/>
     <hyperlink ref="AD70" r:id="rId69"/>
+    <hyperlink ref="AD71" r:id="rId70"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Adyen (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$74</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -5472,12 +5472,12 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>Verisk</t>
+          <t>Adyen</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>VRSK</t>
+          <t>ADYEN</t>
         </is>
       </c>
       <c r="D41" s="10">
@@ -5485,12 +5485,12 @@
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Países Bajos</t>
         </is>
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Financieros</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -5510,32 +5510,32 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K41" s="2">
-        <v>177.63</v>
+        <v>886.1</v>
       </c>
       <c r="L41" s="2">
-        <v>182.74</v>
+        <v>908.88</v>
       </c>
       <c r="M41" s="2">
-        <v>214.96</v>
+        <v>1110.27</v>
       </c>
       <c r="N41" s="3">
-        <v>0.039</v>
+        <v>0.026000000000000002</v>
       </c>
       <c r="O41" s="3">
-        <v>0.221</v>
+        <v>0.253</v>
       </c>
       <c r="P41" s="2">
-        <v>230.94</v>
+        <v>1378.31</v>
       </c>
       <c r="Q41" s="2">
-        <v>175.8</v>
+        <v>865.25</v>
       </c>
       <c r="R41" s="2">
-        <v>241.03</v>
+        <v>1215.17</v>
       </c>
       <c r="S41" s="13" t="inlineStr">
         <is>
@@ -5547,9 +5547,9 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V41" s="4" t="inlineStr">
@@ -5557,14 +5557,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="W41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y41" s="4" t="inlineStr">
@@ -5572,14 +5572,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z41" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA41" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z41" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA41" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB41" s="4" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="AD41" s="11" t="inlineStr">
         <is>
-          <t>informes/verisk-2026-10-12/Verisk - 2026-10-12.pdf</t>
+          <t>informes/adyen-2026-10-12/Adyen - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -5604,25 +5604,25 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Verisk</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>VRSK</t>
         </is>
       </c>
       <c r="D42" s="10">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industriales</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -5642,32 +5642,32 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K42" s="2">
-        <v>191.46</v>
+        <v>177.63</v>
       </c>
       <c r="L42" s="2">
-        <v>191.35</v>
+        <v>182.74</v>
       </c>
       <c r="M42" s="2">
-        <v>230.58</v>
+        <v>214.96</v>
       </c>
       <c r="N42" s="3">
-        <v>0.012</v>
+        <v>0.039</v>
       </c>
       <c r="O42" s="3">
-        <v>0.217</v>
+        <v>0.221</v>
       </c>
       <c r="P42" s="2">
-        <v>210.39</v>
+        <v>230.94</v>
       </c>
       <c r="Q42" s="2">
-        <v>184.46</v>
+        <v>175.8</v>
       </c>
       <c r="R42" s="2">
-        <v>259.09</v>
+        <v>241.03</v>
       </c>
       <c r="S42" s="13" t="inlineStr">
         <is>
@@ -5689,14 +5689,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="W42" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W42" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y42" s="4" t="inlineStr">
@@ -5704,9 +5704,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA42" s="6" t="inlineStr">
@@ -5719,14 +5719,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC42" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD42" s="11" t="inlineStr">
         <is>
-          <t>informes/sap-2026-10-11/SAP - 2026-10-11.pdf</t>
+          <t>informes/verisk-2026-10-12/Verisk - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -5736,25 +5736,25 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>ICON</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="D43" s="10">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
-          <t>Irlanda</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -5774,36 +5774,36 @@
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K43" s="2">
-        <v>164.5</v>
+        <v>191.46</v>
       </c>
       <c r="L43" s="2">
-        <v>163.26</v>
+        <v>191.35</v>
       </c>
       <c r="M43" s="2">
-        <v>194.24</v>
+        <v>230.58</v>
       </c>
       <c r="N43" s="3">
-        <v>-0.008</v>
+        <v>0.012</v>
       </c>
       <c r="O43" s="3">
-        <v>0.18100000000000002</v>
+        <v>0.217</v>
       </c>
       <c r="P43" s="2">
-        <v>184.41</v>
+        <v>210.39</v>
       </c>
       <c r="Q43" s="2">
-        <v>155.42</v>
+        <v>184.46</v>
       </c>
       <c r="R43" s="2">
-        <v>202.28</v>
+        <v>259.09</v>
       </c>
       <c r="S43" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T43" s="13" t="inlineStr">
@@ -5811,29 +5811,29 @@
           <t>Comprar</t>
         </is>
       </c>
-      <c r="U43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V43" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="W43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X43" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Y43" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X43" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z43" s="6" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="AD43" s="11" t="inlineStr">
         <is>
-          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
+          <t>informes/sap-2026-10-11/SAP - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -5868,25 +5868,25 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>Burkhalter</t>
+          <t>ICON</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>BRKN</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="D44" s="10">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Irlanda</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -5906,32 +5906,32 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K44" s="2">
-        <v>124.6</v>
+        <v>164.5</v>
       </c>
       <c r="L44" s="2">
-        <v>111.78</v>
+        <v>163.26</v>
       </c>
       <c r="M44" s="2">
-        <v>136.6</v>
+        <v>194.24</v>
       </c>
       <c r="N44" s="3">
-        <v>-0.061</v>
+        <v>-0.008</v>
       </c>
       <c r="O44" s="3">
-        <v>0.138</v>
+        <v>0.18100000000000002</v>
       </c>
       <c r="P44" s="2">
-        <v>148.18</v>
+        <v>184.41</v>
       </c>
       <c r="Q44" s="2">
-        <v>111.33</v>
+        <v>155.42</v>
       </c>
       <c r="R44" s="2">
-        <v>151.46</v>
+        <v>202.28</v>
       </c>
       <c r="S44" s="13" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="T44" s="13" t="inlineStr">
         <is>
-          <t>Mantener</t>
+          <t>Comprar</t>
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr">
@@ -5948,14 +5948,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="V44" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="X44" s="4" t="inlineStr">
@@ -5963,19 +5963,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Y44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AA44" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="Y44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB44" s="4" t="inlineStr">
@@ -5983,14 +5983,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AC44" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC44" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD44" s="11" t="inlineStr">
         <is>
-          <t>informes/burkhalter-2026-10-11/Burkhalter - 2026-10-11.pdf</t>
+          <t>informes/icon-2026-10-09/ICON - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -6000,20 +6000,20 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>A. O. Smith</t>
+          <t>Burkhalter</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>AOS</t>
+          <t>BRKN</t>
         </is>
       </c>
       <c r="D45" s="10">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F45" s="0" t="inlineStr">
@@ -6028,56 +6028,56 @@
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CHF</t>
         </is>
       </c>
       <c r="K45" s="2">
-        <v>56.56</v>
+        <v>124.6</v>
       </c>
       <c r="L45" s="2">
-        <v>55.24</v>
+        <v>111.78</v>
       </c>
       <c r="M45" s="2">
-        <v>62.35</v>
+        <v>136.6</v>
       </c>
       <c r="N45" s="3">
-        <v>0.002</v>
+        <v>-0.061</v>
       </c>
       <c r="O45" s="3">
-        <v>0.127</v>
+        <v>0.138</v>
       </c>
       <c r="P45" s="2">
-        <v>69.91</v>
+        <v>148.18</v>
       </c>
       <c r="Q45" s="2">
-        <v>55.41</v>
+        <v>111.33</v>
       </c>
       <c r="R45" s="2">
-        <v>65.9</v>
+        <v>151.46</v>
       </c>
       <c r="S45" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T45" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T45" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V45" s="4" t="inlineStr">
@@ -6100,9 +6100,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z45" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Z45" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA45" s="5" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="AD45" s="11" t="inlineStr">
         <is>
-          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
+          <t>informes/burkhalter-2026-10-11/Burkhalter - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6132,16 +6132,16 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>A. O. Smith</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>AOS</t>
         </is>
       </c>
       <c r="D46" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
@@ -6174,28 +6174,28 @@
         </is>
       </c>
       <c r="K46" s="2">
-        <v>70.24</v>
+        <v>56.56</v>
       </c>
       <c r="L46" s="2">
-        <v>73.56</v>
+        <v>55.24</v>
       </c>
       <c r="M46" s="2">
-        <v>80.39</v>
+        <v>62.35</v>
       </c>
       <c r="N46" s="3">
-        <v>0.047</v>
+        <v>0.002</v>
       </c>
       <c r="O46" s="3">
-        <v>0.145</v>
+        <v>0.127</v>
       </c>
       <c r="P46" s="2">
-        <v>100.86</v>
+        <v>69.91</v>
       </c>
       <c r="Q46" s="2">
-        <v>69.88</v>
+        <v>55.41</v>
       </c>
       <c r="R46" s="2">
-        <v>89.38</v>
+        <v>65.9</v>
       </c>
       <c r="S46" s="13" t="inlineStr">
         <is>
@@ -6207,9 +6207,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V46" s="4" t="inlineStr">
@@ -6232,14 +6232,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA46" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z46" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA46" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AB46" s="4" t="inlineStr">
@@ -6254,13 +6254,13 @@
       </c>
       <c r="AD46" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
+          <t>informes/ao-smith-2026-10-09/A. O. Smith - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
         </is>
       </c>
       <c r="D47" s="10">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
@@ -6306,28 +6306,28 @@
         </is>
       </c>
       <c r="K47" s="2">
-        <v>71.51</v>
+        <v>70.24</v>
       </c>
       <c r="L47" s="2">
-        <v>73.59</v>
+        <v>73.56</v>
       </c>
       <c r="M47" s="2">
-        <v>80.42</v>
+        <v>80.39</v>
       </c>
       <c r="N47" s="3">
-        <v>0.028999999999999998</v>
+        <v>0.047</v>
       </c>
       <c r="O47" s="3">
-        <v>0.125</v>
+        <v>0.145</v>
       </c>
       <c r="P47" s="2">
         <v>100.86</v>
       </c>
       <c r="Q47" s="2">
-        <v>69.91</v>
+        <v>69.88</v>
       </c>
       <c r="R47" s="2">
-        <v>89.41</v>
+        <v>89.38</v>
       </c>
       <c r="S47" s="13" t="inlineStr">
         <is>
@@ -6369,9 +6369,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="AA47" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA47" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AB47" s="4" t="inlineStr">
@@ -6386,35 +6386,35 @@
       </c>
       <c r="AD47" s="11" t="inlineStr">
         <is>
-          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
+          <t>informes/uber-2026-10-08/Uber Technologies - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>Almirall</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D48" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -6424,7 +6424,7 @@
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
@@ -6434,32 +6434,32 @@
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K48" s="2">
-        <v>10.18</v>
+        <v>71.51</v>
       </c>
       <c r="L48" s="2">
-        <v>10.41</v>
+        <v>73.59</v>
       </c>
       <c r="M48" s="2">
-        <v>11.23</v>
+        <v>80.42</v>
       </c>
       <c r="N48" s="3">
-        <v>0.040999999999999995</v>
+        <v>0.028999999999999998</v>
       </c>
       <c r="O48" s="3">
-        <v>0.122</v>
+        <v>0.125</v>
       </c>
       <c r="P48" s="2">
-        <v>14.33</v>
+        <v>100.86</v>
       </c>
       <c r="Q48" s="2">
-        <v>9.92</v>
+        <v>69.91</v>
       </c>
       <c r="R48" s="2">
-        <v>12.34</v>
+        <v>89.41</v>
       </c>
       <c r="S48" s="13" t="inlineStr">
         <is>
@@ -6471,14 +6471,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V48" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="U48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W48" s="4" t="inlineStr">
@@ -6486,24 +6486,24 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z48" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA48" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="X48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z48" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA48" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AB48" s="4" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="AD48" s="11" t="inlineStr">
         <is>
-          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
+          <t>informes/uber-2026-10-10/Uber Technologies - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -6528,25 +6528,25 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>ATOSS</t>
+          <t>Almirall</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>AOF</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D49" s="10">
-        <v>46306</v>
+        <v>46302</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
@@ -6570,32 +6570,32 @@
         </is>
       </c>
       <c r="K49" s="2">
-        <v>87.3</v>
+        <v>10.18</v>
       </c>
       <c r="L49" s="2">
-        <v>80.89</v>
+        <v>10.41</v>
       </c>
       <c r="M49" s="2">
-        <v>94.95</v>
+        <v>11.23</v>
       </c>
       <c r="N49" s="3">
-        <v>-0.047</v>
+        <v>0.040999999999999995</v>
       </c>
       <c r="O49" s="3">
-        <v>0.114</v>
+        <v>0.122</v>
       </c>
       <c r="P49" s="2">
-        <v>120.78</v>
+        <v>14.33</v>
       </c>
       <c r="Q49" s="2">
-        <v>79.19</v>
+        <v>9.92</v>
       </c>
       <c r="R49" s="2">
-        <v>101.11</v>
+        <v>12.34</v>
       </c>
       <c r="S49" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T49" s="13" t="inlineStr">
@@ -6603,14 +6603,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V49" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W49" s="4" t="inlineStr">
@@ -6623,9 +6623,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y49" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y49" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z49" s="6" t="inlineStr">
@@ -6638,9 +6638,9 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB49" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB49" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC49" s="4" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="AD49" s="11" t="inlineStr">
         <is>
-          <t>informes/atoss-2026-10-11/ATOSS Software - 2026-10-11.pdf</t>
+          <t>informes/almirall-2026-10-07/Almirall - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>ATOSS</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>AOF</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -6688,12 +6688,12 @@
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
@@ -6702,39 +6702,39 @@
         </is>
       </c>
       <c r="K50" s="2">
-        <v>59.72</v>
+        <v>87.3</v>
       </c>
       <c r="L50" s="2">
-        <v>58.59</v>
+        <v>80.89</v>
       </c>
       <c r="M50" s="2">
-        <v>66.22</v>
+        <v>94.95</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.013999999999999999</v>
+        <v>-0.047</v>
       </c>
       <c r="O50" s="3">
         <v>0.114</v>
       </c>
       <c r="P50" s="2">
-        <v>67.12</v>
+        <v>120.78</v>
       </c>
       <c r="Q50" s="2">
-        <v>57.83</v>
+        <v>79.19</v>
       </c>
       <c r="R50" s="2">
-        <v>73.94</v>
+        <v>101.11</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T50" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6755,9 +6755,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z50" s="6" t="inlineStr">
@@ -6770,19 +6770,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AC50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/atoss-2026-10-11/ATOSS Software - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -6830,32 +6830,32 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K51" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L51" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M51" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N51" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O51" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P51" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q51" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R51" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
@@ -6882,39 +6882,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X51" s="5" t="inlineStr">
+      <c r="X51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA51" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y51" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB51" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -6952,46 +6952,46 @@
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>70.3</v>
+        <v>2702.5</v>
       </c>
       <c r="L52" s="2">
-        <v>61.1</v>
+        <v>2888.64</v>
       </c>
       <c r="M52" s="2">
-        <v>73.49</v>
+        <v>2897.35</v>
       </c>
       <c r="N52" s="3">
-        <v>-0.131</v>
+        <v>0.098</v>
       </c>
       <c r="O52" s="3">
-        <v>0.045</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P52" s="2">
-        <v>92.55</v>
+        <v>4077.5</v>
       </c>
       <c r="Q52" s="2">
-        <v>58.17</v>
+        <v>2585.33</v>
       </c>
       <c r="R52" s="2">
-        <v>81.69</v>
+        <v>3307.49</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T52" s="13" t="inlineStr">
@@ -7014,29 +7014,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA52" s="5" t="inlineStr">
+      <c r="X52" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB52" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC52" s="4" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,16 +7056,16 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J53" s="13" t="inlineStr">
@@ -7098,39 +7098,39 @@
         </is>
       </c>
       <c r="K53" s="2">
-        <v>26.82</v>
+        <v>70.3</v>
       </c>
       <c r="L53" s="2">
-        <v>25.71</v>
+        <v>61.1</v>
       </c>
       <c r="M53" s="2">
-        <v>27.88</v>
+        <v>73.49</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.131</v>
       </c>
       <c r="O53" s="3">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="P53" s="2">
-        <v>39</v>
+        <v>92.55</v>
       </c>
       <c r="Q53" s="2">
-        <v>24.22</v>
+        <v>58.17</v>
       </c>
       <c r="R53" s="2">
-        <v>30.98</v>
+        <v>81.69</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T53" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T53" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U53" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7146,9 +7146,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y53" s="4" t="inlineStr">
@@ -7156,19 +7156,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z53" s="5" t="inlineStr">
+      <c r="Z53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA53" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC53" s="4" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,12 +7188,12 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D54" s="10">
@@ -7201,7 +7201,7 @@
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
@@ -7221,41 +7221,41 @@
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K54" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L54" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M54" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O54" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P54" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q54" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R54" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T54" s="13" t="inlineStr">
@@ -7263,9 +7263,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V54" s="4" t="inlineStr">
@@ -7278,29 +7278,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA54" s="5" t="inlineStr">
+      <c r="X54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC54" s="4" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,25 +7320,25 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>SPGI</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D55" s="10">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -7348,42 +7348,42 @@
       </c>
       <c r="H55" s="13" t="inlineStr">
         <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I55" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K55" s="2">
-        <v>407.82</v>
+        <v>577.5</v>
       </c>
       <c r="L55" s="2">
-        <v>351.69</v>
+        <v>466.62</v>
       </c>
       <c r="M55" s="2">
-        <v>398.1</v>
+        <v>564.55</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.128</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O55" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="P55" s="2">
-        <v>516.86</v>
+        <v>795.86</v>
       </c>
       <c r="Q55" s="2">
-        <v>338.33</v>
+        <v>504.42</v>
       </c>
       <c r="R55" s="2">
-        <v>446.65</v>
+        <v>645.34</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
@@ -7395,44 +7395,44 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V55" s="5" t="inlineStr">
+      <c r="U55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y55" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB55" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC55" s="4" t="inlineStr">
@@ -7442,7 +7442,7 @@
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/sp-global-2026-10-12/S&amp;P Global - 2026-10-12.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,25 +7452,25 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>SPGI</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
@@ -7480,61 +7480,61 @@
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K56" s="2">
-        <v>2000</v>
+        <v>407.82</v>
       </c>
       <c r="L56" s="2">
-        <v>1932.11</v>
+        <v>351.69</v>
       </c>
       <c r="M56" s="2">
-        <v>1939.91</v>
+        <v>398.1</v>
       </c>
       <c r="N56" s="3">
-        <v>-0.019</v>
+        <v>-0.128</v>
       </c>
       <c r="O56" s="3">
-        <v>-0.015</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="P56" s="2">
-        <v>2184.62</v>
+        <v>516.86</v>
       </c>
       <c r="Q56" s="2">
-        <v>1711.85</v>
+        <v>338.33</v>
       </c>
       <c r="R56" s="2">
-        <v>2020.99</v>
+        <v>446.65</v>
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T56" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T56" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V56" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W56" s="4" t="inlineStr">
@@ -7542,39 +7542,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X56" s="5" t="inlineStr">
+      <c r="X56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
       <c r="AB56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/sp-global-2026-10-12/S&amp;P Global - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,25 +7584,25 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -7612,46 +7612,46 @@
       </c>
       <c r="H57" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K57" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L57" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M57" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P57" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q57" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R57" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T57" s="13" t="inlineStr">
@@ -7659,14 +7659,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W57" s="4" t="inlineStr">
@@ -7684,21 +7684,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA57" s="5" t="inlineStr">
+      <c r="Z57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB57" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC57" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7716,25 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -7754,32 +7754,32 @@
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K58" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L58" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M58" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P58" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q58" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R58" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
@@ -7791,46 +7791,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U58" s="5" t="inlineStr">
+      <c r="U58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V58" s="5" t="inlineStr">
+      <c r="Y58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z58" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W58" s="5" t="inlineStr">
+      <c r="AB58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC58" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
@@ -7886,32 +7886,32 @@
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>262.43</v>
+        <v>16.22</v>
       </c>
       <c r="L59" s="2">
-        <v>213.96</v>
+        <v>13.97</v>
       </c>
       <c r="M59" s="2">
-        <v>251.97</v>
+        <v>14.66</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.185</v>
+        <v>-0.077</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.04</v>
+        <v>-0.035</v>
       </c>
       <c r="P59" s="2">
-        <v>331.36</v>
+        <v>17.05</v>
       </c>
       <c r="Q59" s="2">
-        <v>203.69</v>
+        <v>13.61</v>
       </c>
       <c r="R59" s="2">
-        <v>271.09</v>
+        <v>16.41</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7923,19 +7923,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U59" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V59" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W59" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X59" s="5" t="inlineStr">
@@ -7943,14 +7943,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Y59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z59" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y59" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA59" s="5" t="inlineStr">
@@ -7963,14 +7963,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC59" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/amazon-2026-10-12/Amazon - 2026-10-12.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,25 +7980,25 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
@@ -8022,28 +8022,28 @@
         </is>
       </c>
       <c r="K60" s="2">
-        <v>128.3</v>
+        <v>262.43</v>
       </c>
       <c r="L60" s="2">
-        <v>99</v>
+        <v>213.96</v>
       </c>
       <c r="M60" s="2">
-        <v>117</v>
+        <v>251.97</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.185</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.065</v>
+        <v>-0.04</v>
       </c>
       <c r="P60" s="2">
-        <v>128.84</v>
+        <v>331.36</v>
       </c>
       <c r="Q60" s="2">
-        <v>97.02</v>
+        <v>203.69</v>
       </c>
       <c r="R60" s="2">
-        <v>132.07</v>
+        <v>271.09</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8060,29 +8060,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V60" s="5" t="inlineStr">
+      <c r="V60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X60" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="X60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA60" s="5" t="inlineStr">
@@ -8095,14 +8095,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
+          <t>informes/amazon-2026-10-12/Amazon - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,25 +8112,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>6861</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="D61" s="10">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -8150,32 +8150,32 @@
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K61" s="2">
-        <v>81490</v>
+        <v>128.3</v>
       </c>
       <c r="L61" s="2">
-        <v>66566.47</v>
+        <v>99</v>
       </c>
       <c r="M61" s="2">
-        <v>75201.52</v>
+        <v>117</v>
       </c>
       <c r="N61" s="3">
-        <v>-0.17600000000000002</v>
+        <v>-0.20600000000000002</v>
       </c>
       <c r="O61" s="3">
-        <v>-0.07</v>
+        <v>-0.065</v>
       </c>
       <c r="P61" s="2">
-        <v>97866.67</v>
+        <v>128.84</v>
       </c>
       <c r="Q61" s="2">
-        <v>65834.24</v>
+        <v>97.02</v>
       </c>
       <c r="R61" s="2">
-        <v>84206.58</v>
+        <v>132.07</v>
       </c>
       <c r="S61" s="13" t="inlineStr">
         <is>
@@ -8192,29 +8192,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="V61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X61" s="5" t="inlineStr">
+      <c r="V61" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="W61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="X61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z61" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA61" s="5" t="inlineStr">
@@ -8222,19 +8222,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB61" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AC61" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB61" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC61" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD61" s="11" t="inlineStr">
         <is>
-          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
+          <t>informes/csl-2026-10-09/CSL - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -8244,79 +8244,79 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>Cochlear</t>
+          <t>Keyence</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>COH</t>
+          <t>6861</t>
         </is>
       </c>
       <c r="D62" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
-        </is>
-      </c>
-      <c r="G62" s="9" t="inlineStr">
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G62" s="8" t="inlineStr">
+        <is>
+          <t>Mantener</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J62" s="13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="K62" s="2">
+        <v>81490</v>
+      </c>
+      <c r="L62" s="2">
+        <v>66566.47</v>
+      </c>
+      <c r="M62" s="2">
+        <v>75201.52</v>
+      </c>
+      <c r="N62" s="3">
+        <v>-0.17600000000000002</v>
+      </c>
+      <c r="O62" s="3">
+        <v>-0.07</v>
+      </c>
+      <c r="P62" s="2">
+        <v>97866.67</v>
+      </c>
+      <c r="Q62" s="2">
+        <v>65834.24</v>
+      </c>
+      <c r="R62" s="2">
+        <v>84206.58</v>
+      </c>
+      <c r="S62" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H62" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I62" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="J62" s="13" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="K62" s="2">
-        <v>129</v>
-      </c>
-      <c r="L62" s="2">
-        <v>100.16</v>
-      </c>
-      <c r="M62" s="2">
-        <v>115.11</v>
-      </c>
-      <c r="N62" s="3">
-        <v>-0.19699999999999998</v>
-      </c>
-      <c r="O62" s="3">
-        <v>-0.081</v>
-      </c>
-      <c r="P62" s="2">
-        <v>137.09</v>
-      </c>
-      <c r="Q62" s="2">
-        <v>103.06</v>
-      </c>
-      <c r="R62" s="2">
-        <v>128.2</v>
-      </c>
-      <c r="S62" s="13" t="inlineStr">
-        <is>
-          <t>Vender</t>
-        </is>
-      </c>
       <c r="T62" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="U62" s="4" t="inlineStr">
@@ -8334,9 +8334,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X62" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X62" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y62" s="4" t="inlineStr">
@@ -8344,9 +8344,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z62" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA62" s="5" t="inlineStr">
@@ -8354,19 +8354,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB62" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC62" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB62" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC62" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD62" s="11" t="inlineStr">
         <is>
-          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
+          <t>informes/keyence-2026-10-07/Keyence - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8376,25 +8376,25 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>Hermès</t>
+          <t>Cochlear</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>COH</t>
         </is>
       </c>
       <c r="D63" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
@@ -8414,32 +8414,32 @@
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AUD</t>
         </is>
       </c>
       <c r="K63" s="2">
-        <v>1283</v>
+        <v>129</v>
       </c>
       <c r="L63" s="2">
-        <v>937.64</v>
+        <v>100.16</v>
       </c>
       <c r="M63" s="2">
-        <v>1158.7</v>
+        <v>115.11</v>
       </c>
       <c r="N63" s="3">
-        <v>-0.255</v>
+        <v>-0.19699999999999998</v>
       </c>
       <c r="O63" s="3">
-        <v>-0.083</v>
+        <v>-0.081</v>
       </c>
       <c r="P63" s="2">
-        <v>1657.61</v>
+        <v>137.09</v>
       </c>
       <c r="Q63" s="2">
-        <v>909.51</v>
+        <v>103.06</v>
       </c>
       <c r="R63" s="2">
-        <v>1263.94</v>
+        <v>128.2</v>
       </c>
       <c r="S63" s="13" t="inlineStr">
         <is>
@@ -8476,29 +8476,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z63" s="5" t="inlineStr">
+      <c r="Z63" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA63" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA63" s="5" t="inlineStr">
+      <c r="AB63" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB63" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC63" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC63" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD63" s="11" t="inlineStr">
         <is>
-          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
+          <t>informes/cochlear-2026-10-08/Cochlear - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -8508,20 +8508,20 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>Inditex</t>
+          <t>Hermès</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>ITX</t>
+          <t>RMS</t>
         </is>
       </c>
       <c r="D64" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J64" s="13" t="inlineStr">
@@ -8550,28 +8550,28 @@
         </is>
       </c>
       <c r="K64" s="2">
-        <v>53.82</v>
+        <v>1283</v>
       </c>
       <c r="L64" s="2">
-        <v>44.48</v>
+        <v>937.64</v>
       </c>
       <c r="M64" s="2">
-        <v>44.65</v>
+        <v>1158.7</v>
       </c>
       <c r="N64" s="3">
-        <v>-0.151</v>
+        <v>-0.255</v>
       </c>
       <c r="O64" s="3">
-        <v>-0.14800000000000002</v>
+        <v>-0.083</v>
       </c>
       <c r="P64" s="2">
-        <v>60.39</v>
+        <v>1657.61</v>
       </c>
       <c r="Q64" s="2">
-        <v>39.85</v>
+        <v>909.51</v>
       </c>
       <c r="R64" s="2">
-        <v>48.84</v>
+        <v>1263.94</v>
       </c>
       <c r="S64" s="13" t="inlineStr">
         <is>
@@ -8583,9 +8583,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U64" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V64" s="4" t="inlineStr">
@@ -8608,9 +8608,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z64" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z64" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="AA64" s="5" t="inlineStr">
@@ -8623,14 +8623,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC64" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC64" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD64" s="11" t="inlineStr">
         <is>
-          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
+          <t>informes/hermes-2026-10-11/Hermès - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -8640,25 +8640,25 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>Kongsberg</t>
+          <t>Inditex</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>KOG</t>
+          <t>ITX</t>
         </is>
       </c>
       <c r="D65" s="10">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
@@ -8673,37 +8673,37 @@
       </c>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K65" s="2">
-        <v>299</v>
+        <v>53.82</v>
       </c>
       <c r="L65" s="2">
-        <v>204.75</v>
+        <v>44.48</v>
       </c>
       <c r="M65" s="2">
-        <v>239.87</v>
+        <v>44.65</v>
       </c>
       <c r="N65" s="3">
-        <v>-0.308</v>
+        <v>-0.151</v>
       </c>
       <c r="O65" s="3">
-        <v>-0.19</v>
+        <v>-0.14800000000000002</v>
       </c>
       <c r="P65" s="2">
-        <v>397.27</v>
+        <v>60.39</v>
       </c>
       <c r="Q65" s="2">
-        <v>210.48</v>
+        <v>39.85</v>
       </c>
       <c r="R65" s="2">
-        <v>269.04</v>
+        <v>48.84</v>
       </c>
       <c r="S65" s="13" t="inlineStr">
         <is>
@@ -8715,9 +8715,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U65" s="13" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="U65" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="V65" s="4" t="inlineStr">
@@ -8730,39 +8730,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X65" s="5" t="inlineStr">
+      <c r="X65" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z65" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA65" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z65" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA65" s="5" t="inlineStr">
+      <c r="AB65" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB65" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AC65" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC65" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD65" s="11" t="inlineStr">
         <is>
-          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
+          <t>informes/inditex-2026-10-06/Inditex - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8772,25 +8772,25 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Kongsberg</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>KOG</t>
         </is>
       </c>
       <c r="D66" s="10">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G66" s="9" t="inlineStr">
@@ -8805,37 +8805,37 @@
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="K66" s="2">
-        <v>350.5</v>
+        <v>299</v>
       </c>
       <c r="L66" s="2">
-        <v>252.74</v>
+        <v>204.75</v>
       </c>
       <c r="M66" s="2">
-        <v>281.33</v>
+        <v>239.87</v>
       </c>
       <c r="N66" s="3">
-        <v>-0.276</v>
+        <v>-0.308</v>
       </c>
       <c r="O66" s="3">
-        <v>-0.195</v>
+        <v>-0.19</v>
       </c>
       <c r="P66" s="2">
-        <v>429.47</v>
+        <v>397.27</v>
       </c>
       <c r="Q66" s="2">
-        <v>245.16</v>
+        <v>210.48</v>
       </c>
       <c r="R66" s="2">
-        <v>313.65</v>
+        <v>269.04</v>
       </c>
       <c r="S66" s="13" t="inlineStr">
         <is>
@@ -8847,9 +8847,9 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U66" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U66" s="13" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="V66" s="4" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="AD66" s="11" t="inlineStr">
         <is>
-          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
+          <t>informes/kongsberg-2026-10-07/Kongsberg - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -8904,25 +8904,25 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>Fanuc</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>6954</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D67" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -8937,37 +8937,37 @@
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J67" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K67" s="2">
-        <v>6220</v>
+        <v>350.5</v>
       </c>
       <c r="L67" s="2">
-        <v>4460.49</v>
+        <v>252.74</v>
       </c>
       <c r="M67" s="2">
-        <v>4713.09</v>
+        <v>281.33</v>
       </c>
       <c r="N67" s="3">
-        <v>-0.266</v>
+        <v>-0.276</v>
       </c>
       <c r="O67" s="3">
-        <v>-0.225</v>
+        <v>-0.195</v>
       </c>
       <c r="P67" s="2">
-        <v>7278.89</v>
+        <v>429.47</v>
       </c>
       <c r="Q67" s="2">
-        <v>4188.4</v>
+        <v>245.16</v>
       </c>
       <c r="R67" s="2">
-        <v>4821.79</v>
+        <v>313.65</v>
       </c>
       <c r="S67" s="13" t="inlineStr">
         <is>
@@ -8979,14 +8979,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U67" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V67" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U67" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V67" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="W67" s="4" t="inlineStr">
@@ -8994,9 +8994,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X67" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X67" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Y67" s="4" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="AD67" s="11" t="inlineStr">
         <is>
-          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
+          <t>informes/alphabet-2026-10-08/Alphabet - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -9036,25 +9036,25 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>Games Workshop</t>
+          <t>Fanuc</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>GAW</t>
+          <t>6954</t>
         </is>
       </c>
       <c r="D68" s="10">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I68" s="13" t="inlineStr">
@@ -9074,32 +9074,32 @@
       </c>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K68" s="2">
-        <v>163.9</v>
+        <v>6220</v>
       </c>
       <c r="L68" s="2">
-        <v>102</v>
+        <v>4460.49</v>
       </c>
       <c r="M68" s="2">
-        <v>116.59</v>
+        <v>4713.09</v>
       </c>
       <c r="N68" s="3">
-        <v>-0.348</v>
+        <v>-0.266</v>
       </c>
       <c r="O68" s="3">
-        <v>-0.259</v>
+        <v>-0.225</v>
       </c>
       <c r="P68" s="2">
-        <v>220.75</v>
+        <v>7278.89</v>
       </c>
       <c r="Q68" s="2">
-        <v>101.69</v>
+        <v>4188.4</v>
       </c>
       <c r="R68" s="2">
-        <v>131.58</v>
+        <v>4821.79</v>
       </c>
       <c r="S68" s="13" t="inlineStr">
         <is>
@@ -9111,14 +9111,14 @@
           <t>Vender</t>
         </is>
       </c>
-      <c r="U68" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V68" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U68" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V68" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W68" s="4" t="inlineStr">
@@ -9136,9 +9136,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z68" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z68" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA68" s="5" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="AD68" s="11" t="inlineStr">
         <is>
-          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
+          <t>informes/fanuc-2026-10-07/Fanuc - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -9168,25 +9168,25 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Games Workshop</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>GAW</t>
         </is>
       </c>
       <c r="D69" s="10">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Reino Unido</t>
         </is>
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="H69" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I69" s="13" t="inlineStr">
@@ -9206,32 +9206,32 @@
       </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="K69" s="2">
-        <v>253.14</v>
+        <v>163.9</v>
       </c>
       <c r="L69" s="2">
-        <v>168.18</v>
+        <v>102</v>
       </c>
       <c r="M69" s="2">
-        <v>168.18</v>
+        <v>116.59</v>
       </c>
       <c r="N69" s="3">
-        <v>-0.335</v>
+        <v>-0.348</v>
       </c>
       <c r="O69" s="3">
-        <v>-0.335</v>
+        <v>-0.259</v>
       </c>
       <c r="P69" s="2">
-        <v>337.43</v>
+        <v>220.75</v>
       </c>
       <c r="Q69" s="2">
-        <v>146.32</v>
+        <v>101.69</v>
       </c>
       <c r="R69" s="2">
-        <v>187.18</v>
+        <v>131.58</v>
       </c>
       <c r="S69" s="13" t="inlineStr">
         <is>
@@ -9263,14 +9263,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y69" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z69" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y69" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z69" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA69" s="5" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="AD69" s="11" t="inlineStr">
         <is>
-          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
+          <t>informes/games-workshop-2026-10-10/Games Workshop - 2026-10-10.pdf</t>
         </is>
       </c>
     </row>
@@ -9300,16 +9300,16 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>Medpace</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D70" s="10">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
@@ -9318,7 +9318,7 @@
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
@@ -9328,7 +9328,7 @@
       </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I70" s="13" t="inlineStr">
@@ -9342,28 +9342,28 @@
         </is>
       </c>
       <c r="K70" s="2">
-        <v>612.05</v>
+        <v>253.14</v>
       </c>
       <c r="L70" s="2">
-        <v>326.15</v>
+        <v>168.18</v>
       </c>
       <c r="M70" s="2">
-        <v>382.27</v>
+        <v>168.18</v>
       </c>
       <c r="N70" s="3">
-        <v>-0.467</v>
+        <v>-0.335</v>
       </c>
       <c r="O70" s="3">
-        <v>-0.375</v>
+        <v>-0.335</v>
       </c>
       <c r="P70" s="2">
-        <v>595.92</v>
+        <v>337.43</v>
       </c>
       <c r="Q70" s="2">
-        <v>310.49</v>
+        <v>146.32</v>
       </c>
       <c r="R70" s="2">
-        <v>424.97</v>
+        <v>187.18</v>
       </c>
       <c r="S70" s="13" t="inlineStr">
         <is>
@@ -9395,9 +9395,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y70" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Y70" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Z70" s="6" t="inlineStr">
@@ -9415,14 +9415,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC70" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AC70" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD70" s="11" t="inlineStr">
         <is>
-          <t>informes/medpace-2026-10-12/Medpace - 2026-10-12.pdf</t>
+          <t>informes/vertiv-2026-10-07/Vertiv - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -9432,16 +9432,16 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>Intuitive</t>
+          <t>Medpace</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="D71" s="10">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="H71" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I71" s="13" t="inlineStr">
@@ -9474,28 +9474,28 @@
         </is>
       </c>
       <c r="K71" s="2">
-        <v>404.76</v>
+        <v>612.05</v>
       </c>
       <c r="L71" s="2">
-        <v>222.49</v>
+        <v>326.15</v>
       </c>
       <c r="M71" s="2">
-        <v>222.49</v>
+        <v>382.27</v>
       </c>
       <c r="N71" s="3">
-        <v>-0.45</v>
+        <v>-0.467</v>
       </c>
       <c r="O71" s="3">
-        <v>-0.45</v>
+        <v>-0.375</v>
       </c>
       <c r="P71" s="2">
-        <v>477.21</v>
+        <v>595.92</v>
       </c>
       <c r="Q71" s="2">
-        <v>193.34</v>
+        <v>310.49</v>
       </c>
       <c r="R71" s="2">
-        <v>247.41</v>
+        <v>424.97</v>
       </c>
       <c r="S71" s="13" t="inlineStr">
         <is>
@@ -9522,39 +9522,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X71" s="5" t="inlineStr">
+      <c r="X71" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y71" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z71" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y71" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z71" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA71" s="5" t="inlineStr">
+      <c r="AB71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB71" s="5" t="inlineStr">
+      <c r="AC71" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC71" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AD71" s="11" t="inlineStr">
         <is>
-          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
+          <t>informes/medpace-2026-10-12/Medpace - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -9564,12 +9564,12 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Intuitive</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>VACN</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="D72" s="10">
@@ -9577,12 +9577,12 @@
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
@@ -9602,32 +9602,32 @@
       </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K72" s="2">
-        <v>698.2</v>
+        <v>404.76</v>
       </c>
       <c r="L72" s="2">
-        <v>272.01</v>
+        <v>222.49</v>
       </c>
       <c r="M72" s="2">
-        <v>348.9</v>
+        <v>222.49</v>
       </c>
       <c r="N72" s="3">
-        <v>-0.6</v>
+        <v>-0.45</v>
       </c>
       <c r="O72" s="3">
-        <v>-0.49</v>
+        <v>-0.45</v>
       </c>
       <c r="P72" s="2">
-        <v>713.11</v>
+        <v>477.21</v>
       </c>
       <c r="Q72" s="2">
-        <v>282.35</v>
+        <v>193.34</v>
       </c>
       <c r="R72" s="2">
-        <v>395.5</v>
+        <v>247.41</v>
       </c>
       <c r="S72" s="13" t="inlineStr">
         <is>
@@ -9664,9 +9664,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z72" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="Z72" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AA72" s="5" t="inlineStr">
@@ -9679,14 +9679,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC72" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC72" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD72" s="11" t="inlineStr">
         <is>
-          <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
+          <t>informes/intuitive-2026-10-06/Intuitive Surgical - 2026-10-06 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -9696,134 +9696,266 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>VACN</t>
+        </is>
+      </c>
+      <c r="D73" s="10">
+        <v>46301</v>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>Suiza</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>Tecnologías de la información</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="H73" s="13" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="K73" s="2">
+        <v>698.2</v>
+      </c>
+      <c r="L73" s="2">
+        <v>272.01</v>
+      </c>
+      <c r="M73" s="2">
+        <v>348.9</v>
+      </c>
+      <c r="N73" s="3">
+        <v>-0.6</v>
+      </c>
+      <c r="O73" s="3">
+        <v>-0.49</v>
+      </c>
+      <c r="P73" s="2">
+        <v>713.11</v>
+      </c>
+      <c r="Q73" s="2">
+        <v>282.35</v>
+      </c>
+      <c r="R73" s="2">
+        <v>395.5</v>
+      </c>
+      <c r="S73" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T73" s="13" t="inlineStr">
+        <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="U73" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V73" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W73" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X73" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Y73" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z73" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA73" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AB73" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="AC73" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AD73" s="11" t="inlineStr">
+        <is>
+          <t>informes/vat-2026-10-06/VAT Group - 2026-10-06 v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13">
+        <v>1</v>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
           <t>Pro Medicus</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C74" s="13" t="inlineStr">
         <is>
           <t>PME</t>
         </is>
       </c>
-      <c r="D73" s="10">
+      <c r="D74" s="10">
         <v>46307</v>
       </c>
-      <c r="E73" s="0" t="inlineStr">
+      <c r="E74" s="0" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="F73" s="0" t="inlineStr">
+      <c r="F74" s="0" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="G73" s="9" t="inlineStr">
+      <c r="G74" s="9" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="H73" s="13" t="inlineStr">
+      <c r="H74" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="I73" s="13" t="inlineStr">
+      <c r="I74" s="13" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="J73" s="13" t="inlineStr">
+      <c r="J74" s="13" t="inlineStr">
         <is>
           <t>AUD</t>
         </is>
       </c>
-      <c r="K73" s="2">
+      <c r="K74" s="2">
         <v>168.37</v>
       </c>
-      <c r="L73" s="2">
+      <c r="L74" s="2">
         <v>50.61</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M74" s="2">
         <v>58.79</v>
       </c>
-      <c r="N73" s="3">
+      <c r="N74" s="3">
         <v>-0.695</v>
       </c>
-      <c r="O73" s="3">
+      <c r="O74" s="3">
         <v>-0.647</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P74" s="2">
         <v>202.47</v>
       </c>
-      <c r="Q73" s="2">
+      <c r="Q74" s="2">
         <v>48.84</v>
       </c>
-      <c r="R73" s="2">
+      <c r="R74" s="2">
         <v>66.1</v>
       </c>
-      <c r="S73" s="13" t="inlineStr">
+      <c r="S74" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="T73" s="13" t="inlineStr">
+      <c r="T74" s="13" t="inlineStr">
         <is>
           <t>Vender</t>
         </is>
       </c>
-      <c r="U73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X73" s="5" t="inlineStr">
+      <c r="U74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X74" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA73" s="5" t="inlineStr">
+      <c r="Y74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA74" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB73" s="5" t="inlineStr">
+      <c r="AB74" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC73" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AD73" s="11" t="inlineStr">
+      <c r="AC74" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AD74" s="11" t="inlineStr">
         <is>
           <t>informes/pro-medicus-2026-10-12/Pro Medicus - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD73"/>
+  <autoFilter ref="A1:AD74"/>
   <hyperlinks>
     <hyperlink ref="AD2" r:id="rId1"/>
     <hyperlink ref="AD3" r:id="rId2"/>
@@ -9897,6 +10029,7 @@
     <hyperlink ref="AD71" r:id="rId70"/>
     <hyperlink ref="AD72" r:id="rId71"/>
     <hyperlink ref="AD73" r:id="rId72"/>
+    <hyperlink ref="AD74" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Informe de Paychex (Mantener, convicción baja)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento.xlsx
+++ b/seguimiento.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Criterios" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Seguimiento!$A$1:$AD$75</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -6660,25 +6660,25 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>ATOSS</t>
+          <t>Paychex</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>AOF</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="D50" s="10">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -6698,32 +6698,32 @@
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K50" s="2">
-        <v>87.3</v>
+        <v>103.98</v>
       </c>
       <c r="L50" s="2">
-        <v>80.89</v>
+        <v>97.19</v>
       </c>
       <c r="M50" s="2">
-        <v>94.95</v>
+        <v>111.76</v>
       </c>
       <c r="N50" s="3">
-        <v>-0.047</v>
+        <v>-0.022000000000000002</v>
       </c>
       <c r="O50" s="3">
-        <v>0.114</v>
+        <v>0.11800000000000001</v>
       </c>
       <c r="P50" s="2">
-        <v>120.78</v>
+        <v>113.93</v>
       </c>
       <c r="Q50" s="2">
-        <v>79.19</v>
+        <v>96.8</v>
       </c>
       <c r="R50" s="2">
-        <v>101.11</v>
+        <v>119.74</v>
       </c>
       <c r="S50" s="13" t="inlineStr">
         <is>
@@ -6750,9 +6750,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X50" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="X50" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Y50" s="4" t="inlineStr">
@@ -6775,14 +6775,14 @@
           <t>=</t>
         </is>
       </c>
-      <c r="AC50" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC50" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD50" s="11" t="inlineStr">
         <is>
-          <t>informes/atoss-2026-10-11/ATOSS Software - 2026-10-11.pdf</t>
+          <t>informes/paychex-2026-10-12/Paychex - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -6792,25 +6792,25 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>Indra</t>
+          <t>ATOSS</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>AOF</t>
         </is>
       </c>
       <c r="D51" s="10">
-        <v>46301</v>
+        <v>46306</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -6820,12 +6820,12 @@
       </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
@@ -6834,39 +6834,39 @@
         </is>
       </c>
       <c r="K51" s="2">
-        <v>59.72</v>
+        <v>87.3</v>
       </c>
       <c r="L51" s="2">
-        <v>58.59</v>
+        <v>80.89</v>
       </c>
       <c r="M51" s="2">
-        <v>66.22</v>
+        <v>94.95</v>
       </c>
       <c r="N51" s="3">
-        <v>-0.013999999999999999</v>
+        <v>-0.047</v>
       </c>
       <c r="O51" s="3">
         <v>0.114</v>
       </c>
       <c r="P51" s="2">
-        <v>67.12</v>
+        <v>120.78</v>
       </c>
       <c r="Q51" s="2">
-        <v>57.83</v>
+        <v>79.19</v>
       </c>
       <c r="R51" s="2">
-        <v>73.94</v>
+        <v>101.11</v>
       </c>
       <c r="S51" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T51" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T51" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U51" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6887,9 +6887,9 @@
           <t>=</t>
         </is>
       </c>
-      <c r="Y51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Z51" s="6" t="inlineStr">
@@ -6902,19 +6902,19 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AB51" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AC51" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AB51" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AC51" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD51" s="11" t="inlineStr">
         <is>
-          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
+          <t>informes/atoss-2026-10-11/ATOSS Software - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -6924,25 +6924,25 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Indra</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>4568</t>
+          <t>IDR</t>
         </is>
       </c>
       <c r="D52" s="10">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -6962,32 +6962,32 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K52" s="2">
-        <v>2702.5</v>
+        <v>59.72</v>
       </c>
       <c r="L52" s="2">
-        <v>2888.64</v>
+        <v>58.59</v>
       </c>
       <c r="M52" s="2">
-        <v>2897.35</v>
+        <v>66.22</v>
       </c>
       <c r="N52" s="3">
-        <v>0.098</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="O52" s="3">
-        <v>0.10099999999999999</v>
+        <v>0.114</v>
       </c>
       <c r="P52" s="2">
-        <v>4077.5</v>
+        <v>67.12</v>
       </c>
       <c r="Q52" s="2">
-        <v>2585.33</v>
+        <v>57.83</v>
       </c>
       <c r="R52" s="2">
-        <v>3307.49</v>
+        <v>73.94</v>
       </c>
       <c r="S52" s="13" t="inlineStr">
         <is>
@@ -7014,39 +7014,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X52" s="5" t="inlineStr">
+      <c r="X52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y52" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z52" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="AB52" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="AC52" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC52" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD52" s="11" t="inlineStr">
         <is>
-          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
+          <t>informes/indra-2026-10-06/Indra - 2026-10-06 v3.pdf</t>
         </is>
       </c>
     </row>
@@ -7056,25 +7056,25 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>4568</t>
         </is>
       </c>
       <c r="D53" s="10">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>Servicios de comunicación</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -7084,46 +7084,46 @@
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K53" s="2">
-        <v>70.3</v>
+        <v>2702.5</v>
       </c>
       <c r="L53" s="2">
-        <v>61.1</v>
+        <v>2888.64</v>
       </c>
       <c r="M53" s="2">
-        <v>73.49</v>
+        <v>2897.35</v>
       </c>
       <c r="N53" s="3">
-        <v>-0.131</v>
+        <v>0.098</v>
       </c>
       <c r="O53" s="3">
-        <v>0.045</v>
+        <v>0.10099999999999999</v>
       </c>
       <c r="P53" s="2">
-        <v>92.55</v>
+        <v>4077.5</v>
       </c>
       <c r="Q53" s="2">
-        <v>58.17</v>
+        <v>2585.33</v>
       </c>
       <c r="R53" s="2">
-        <v>81.69</v>
+        <v>3307.49</v>
       </c>
       <c r="S53" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T53" s="13" t="inlineStr">
@@ -7146,29 +7146,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z53" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA53" s="5" t="inlineStr">
+      <c r="X53" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB53" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y53" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z53" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AB53" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC53" s="4" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="AD53" s="11" t="inlineStr">
         <is>
-          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
+          <t>informes/daiichi-sankyo-2026-10-08/Daiichi Sankyo - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7188,16 +7188,16 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Copart</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D54" s="10">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>Industria</t>
+          <t>Servicios de comunicación</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
@@ -7216,12 +7216,12 @@
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
@@ -7230,39 +7230,39 @@
         </is>
       </c>
       <c r="K54" s="2">
-        <v>26.82</v>
+        <v>70.3</v>
       </c>
       <c r="L54" s="2">
-        <v>25.71</v>
+        <v>61.1</v>
       </c>
       <c r="M54" s="2">
-        <v>27.88</v>
+        <v>73.49</v>
       </c>
       <c r="N54" s="3">
-        <v>-0.040999999999999995</v>
+        <v>-0.131</v>
       </c>
       <c r="O54" s="3">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="P54" s="2">
-        <v>39</v>
+        <v>92.55</v>
       </c>
       <c r="Q54" s="2">
-        <v>24.22</v>
+        <v>58.17</v>
       </c>
       <c r="R54" s="2">
-        <v>30.98</v>
+        <v>81.69</v>
       </c>
       <c r="S54" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T54" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T54" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7278,9 +7278,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="X54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="Y54" s="4" t="inlineStr">
@@ -7288,19 +7288,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z54" s="5" t="inlineStr">
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA54" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AA54" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AB54" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AB54" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC54" s="4" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="AD54" s="11" t="inlineStr">
         <is>
-          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
+          <t>informes/netflix-2026-10-11/Netflix - 2026-10-11.pdf</t>
         </is>
       </c>
     </row>
@@ -7320,12 +7320,12 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Rational</t>
+          <t>Copart</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>RAA</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="D55" s="10">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F55" s="0" t="inlineStr">
@@ -7353,41 +7353,41 @@
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K55" s="2">
-        <v>577.5</v>
+        <v>26.82</v>
       </c>
       <c r="L55" s="2">
-        <v>466.62</v>
+        <v>25.71</v>
       </c>
       <c r="M55" s="2">
-        <v>564.55</v>
+        <v>27.88</v>
       </c>
       <c r="N55" s="3">
-        <v>-0.16399999999999998</v>
+        <v>-0.040999999999999995</v>
       </c>
       <c r="O55" s="3">
-        <v>0.005</v>
+        <v>0.04</v>
       </c>
       <c r="P55" s="2">
-        <v>795.86</v>
+        <v>39</v>
       </c>
       <c r="Q55" s="2">
-        <v>504.42</v>
+        <v>24.22</v>
       </c>
       <c r="R55" s="2">
-        <v>645.34</v>
+        <v>30.98</v>
       </c>
       <c r="S55" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T55" s="13" t="inlineStr">
@@ -7395,9 +7395,9 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="V55" s="4" t="inlineStr">
@@ -7410,29 +7410,29 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Z55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA55" s="5" t="inlineStr">
+      <c r="X55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Y55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z55" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB55" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AA55" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB55" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AC55" s="4" t="inlineStr">
@@ -7442,7 +7442,7 @@
       </c>
       <c r="AD55" s="11" t="inlineStr">
         <is>
-          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
+          <t>informes/copart-2026-10-07/Copart - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7452,25 +7452,25 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>Rational</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>SPGI</t>
+          <t>RAA</t>
         </is>
       </c>
       <c r="D56" s="10">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>Finanzas</t>
+          <t>Industria</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
@@ -7480,42 +7480,42 @@
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K56" s="2">
-        <v>407.82</v>
+        <v>577.5</v>
       </c>
       <c r="L56" s="2">
-        <v>351.69</v>
+        <v>466.62</v>
       </c>
       <c r="M56" s="2">
-        <v>398.1</v>
+        <v>564.55</v>
       </c>
       <c r="N56" s="3">
-        <v>-0.128</v>
+        <v>-0.16399999999999998</v>
       </c>
       <c r="O56" s="3">
-        <v>-0.013999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="P56" s="2">
-        <v>516.86</v>
+        <v>795.86</v>
       </c>
       <c r="Q56" s="2">
-        <v>338.33</v>
+        <v>504.42</v>
       </c>
       <c r="R56" s="2">
-        <v>446.65</v>
+        <v>645.34</v>
       </c>
       <c r="S56" s="13" t="inlineStr">
         <is>
@@ -7527,44 +7527,44 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V56" s="5" t="inlineStr">
+      <c r="U56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W56" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Z56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="X56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="Y56" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z56" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA56" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB56" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="AB56" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AC56" s="4" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="AD56" s="11" t="inlineStr">
         <is>
-          <t>informes/sp-global-2026-10-12/S&amp;P Global - 2026-10-12.pdf</t>
+          <t>informes/rational-2026-10-07/Rational - 2026-10-07.pdf</t>
         </is>
       </c>
     </row>
@@ -7584,25 +7584,25 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>7733</t>
+          <t>SPGI</t>
         </is>
       </c>
       <c r="D57" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Japón</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -7612,61 +7612,61 @@
       </c>
       <c r="H57" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K57" s="2">
-        <v>2000</v>
+        <v>407.82</v>
       </c>
       <c r="L57" s="2">
-        <v>1932.11</v>
+        <v>351.69</v>
       </c>
       <c r="M57" s="2">
-        <v>1939.91</v>
+        <v>398.1</v>
       </c>
       <c r="N57" s="3">
-        <v>-0.019</v>
+        <v>-0.128</v>
       </c>
       <c r="O57" s="3">
-        <v>-0.015</v>
+        <v>-0.013999999999999999</v>
       </c>
       <c r="P57" s="2">
-        <v>2184.62</v>
+        <v>516.86</v>
       </c>
       <c r="Q57" s="2">
-        <v>1711.85</v>
+        <v>338.33</v>
       </c>
       <c r="R57" s="2">
-        <v>2020.99</v>
+        <v>446.65</v>
       </c>
       <c r="S57" s="13" t="inlineStr">
         <is>
+          <t>Vender</t>
+        </is>
+      </c>
+      <c r="T57" s="13" t="inlineStr">
+        <is>
           <t>Mantener</t>
         </is>
       </c>
-      <c r="T57" s="13" t="inlineStr">
-        <is>
-          <t>Mantener</t>
-        </is>
-      </c>
-      <c r="U57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="V57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V57" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="W57" s="4" t="inlineStr">
@@ -7674,39 +7674,39 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="X57" s="5" t="inlineStr">
+      <c r="X57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z57" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="Y57" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="AA57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
       <c r="AB57" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AC57" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="AC57" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AD57" s="11" t="inlineStr">
         <is>
-          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
+          <t>informes/sp-global-2026-10-12/S&amp;P Global - 2026-10-12.pdf</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7716,25 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>7733</t>
         </is>
       </c>
       <c r="D58" s="10">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Japón</t>
         </is>
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>Tecnologías de la información</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -7744,46 +7744,46 @@
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="K58" s="2">
-        <v>529.76</v>
+        <v>2000</v>
       </c>
       <c r="L58" s="2">
-        <v>450.46</v>
+        <v>1932.11</v>
       </c>
       <c r="M58" s="2">
-        <v>511.38</v>
+        <v>1939.91</v>
       </c>
       <c r="N58" s="3">
-        <v>-0.14300000000000002</v>
+        <v>-0.019</v>
       </c>
       <c r="O58" s="3">
-        <v>-0.027999999999999997</v>
+        <v>-0.015</v>
       </c>
       <c r="P58" s="2">
-        <v>587.63</v>
+        <v>2184.62</v>
       </c>
       <c r="Q58" s="2">
-        <v>447.76</v>
+        <v>1711.85</v>
       </c>
       <c r="R58" s="2">
-        <v>568.48</v>
+        <v>2020.99</v>
       </c>
       <c r="S58" s="13" t="inlineStr">
         <is>
-          <t>Vender</t>
+          <t>Mantener</t>
         </is>
       </c>
       <c r="T58" s="13" t="inlineStr">
@@ -7791,14 +7791,14 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="V58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="W58" s="4" t="inlineStr">
@@ -7816,21 +7816,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Z58" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA58" s="5" t="inlineStr">
+      <c r="Z58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AA58" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="AB58" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="AB58" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC58" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="AD58" s="11" t="inlineStr">
         <is>
-          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
+          <t>informes/olympus-2026-10-09/Olympus - 2026-10-09.pdf</t>
         </is>
       </c>
     </row>
@@ -7848,25 +7848,25 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Enagás</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D59" s="10">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Tecnologías de la información</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
@@ -7886,32 +7886,32 @@
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K59" s="2">
-        <v>16.22</v>
+        <v>529.76</v>
       </c>
       <c r="L59" s="2">
-        <v>13.97</v>
+        <v>450.46</v>
       </c>
       <c r="M59" s="2">
-        <v>14.66</v>
+        <v>511.38</v>
       </c>
       <c r="N59" s="3">
-        <v>-0.077</v>
+        <v>-0.14300000000000002</v>
       </c>
       <c r="O59" s="3">
-        <v>-0.035</v>
+        <v>-0.027999999999999997</v>
       </c>
       <c r="P59" s="2">
-        <v>17.05</v>
+        <v>587.63</v>
       </c>
       <c r="Q59" s="2">
-        <v>13.61</v>
+        <v>447.76</v>
       </c>
       <c r="R59" s="2">
-        <v>16.41</v>
+        <v>568.48</v>
       </c>
       <c r="S59" s="13" t="inlineStr">
         <is>
@@ -7923,46 +7923,46 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U59" s="5" t="inlineStr">
+      <c r="U59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="V59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="W59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="X59" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="V59" s="5" t="inlineStr">
+      <c r="Y59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="Z59" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="AA59" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="W59" s="5" t="inlineStr">
+      <c r="AB59" s="5" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="X59" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Y59" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="Z59" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="AA59" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="AB59" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="AC59" s="6" t="inlineStr">
         <is>
           <t>=</t>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="AD59" s="11" t="inlineStr">
         <is>
-          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
+          <t>informes/microsoft-2026-10-08/Microsoft - 2026-10-08.pdf</t>
         </is>
       </c>
     </row>
@@ -7980,25 +7980,25 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Enagás</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="D60" s="10">
-        <v>46307</v>
+        <v>46302</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>Consumo discrecional</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
@@ -8018,32 +8018,32 @@
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="K60" s="2">
-        <v>262.43</v>
+        <v>16.22</v>
       </c>
       <c r="L60" s="2">
-        <v>213.96</v>
+        <v>13.97</v>
       </c>
       <c r="M60" s="2">
-        <v>251.97</v>
+        <v>14.66</v>
       </c>
       <c r="N60" s="3">
-        <v>-0.185</v>
+        <v>-0.077</v>
       </c>
       <c r="O60" s="3">
-        <v>-0.04</v>
+        <v>-0.035</v>
       </c>
       <c r="P60" s="2">
-        <v>331.36</v>
+        <v>17.05</v>
       </c>
       <c r="Q60" s="2">
-        <v>203.69</v>
+        <v>13.61</v>
       </c>
       <c r="R60" s="2">
-        <v>271.09</v>
+        <v>16.41</v>
       </c>
       <c r="S60" s="13" t="inlineStr">
         <is>
@@ -8055,19 +8055,19 @@
           <t>Mantener</t>
         </is>
       </c>
-      <c r="U60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="V60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="W60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="U60" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="V60" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="W60" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="X60" s="5" t="inlineStr">
@@ -8075,14 +8075,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="Y60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Z60" s="6" t="inlineStr">
-        <is>
-          <t>=</t>
+      <c r="Y60" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="Z60" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="AA60" s="5" t="inlineStr">
@@ -8095,14 +8095,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="AC60" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="AC60" s="6" t="inlineStr">
+        <is>
+          <t>=</t>
         </is>
       </c>
       <c r="AD60" s="11" t="inlineStr">
         <is>
-          <t>informes/amazon-2026-10-12/Amazon - 2026-10-12.pdf</t>
+          <t>informes/enagas-2026-10-07/Enagás - 2026-10-07 v2.pdf</t>
         </is>
       </c>
     </row>
@@ -8112,25 +8112,25 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D61" s="10">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Consumo discrecional</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -8154,28 +8154,28 @@
         </is>
       </c>
       <c r="K61" s="2">
-        <v>128.3</v>
+        <v>262.43</v>
       </c>
       <c r="L61" s="2">
-        <v>99</v>
+        <v>213.96</v>
       </c>
       <c r="M61" s="2">
-        <v>117</v>
+        <v>251.97</v>
       </c>
       <c r="N61" s="3">
-        <v>-0.20600000000000002</v>
+        <v>-0.185</v>
       </c>
       <c r="O61" s="3">
-        <v